<commit_message>
Use PCD formula Q = 1.38 H^2.5 in workbook with ISO 1438 comparison
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXLmoKkgGBxM2QbbegGKn7
</commit_message>
<xml_diff>
--- a/weir_design.xlsx
+++ b/weir_design.xlsx
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="143">
   <si>
     <t xml:space="preserve">1) ข้อมูลออกแบบ — บ่อ 3 ช่อง: ปั๊มจุ่ม | โชว์น้ำใส | V-notch 90°</t>
   </si>
@@ -174,19 +174,25 @@
     <t xml:space="preserve">m/s²</t>
   </si>
   <si>
+    <t xml:space="preserve">ค่าคงที่ V-notch 90° กรมควบคุมมลพิษ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">สูตรหลัก: Q = 1.38 × H^2.5 (Thomson)</t>
+  </si>
+  <si>
     <t xml:space="preserve">สัมประสิทธิ์อัตราไหล V-notch 90° (Ce)</t>
   </si>
   <si>
-    <t xml:space="preserve">-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ISO 1438 / USBR, สมการ Kindsvater–Shen</t>
+    <t xml:space="preserve">ใช้เทียบ: ISO 1438 (Kindsvater–Shen)</t>
   </si>
   <si>
     <t xml:space="preserve">ค่าปรับความสูงน้ำ V-notch 90° (kh)</t>
   </si>
   <si>
-    <t xml:space="preserve">ISO 1438 / USBR</t>
+    <t xml:space="preserve">ใช้เทียบ: ISO 1438</t>
   </si>
   <si>
     <t xml:space="preserve">สัมประสิทธิ์สันปลายตรง (Francis)</t>
@@ -225,22 +231,28 @@
     <t xml:space="preserve">สูตรคำนวณ ห้ามพิมพ์ทับ</t>
   </si>
   <si>
-    <t xml:space="preserve">2) เวียร์ V-notch 90° — หาความสูงน้ำ h จากอัตราการไหล</t>
-  </si>
-  <si>
-    <t xml:space="preserve">สูตร ISO 1438:  Q = Ce × (8/15) × √(2g) × (h + kh)^2.5   →   h = (Q ÷ K)^0.4 − kh   โดย K = Ce × (8/15) × √(2g)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ขั้นที่ 1  หาค่าคงที่ K</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K = Ce × (8/15) × √(2g)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">≈ 1.365 สำหรับ V-notch 90°</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ขั้นที่ 2  แปลงอัตราการไหล แล้วหา h</t>
+    <t xml:space="preserve">2) เวียร์ V-notch 90° — หาความสูงน้ำ H จากอัตราการไหล</t>
+  </si>
+  <si>
+    <t xml:space="preserve">สูตรหลัก (กรมควบคุมมลพิษ): Q = 1.38 × H^2.5  →  H = (Q ÷ 1.38)^0.4     |     สูตรเทียบ (ISO 1438): Q = K × (H + kh)^2.5  →  H = (Q ÷ K)^0.4 − kh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ขั้นที่ 1  ค่าคงที่ของแต่ละสูตร</t>
+  </si>
+  <si>
+    <t xml:space="preserve">สูตรกรมควบคุมมลพิษ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ค่าคงที่ตายตัว</t>
+  </si>
+  <si>
+    <t xml:space="preserve">สูตร ISO: K = Ce × (8/15) × √(2g)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≈ 1.365 และบวก kh ที่ H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ขั้นที่ 2  แปลงอัตราการไหล แล้วหา H ทั้ง 2 สูตร</t>
   </si>
   <si>
     <t xml:space="preserve">กรณี</t>
@@ -255,18 +267,24 @@
 = ÷3600</t>
   </si>
   <si>
-    <t xml:space="preserve">h
-(m)
+    <t xml:space="preserve">H กรมฯ
+(cm)
+= (Q÷1.38)^0.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H ISO
+(cm)
 = (Q÷K)^0.4 − kh</t>
   </si>
   <si>
-    <t xml:space="preserve">h
-(cm)</t>
+    <t xml:space="preserve">ต่างกัน
+(cm)
+= กรมฯ − ISO</t>
   </si>
   <si>
     <t xml:space="preserve">ระดับน้ำ ช่อง 3
 (m จากพื้น)
-= P + h</t>
+= P + H กรมฯ</t>
   </si>
   <si>
     <t xml:space="preserve">น้ำเข้าต่ำสุด ปั๊มเดิน</t>
@@ -281,7 +299,7 @@
     <t xml:space="preserve">น้ำเข้าสูงสุด ปั๊มหยุด (ใช้ออกแบบ)</t>
   </si>
   <si>
-    <t xml:space="preserve">ขั้นที่ 3  ตรวจสอบเกณฑ์ (ใช้ hmax = กรณีสุดท้าย)</t>
+    <t xml:space="preserve">ขั้นที่ 3  ตรวจสอบเกณฑ์ ISO 1438 (ใช้ H กรมฯ, hmax = กรณีสุดท้าย)</t>
   </si>
   <si>
     <t xml:space="preserve">รายการตรวจ</t>
@@ -296,25 +314,25 @@
     <t xml:space="preserve">ผล</t>
   </si>
   <si>
-    <t xml:space="preserve">h ต่ำสุด ≥ 0.05 m (ต่ำกว่านี้วัดไม่แม่น)</t>
+    <t xml:space="preserve">H ต่ำสุด ≥ 0.05 m (ต่ำกว่านี้วัดไม่แม่น)</t>
   </si>
   <si>
     <t xml:space="preserve">≥ 0.05 m</t>
   </si>
   <si>
-    <t xml:space="preserve">hmax ≤ 0.38 m</t>
+    <t xml:space="preserve">Hmax ≤ 0.38 m</t>
   </si>
   <si>
     <t xml:space="preserve">≤ 0.38 m</t>
   </si>
   <si>
-    <t xml:space="preserve">h / P</t>
+    <t xml:space="preserve">H / P</t>
   </si>
   <si>
     <t xml:space="preserve">≤ 0.4</t>
   </si>
   <si>
-    <t xml:space="preserve">h / B</t>
+    <t xml:space="preserve">H / B</t>
   </si>
   <si>
     <t xml:space="preserve">≤ 0.2</t>
@@ -332,22 +350,34 @@
     <t xml:space="preserve">≥ 0.90 m</t>
   </si>
   <si>
-    <t xml:space="preserve">ร่อง V ลึกกว่า hmax อย่างน้อย (m)</t>
+    <t xml:space="preserve">ร่อง V ลึกกว่า Hmax อย่างน้อย (m)</t>
   </si>
   <si>
     <t xml:space="preserve">≥ 0.08 m</t>
   </si>
   <si>
-    <t xml:space="preserve">ช่วงตรงหน้าเวียร์ ÷ hmax</t>
+    <t xml:space="preserve">ช่วงตรงหน้าเวียร์ ÷ Hmax</t>
   </si>
   <si>
     <t xml:space="preserve">≥ 10 เท่า</t>
   </si>
   <si>
-    <t xml:space="preserve">ระยะจุดวัด h ÷ hmax</t>
+    <t xml:space="preserve">ระยะจุดวัด H ÷ Hmax</t>
   </si>
   <si>
     <t xml:space="preserve">4–5 เท่า</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ทำไม 2 สูตรต่างกัน</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• ทั้งคู่มาจาก Q = Cd × (8/15) × √(2g) × H^2.5 ต่างกันที่ Cd: กรมฯ 0.584 (→ 1.38) / ISO 0.578 (→ 1.365)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• ISO บวก kh = 0.85 mm ที่ H เพื่อชดเชยแรงตึงผิวตอนน้ำตื้น จึงต่างกันมากเฉพาะ H &lt; 10 cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• ช่วงใช้งานบ่อนี้ (H 14–21 cm) ต่างกันไม่ถึง 0.5% — รายงานราชการให้ใช้สูตรกรมฯ</t>
   </si>
   <si>
     <t xml:space="preserve">3) ช่อง 2 โชว์น้ำใส — ชั้นน้ำบนพื้นยกหนาเท่าไร</t>
@@ -441,7 +471,7 @@
     <t xml:space="preserve">น้ำ ช่อง 3 สูงสุด</t>
   </si>
   <si>
-    <t xml:space="preserve">P + hmax</t>
+    <t xml:space="preserve">P + Hmax (สูตรกรมฯ)</t>
   </si>
   <si>
     <t xml:space="preserve">ยอด V (h = 0)</t>
@@ -465,29 +495,41 @@
     <t xml:space="preserve">สันกำแพงสูงกว่าน้ำช่อง 1 (m)</t>
   </si>
   <si>
-    <t xml:space="preserve">5) ตาราง h → Q สำหรับอ่านค่าหน้างาน</t>
-  </si>
-  <si>
-    <t xml:space="preserve">วัด h จากยอด V (cm) แล้วอ่าน Q   |   Q = K × (h + kh)^2.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">h (cm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Q (m³/h)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Q (L/s)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Q (m³/วัน)</t>
+    <t xml:space="preserve">5) ตาราง H → Q สำหรับอ่านค่าหน้างาน</t>
+  </si>
+  <si>
+    <t xml:space="preserve">วัด H จากยอด V (cm) แล้วอ่าน Q   |   กรมฯ: Q = 1.38 × H^2.5   |   ISO: Q = K × (H + kh)^2.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H (cm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q กรมฯ
+(m³/h)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q ISO
+(m³/h)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ต่างกัน
+(%)
+= กรมฯ ÷ ISO − 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q กรมฯ
+(L/s)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q กรมฯ
+(m³/วัน)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="11">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="0.00"/>
@@ -495,8 +537,10 @@
     <numFmt numFmtId="168" formatCode="0.000"/>
     <numFmt numFmtId="169" formatCode="0.00000"/>
     <numFmt numFmtId="170" formatCode="0.0000"/>
-    <numFmt numFmtId="171" formatCode="\+0.000;\-0.000;\±0.000"/>
-    <numFmt numFmtId="172" formatCode="0"/>
+    <numFmt numFmtId="171" formatCode="\+0.00;\-0.00;0.00"/>
+    <numFmt numFmtId="172" formatCode="\+0.000;\-0.000;\±0.000"/>
+    <numFmt numFmtId="173" formatCode="0"/>
+    <numFmt numFmtId="174" formatCode="\+0.0%;\-0.0%;0.0%"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -680,7 +724,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -745,8 +789,16 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="171" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -757,11 +809,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="172" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="173" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="174" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1021,7 +1077,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:E27"/>
+  <dimension ref="B1:E28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -1249,7 +1305,7 @@
         <v>34</v>
       </c>
       <c r="C20" s="10" t="n">
-        <v>0.578</v>
+        <v>1.38</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>35</v>
@@ -1262,11 +1318,11 @@
       <c r="B21" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C21" s="11" t="n">
-        <v>0.00085</v>
+      <c r="C21" s="10" t="n">
+        <v>0.578</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>38</v>
@@ -1276,58 +1332,72 @@
       <c r="B22" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C22" s="10" t="n">
-        <v>1.84</v>
+      <c r="C22" s="11" t="n">
+        <v>0.00085</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="E22" s="4" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="8" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
+      <c r="C23" s="10" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C25" s="12" t="s">
+      <c r="B25" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="D25" s="4"/>
-      <c r="E25" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C26" s="12" t="s">
         <v>45</v>
-      </c>
-      <c r="C26" s="13" t="s">
-        <v>46</v>
       </c>
       <c r="D26" s="4"/>
       <c r="E26" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C27" s="13" t="s">
         <v>48</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>49</v>
       </c>
       <c r="D27" s="4"/>
       <c r="E27" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="4" t="s">
         <v>50</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1347,223 +1417,263 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:G25"/>
+  <dimension ref="B1:H30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="40"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C4" s="9"/>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
       <c r="F4" s="9"/>
       <c r="G4" s="9"/>
-    </row>
-    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H4" s="9"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C5" s="14" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$20*(8/15)*SQRT(2*'1 ข้อมูล'!$C$19)</f>
-        <v>1.36545083661038</v>
+        <v>56</v>
+      </c>
+      <c r="C5" s="10" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$20</f>
+        <v>1.38</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>35</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-    </row>
-    <row r="8" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C8" s="3" t="s">
+      <c r="H5" s="4"/>
+    </row>
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="C6" s="14" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$21*(8/15)*SQRT(2*'1 ข้อมูล'!$C$19)</f>
+        <v>1.36545083661038</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="4"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+    </row>
+    <row r="9" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="4" t="s">
+      <c r="D9" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="E9" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C10" s="7" t="n">
         <f aca="false">'1 ข้อมูล'!$C$6-'1 ข้อมูล'!$C$8</f>
         <v>40</v>
       </c>
-      <c r="D9" s="11" t="n">
-        <f aca="false">C9/3600</f>
+      <c r="D10" s="11" t="n">
+        <f aca="false">C10/3600</f>
         <v>0.0111111111111111</v>
       </c>
-      <c r="E9" s="14" t="n">
-        <f aca="false">(D9/'2 เวียร์'!$C$5)^0.4-'1 ข้อมูล'!$C$21</f>
-        <v>0.145096125168743</v>
-      </c>
-      <c r="F9" s="15" t="n">
-        <f aca="false">E9*100</f>
+      <c r="E10" s="15" t="n">
+        <f aca="false">(D10/'2 เวียร์'!$C$5)^0.4*100</f>
+        <v>14.532869095236</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <f aca="false">((D10/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$22)*100</f>
         <v>14.5096125168743</v>
       </c>
-      <c r="G9" s="10" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$10+E9</f>
-        <v>0.745096125168743</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="C10" s="7" t="n">
+      <c r="G10" s="16" t="n">
+        <f aca="false">E10-F10</f>
+        <v>0.0232565783616678</v>
+      </c>
+      <c r="H10" s="17" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$10+E10/100</f>
+        <v>0.74532869095236</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C11" s="7" t="n">
         <f aca="false">'1 ข้อมูล'!$C$16-'1 ข้อมูล'!$C$8</f>
         <v>52.7916666666667</v>
       </c>
-      <c r="D10" s="11" t="n">
-        <f aca="false">C10/3600</f>
+      <c r="D11" s="11" t="n">
+        <f aca="false">C11/3600</f>
         <v>0.0146643518518519</v>
       </c>
-      <c r="E10" s="14" t="n">
-        <f aca="false">(D10/'2 เวียร์'!$C$5)^0.4-'1 ข้อมูล'!$C$21</f>
-        <v>0.162227754127948</v>
-      </c>
-      <c r="F10" s="15" t="n">
-        <f aca="false">E10*100</f>
+      <c r="E11" s="15" t="n">
+        <f aca="false">(D11/'2 เวียร์'!$C$5)^0.4*100</f>
+        <v>16.2387843483091</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <f aca="false">((D11/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$22)*100</f>
         <v>16.2227754127948</v>
       </c>
-      <c r="G10" s="10" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$10+E10</f>
-        <v>0.762227754127948</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="C11" s="7" t="n">
+      <c r="G11" s="16" t="n">
+        <f aca="false">E11-F11</f>
+        <v>0.0160089355143072</v>
+      </c>
+      <c r="H11" s="17" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$10+E11/100</f>
+        <v>0.762387843483091</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C12" s="7" t="n">
         <f aca="false">'1 ข้อมูล'!$C$7-'1 ข้อมูล'!$C$8</f>
         <v>90</v>
       </c>
-      <c r="D11" s="11" t="n">
-        <f aca="false">C11/3600</f>
+      <c r="D12" s="11" t="n">
+        <f aca="false">C12/3600</f>
         <v>0.025</v>
       </c>
-      <c r="E11" s="14" t="n">
-        <f aca="false">(D11/'2 เวียร์'!$C$5)^0.4-'1 ข้อมูล'!$C$21</f>
-        <v>0.201017115002301</v>
-      </c>
-      <c r="F11" s="15" t="n">
-        <f aca="false">E11*100</f>
+      <c r="E12" s="15" t="n">
+        <f aca="false">(D12/'2 เวียร์'!$C$5)^0.4*100</f>
+        <v>20.1013103538681</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <f aca="false">((D12/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$22)*100</f>
         <v>20.1017115002301</v>
       </c>
-      <c r="G11" s="10" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$10+E11</f>
-        <v>0.801017115002301</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="C12" s="7" t="n">
+      <c r="G12" s="16" t="n">
+        <f aca="false">E12-F12</f>
+        <v>-0.000401146361987514</v>
+      </c>
+      <c r="H12" s="17" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$10+E12/100</f>
+        <v>0.801013103538681</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="C13" s="7" t="n">
         <f aca="false">'1 ข้อมูล'!$C$7</f>
         <v>100</v>
       </c>
-      <c r="D12" s="11" t="n">
-        <f aca="false">C12/3600</f>
+      <c r="D13" s="11" t="n">
+        <f aca="false">C13/3600</f>
         <v>0.0277777777777778</v>
       </c>
-      <c r="E12" s="14" t="n">
-        <f aca="false">(D12/'2 เวียร์'!$C$5)^0.4-'1 ข้อมูล'!$C$21</f>
-        <v>0.209706461048468</v>
-      </c>
-      <c r="F12" s="15" t="n">
-        <f aca="false">E12*100</f>
+      <c r="E13" s="15" t="n">
+        <f aca="false">(D13/'2 เวียร์'!$C$5)^0.4*100</f>
+        <v>20.9665688762588</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <f aca="false">((D13/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$22)*100</f>
         <v>20.9706461048468</v>
       </c>
-      <c r="G12" s="10" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$10+E12</f>
-        <v>0.809706461048468</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="16"/>
+      <c r="G13" s="16" t="n">
+        <f aca="false">E13-F13</f>
+        <v>-0.00407722858800952</v>
+      </c>
+      <c r="H13" s="17" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$10+E13/100</f>
+        <v>0.809665688762588</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="8" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C15" s="9"/>
       <c r="D15" s="9"/>
       <c r="E15" s="9"/>
       <c r="F15" s="9"/>
       <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="3" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="4" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="D17" s="10" t="n">
-        <f aca="false">E9</f>
-        <v>0.145096125168743</v>
+        <f aca="false">E10/100</f>
+        <v>0.14532869095236</v>
       </c>
       <c r="E17" s="13" t="str">
         <f aca="false">IF(D17&gt;=0.05,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
@@ -1571,17 +1681,18 @@
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="4" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D18" s="10" t="n">
-        <f aca="false">E12</f>
-        <v>0.209706461048468</v>
+        <f aca="false">E13/100</f>
+        <v>0.209665688762588</v>
       </c>
       <c r="E18" s="13" t="str">
         <f aca="false">IF(D18&lt;=0.38,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
@@ -1589,17 +1700,18 @@
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="D19" s="17" t="n">
-        <f aca="false">E12/'1 ข้อมูล'!$C$10</f>
-        <v>0.349510768414113</v>
+        <v>82</v>
+      </c>
+      <c r="D19" s="19" t="n">
+        <f aca="false">E13/100/'1 ข้อมูล'!$C$10</f>
+        <v>0.349442814604313</v>
       </c>
       <c r="E19" s="13" t="str">
         <f aca="false">IF(D19&lt;=0.4,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
@@ -1607,17 +1719,18 @@
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="4" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="D20" s="17" t="n">
-        <f aca="false">E12/'1 ข้อมูล'!$C$9</f>
-        <v>0.174755384207057</v>
+        <v>84</v>
+      </c>
+      <c r="D20" s="19" t="n">
+        <f aca="false">E13/100/'1 ข้อมูล'!$C$9</f>
+        <v>0.174721407302157</v>
       </c>
       <c r="E20" s="13" t="str">
         <f aca="false">IF(D20&lt;=0.2,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
@@ -1625,15 +1738,16 @@
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="4" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="D21" s="17" t="n">
+        <v>86</v>
+      </c>
+      <c r="D21" s="19" t="n">
         <f aca="false">'1 ข้อมูล'!$C$10</f>
         <v>0.6</v>
       </c>
@@ -1643,15 +1757,16 @@
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="4" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="D22" s="17" t="n">
+        <v>88</v>
+      </c>
+      <c r="D22" s="19" t="n">
         <f aca="false">'1 ข้อมูล'!$C$9</f>
         <v>1.2</v>
       </c>
@@ -1661,17 +1776,18 @@
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
+      <c r="H22" s="4"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="4" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D23" s="10" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$11-E12</f>
-        <v>0.0902935389515321</v>
+        <f aca="false">'1 ข้อมูล'!$C$11-E13/100</f>
+        <v>0.0903343112374122</v>
       </c>
       <c r="E23" s="13" t="str">
         <f aca="false">IF(D23&gt;=0.08,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
@@ -1679,17 +1795,18 @@
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
+      <c r="H23" s="4"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="4" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="D24" s="7" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$12/E12</f>
-        <v>10.4908546403419</v>
+        <f aca="false">'1 ข้อมูล'!$C$12/(E13/100)</f>
+        <v>10.4928947267626</v>
       </c>
       <c r="E24" s="13" t="str">
         <f aca="false">IF(D24&gt;=10,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
@@ -1697,17 +1814,18 @@
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
+      <c r="H24" s="4"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="4" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="D25" s="7" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$13/E12</f>
-        <v>4.76857029106451</v>
+        <f aca="false">'1 ข้อมูล'!$C$13/(E13/100)</f>
+        <v>4.7694976030739</v>
       </c>
       <c r="E25" s="13" t="str">
         <f aca="false">IF(AND(D25&gt;=4,D25&lt;=5),"ผ่าน ✔","ไม่ผ่าน ✘")</f>
@@ -1715,6 +1833,33 @@
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="9"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="20" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="20" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="20" t="s">
+        <v>98</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1748,43 +1893,43 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="4" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C5" s="7" t="n">
         <f aca="false">'1 ข้อมูล'!$C$6-'1 ข้อมูล'!$C$8</f>
@@ -1795,18 +1940,18 @@
         <v>0.0111111111111111</v>
       </c>
       <c r="E5" s="7" t="n">
-        <f aca="false">(D5/('1 ข้อมูล'!$C$22*'1 ข้อมูล'!$C$9))^(2/3)*100</f>
+        <f aca="false">(D5/('1 ข้อมูล'!$C$23*'1 ข้อมูล'!$C$9))^(2/3)*100</f>
         <v>2.93656046563664</v>
       </c>
       <c r="F5" s="15" t="n">
         <f aca="false">'1 ข้อมูล'!$C$15*100+E5</f>
         <v>4.93656046563664</v>
       </c>
-      <c r="G5" s="17" t="n">
+      <c r="G5" s="19" t="n">
         <f aca="false">D5/('1 ข้อมูล'!$C$9*F5/100)</f>
         <v>0.187564992340576</v>
       </c>
-      <c r="H5" s="17" t="n">
+      <c r="H5" s="19" t="n">
         <f aca="false">G5/SQRT('1 ข้อมูล'!$C$19*F5/100)</f>
         <v>0.269528720442653</v>
       </c>
@@ -1817,7 +1962,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="4" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="C6" s="7" t="n">
         <f aca="false">'1 ข้อมูล'!$C$16-'1 ข้อมูล'!$C$8</f>
@@ -1828,18 +1973,18 @@
         <v>0.0146643518518519</v>
       </c>
       <c r="E6" s="7" t="n">
-        <f aca="false">(D6/('1 ข้อมูล'!$C$22*'1 ข้อมูล'!$C$9))^(2/3)*100</f>
+        <f aca="false">(D6/('1 ข้อมูล'!$C$23*'1 ข้อมูล'!$C$9))^(2/3)*100</f>
         <v>3.53326221375287</v>
       </c>
       <c r="F6" s="15" t="n">
         <f aca="false">'1 ข้อมูล'!$C$15*100+E6</f>
         <v>5.53326221375287</v>
       </c>
-      <c r="G6" s="17" t="n">
+      <c r="G6" s="19" t="n">
         <f aca="false">D6/('1 ข้อมูล'!$C$9*F6/100)</f>
         <v>0.220851511058036</v>
       </c>
-      <c r="H6" s="17" t="n">
+      <c r="H6" s="19" t="n">
         <f aca="false">G6/SQRT('1 ข้อมูล'!$C$19*F6/100)</f>
         <v>0.29976108061034</v>
       </c>
@@ -1850,7 +1995,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="4" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C7" s="7" t="n">
         <f aca="false">'1 ข้อมูล'!$C$7-'1 ข้อมูล'!$C$8</f>
@@ -1861,18 +2006,18 @@
         <v>0.025</v>
       </c>
       <c r="E7" s="7" t="n">
-        <f aca="false">(D7/('1 ข้อมูล'!$C$22*'1 ข้อมูล'!$C$9))^(2/3)*100</f>
+        <f aca="false">(D7/('1 ข้อมูล'!$C$23*'1 ข้อมูล'!$C$9))^(2/3)*100</f>
         <v>5.04228388369996</v>
       </c>
       <c r="F7" s="15" t="n">
         <f aca="false">'1 ข้อมูล'!$C$15*100+E7</f>
         <v>7.04228388369996</v>
       </c>
-      <c r="G7" s="17" t="n">
+      <c r="G7" s="19" t="n">
         <f aca="false">D7/('1 ข้อมูล'!$C$9*F7/100)</f>
         <v>0.295832057857737</v>
       </c>
-      <c r="H7" s="17" t="n">
+      <c r="H7" s="19" t="n">
         <f aca="false">G7/SQRT('1 ข้อมูล'!$C$19*F7/100)</f>
         <v>0.35592129002886</v>
       </c>
@@ -1883,7 +2028,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="4" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C8" s="7" t="n">
         <f aca="false">'1 ข้อมูล'!$C$7</f>
@@ -1894,18 +2039,18 @@
         <v>0.0277777777777778</v>
       </c>
       <c r="E8" s="7" t="n">
-        <f aca="false">(D8/('1 ข้อมูล'!$C$22*'1 ข้อมูล'!$C$9))^(2/3)*100</f>
+        <f aca="false">(D8/('1 ข้อมูล'!$C$23*'1 ข้อมูล'!$C$9))^(2/3)*100</f>
         <v>5.40919062653374</v>
       </c>
       <c r="F8" s="15" t="n">
         <f aca="false">'1 ข้อมูล'!$C$15*100+E8</f>
         <v>7.40919062653374</v>
       </c>
-      <c r="G8" s="17" t="n">
+      <c r="G8" s="19" t="n">
         <f aca="false">D8/('1 ข้อมูล'!$C$9*F8/100)</f>
         <v>0.312424788549105</v>
       </c>
-      <c r="H8" s="17" t="n">
+      <c r="H8" s="19" t="n">
         <f aca="false">G8/SQRT('1 ข้อมูล'!$C$19*F8/100)</f>
         <v>0.36645917247664</v>
       </c>
@@ -1916,7 +2061,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="8" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="C10" s="9"/>
       <c r="D10" s="9"/>
@@ -1927,18 +2072,18 @@
       <c r="I10" s="9"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="18" t="s">
-        <v>100</v>
+      <c r="B11" s="20" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="18" t="s">
-        <v>101</v>
+      <c r="B12" s="20" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="18" t="s">
-        <v>102</v>
+      <c r="B13" s="20" t="s">
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -1968,144 +2113,144 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="C5" s="19" t="n">
+        <v>116</v>
+      </c>
+      <c r="C5" s="21" t="n">
         <f aca="false">C6+0.2</f>
         <v>1.18155438703751</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="C6" s="19" t="n">
+        <v>118</v>
+      </c>
+      <c r="C6" s="21" t="n">
         <f aca="false">C8+'3 ช่องโชว์น้ำ'!F8/100+1.5*'3 ช่องโชว์น้ำ'!G8^2/(2*'1 ข้อมูล'!$C$19)</f>
         <v>0.981554387037505</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="C7" s="19" t="n">
+        <v>120</v>
+      </c>
+      <c r="C7" s="21" t="n">
         <f aca="false">C8+'1 ข้อมูล'!$C$15</f>
         <v>0.92</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="C8" s="19" t="n">
+        <v>122</v>
+      </c>
+      <c r="C8" s="21" t="n">
         <f aca="false">'1 ข้อมูล'!$C$14</f>
         <v>0.9</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="C9" s="19" t="n">
+        <v>124</v>
+      </c>
+      <c r="C9" s="21" t="n">
         <f aca="false">'1 ข้อมูล'!$C$10+'1 ข้อมูล'!$C$11</f>
         <v>0.9</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="C10" s="19" t="n">
-        <f aca="false">'2 เวียร์'!G12</f>
-        <v>0.809706461048468</v>
+        <v>126</v>
+      </c>
+      <c r="C10" s="21" t="n">
+        <f aca="false">'2 เวียร์'!H13</f>
+        <v>0.809665688762588</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="C11" s="19" t="n">
+        <v>128</v>
+      </c>
+      <c r="C11" s="21" t="n">
         <f aca="false">'1 ข้อมูล'!$C$10</f>
         <v>0.6</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="C12" s="19" t="n">
+        <v>129</v>
+      </c>
+      <c r="C12" s="21" t="n">
         <f aca="false">'1 ข้อมูล'!$C$10-0.06</f>
         <v>0.54</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="C13" s="19" t="n">
+        <v>131</v>
+      </c>
+      <c r="C13" s="21" t="n">
         <v>0</v>
       </c>
       <c r="D13" s="4"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="8" t="s">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="C15" s="9"/>
       <c r="D15" s="9"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="4" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="C16" s="10" t="n">
         <f aca="false">C7-C10</f>
-        <v>0.110293538951532</v>
+        <v>0.110334311237412</v>
       </c>
       <c r="D16" s="13" t="str">
         <f aca="false">IF(C16&gt;=0.1,"ผ่าน ✔ ม่านน้ำตกอิสระ","ไม่ผ่าน ✘ น้ำช่อง 3 จะย้อนขึ้นช่อง 2")</f>
@@ -2114,7 +2259,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="4" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="C17" s="10" t="n">
         <f aca="false">C5-C6</f>
@@ -2141,395 +2286,570 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:E25"/>
+  <dimension ref="B1:G25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>131</v>
+        <v>140</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="20" t="n">
+      <c r="B5" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="C5" s="7" t="n">
-        <f aca="false">'2 เวียร์'!$C$5*(B5/100+'1 ข้อมูล'!$C$21)^2.5*3600</f>
+      <c r="C5" s="15" t="n">
+        <f aca="false">'2 เวียร์'!$C$5*(B5/100)^2.5*3600</f>
+        <v>2.77719642805474</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <f aca="false">'2 เวียร์'!$C$6*(B5/100+'1 ข้อมูล'!$C$22)^2.5*3600</f>
         <v>2.86619650300861</v>
       </c>
-      <c r="D5" s="17" t="n">
+      <c r="E5" s="23" t="n">
+        <f aca="false">C5/D5-1</f>
+        <v>-0.0310516305704971</v>
+      </c>
+      <c r="F5" s="19" t="n">
         <f aca="false">C5/3.6</f>
-        <v>0.79616569528017</v>
-      </c>
-      <c r="E5" s="21" t="n">
+        <v>0.771443452237427</v>
+      </c>
+      <c r="G5" s="24" t="n">
         <f aca="false">C5*24</f>
-        <v>68.7887160722067</v>
+        <v>66.6527142733137</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="20" t="n">
+      <c r="B6" s="22" t="n">
         <v>6</v>
       </c>
-      <c r="C6" s="7" t="n">
-        <f aca="false">'2 เวียร์'!$C$5*(B6/100+'1 ข้อมูล'!$C$21)^2.5*3600</f>
+      <c r="C6" s="15" t="n">
+        <f aca="false">'2 เวียร์'!$C$5*(B6/100)^2.5*3600</f>
+        <v>4.38086341517286</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <f aca="false">'2 เวียร์'!$C$6*(B6/100+'1 ข้อมูล'!$C$22)^2.5*3600</f>
         <v>4.48983131905459</v>
       </c>
-      <c r="D6" s="17" t="n">
+      <c r="E6" s="23" t="n">
+        <f aca="false">C6/D6-1</f>
+        <v>-0.0242699326852838</v>
+      </c>
+      <c r="F6" s="19" t="n">
         <f aca="false">C6/3.6</f>
-        <v>1.24717536640405</v>
-      </c>
-      <c r="E6" s="21" t="n">
+        <v>1.21690650421468</v>
+      </c>
+      <c r="G6" s="24" t="n">
         <f aca="false">C6*24</f>
-        <v>107.75595165731</v>
+        <v>105.140721964149</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="20" t="n">
+      <c r="B7" s="22" t="n">
         <v>7</v>
       </c>
-      <c r="C7" s="7" t="n">
-        <f aca="false">'2 เวียร์'!$C$5*(B7/100+'1 ข้อมูล'!$C$21)^2.5*3600</f>
+      <c r="C7" s="15" t="n">
+        <f aca="false">'2 เวียร์'!$C$5*(B7/100)^2.5*3600</f>
+        <v>6.44060533155076</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <f aca="false">'2 เวียร์'!$C$6*(B7/100+'1 ข้อมูล'!$C$22)^2.5*3600</f>
         <v>6.56792530595593</v>
       </c>
-      <c r="D7" s="17" t="n">
+      <c r="E7" s="23" t="n">
+        <f aca="false">C7/D7-1</f>
+        <v>-0.0193851130264402</v>
+      </c>
+      <c r="F7" s="19" t="n">
         <f aca="false">C7/3.6</f>
-        <v>1.82442369609887</v>
-      </c>
-      <c r="E7" s="21" t="n">
+        <v>1.78905703654188</v>
+      </c>
+      <c r="G7" s="24" t="n">
         <f aca="false">C7*24</f>
-        <v>157.630207342942</v>
+        <v>154.574527957218</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="20" t="n">
+      <c r="B8" s="22" t="n">
         <v>8</v>
       </c>
-      <c r="C8" s="7" t="n">
-        <f aca="false">'2 เวียร์'!$C$5*(B8/100+'1 ข้อมูล'!$C$21)^2.5*3600</f>
+      <c r="C8" s="15" t="n">
+        <f aca="false">'2 เวียร์'!$C$5*(B8/100)^2.5*3600</f>
+        <v>8.99304061167301</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <f aca="false">'2 เวียร์'!$C$6*(B8/100+'1 ข้อมูล'!$C$22)^2.5*3600</f>
         <v>9.13647413844802</v>
       </c>
-      <c r="D8" s="17" t="n">
+      <c r="E8" s="23" t="n">
+        <f aca="false">C8/D8-1</f>
+        <v>-0.0156990021097324</v>
+      </c>
+      <c r="F8" s="19" t="n">
         <f aca="false">C8/3.6</f>
-        <v>2.53790948290223</v>
-      </c>
-      <c r="E8" s="21" t="n">
+        <v>2.49806683657584</v>
+      </c>
+      <c r="G8" s="24" t="n">
         <f aca="false">C8*24</f>
-        <v>219.275379322752</v>
+        <v>215.832974680152</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="20" t="n">
+      <c r="B9" s="22" t="n">
         <v>9</v>
       </c>
-      <c r="C9" s="7" t="n">
-        <f aca="false">'2 เวียร์'!$C$5*(B9/100+'1 ข้อมูล'!$C$21)^2.5*3600</f>
+      <c r="C9" s="15" t="n">
+        <f aca="false">'2 เวียร์'!$C$5*(B9/100)^2.5*3600</f>
+        <v>12.07224</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <f aca="false">'2 เวียร์'!$C$6*(B9/100+'1 ข้อมูล'!$C$22)^2.5*3600</f>
         <v>12.2289986697729</v>
       </c>
-      <c r="D9" s="17" t="n">
+      <c r="E9" s="23" t="n">
+        <f aca="false">C9/D9-1</f>
+        <v>-0.0128186022425818</v>
+      </c>
+      <c r="F9" s="19" t="n">
         <f aca="false">C9/3.6</f>
-        <v>3.39694407493691</v>
-      </c>
-      <c r="E9" s="21" t="n">
+        <v>3.3534</v>
+      </c>
+      <c r="G9" s="24" t="n">
         <f aca="false">C9*24</f>
-        <v>293.495968074549</v>
+        <v>289.73376</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="20" t="n">
+      <c r="B10" s="22" t="n">
         <v>10</v>
       </c>
-      <c r="C10" s="7" t="n">
-        <f aca="false">'2 เวียร์'!$C$5*(B10/100+'1 ข้อมูล'!$C$21)^2.5*3600</f>
+      <c r="C10" s="15" t="n">
+        <f aca="false">'2 เวียร์'!$C$5*(B10/100)^2.5*3600</f>
+        <v>15.7101954157165</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <f aca="false">'2 เวียร์'!$C$6*(B10/100+'1 ข้อมูล'!$C$22)^2.5*3600</f>
         <v>15.8769956216084</v>
       </c>
-      <c r="D10" s="17" t="n">
+      <c r="E10" s="23" t="n">
+        <f aca="false">C10/D10-1</f>
+        <v>-0.0105057789185823</v>
+      </c>
+      <c r="F10" s="19" t="n">
         <f aca="false">C10/3.6</f>
-        <v>4.4102765615579</v>
-      </c>
-      <c r="E10" s="21" t="n">
+        <v>4.36394317103236</v>
+      </c>
+      <c r="G10" s="24" t="n">
         <f aca="false">C10*24</f>
-        <v>381.047894918602</v>
+        <v>377.044689977196</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="20" t="n">
+      <c r="B11" s="22" t="n">
         <v>11</v>
       </c>
-      <c r="C11" s="7" t="n">
-        <f aca="false">'2 เวียร์'!$C$5*(B11/100+'1 ข้อมูล'!$C$21)^2.5*3600</f>
+      <c r="C11" s="15" t="n">
+        <f aca="false">'2 เวียร์'!$C$5*(B11/100)^2.5*3600</f>
+        <v>19.9371602697676</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <f aca="false">'2 เวียร์'!$C$6*(B11/100+'1 ข้อมูล'!$C$22)^2.5*3600</f>
         <v>20.1102658699656</v>
       </c>
-      <c r="D11" s="17" t="n">
+      <c r="E11" s="23" t="n">
+        <f aca="false">C11/D11-1</f>
+        <v>-0.00860782255775738</v>
+      </c>
+      <c r="F11" s="19" t="n">
         <f aca="false">C11/3.6</f>
-        <v>5.58618496387933</v>
-      </c>
-      <c r="E11" s="21" t="n">
+        <v>5.53810007493545</v>
+      </c>
+      <c r="G11" s="24" t="n">
         <f aca="false">C11*24</f>
-        <v>482.646380879174</v>
+        <v>478.491846474423</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="20" t="n">
+      <c r="B12" s="22" t="n">
         <v>12</v>
       </c>
-      <c r="C12" s="7" t="n">
-        <f aca="false">'2 เวียร์'!$C$5*(B12/100+'1 ข้อมูล'!$C$21)^2.5*3600</f>
+      <c r="C12" s="15" t="n">
+        <f aca="false">'2 เวียร์'!$C$5*(B12/100)^2.5*3600</f>
+        <v>24.7819058265663</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <f aca="false">'2 เวียร์'!$C$6*(B12/100+'1 ข้อมูล'!$C$22)^2.5*3600</f>
         <v>24.9571624264048</v>
       </c>
-      <c r="D12" s="17" t="n">
+      <c r="E12" s="23" t="n">
+        <f aca="false">C12/D12-1</f>
+        <v>-0.00702229671964116</v>
+      </c>
+      <c r="F12" s="19" t="n">
         <f aca="false">C12/3.6</f>
-        <v>6.93254511844577</v>
-      </c>
-      <c r="E12" s="21" t="n">
+        <v>6.88386272960174</v>
+      </c>
+      <c r="G12" s="24" t="n">
         <f aca="false">C12*24</f>
-        <v>598.971898233715</v>
+        <v>594.765739837591</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="20" t="n">
+      <c r="B13" s="22" t="n">
         <v>13</v>
       </c>
-      <c r="C13" s="7" t="n">
-        <f aca="false">'2 เวียร์'!$C$5*(B13/100+'1 ข้อมูล'!$C$21)^2.5*3600</f>
+      <c r="C13" s="15" t="n">
+        <f aca="false">'2 เวียร์'!$C$5*(B13/100)^2.5*3600</f>
+        <v>30.2719200646936</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <f aca="false">'2 เวียร์'!$C$6*(B13/100+'1 ข้อมูล'!$C$22)^2.5*3600</f>
         <v>30.4447832233961</v>
       </c>
-      <c r="D13" s="17" t="n">
+      <c r="E13" s="23" t="n">
+        <f aca="false">C13/D13-1</f>
+        <v>-0.0056779237820157</v>
+      </c>
+      <c r="F13" s="19" t="n">
         <f aca="false">C13/3.6</f>
-        <v>8.45688422872113</v>
-      </c>
-      <c r="E13" s="21" t="n">
+        <v>8.40886668463712</v>
+      </c>
+      <c r="G13" s="24" t="n">
         <f aca="false">C13*24</f>
-        <v>730.674797361505</v>
+        <v>726.526081552647</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="20" t="n">
+      <c r="B14" s="22" t="n">
         <v>14</v>
       </c>
-      <c r="C14" s="7" t="n">
-        <f aca="false">'2 เวียร์'!$C$5*(B14/100+'1 ข้อมูล'!$C$21)^2.5*3600</f>
+      <c r="C14" s="15" t="n">
+        <f aca="false">'2 เวียร์'!$C$5*(B14/100)^2.5*3600</f>
+        <v>36.4335656390862</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <f aca="false">'2 เวียร์'!$C$6*(B14/100+'1 ข้อมูล'!$C$22)^2.5*3600</f>
         <v>36.599124528368</v>
       </c>
-      <c r="D14" s="17" t="n">
+      <c r="E14" s="23" t="n">
+        <f aca="false">C14/D14-1</f>
+        <v>-0.00452357512413992</v>
+      </c>
+      <c r="F14" s="19" t="n">
         <f aca="false">C14/3.6</f>
-        <v>10.1664234801022</v>
-      </c>
-      <c r="E14" s="21" t="n">
+        <v>10.1204348997462</v>
+      </c>
+      <c r="G14" s="24" t="n">
         <f aca="false">C14*24</f>
-        <v>878.378988680832</v>
+        <v>874.405575338068</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="20" t="n">
+      <c r="B15" s="22" t="n">
         <v>15</v>
       </c>
-      <c r="C15" s="7" t="n">
-        <f aca="false">'2 เวียร์'!$C$5*(B15/100+'1 ข้อมูล'!$C$21)^2.5*3600</f>
+      <c r="C15" s="15" t="n">
+        <f aca="false">'2 เวียร์'!$C$5*(B15/100)^2.5*3600</f>
+        <v>43.2922078439065</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <f aca="false">'2 เวียร์'!$C$6*(B15/100+'1 ข้อมูล'!$C$22)^2.5*3600</f>
         <v>43.4452054104805</v>
       </c>
-      <c r="D15" s="17" t="n">
+      <c r="E15" s="23" t="n">
+        <f aca="false">C15/D15-1</f>
+        <v>-0.00352162143390655</v>
+      </c>
+      <c r="F15" s="19" t="n">
         <f aca="false">C15/3.6</f>
-        <v>12.0681126140224</v>
-      </c>
-      <c r="E15" s="21" t="n">
+        <v>12.025613289974</v>
+      </c>
+      <c r="G15" s="24" t="n">
         <f aca="false">C15*24</f>
-        <v>1042.68492985153</v>
+        <v>1039.01298825376</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="20" t="n">
+      <c r="B16" s="22" t="n">
         <v>16</v>
       </c>
-      <c r="C16" s="7" t="n">
-        <f aca="false">'2 เวียร์'!$C$5*(B16/100+'1 ข้อมูล'!$C$21)^2.5*3600</f>
+      <c r="C16" s="15" t="n">
+        <f aca="false">'2 เวียร์'!$C$5*(B16/100)^2.5*3600</f>
+        <v>50.87232</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <f aca="false">'2 เวียร์'!$C$6*(B16/100+'1 ข้อมูล'!$C$22)^2.5*3600</f>
         <v>51.0071703805085</v>
       </c>
-      <c r="D16" s="17" t="n">
+      <c r="E16" s="23" t="n">
+        <f aca="false">C16/D16-1</f>
+        <v>-0.0026437534076581</v>
+      </c>
+      <c r="F16" s="19" t="n">
         <f aca="false">C16/3.6</f>
-        <v>14.1686584390301</v>
-      </c>
-      <c r="E16" s="21" t="n">
+        <v>14.1312</v>
+      </c>
+      <c r="G16" s="24" t="n">
         <f aca="false">C16*24</f>
-        <v>1224.1720891322</v>
+        <v>1220.93568</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="20" t="n">
+      <c r="B17" s="22" t="n">
         <v>17</v>
       </c>
-      <c r="C17" s="7" t="n">
-        <f aca="false">'2 เวียร์'!$C$5*(B17/100+'1 ข้อมูล'!$C$21)^2.5*3600</f>
+      <c r="C17" s="15" t="n">
+        <f aca="false">'2 เวียร์'!$C$5*(B17/100)^2.5*3600</f>
+        <v>59.1975714819181</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <f aca="false">'2 เวียร์'!$C$6*(B17/100+'1 ข้อมูล'!$C$22)^2.5*3600</f>
         <v>59.3083752175669</v>
       </c>
-      <c r="D17" s="17" t="n">
+      <c r="E17" s="23" t="n">
+        <f aca="false">C17/D17-1</f>
+        <v>-0.00186826456200051</v>
+      </c>
+      <c r="F17" s="19" t="n">
         <f aca="false">C17/3.6</f>
-        <v>16.4745486715464</v>
-      </c>
-      <c r="E17" s="21" t="n">
+        <v>16.4437698560884</v>
+      </c>
+      <c r="G17" s="24" t="n">
         <f aca="false">C17*24</f>
-        <v>1423.40100522161</v>
+        <v>1420.74171556603</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="20" t="n">
+      <c r="B18" s="22" t="n">
         <v>18</v>
       </c>
-      <c r="C18" s="7" t="n">
-        <f aca="false">'2 เวียร์'!$C$5*(B18/100+'1 ข้อมูล'!$C$21)^2.5*3600</f>
+      <c r="C18" s="15" t="n">
+        <f aca="false">'2 เวียร์'!$C$5*(B18/100)^2.5*3600</f>
+        <v>68.2909021448919</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <f aca="false">'2 เวียร์'!$C$6*(B18/100+'1 ข้อมูล'!$C$22)^2.5*3600</f>
         <v>68.3714596053392</v>
       </c>
-      <c r="D18" s="17" t="n">
+      <c r="E18" s="23" t="n">
+        <f aca="false">C18/D18-1</f>
+        <v>-0.00117823227575298</v>
+      </c>
+      <c r="F18" s="19" t="n">
         <f aca="false">C18/3.6</f>
-        <v>18.9920721125942</v>
-      </c>
-      <c r="E18" s="21" t="n">
+        <v>18.9696950402477</v>
+      </c>
+      <c r="G18" s="24" t="n">
         <f aca="false">C18*24</f>
-        <v>1640.91503052814</v>
+        <v>1638.98165147741</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="20" t="n">
+      <c r="B19" s="22" t="n">
         <v>19</v>
       </c>
-      <c r="C19" s="7" t="n">
-        <f aca="false">'2 เวียร์'!$C$5*(B19/100+'1 ข้อมูล'!$C$21)^2.5*3600</f>
+      <c r="C19" s="15" t="n">
+        <f aca="false">'2 เวียร์'!$C$5*(B19/100)^2.5*3600</f>
+        <v>78.1745859249513</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <f aca="false">'2 เวียร์'!$C$6*(B19/100+'1 ข้อมูล'!$C$22)^2.5*3600</f>
         <v>78.2184092541632</v>
       </c>
-      <c r="D19" s="17" t="n">
+      <c r="E19" s="23" t="n">
+        <f aca="false">C19/D19-1</f>
+        <v>-0.000560268735067315</v>
+      </c>
+      <c r="F19" s="19" t="n">
         <f aca="false">C19/3.6</f>
-        <v>21.7273359039342</v>
-      </c>
-      <c r="E19" s="21" t="n">
+        <v>21.7151627569309</v>
+      </c>
+      <c r="G19" s="24" t="n">
         <f aca="false">C19*24</f>
-        <v>1877.24182209992</v>
+        <v>1876.19006219883</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="20" t="n">
+      <c r="B20" s="22" t="n">
         <v>20</v>
       </c>
-      <c r="C20" s="7" t="n">
-        <f aca="false">'2 เวียร์'!$C$5*(B20/100+'1 ข้อมูล'!$C$21)^2.5*3600</f>
+      <c r="C20" s="15" t="n">
+        <f aca="false">'2 เวียร์'!$C$5*(B20/100)^2.5*3600</f>
+        <v>88.8702856977516</v>
+      </c>
+      <c r="D20" s="7" t="n">
+        <f aca="false">'2 เวียร์'!$C$6*(B20/100+'1 ข้อมูล'!$C$22)^2.5*3600</f>
         <v>88.8706095248216</v>
       </c>
-      <c r="D20" s="17" t="n">
+      <c r="E20" s="23" t="n">
+        <f aca="false">C20/D20-1</f>
+        <v>-3.64380385908802E-006</v>
+      </c>
+      <c r="F20" s="19" t="n">
         <f aca="false">C20/3.6</f>
-        <v>24.6862804235616</v>
-      </c>
-      <c r="E20" s="21" t="n">
+        <v>24.6861904715977</v>
+      </c>
+      <c r="G20" s="24" t="n">
         <f aca="false">C20*24</f>
-        <v>2132.89462859572</v>
+        <v>2132.88685674604</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="20" t="n">
+      <c r="B21" s="22" t="n">
         <v>21</v>
       </c>
-      <c r="C21" s="7" t="n">
-        <f aca="false">'2 เวียร์'!$C$5*(B21/100+'1 ข้อมูล'!$C$21)^2.5*3600</f>
+      <c r="C21" s="15" t="n">
+        <f aca="false">'2 เวียร์'!$C$5*(B21/100)^2.5*3600</f>
+        <v>100.399100991704</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <f aca="false">'2 เวียร์'!$C$6*(B21/100+'1 ข้อมูล'!$C$22)^2.5*3600</f>
         <v>100.348892098404</v>
       </c>
-      <c r="D21" s="17" t="n">
+      <c r="E21" s="23" t="n">
+        <f aca="false">C21/D21-1</f>
+        <v>0.000500343274847825</v>
+      </c>
+      <c r="F21" s="19" t="n">
         <f aca="false">C21/3.6</f>
-        <v>27.8746922495567</v>
-      </c>
-      <c r="E21" s="21" t="n">
+        <v>27.8886391643623</v>
+      </c>
+      <c r="G21" s="24" t="n">
         <f aca="false">C21*24</f>
-        <v>2408.3734103617</v>
+        <v>2409.5784238009</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="20" t="n">
+      <c r="B22" s="22" t="n">
         <v>22</v>
       </c>
-      <c r="C22" s="7" t="n">
-        <f aca="false">'2 เวียร์'!$C$5*(B22/100+'1 ข้อมูล'!$C$21)^2.5*3600</f>
+      <c r="C22" s="15" t="n">
+        <f aca="false">'2 เวียร์'!$C$5*(B22/100)^2.5*3600</f>
+        <v>112.781609794846</v>
+      </c>
+      <c r="D22" s="7" t="n">
+        <f aca="false">'2 เวียร์'!$C$6*(B22/100+'1 ข้อมูล'!$C$22)^2.5*3600</f>
         <v>112.673575893332</v>
       </c>
-      <c r="D22" s="17" t="n">
+      <c r="E22" s="23" t="n">
+        <f aca="false">C22/D22-1</f>
+        <v>0.00095882198338515</v>
+      </c>
+      <c r="F22" s="19" t="n">
         <f aca="false">C22/3.6</f>
-        <v>31.2982155259257</v>
-      </c>
-      <c r="E22" s="21" t="n">
+        <v>31.3282249430127</v>
+      </c>
+      <c r="G22" s="24" t="n">
         <f aca="false">C22*24</f>
-        <v>2704.16582143998</v>
+        <v>2706.75863507629</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="20" t="n">
+      <c r="B23" s="22" t="n">
         <v>23</v>
       </c>
-      <c r="C23" s="7" t="n">
-        <f aca="false">'2 เวียร์'!$C$5*(B23/100+'1 ข้อมูล'!$C$21)^2.5*3600</f>
+      <c r="C23" s="15" t="n">
+        <f aca="false">'2 เวียร์'!$C$5*(B23/100)^2.5*3600</f>
+        <v>126.037905431355</v>
+      </c>
+      <c r="D23" s="7" t="n">
+        <f aca="false">'2 เวียร์'!$C$6*(B23/100+'1 ข้อมูล'!$C$22)^2.5*3600</f>
         <v>125.864503176292</v>
       </c>
-      <c r="D23" s="17" t="n">
+      <c r="E23" s="23" t="n">
+        <f aca="false">C23/D23-1</f>
+        <v>0.00137768990213294</v>
+      </c>
+      <c r="F23" s="19" t="n">
         <f aca="false">C23/3.6</f>
-        <v>34.9623619934145</v>
-      </c>
-      <c r="E23" s="21" t="n">
+        <v>35.0105292864875</v>
+      </c>
+      <c r="G23" s="24" t="n">
         <f aca="false">C23*24</f>
-        <v>3020.74807623101</v>
+        <v>3024.90973035252</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="20" t="n">
+      <c r="B24" s="22" t="n">
         <v>24</v>
       </c>
-      <c r="C24" s="7" t="n">
-        <f aca="false">'2 เวียร์'!$C$5*(B24/100+'1 ข้อมูล'!$C$21)^2.5*3600</f>
+      <c r="C24" s="15" t="n">
+        <f aca="false">'2 เวียร์'!$C$5*(B24/100)^2.5*3600</f>
+        <v>140.187629285531</v>
+      </c>
+      <c r="D24" s="7" t="n">
+        <f aca="false">'2 เวียร์'!$C$6*(B24/100+'1 ข้อมูล'!$C$22)^2.5*3600</f>
         <v>139.941071622383</v>
       </c>
-      <c r="D24" s="17" t="n">
+      <c r="E24" s="23" t="n">
+        <f aca="false">C24/D24-1</f>
+        <v>0.00176186776540921</v>
+      </c>
+      <c r="F24" s="19" t="n">
         <f aca="false">C24/3.6</f>
-        <v>38.8725198951064</v>
-      </c>
-      <c r="E24" s="21" t="n">
+        <v>38.9410081348699</v>
+      </c>
+      <c r="G24" s="24" t="n">
         <f aca="false">C24*24</f>
-        <v>3358.5857189372</v>
+        <v>3364.50310285276</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="20" t="n">
+      <c r="B25" s="22" t="n">
         <v>25</v>
       </c>
-      <c r="C25" s="7" t="n">
-        <f aca="false">'2 เวียร์'!$C$5*(B25/100+'1 ข้อมูล'!$C$21)^2.5*3600</f>
+      <c r="C25" s="15" t="n">
+        <f aca="false">'2 เวียร์'!$C$5*(B25/100)^2.5*3600</f>
+        <v>155.25</v>
+      </c>
+      <c r="D25" s="7" t="n">
+        <f aca="false">'2 เวียร์'!$C$6*(B25/100+'1 ข้อมูล'!$C$22)^2.5*3600</f>
         <v>154.922262933655</v>
       </c>
-      <c r="D25" s="17" t="n">
+      <c r="E25" s="23" t="n">
+        <f aca="false">C25/D25-1</f>
+        <v>0.00211549366849639</v>
+      </c>
+      <c r="F25" s="19" t="n">
         <f aca="false">C25/3.6</f>
-        <v>43.0339619260152</v>
-      </c>
-      <c r="E25" s="21" t="n">
+        <v>43.125</v>
+      </c>
+      <c r="G25" s="24" t="n">
         <f aca="false">C25*24</f>
-        <v>3718.13431040771</v>
+        <v>3726</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Shorten clear-water section to 1.00 m (tank 6.75 m external)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXLmoKkgGBxM2QbbegGKn7
</commit_message>
<xml_diff>
--- a/weir_design.xlsx
+++ b/weir_design.xlsx
@@ -1739,7 +1739,7 @@
         <v>29</v>
       </c>
       <c r="C18" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>19</v>
@@ -3006,7 +3006,7 @@
       <c r="D37" s="13"/>
       <c r="E37" s="23" t="n">
         <f aca="false">'1 ข้อมูล'!$C$18</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F37" s="6" t="s">
         <v>19</v>
@@ -3020,7 +3020,7 @@
       <c r="C38" s="6"/>
       <c r="D38" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$37-'3 ขนาดบ่อ'!$E$36</f>
-        <v>1.2</v>
+        <v>0.2</v>
       </c>
       <c r="E38" s="17" t="str">
         <f aca="false">IF(D38&gt;=0,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
@@ -3546,7 +3546,7 @@
       <c r="D74" s="13"/>
       <c r="E74" s="23" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$45+'3 ขนาดบ่อ'!$E$37+'3 ขนาดบ่อ'!$E$73</f>
-        <v>7.35</v>
+        <v>6.35</v>
       </c>
       <c r="F74" s="6" t="s">
         <v>19</v>
@@ -3597,7 +3597,7 @@
       <c r="D77" s="13"/>
       <c r="E77" s="23" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$74+2*'1 ข้อมูล'!$C$35</f>
-        <v>7.75</v>
+        <v>6.75</v>
       </c>
       <c r="F77" s="6" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
Replace perforated plate with under-flow baffle and sill in compartment 3
Plain SS304 6 mm plates: under-flow baffle with 0.30 m gap and a 0.40 m
sill 0.30 m downstream, sized for <= 0.10 m/s. Adds sizing rows and
checks to the workbook, a close-up detail drawing, and updates plan,
section, dimension sheet and animation (tank now 7.05 m external).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXLmoKkgGBxM2QbbegGKn7
</commit_message>
<xml_diff>
--- a/weir_design.xlsx
+++ b/weir_design.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="315">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="332">
   <si>
     <t xml:space="preserve">1) ข้อมูลออกแบบ — บ่อ 3 ช่อง: ปั๊มจุ่ม | โชว์น้ำใส | V-notch 90°</t>
   </si>
@@ -163,6 +163,12 @@
   </si>
   <si>
     <t xml:space="preserve">ไม่ให้เกิดกระแสวน / ยกปั๊มขึ้นซ่อมได้</t>
+  </si>
+  <si>
+    <t xml:space="preserve">สันล้นช่อง 3 สูงกว่าช่องลอดใต้</t>
+  </si>
+  <si>
+    <t xml:space="preserve">บังคับให้น้ำที่ลอดใต้ต้องยกตัวขึ้น</t>
   </si>
   <si>
     <t xml:space="preserve">ความเร็วลอยตัวฟองอากาศ</t>
@@ -552,7 +558,7 @@
     <t xml:space="preserve">ม่านน้ำพุ่งไกล + เผื่อ 0.20</t>
   </si>
   <si>
-    <t xml:space="preserve">ค. โซนรับน้ำตก ช่อง 3 (ให้ฟองอากาศลอยหมดก่อนถึงแผ่นรูพรุน)</t>
+    <t xml:space="preserve">ค. โซนรับน้ำตก + ผนังลอดใต้ + สันล้น ช่อง 3 (ทำให้น้ำนิ่งก่อนเข้าช่วงตรง)</t>
   </si>
   <si>
     <t xml:space="preserve">ความลึกน้ำช่อง 3 สูงสุด</t>
@@ -579,6 +585,51 @@
     <t xml:space="preserve">MAX(ระยะทำงาน 0.50, ระยะฟอง)</t>
   </si>
   <si>
+    <t xml:space="preserve">ฟองลอยหมดก่อนถึงผนังลอดใต้</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ช่องลอดใต้ผนัง ช่อง 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q ÷ (B × v ไม่เกิน 0.10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ผนังลอดใต้ = แผ่น SS304 6 mm ขอบบนเสมอสันกำแพง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ระยะผนังลอดใต้ ถึง สันล้น</t>
+  </si>
+  <si>
+    <t xml:space="preserve">เท่าช่องลอด (น้ำเลี้ยวขึ้นเรียบ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ความสูงสันล้น</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ช่องลอด + 0.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">สันล้น = แผ่น SS304 6 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ความเร็วน้ำข้ามสันล้น (สูงสุด)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q ÷ (B × (น้ำช่อง 3 − สันล้น))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ตรวจ: ความเร็วข้ามสันล้น ≤ 0.10 m/s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ตรวจ: น้ำเหนือสันล้น ที่น้ำต่ำสุด (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≥ 0.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">น้ำ 50 m³/h ยังข้ามสันได้สบาย</t>
+  </si>
+  <si>
     <t xml:space="preserve">ง. ช่อง 2 โชว์น้ำใส</t>
   </si>
   <si>
@@ -621,9 +672,6 @@
     <t xml:space="preserve">ช่องลอดใต้ผนังกั้น</t>
   </si>
   <si>
-    <t xml:space="preserve">Q ÷ (B × v ไม่เกิน 0.10)</t>
-  </si>
-  <si>
     <t xml:space="preserve">โซนน้ำเข้า</t>
   </si>
   <si>
@@ -813,7 +861,10 @@
     <t xml:space="preserve">ความยาวช่อง 3</t>
   </si>
   <si>
-    <t xml:space="preserve">รับน้ำตก + ช่วงตรง + กำแพงเวียร์ + ท้ายเวียร์</t>
+    <t xml:space="preserve">รับน้ำตก + ลอดใต้–สันล้น + ช่วงตรง + กำแพงเวียร์ + ท้ายเวียร์</t>
+  </si>
+  <si>
+    <t xml:space="preserve">แผ่น SS 6 mm รวมอยู่ในระยะ</t>
   </si>
   <si>
     <t xml:space="preserve">ความยาวภายใน</t>
@@ -1543,7 +1594,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:E54"/>
+  <dimension ref="B1:E55"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -1854,7 +1905,7 @@
         <v>0.1</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>47</v>
@@ -1865,10 +1916,10 @@
         <v>48</v>
       </c>
       <c r="C27" s="10" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="E27" s="6" t="s">
         <v>49</v>
@@ -1879,7 +1930,7 @@
         <v>50</v>
       </c>
       <c r="C28" s="10" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="D28" s="6" t="s">
         <v>19</v>
@@ -1898,21 +1949,21 @@
       <c r="D29" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E29" s="6"/>
+      <c r="E29" s="6" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C30" s="10" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="D30" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E30" s="6" t="s">
-        <v>54</v>
-      </c>
+      <c r="E30" s="6"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="6" t="s">
@@ -1924,11 +1975,13 @@
       <c r="D31" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E31" s="6"/>
+      <c r="E31" s="6" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C32" s="10" t="n">
         <v>0.1</v>
@@ -1936,9 +1989,7 @@
       <c r="D32" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E32" s="6" t="s">
-        <v>57</v>
-      </c>
+      <c r="E32" s="6"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="6" t="s">
@@ -1958,27 +2009,27 @@
       <c r="B34" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="C34" s="11" t="n">
-        <v>0.006</v>
+      <c r="C34" s="10" t="n">
+        <v>0.1</v>
       </c>
       <c r="D34" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E34" s="6"/>
+      <c r="E34" s="6" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="C35" s="10" t="n">
-        <v>0.2</v>
+        <v>62</v>
+      </c>
+      <c r="C35" s="11" t="n">
+        <v>0.006</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E35" s="6" t="s">
-        <v>62</v>
-      </c>
+      <c r="E35" s="6"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="6" t="s">
@@ -1990,41 +2041,43 @@
       <c r="D36" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E36" s="6"/>
+      <c r="E36" s="6" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C37" s="10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E37" s="6"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B38" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="C38" s="10" t="n">
         <v>0.05</v>
       </c>
-      <c r="D37" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="C39" s="5"/>
-      <c r="D39" s="5"/>
-      <c r="E39" s="5"/>
+      <c r="D38" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E38" s="6" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="C40" s="12" t="n">
-        <v>9.81</v>
-      </c>
-      <c r="D40" s="6" t="s">
+      <c r="B40" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="E40" s="6"/>
+      <c r="C40" s="5"/>
+      <c r="D40" s="5"/>
+      <c r="E40" s="5"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="6" t="s">
@@ -2042,25 +2095,23 @@
       <c r="B42" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="C42" s="13" t="n">
-        <v>1.38</v>
+      <c r="C42" s="12" t="n">
+        <v>9.81</v>
       </c>
       <c r="D42" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="E42" s="6" t="s">
-        <v>73</v>
-      </c>
+      <c r="E42" s="6"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C43" s="13" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="D43" s="6" t="s">
         <v>74</v>
-      </c>
-      <c r="C43" s="13" t="n">
-        <v>0.578</v>
-      </c>
-      <c r="D43" s="6" t="s">
-        <v>72</v>
       </c>
       <c r="E43" s="6" t="s">
         <v>75</v>
@@ -2070,28 +2121,28 @@
       <c r="B44" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="C44" s="14" t="n">
-        <v>0.00085</v>
+      <c r="C44" s="13" t="n">
+        <v>0.578</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>19</v>
+        <v>74</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C45" s="14" t="n">
+        <v>0.00085</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E45" s="6" t="s">
         <v>77</v>
-      </c>
-      <c r="C45" s="12" t="n">
-        <v>1.84</v>
-      </c>
-      <c r="D45" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="E45" s="6" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2099,10 +2150,10 @@
         <v>79</v>
       </c>
       <c r="C46" s="12" t="n">
-        <v>0.6</v>
+        <v>1.84</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>80</v>
@@ -2112,80 +2163,94 @@
       <c r="B47" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="C47" s="15" t="n">
-        <v>205</v>
+      <c r="C47" s="12" t="n">
+        <v>0.6</v>
       </c>
       <c r="D47" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="E47" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="E47" s="6"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="6" t="s">
         <v>83</v>
       </c>
       <c r="C48" s="15" t="n">
-        <v>400</v>
+        <v>205</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E48" s="6"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C49" s="15" t="n">
+        <v>400</v>
+      </c>
+      <c r="D49" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="C49" s="9" t="n">
+      <c r="E49" s="6"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B50" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C50" s="9" t="n">
         <v>1.7</v>
       </c>
-      <c r="D49" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="E49" s="6"/>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="C51" s="5"/>
-      <c r="D51" s="5"/>
-      <c r="E51" s="5"/>
+      <c r="D50" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="E50" s="6"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B52" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="C52" s="16" t="s">
+      <c r="B52" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="D52" s="6"/>
-      <c r="E52" s="6" t="s">
-        <v>88</v>
-      </c>
+      <c r="C52" s="5"/>
+      <c r="D52" s="5"/>
+      <c r="E52" s="5"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C53" s="16" t="s">
         <v>89</v>
-      </c>
-      <c r="C53" s="17" t="s">
-        <v>90</v>
       </c>
       <c r="D53" s="6"/>
       <c r="E53" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="C54" s="17" t="s">
         <v>92</v>
-      </c>
-      <c r="C54" s="6" t="s">
-        <v>93</v>
       </c>
       <c r="D54" s="6"/>
       <c r="E54" s="6" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B55" s="6" t="s">
         <v>94</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="D55" s="6"/>
+      <c r="E55" s="6" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -2219,17 +2284,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="4" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="5"/>
@@ -2240,17 +2305,17 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C5" s="13" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$42</f>
+        <f aca="false">'1 ข้อมูล'!$C$43</f>
         <v>1.38</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
@@ -2258,17 +2323,17 @@
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C6" s="18" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$43*(8/15)*SQRT(2*'1 ข้อมูล'!$C$40)</f>
+        <f aca="false">'1 ข้อมูล'!$C$44*(8/15)*SQRT(2*'1 ข้อมูล'!$C$41)</f>
         <v>1.36545083661038</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
@@ -2276,7 +2341,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="4" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
@@ -2287,30 +2352,30 @@
     </row>
     <row r="9" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C10" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$7-'1 ข้อมูล'!$C$9</f>
@@ -2325,7 +2390,7 @@
         <v>14.532869095236</v>
       </c>
       <c r="F10" s="9" t="n">
-        <f aca="false">((D10/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$44)*100</f>
+        <f aca="false">((D10/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$45)*100</f>
         <v>14.5096125168743</v>
       </c>
       <c r="G10" s="20" t="n">
@@ -2336,7 +2401,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C11" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$10-'1 ข้อมูล'!$C$9</f>
@@ -2351,7 +2416,7 @@
         <v>16.2387843483091</v>
       </c>
       <c r="F11" s="9" t="n">
-        <f aca="false">((D11/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$44)*100</f>
+        <f aca="false">((D11/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$45)*100</f>
         <v>16.2227754127948</v>
       </c>
       <c r="G11" s="20" t="n">
@@ -2359,12 +2424,12 @@
         <v>0.0160089355143072</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C12" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8-'1 ข้อมูล'!$C$9</f>
@@ -2379,7 +2444,7 @@
         <v>20.1013103538681</v>
       </c>
       <c r="F12" s="9" t="n">
-        <f aca="false">((D12/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$44)*100</f>
+        <f aca="false">((D12/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$45)*100</f>
         <v>20.1017115002301</v>
       </c>
       <c r="G12" s="20" t="n">
@@ -2390,7 +2455,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="21" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C13" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8</f>
@@ -2405,7 +2470,7 @@
         <v>20.9665688762588</v>
       </c>
       <c r="F13" s="9" t="n">
-        <f aca="false">((D13/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$44)*100</f>
+        <f aca="false">((D13/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$45)*100</f>
         <v>20.9706461048468</v>
       </c>
       <c r="G13" s="20" t="n">
@@ -2413,22 +2478,22 @@
         <v>-0.00407722858800952</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="22" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="22" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="22" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -2447,7 +2512,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:G79"/>
+  <dimension ref="B1:G85"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -2460,12 +2525,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2473,24 +2538,24 @@
         <v>2</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>4</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="4" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -2500,10 +2565,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D7" s="13"/>
       <c r="E7" s="23" t="n">
@@ -2514,15 +2579,15 @@
         <v>19</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D8" s="13" t="n">
         <f aca="false">MAX(0.45,'3 ขนาดบ่อ'!$E$7/0.4)+'1 ข้อมูล'!$C$14</f>
@@ -2536,15 +2601,15 @@
         <v>19</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D9" s="13" t="n">
         <f aca="false">MAX(0.9,'3 ขนาดบ่อ'!$E$7/0.2)</f>
@@ -2558,15 +2623,15 @@
         <v>19</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D10" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$7+'1 ข้อมูล'!$C$15</f>
@@ -2580,15 +2645,15 @@
         <v>19</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D11" s="13"/>
       <c r="E11" s="23" t="n">
@@ -2599,15 +2664,15 @@
         <v>19</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D12" s="13" t="n">
         <f aca="false">10*'3 ขนาดบ่อ'!$E$7</f>
@@ -2621,15 +2686,15 @@
         <v>19</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D13" s="13" t="n">
         <f aca="false">4.5*'3 ขนาดบ่อ'!$E$7</f>
@@ -2643,15 +2708,15 @@
         <v>19</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="6" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D14" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$7/'3 ขนาดบ่อ'!$E$8</f>
@@ -2666,10 +2731,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="6" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D15" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$7/'3 ขนาดบ่อ'!$E$9</f>
@@ -2684,10 +2749,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D16" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$13/'3 ขนาดบ่อ'!$E$7</f>
@@ -2702,10 +2767,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D17" s="13" t="n">
         <f aca="false">'2 เวียร์'!$E$10/100</f>
@@ -2717,12 +2782,12 @@
       </c>
       <c r="F17" s="6"/>
       <c r="G17" s="6" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="4" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5"/>
@@ -2732,14 +2797,14 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="6" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D20" s="13"/>
       <c r="E20" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$29/2+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$46*PI()*'1 ข้อมูล'!$C$29^2/4))^2/(2*'1 ข้อมูล'!$C$40)</f>
+        <f aca="false">'1 ข้อมูล'!$C$30/2+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$47*PI()*'1 ข้อมูล'!$C$30^2/4))^2/(2*'1 ข้อมูล'!$C$41)</f>
         <v>0.210686269183871</v>
       </c>
       <c r="F20" s="6" t="s">
@@ -2749,10 +2814,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="6" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D21" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8-'3 ขนาดบ่อ'!$E$20</f>
@@ -2764,34 +2829,34 @@
       </c>
       <c r="F21" s="6"/>
       <c r="G21" s="6" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="6" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D22" s="13"/>
       <c r="E22" s="23" t="n">
-        <f aca="false">SQRT(2*'1 ข้อมูล'!$C$40*'3 ขนาดบ่อ'!$E$7)</f>
+        <f aca="false">SQRT(2*'1 ข้อมูล'!$C$41*'3 ขนาดบ่อ'!$E$7)</f>
         <v>2.02821123493634</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>34</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="6" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D23" s="13"/>
       <c r="E23" s="23" t="n">
@@ -2805,32 +2870,32 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="6" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D24" s="13"/>
       <c r="E24" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$22*SQRT(2*'3 ขนาดบ่อ'!$E$23/'1 ข้อมูล'!$C$40)</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$22*SQRT(2*'3 ขนาดบ่อ'!$E$23/'1 ข้อมูล'!$C$41)</f>
         <v>0.708760700266562</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="6" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D25" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$24+'1 ข้อมูล'!$C$28</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$24+'1 ข้อมูล'!$C$29</f>
         <v>0.908760700266562</v>
       </c>
       <c r="E25" s="23" t="n">
@@ -2844,7 +2909,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="4" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C27" s="5"/>
       <c r="D27" s="5"/>
@@ -2854,10 +2919,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="6" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D28" s="13"/>
       <c r="E28" s="23" t="n">
@@ -2871,10 +2936,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="6" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D29" s="13"/>
       <c r="E29" s="23" t="n">
@@ -2888,14 +2953,14 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="6" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D30" s="13"/>
       <c r="E30" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$28/'1 ข้อมูล'!$C$26*'3 ขนาดบ่อ'!$E$29</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$28/'1 ข้อมูล'!$C$27*'3 ขนาดบ่อ'!$E$29</f>
         <v>0.264550264550265</v>
       </c>
       <c r="F30" s="6" t="s">
@@ -2905,13 +2970,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="6" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D31" s="13" t="n">
-        <f aca="false">MAX('1 ข้อมูล'!$C$27,'3 ขนาดบ่อ'!$E$30)</f>
+        <f aca="false">MAX('1 ข้อมูล'!$C$28,'3 ขนาดบ่อ'!$E$30)</f>
         <v>0.5</v>
       </c>
       <c r="E31" s="23" t="n">
@@ -2921,722 +2986,840 @@
       <c r="F31" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G31" s="6"/>
+      <c r="G31" s="6" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="D32" s="13" t="n">
+        <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$9*'1 ข้อมูล'!$C$20)</f>
+        <v>0.264550264550265</v>
+      </c>
+      <c r="E32" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D32,4),'1 ข้อมูล'!$C$13)</f>
+        <v>0.3</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G32" s="6" t="s">
+        <v>186</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="C33" s="5"/>
-      <c r="D33" s="5"/>
-      <c r="E33" s="5"/>
-      <c r="F33" s="5"/>
-      <c r="G33" s="5"/>
+      <c r="B33" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="D33" s="13"/>
+      <c r="E33" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$32</f>
+        <v>0.3</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G33" s="6"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="6" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="D34" s="13"/>
+        <v>190</v>
+      </c>
+      <c r="D34" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$32+'1 ข้อมูล'!$C$26</f>
+        <v>0.4</v>
+      </c>
       <c r="E34" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$17+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$45*'3 ขนาดบ่อ'!$E$9))^(2/3)</f>
-        <v>0.0791280538460372</v>
+        <f aca="false">CEILING(ROUND(D34,4),'1 ข้อมูล'!$C$13)</f>
+        <v>0.4</v>
       </c>
       <c r="F34" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="6" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>186</v>
-      </c>
-      <c r="D35" s="13" t="n">
+        <v>193</v>
+      </c>
+      <c r="D35" s="13"/>
+      <c r="E35" s="23" t="n">
+        <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$9*('3 ขนาดบ่อ'!$E$28-'3 ขนาดบ่อ'!$E$34))</f>
+        <v>0.0645771105091445</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="G35" s="6"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B36" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="C36" s="6"/>
+      <c r="D36" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$35</f>
+        <v>0.0645771105091445</v>
+      </c>
+      <c r="E36" s="17" t="str">
+        <f aca="false">IF(D36&lt;=0.1,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F36" s="6"/>
+      <c r="G36" s="6"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B37" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="D37" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$8+'2 เวียร์'!$E$10/100-'3 ขนาดบ่อ'!$E$34</f>
+        <v>0.34532869095236</v>
+      </c>
+      <c r="E37" s="17" t="str">
+        <f aca="false">IF(D37&gt;=0.1,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F37" s="6"/>
+      <c r="G37" s="6" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B39" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="C39" s="5"/>
+      <c r="D39" s="5"/>
+      <c r="E39" s="5"/>
+      <c r="F39" s="5"/>
+      <c r="G39" s="5"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B40" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="D40" s="13"/>
+      <c r="E40" s="23" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$17+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$46*'3 ขนาดบ่อ'!$E$9))^(2/3)</f>
+        <v>0.0791280538460372</v>
+      </c>
+      <c r="F40" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G40" s="6" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B41" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="D41" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$28+'1 ข้อมูล'!$C$16-'1 ข้อมูล'!$C$17</f>
         <v>0.889665688762588</v>
       </c>
-      <c r="E35" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D35,4),'1 ข้อมูล'!$C$13)</f>
+      <c r="E41" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D41,4),'1 ข้อมูล'!$C$13)</f>
         <v>0.9</v>
       </c>
-      <c r="F35" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G35" s="6" t="s">
+      <c r="F41" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G41" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="C36" s="6" t="s">
-        <v>188</v>
-      </c>
-      <c r="D36" s="13" t="n">
-        <f aca="false">10*'3 ขนาดบ่อ'!$E$34</f>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B42" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="D42" s="13" t="n">
+        <f aca="false">10*'3 ขนาดบ่อ'!$E$40</f>
         <v>0.791280538460372</v>
       </c>
-      <c r="E36" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D36,4),'1 ข้อมูล'!$C$13)</f>
+      <c r="E42" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D42,4),'1 ข้อมูล'!$C$13)</f>
         <v>0.8</v>
       </c>
-      <c r="F36" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G36" s="6" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="6" t="s">
-        <v>190</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>191</v>
-      </c>
-      <c r="D37" s="13"/>
-      <c r="E37" s="23" t="n">
+      <c r="F42" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G42" s="6" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B43" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="D43" s="13"/>
+      <c r="E43" s="23" t="n">
         <f aca="false">'1 ข้อมูล'!$C$18</f>
         <v>1</v>
       </c>
-      <c r="F37" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G37" s="6"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="6" t="s">
-        <v>192</v>
-      </c>
-      <c r="C38" s="6"/>
-      <c r="D38" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$37-'3 ขนาดบ่อ'!$E$36</f>
+      <c r="F43" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G43" s="6"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B44" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="C44" s="6"/>
+      <c r="D44" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$43-'3 ขนาดบ่อ'!$E$42</f>
         <v>0.2</v>
       </c>
-      <c r="E38" s="17" t="str">
-        <f aca="false">IF(D38&gt;=0,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+      <c r="E44" s="17" t="str">
+        <f aca="false">IF(D44&gt;=0,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
-      <c r="F38" s="6"/>
-      <c r="G38" s="6"/>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="C40" s="5"/>
-      <c r="D40" s="5"/>
-      <c r="E40" s="5"/>
-      <c r="F40" s="5"/>
-      <c r="G40" s="5"/>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="C41" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="D41" s="13" t="n">
+      <c r="F44" s="6"/>
+      <c r="G44" s="6"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B46" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="C46" s="5"/>
+      <c r="D46" s="5"/>
+      <c r="E46" s="5"/>
+      <c r="F46" s="5"/>
+      <c r="G46" s="5"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B47" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="D47" s="13" t="n">
         <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$9*'1 ข้อมูล'!$C$20)</f>
         <v>0.264550264550265</v>
       </c>
-      <c r="E41" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D41,4),'1 ข้อมูล'!$C$13)</f>
+      <c r="E47" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D47,4),'1 ข้อมูล'!$C$13)</f>
         <v>0.3</v>
       </c>
-      <c r="F41" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G41" s="6"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="D42" s="13" t="n">
+      <c r="F47" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G47" s="6"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B48" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="D48" s="13" t="n">
         <f aca="false">'1 ข้อมูล'!$C$21+2*'1 ข้อมูล'!$C$22</f>
         <v>0.468</v>
       </c>
-      <c r="E42" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D42,4),'1 ข้อมูล'!$C$13)</f>
+      <c r="E48" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D48,4),'1 ข้อมูล'!$C$13)</f>
         <v>0.5</v>
       </c>
-      <c r="F42" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G42" s="6"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="D43" s="13"/>
-      <c r="E43" s="23" t="n">
+      <c r="F48" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G48" s="6"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B49" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="D49" s="13"/>
+      <c r="E49" s="23" t="n">
         <f aca="false">'1 ข้อมูล'!$C$23</f>
         <v>0.1</v>
       </c>
-      <c r="F43" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G43" s="6"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="6" t="s">
-        <v>200</v>
-      </c>
-      <c r="C44" s="6" t="s">
-        <v>201</v>
-      </c>
-      <c r="D44" s="13" t="n">
+      <c r="F49" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G49" s="6"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B50" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="D50" s="13" t="n">
         <f aca="false">'1 ข้อมูล'!$C$24+2*'1 ข้อมูล'!$C$25</f>
         <v>1</v>
       </c>
-      <c r="E44" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D44,4),'1 ข้อมูล'!$C$13)</f>
-        <v>1</v>
-      </c>
-      <c r="F44" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G44" s="6"/>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="C45" s="6" t="s">
-        <v>203</v>
-      </c>
-      <c r="D45" s="13"/>
-      <c r="E45" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$42+'3 ขนาดบ่อ'!$E$43+'3 ขนาดบ่อ'!$E$44</f>
-        <v>1.6</v>
-      </c>
-      <c r="F45" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G45" s="6"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="C46" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="D46" s="13"/>
-      <c r="E46" s="23" t="n">
-        <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$9*'3 ขนาดบ่อ'!$E$34)</f>
-        <v>0.334331822522782</v>
-      </c>
-      <c r="F46" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="G46" s="6"/>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="6" t="s">
-        <v>206</v>
-      </c>
-      <c r="C47" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="D47" s="13"/>
-      <c r="E47" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$35+'3 ขนาดบ่อ'!$E$34+1.5*'3 ขนาดบ่อ'!$E$46^2/(2*'1 ข้อมูล'!$C$40)</f>
-        <v>0.987673754729172</v>
-      </c>
-      <c r="F47" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G47" s="6" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B49" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="C49" s="5"/>
-      <c r="D49" s="5"/>
-      <c r="E49" s="5"/>
-      <c r="F49" s="5"/>
-      <c r="G49" s="5"/>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B50" s="6" t="s">
-        <v>210</v>
-      </c>
-      <c r="C50" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="D50" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$47+'1 ข้อมูล'!$C$19</f>
-        <v>1.18767375472917</v>
-      </c>
       <c r="E50" s="23" t="n">
         <f aca="false">CEILING(ROUND(D50,4),'1 ข้อมูล'!$C$13)</f>
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="F50" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G50" s="6" t="s">
-        <v>212</v>
-      </c>
+      <c r="G50" s="6"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B51" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="D51" s="13"/>
+      <c r="E51" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$48+'3 ขนาดบ่อ'!$E$49+'3 ขนาดบ่อ'!$E$50</f>
+        <v>1.6</v>
+      </c>
+      <c r="F51" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G51" s="6"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B52" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="C52" s="5"/>
-      <c r="D52" s="5"/>
-      <c r="E52" s="5"/>
-      <c r="F52" s="5"/>
-      <c r="G52" s="5"/>
+      <c r="B52" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C52" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="D52" s="13"/>
+      <c r="E52" s="23" t="n">
+        <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$9*'3 ขนาดบ่อ'!$E$40)</f>
+        <v>0.334331822522782</v>
+      </c>
+      <c r="F52" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="G52" s="6"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="6" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="D53" s="13"/>
       <c r="E53" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$8-'1 ข้อมูล'!$C$30</f>
-        <v>0.5</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$41+'3 ขนาดบ่อ'!$E$40+1.5*'3 ขนาดบ่อ'!$E$52^2/(2*'1 ข้อมูล'!$C$41)</f>
+        <v>0.987673754729172</v>
       </c>
       <c r="F53" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G53" s="6" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B54" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="C54" s="6" t="s">
-        <v>218</v>
-      </c>
-      <c r="D54" s="13"/>
-      <c r="E54" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$9+2*'1 ข้อมูล'!$C$33</f>
-        <v>1.25</v>
-      </c>
-      <c r="F54" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G54" s="6"/>
+        <v>224</v>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B55" s="6" t="s">
-        <v>219</v>
-      </c>
-      <c r="C55" s="6" t="s">
-        <v>220</v>
-      </c>
-      <c r="D55" s="13"/>
-      <c r="E55" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$53-'1 ข้อมูล'!$C$31</f>
-        <v>0.4</v>
-      </c>
-      <c r="F55" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G55" s="6" t="s">
-        <v>221</v>
-      </c>
+      <c r="B55" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="C55" s="5"/>
+      <c r="D55" s="5"/>
+      <c r="E55" s="5"/>
+      <c r="F55" s="5"/>
+      <c r="G55" s="5"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="6" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>223</v>
-      </c>
-      <c r="D56" s="13"/>
+        <v>227</v>
+      </c>
+      <c r="D56" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$53+'1 ข้อมูล'!$C$19</f>
+        <v>1.18767375472917</v>
+      </c>
       <c r="E56" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$10+'1 ข้อมูล'!$C$32</f>
-        <v>1</v>
+        <f aca="false">CEILING(ROUND(D56,4),'1 ข้อมูล'!$C$13)</f>
+        <v>1.2</v>
       </c>
       <c r="F56" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G56" s="6"/>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B57" s="6" t="s">
-        <v>224</v>
-      </c>
-      <c r="C57" s="6" t="s">
-        <v>225</v>
-      </c>
-      <c r="D57" s="13"/>
-      <c r="E57" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$56-'3 ขนาดบ่อ'!$E$55</f>
-        <v>0.6</v>
-      </c>
-      <c r="F57" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G57" s="6"/>
+      <c r="G56" s="6" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B58" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="C58" s="6" t="s">
-        <v>227</v>
-      </c>
-      <c r="D58" s="13"/>
-      <c r="E58" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$28-'3 ขนาดบ่อ'!$E$53</f>
-        <v>0.309665688762588</v>
-      </c>
-      <c r="F58" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G58" s="6"/>
+      <c r="B58" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="C58" s="5"/>
+      <c r="D58" s="5"/>
+      <c r="E58" s="5"/>
+      <c r="F58" s="5"/>
+      <c r="G58" s="5"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="6" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="D59" s="13"/>
       <c r="E59" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$41*'3 ขนาดบ่อ'!$E$58^3/6</f>
-        <v>0.0485508704265308</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$8-'1 ข้อมูล'!$C$31</f>
+        <v>0.5</v>
       </c>
       <c r="F59" s="6" t="s">
-        <v>230</v>
+        <v>19</v>
       </c>
       <c r="G59" s="6" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="6" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D60" s="13"/>
       <c r="E60" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$59/('1 ข้อมูล'!$C$34^2/6)/1000</f>
-        <v>8.09181173775513</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$9+2*'1 ข้อมูล'!$C$34</f>
+        <v>1.25</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>82</v>
+        <v>19</v>
       </c>
       <c r="G60" s="6"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="6" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>235</v>
-      </c>
-      <c r="D61" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$60</f>
-        <v>8.09181173775513</v>
-      </c>
-      <c r="E61" s="17" t="str">
-        <f aca="false">IF(D61&lt;=0.6*'1 ข้อมูล'!$C$47,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
-        <v>ผ่าน ✔</v>
-      </c>
-      <c r="F61" s="6"/>
+        <v>236</v>
+      </c>
+      <c r="D61" s="13"/>
+      <c r="E61" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$59-'1 ข้อมูล'!$C$32</f>
+        <v>0.4</v>
+      </c>
+      <c r="F61" s="6" t="s">
+        <v>19</v>
+      </c>
       <c r="G61" s="6" t="s">
-        <v>236</v>
-      </c>
+        <v>237</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B62" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="D62" s="13"/>
+      <c r="E62" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$10+'1 ข้อมูล'!$C$33</f>
+        <v>1</v>
+      </c>
+      <c r="F62" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G62" s="6"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B63" s="4" t="s">
-        <v>237</v>
-      </c>
-      <c r="C63" s="5"/>
-      <c r="D63" s="5"/>
-      <c r="E63" s="5"/>
-      <c r="F63" s="5"/>
-      <c r="G63" s="5"/>
+      <c r="B63" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="D63" s="13"/>
+      <c r="E63" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$62-'3 ขนาดบ่อ'!$E$61</f>
+        <v>0.6</v>
+      </c>
+      <c r="F63" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G63" s="6"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B64" s="6" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="D64" s="13"/>
       <c r="E64" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$41*'3 ขนาดบ่อ'!$E$50^3/6</f>
-        <v>2.82528</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$28-'3 ขนาดบ่อ'!$E$59</f>
+        <v>0.309665688762588</v>
       </c>
       <c r="F64" s="6" t="s">
-        <v>230</v>
-      </c>
-      <c r="G64" s="6" t="s">
-        <v>240</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="G64" s="6"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="6" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="D65" s="13"/>
       <c r="E65" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$49*'3 ขนาดบ่อ'!$E$64</f>
-        <v>4.802976</v>
+        <f aca="false">'1 ข้อมูล'!$C$42*'3 ขนาดบ่อ'!$E$64^3/6</f>
+        <v>0.0485508704265308</v>
       </c>
       <c r="F65" s="6" t="s">
-        <v>230</v>
-      </c>
-      <c r="G65" s="6"/>
+        <v>246</v>
+      </c>
+      <c r="G65" s="6" t="s">
+        <v>247</v>
+      </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="6" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="D66" s="13"/>
       <c r="E66" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$35-'1 ข้อมูล'!$C$37-0.006</f>
-        <v>0.144</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$65/('1 ข้อมูล'!$C$35^2/6)/1000</f>
+        <v>8.09181173775513</v>
       </c>
       <c r="F66" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G66" s="6" t="s">
-        <v>245</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="G66" s="6"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="6" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>247</v>
-      </c>
-      <c r="D67" s="13"/>
-      <c r="E67" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$65/(0.9*'1 ข้อมูล'!$C$48*1000*0.9*'3 ขนาดบ่อ'!$E$66)*1000000</f>
-        <v>102.944444444444</v>
-      </c>
-      <c r="F67" s="6" t="s">
-        <v>248</v>
-      </c>
-      <c r="G67" s="6"/>
-    </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B68" s="6" t="s">
-        <v>249</v>
-      </c>
-      <c r="C68" s="6" t="s">
-        <v>250</v>
-      </c>
-      <c r="D68" s="13"/>
-      <c r="E68" s="23" t="n">
-        <f aca="false">0.003*1000*'1 ข้อมูล'!$C$35*1000</f>
-        <v>600</v>
-      </c>
-      <c r="F68" s="6" t="s">
-        <v>248</v>
-      </c>
-      <c r="G68" s="6" t="s">
         <v>251</v>
       </c>
+      <c r="D67" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$66</f>
+        <v>8.09181173775513</v>
+      </c>
+      <c r="E67" s="17" t="str">
+        <f aca="false">IF(D67&lt;=0.6*'1 ข้อมูล'!$C$48,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F67" s="6"/>
+      <c r="G67" s="6" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B69" s="6" t="s">
-        <v>252</v>
-      </c>
-      <c r="C69" s="6" t="s">
+      <c r="B69" s="4" t="s">
         <v>253</v>
       </c>
-      <c r="D69" s="13"/>
-      <c r="E69" s="23" t="n">
-        <f aca="false">FLOOR(113/MAX('3 ขนาดบ่อ'!$E$67,'3 ขนาดบ่อ'!$E$68)*1000,25)</f>
-        <v>175</v>
-      </c>
-      <c r="F69" s="6" t="s">
-        <v>254</v>
-      </c>
-      <c r="G69" s="6"/>
+      <c r="C69" s="5"/>
+      <c r="D69" s="5"/>
+      <c r="E69" s="5"/>
+      <c r="F69" s="5"/>
+      <c r="G69" s="5"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B70" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="C70" s="6" t="s">
         <v>255</v>
       </c>
-      <c r="C70" s="6"/>
-      <c r="D70" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$69</f>
-        <v>175</v>
-      </c>
-      <c r="E70" s="17" t="str">
-        <f aca="false">IF(D70&gt;=100,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
-        <v>ผ่าน ✔</v>
-      </c>
-      <c r="F70" s="6"/>
+      <c r="D70" s="13"/>
+      <c r="E70" s="23" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$42*'3 ขนาดบ่อ'!$E$56^3/6</f>
+        <v>2.82528</v>
+      </c>
+      <c r="F70" s="6" t="s">
+        <v>246</v>
+      </c>
       <c r="G70" s="6" t="s">
         <v>256</v>
       </c>
     </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B71" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="D71" s="13"/>
+      <c r="E71" s="23" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$50*'3 ขนาดบ่อ'!$E$70</f>
+        <v>4.802976</v>
+      </c>
+      <c r="F71" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="G71" s="6"/>
+    </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B72" s="4" t="s">
-        <v>257</v>
-      </c>
-      <c r="C72" s="5"/>
-      <c r="D72" s="5"/>
-      <c r="E72" s="5"/>
-      <c r="F72" s="5"/>
-      <c r="G72" s="5"/>
+      <c r="B72" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C72" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="D72" s="13"/>
+      <c r="E72" s="23" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$36-'1 ข้อมูล'!$C$38-0.006</f>
+        <v>0.144</v>
+      </c>
+      <c r="F72" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G72" s="6" t="s">
+        <v>261</v>
+      </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B73" s="6" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="D73" s="13"/>
       <c r="E73" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$31+'3 ขนาดบ่อ'!$E$12+'1 ข้อมูล'!$C$35+'3 ขนาดบ่อ'!$E$25</f>
-        <v>3.75</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$71/(0.9*'1 ข้อมูล'!$C$49*1000*0.9*'3 ขนาดบ่อ'!$E$72)*1000000</f>
+        <v>102.944444444444</v>
       </c>
       <c r="F73" s="6" t="s">
-        <v>19</v>
+        <v>264</v>
       </c>
       <c r="G73" s="6"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B74" s="6" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="D74" s="13"/>
       <c r="E74" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$45+'3 ขนาดบ่อ'!$E$37+'3 ขนาดบ่อ'!$E$73</f>
-        <v>6.35</v>
+        <f aca="false">0.003*1000*'1 ข้อมูล'!$C$36*1000</f>
+        <v>600</v>
       </c>
       <c r="F74" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G74" s="6"/>
+        <v>264</v>
+      </c>
+      <c r="G74" s="6" t="s">
+        <v>267</v>
+      </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B75" s="6" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="D75" s="13"/>
       <c r="E75" s="23" t="n">
+        <f aca="false">FLOOR(113/MAX('3 ขนาดบ่อ'!$E$73,'3 ขนาดบ่อ'!$E$74)*1000,25)</f>
+        <v>175</v>
+      </c>
+      <c r="F75" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="G75" s="6"/>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B76" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="C76" s="6"/>
+      <c r="D76" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$75</f>
+        <v>175</v>
+      </c>
+      <c r="E76" s="17" t="str">
+        <f aca="false">IF(D76&gt;=100,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F76" s="6"/>
+      <c r="G76" s="6" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B78" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="C78" s="5"/>
+      <c r="D78" s="5"/>
+      <c r="E78" s="5"/>
+      <c r="F78" s="5"/>
+      <c r="G78" s="5"/>
+    </row>
+    <row r="79" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B79" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="C79" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="D79" s="13"/>
+      <c r="E79" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$31+'3 ขนาดบ่อ'!$E$33+'3 ขนาดบ่อ'!$E$12+'1 ข้อมูล'!$C$36+'3 ขนาดบ่อ'!$E$25</f>
+        <v>4.05</v>
+      </c>
+      <c r="F79" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G79" s="6" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B80" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="C80" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="D80" s="13"/>
+      <c r="E80" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$51+'3 ขนาดบ่อ'!$E$43+'3 ขนาดบ่อ'!$E$79</f>
+        <v>6.65</v>
+      </c>
+      <c r="F80" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G80" s="6"/>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B81" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="C81" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="D81" s="13"/>
+      <c r="E81" s="23" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$9</f>
         <v>1.05</v>
       </c>
-      <c r="F75" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G75" s="6"/>
-    </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B76" s="6" t="s">
-        <v>264</v>
-      </c>
-      <c r="C76" s="6" t="s">
-        <v>265</v>
-      </c>
-      <c r="D76" s="13"/>
-      <c r="E76" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$50</f>
+      <c r="F81" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G81" s="6"/>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B82" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="C82" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="D82" s="13"/>
+      <c r="E82" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$56</f>
         <v>1.2</v>
       </c>
-      <c r="F76" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G76" s="6"/>
-    </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B77" s="6" t="s">
-        <v>266</v>
-      </c>
-      <c r="C77" s="6" t="s">
-        <v>267</v>
-      </c>
-      <c r="D77" s="13"/>
-      <c r="E77" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$74+2*'1 ข้อมูล'!$C$35</f>
-        <v>6.75</v>
-      </c>
-      <c r="F77" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G77" s="6"/>
-    </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B78" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="C78" s="6" t="s">
-        <v>267</v>
-      </c>
-      <c r="D78" s="13"/>
-      <c r="E78" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$75+2*'1 ข้อมูล'!$C$35</f>
+      <c r="F82" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G82" s="6"/>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B83" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="C83" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="D83" s="13"/>
+      <c r="E83" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$80+2*'1 ข้อมูล'!$C$36</f>
+        <v>7.05</v>
+      </c>
+      <c r="F83" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G83" s="6"/>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B84" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="C84" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="D84" s="13"/>
+      <c r="E84" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$81+2*'1 ข้อมูล'!$C$36</f>
         <v>1.45</v>
       </c>
-      <c r="F78" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G78" s="6"/>
-    </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B79" s="6" t="s">
-        <v>269</v>
-      </c>
-      <c r="C79" s="6" t="s">
-        <v>270</v>
-      </c>
-      <c r="D79" s="13"/>
-      <c r="E79" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$76+'1 ข้อมูล'!$C$36</f>
+      <c r="F84" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G84" s="6"/>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B85" s="6" t="s">
+        <v>286</v>
+      </c>
+      <c r="C85" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="D85" s="13"/>
+      <c r="E85" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$82+'1 ข้อมูล'!$C$37</f>
         <v>1.4</v>
       </c>
-      <c r="F79" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G79" s="6"/>
+      <c r="F85" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G85" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -3670,43 +3853,43 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>271</v>
+        <v>288</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>272</v>
+        <v>289</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>273</v>
+        <v>290</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>274</v>
+        <v>291</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>275</v>
+        <v>292</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>276</v>
+        <v>293</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>277</v>
+        <v>294</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>278</v>
+        <v>295</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>279</v>
+        <v>296</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C5" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$7-'1 ข้อมูล'!$C$9</f>
@@ -3717,7 +3900,7 @@
         <v>0.0111111111111111</v>
       </c>
       <c r="E5" s="9" t="n">
-        <f aca="false">(D5/('1 ข้อมูล'!$C$45*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
+        <f aca="false">(D5/('1 ข้อมูล'!$C$46*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
         <v>3.20996461989311</v>
       </c>
       <c r="F5" s="19" t="n">
@@ -3729,7 +3912,7 @@
         <v>0.203110987387621</v>
       </c>
       <c r="H5" s="12" t="n">
-        <f aca="false">G5/SQRT('1 ข้อมูล'!$C$40*F5/100)</f>
+        <f aca="false">G5/SQRT('1 ข้อมูล'!$C$41*F5/100)</f>
         <v>0.284106733367315</v>
       </c>
       <c r="I5" s="17" t="str">
@@ -3739,7 +3922,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C6" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$10-'1 ข้อมูล'!$C$9</f>
@@ -3750,7 +3933,7 @@
         <v>0.0146643518518519</v>
       </c>
       <c r="E6" s="9" t="n">
-        <f aca="false">(D6/('1 ข้อมูล'!$C$45*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
+        <f aca="false">(D6/('1 ข้อมูล'!$C$46*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
         <v>3.86222140891387</v>
       </c>
       <c r="F6" s="19" t="n">
@@ -3762,7 +3945,7 @@
         <v>0.23823817642711</v>
       </c>
       <c r="H6" s="12" t="n">
-        <f aca="false">G6/SQRT('1 ข้อมูล'!$C$40*F6/100)</f>
+        <f aca="false">G6/SQRT('1 ข้อมูล'!$C$41*F6/100)</f>
         <v>0.314156278671783</v>
       </c>
       <c r="I6" s="17" t="str">
@@ -3772,7 +3955,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C7" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8-'1 ข้อมูล'!$C$9</f>
@@ -3783,7 +3966,7 @@
         <v>0.025</v>
       </c>
       <c r="E7" s="9" t="n">
-        <f aca="false">(D7/('1 ข้อมูล'!$C$45*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
+        <f aca="false">(D7/('1 ข้อมูล'!$C$46*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
         <v>5.5117383277259</v>
       </c>
       <c r="F7" s="19" t="n">
@@ -3795,7 +3978,7 @@
         <v>0.316964233453695</v>
       </c>
       <c r="H7" s="12" t="n">
-        <f aca="false">G7/SQRT('1 ข้อมูล'!$C$40*F7/100)</f>
+        <f aca="false">G7/SQRT('1 ข้อมูล'!$C$41*F7/100)</f>
         <v>0.369237268621783</v>
       </c>
       <c r="I7" s="17" t="str">
@@ -3805,7 +3988,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C8" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8</f>
@@ -3816,7 +3999,7 @@
         <v>0.0277777777777778</v>
       </c>
       <c r="E8" s="9" t="n">
-        <f aca="false">(D8/('1 ข้อมูล'!$C$45*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
+        <f aca="false">(D8/('1 ข้อมูล'!$C$46*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
         <v>5.91280538460372</v>
       </c>
       <c r="F8" s="19" t="n">
@@ -3828,7 +4011,7 @@
         <v>0.334331822522782</v>
       </c>
       <c r="H8" s="12" t="n">
-        <f aca="false">G8/SQRT('1 ข้อมูล'!$C$40*F8/100)</f>
+        <f aca="false">G8/SQRT('1 ข้อมูล'!$C$41*F8/100)</f>
         <v>0.379470456623503</v>
       </c>
       <c r="I8" s="17" t="str">
@@ -3838,17 +4021,17 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="22" t="s">
-        <v>280</v>
+        <v>297</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="22" t="s">
-        <v>281</v>
+        <v>298</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="22" t="s">
-        <v>282</v>
+        <v>299</v>
       </c>
     </row>
   </sheetData>
@@ -3878,172 +4061,172 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>283</v>
+        <v>300</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>284</v>
+        <v>301</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>285</v>
+        <v>302</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>19</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>286</v>
+        <v>303</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="6" t="s">
-        <v>265</v>
+        <v>282</v>
       </c>
       <c r="C5" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$50</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$56</f>
         <v>1.2</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>211</v>
+        <v>227</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>287</v>
+        <v>304</v>
       </c>
       <c r="C6" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$47</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$53</f>
         <v>0.987673754729172</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>288</v>
+        <v>305</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>289</v>
+        <v>306</v>
       </c>
       <c r="C7" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$35+'1 ข้อมูล'!$C$17</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$41+'1 ข้อมูล'!$C$17</f>
         <v>0.92</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>290</v>
+        <v>307</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>291</v>
+        <v>308</v>
       </c>
       <c r="C8" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$35</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$41</f>
         <v>0.9</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>186</v>
+        <v>203</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="6" t="s">
-        <v>292</v>
+        <v>309</v>
       </c>
       <c r="C9" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$56</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$62</f>
         <v>1</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>223</v>
+        <v>239</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>293</v>
+        <v>310</v>
       </c>
       <c r="C10" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$10</f>
         <v>0.9</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>294</v>
+        <v>311</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
-        <v>295</v>
+        <v>312</v>
       </c>
       <c r="C11" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$28</f>
         <v>0.809665688762588</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>296</v>
+        <v>313</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>297</v>
+        <v>314</v>
       </c>
       <c r="C12" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8</f>
         <v>0.6</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>298</v>
+        <v>315</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="6" t="s">
-        <v>299</v>
+        <v>316</v>
       </c>
       <c r="C13" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$53</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$59</f>
         <v>0.5</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>215</v>
+        <v>231</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="6" t="s">
-        <v>300</v>
+        <v>317</v>
       </c>
       <c r="C14" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$55</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$61</f>
         <v>0.4</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>301</v>
+        <v>318</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="6" t="s">
-        <v>302</v>
+        <v>319</v>
       </c>
       <c r="C15" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$41</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$47</f>
         <v>0.3</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>303</v>
+        <v>320</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="s">
-        <v>304</v>
+        <v>321</v>
       </c>
       <c r="C16" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$20</f>
         <v>0.210686269183871</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>305</v>
+        <v>322</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="s">
-        <v>306</v>
+        <v>323</v>
       </c>
       <c r="C17" s="24" t="n">
         <f aca="false">0</f>
@@ -4079,32 +4262,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>307</v>
+        <v>324</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>308</v>
+        <v>325</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>309</v>
+        <v>326</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>310</v>
+        <v>327</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>311</v>
+        <v>328</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>312</v>
+        <v>329</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>313</v>
+        <v>330</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>314</v>
+        <v>331</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4116,7 +4299,7 @@
         <v>2.77719642805474</v>
       </c>
       <c r="D5" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B5/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B5/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
         <v>2.86619650300861</v>
       </c>
       <c r="E5" s="25" t="n">
@@ -4141,7 +4324,7 @@
         <v>4.38086341517286</v>
       </c>
       <c r="D6" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B6/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B6/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
         <v>4.48983131905459</v>
       </c>
       <c r="E6" s="25" t="n">
@@ -4166,7 +4349,7 @@
         <v>6.44060533155076</v>
       </c>
       <c r="D7" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B7/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B7/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
         <v>6.56792530595593</v>
       </c>
       <c r="E7" s="25" t="n">
@@ -4191,7 +4374,7 @@
         <v>8.99304061167301</v>
       </c>
       <c r="D8" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B8/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B8/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
         <v>9.13647413844802</v>
       </c>
       <c r="E8" s="25" t="n">
@@ -4216,7 +4399,7 @@
         <v>12.07224</v>
       </c>
       <c r="D9" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B9/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B9/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
         <v>12.2289986697729</v>
       </c>
       <c r="E9" s="25" t="n">
@@ -4241,7 +4424,7 @@
         <v>15.7101954157165</v>
       </c>
       <c r="D10" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B10/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B10/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
         <v>15.8769956216084</v>
       </c>
       <c r="E10" s="25" t="n">
@@ -4266,7 +4449,7 @@
         <v>19.9371602697676</v>
       </c>
       <c r="D11" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B11/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B11/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
         <v>20.1102658699656</v>
       </c>
       <c r="E11" s="25" t="n">
@@ -4291,7 +4474,7 @@
         <v>24.7819058265663</v>
       </c>
       <c r="D12" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B12/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B12/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
         <v>24.9571624264048</v>
       </c>
       <c r="E12" s="25" t="n">
@@ -4316,7 +4499,7 @@
         <v>30.2719200646936</v>
       </c>
       <c r="D13" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B13/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B13/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
         <v>30.4447832233961</v>
       </c>
       <c r="E13" s="25" t="n">
@@ -4341,7 +4524,7 @@
         <v>36.4335656390862</v>
       </c>
       <c r="D14" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B14/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B14/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
         <v>36.599124528368</v>
       </c>
       <c r="E14" s="25" t="n">
@@ -4366,7 +4549,7 @@
         <v>43.2922078439065</v>
       </c>
       <c r="D15" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B15/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B15/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
         <v>43.4452054104805</v>
       </c>
       <c r="E15" s="25" t="n">
@@ -4391,7 +4574,7 @@
         <v>50.87232</v>
       </c>
       <c r="D16" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B16/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B16/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
         <v>51.0071703805085</v>
       </c>
       <c r="E16" s="25" t="n">
@@ -4416,7 +4599,7 @@
         <v>59.1975714819181</v>
       </c>
       <c r="D17" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B17/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B17/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
         <v>59.3083752175669</v>
       </c>
       <c r="E17" s="25" t="n">
@@ -4441,7 +4624,7 @@
         <v>68.2909021448919</v>
       </c>
       <c r="D18" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B18/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B18/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
         <v>68.3714596053392</v>
       </c>
       <c r="E18" s="25" t="n">
@@ -4466,7 +4649,7 @@
         <v>78.1745859249513</v>
       </c>
       <c r="D19" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B19/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B19/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
         <v>78.2184092541632</v>
       </c>
       <c r="E19" s="25" t="n">
@@ -4491,7 +4674,7 @@
         <v>88.8702856977516</v>
       </c>
       <c r="D20" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B20/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B20/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
         <v>88.8706095248216</v>
       </c>
       <c r="E20" s="25" t="n">
@@ -4516,7 +4699,7 @@
         <v>100.399100991704</v>
       </c>
       <c r="D21" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B21/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B21/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
         <v>100.348892098404</v>
       </c>
       <c r="E21" s="25" t="n">
@@ -4541,7 +4724,7 @@
         <v>112.781609794846</v>
       </c>
       <c r="D22" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B22/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B22/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
         <v>112.673575893332</v>
       </c>
       <c r="E22" s="25" t="n">
@@ -4566,7 +4749,7 @@
         <v>126.037905431355</v>
       </c>
       <c r="D23" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B23/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B23/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
         <v>125.864503176292</v>
       </c>
       <c r="E23" s="25" t="n">
@@ -4591,7 +4774,7 @@
         <v>140.187629285531</v>
       </c>
       <c r="D24" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B24/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B24/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
         <v>139.941071622383</v>
       </c>
       <c r="E24" s="25" t="n">
@@ -4616,7 +4799,7 @@
         <v>155.25</v>
       </c>
       <c r="D25" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B25/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B25/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
         <v>154.922262933655</v>
       </c>
       <c r="E25" s="25" t="n">

</xml_diff>

<commit_message>
Make compartment 3 baffle and sill cast-in-place RC (0.10 m)
V-notch plate stays SS304. Tank now 7.25 m external.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXLmoKkgGBxM2QbbegGKn7
</commit_message>
<xml_diff>
--- a/weir_design.xlsx
+++ b/weir_design.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="332">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="333">
   <si>
     <t xml:space="preserve">1) ข้อมูลออกแบบ — บ่อ 3 ช่อง: ปั๊มจุ่ม | โชว์น้ำใส | V-notch 90°</t>
   </si>
@@ -169,6 +169,12 @@
   </si>
   <si>
     <t xml:space="preserve">บังคับให้น้ำที่ลอดใต้ต้องยกตัวขึ้น</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ความหนาผนังลอดใต้ / สันล้น ช่อง 3 (คสล.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">หล่อพร้อมบ่อ</t>
   </si>
   <si>
     <t xml:space="preserve">ความเร็วลอยตัวฟองอากาศ</t>
@@ -594,10 +600,10 @@
     <t xml:space="preserve">Q ÷ (B × v ไม่เกิน 0.10)</t>
   </si>
   <si>
-    <t xml:space="preserve">ผนังลอดใต้ = แผ่น SS304 6 mm ขอบบนเสมอสันกำแพง</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ระยะผนังลอดใต้ ถึง สันล้น</t>
+    <t xml:space="preserve">ผนังลอดใต้ คสล. ขอบบนเสมอสันกำแพง ผูกเหล็กเข้าผนังบ่อ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ระยะผนังลอดใต้ ถึง สันล้น (ผิวถึงผิว)</t>
   </si>
   <si>
     <t xml:space="preserve">เท่าช่องลอด (น้ำเลี้ยวขึ้นเรียบ)</t>
@@ -609,7 +615,7 @@
     <t xml:space="preserve">ช่องลอด + 0.10</t>
   </si>
   <si>
-    <t xml:space="preserve">สันล้น = แผ่น SS304 6 mm</t>
+    <t xml:space="preserve">สันล้น คสล. หล่อพร้อมพื้น</t>
   </si>
   <si>
     <t xml:space="preserve">ความเร็วน้ำข้ามสันล้น (สูงสุด)</t>
@@ -861,10 +867,7 @@
     <t xml:space="preserve">ความยาวช่อง 3</t>
   </si>
   <si>
-    <t xml:space="preserve">รับน้ำตก + ลอดใต้–สันล้น + ช่วงตรง + กำแพงเวียร์ + ท้ายเวียร์</t>
-  </si>
-  <si>
-    <t xml:space="preserve">แผ่น SS 6 mm รวมอยู่ในระยะ</t>
+    <t xml:space="preserve">รับน้ำตก + ผนัง + ระยะห่าง + สันล้น + ช่วงตรง + กำแพงเวียร์ + ท้ายเวียร์</t>
   </si>
   <si>
     <t xml:space="preserve">ความยาวภายใน</t>
@@ -1594,7 +1597,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:E55"/>
+  <dimension ref="B1:E56"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -1919,7 +1922,7 @@
         <v>0.1</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="E27" s="6" t="s">
         <v>49</v>
@@ -1930,10 +1933,10 @@
         <v>50</v>
       </c>
       <c r="C28" s="10" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>51</v>
@@ -1944,7 +1947,7 @@
         <v>52</v>
       </c>
       <c r="C29" s="10" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>19</v>
@@ -1963,21 +1966,21 @@
       <c r="D30" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E30" s="6"/>
+      <c r="E30" s="6" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C31" s="10" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="D31" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E31" s="6" t="s">
-        <v>56</v>
-      </c>
+      <c r="E31" s="6"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="6" t="s">
@@ -1989,11 +1992,13 @@
       <c r="D32" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E32" s="6"/>
+      <c r="E32" s="6" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C33" s="10" t="n">
         <v>0.1</v>
@@ -2001,9 +2006,7 @@
       <c r="D33" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E33" s="6" t="s">
-        <v>59</v>
-      </c>
+      <c r="E33" s="6"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="6" t="s">
@@ -2023,27 +2026,27 @@
       <c r="B35" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="C35" s="11" t="n">
-        <v>0.006</v>
+      <c r="C35" s="10" t="n">
+        <v>0.1</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E35" s="6"/>
+      <c r="E35" s="6" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="C36" s="10" t="n">
-        <v>0.2</v>
+        <v>64</v>
+      </c>
+      <c r="C36" s="11" t="n">
+        <v>0.006</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E36" s="6" t="s">
-        <v>64</v>
-      </c>
+      <c r="E36" s="6"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="6" t="s">
@@ -2055,41 +2058,43 @@
       <c r="D37" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E37" s="6"/>
+      <c r="E37" s="6" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C38" s="10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E38" s="6"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B39" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C39" s="10" t="n">
         <v>0.05</v>
       </c>
-      <c r="D38" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E38" s="6" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C40" s="5"/>
-      <c r="D40" s="5"/>
-      <c r="E40" s="5"/>
+      <c r="D39" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="C41" s="12" t="n">
-        <v>9.81</v>
-      </c>
-      <c r="D41" s="6" t="s">
+      <c r="B41" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="E41" s="6"/>
+      <c r="C41" s="5"/>
+      <c r="D41" s="5"/>
+      <c r="E41" s="5"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="6" t="s">
@@ -2107,25 +2112,23 @@
       <c r="B43" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="C43" s="13" t="n">
-        <v>1.38</v>
+      <c r="C43" s="12" t="n">
+        <v>9.81</v>
       </c>
       <c r="D43" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="E43" s="6" t="s">
-        <v>75</v>
-      </c>
+      <c r="E43" s="6"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C44" s="13" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="D44" s="6" t="s">
         <v>76</v>
-      </c>
-      <c r="C44" s="13" t="n">
-        <v>0.578</v>
-      </c>
-      <c r="D44" s="6" t="s">
-        <v>74</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>77</v>
@@ -2135,28 +2138,28 @@
       <c r="B45" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="C45" s="14" t="n">
-        <v>0.00085</v>
+      <c r="C45" s="13" t="n">
+        <v>0.578</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>19</v>
+        <v>76</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C46" s="14" t="n">
+        <v>0.00085</v>
+      </c>
+      <c r="D46" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E46" s="6" t="s">
         <v>79</v>
-      </c>
-      <c r="C46" s="12" t="n">
-        <v>1.84</v>
-      </c>
-      <c r="D46" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2164,10 +2167,10 @@
         <v>81</v>
       </c>
       <c r="C47" s="12" t="n">
-        <v>0.6</v>
+        <v>1.84</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E47" s="6" t="s">
         <v>82</v>
@@ -2177,80 +2180,94 @@
       <c r="B48" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="C48" s="15" t="n">
-        <v>205</v>
+      <c r="C48" s="12" t="n">
+        <v>0.6</v>
       </c>
       <c r="D48" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="E48" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="E48" s="6"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="6" t="s">
         <v>85</v>
       </c>
       <c r="C49" s="15" t="n">
-        <v>400</v>
+        <v>205</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E49" s="6"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="C50" s="15" t="n">
+        <v>400</v>
+      </c>
+      <c r="D50" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="C50" s="9" t="n">
+      <c r="E50" s="6"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B51" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C51" s="9" t="n">
         <v>1.7</v>
       </c>
-      <c r="D50" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="E50" s="6"/>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B52" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="C52" s="5"/>
-      <c r="D52" s="5"/>
-      <c r="E52" s="5"/>
+      <c r="D51" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="E51" s="6"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="C53" s="16" t="s">
+      <c r="B53" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="D53" s="6"/>
-      <c r="E53" s="6" t="s">
-        <v>90</v>
-      </c>
+      <c r="C53" s="5"/>
+      <c r="D53" s="5"/>
+      <c r="E53" s="5"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C54" s="16" t="s">
         <v>91</v>
-      </c>
-      <c r="C54" s="17" t="s">
-        <v>92</v>
       </c>
       <c r="D54" s="6"/>
       <c r="E54" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C55" s="17" t="s">
         <v>94</v>
-      </c>
-      <c r="C55" s="6" t="s">
-        <v>95</v>
       </c>
       <c r="D55" s="6"/>
       <c r="E55" s="6" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B56" s="6" t="s">
         <v>96</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D56" s="6"/>
+      <c r="E56" s="6" t="s">
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -2284,17 +2301,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="4" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="5"/>
@@ -2305,17 +2322,17 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C5" s="13" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$43</f>
+        <f aca="false">'1 ข้อมูล'!$C$44</f>
         <v>1.38</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
@@ -2323,17 +2340,17 @@
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C6" s="18" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$44*(8/15)*SQRT(2*'1 ข้อมูล'!$C$41)</f>
+        <f aca="false">'1 ข้อมูล'!$C$45*(8/15)*SQRT(2*'1 ข้อมูล'!$C$42)</f>
         <v>1.36545083661038</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
@@ -2341,7 +2358,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
@@ -2352,30 +2369,30 @@
     </row>
     <row r="9" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C10" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$7-'1 ข้อมูล'!$C$9</f>
@@ -2390,7 +2407,7 @@
         <v>14.532869095236</v>
       </c>
       <c r="F10" s="9" t="n">
-        <f aca="false">((D10/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$45)*100</f>
+        <f aca="false">((D10/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$46)*100</f>
         <v>14.5096125168743</v>
       </c>
       <c r="G10" s="20" t="n">
@@ -2401,7 +2418,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C11" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$10-'1 ข้อมูล'!$C$9</f>
@@ -2416,7 +2433,7 @@
         <v>16.2387843483091</v>
       </c>
       <c r="F11" s="9" t="n">
-        <f aca="false">((D11/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$45)*100</f>
+        <f aca="false">((D11/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$46)*100</f>
         <v>16.2227754127948</v>
       </c>
       <c r="G11" s="20" t="n">
@@ -2424,12 +2441,12 @@
         <v>0.0160089355143072</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C12" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8-'1 ข้อมูล'!$C$9</f>
@@ -2444,7 +2461,7 @@
         <v>20.1013103538681</v>
       </c>
       <c r="F12" s="9" t="n">
-        <f aca="false">((D12/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$45)*100</f>
+        <f aca="false">((D12/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$46)*100</f>
         <v>20.1017115002301</v>
       </c>
       <c r="G12" s="20" t="n">
@@ -2455,7 +2472,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="21" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C13" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8</f>
@@ -2470,7 +2487,7 @@
         <v>20.9665688762588</v>
       </c>
       <c r="F13" s="9" t="n">
-        <f aca="false">((D13/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$45)*100</f>
+        <f aca="false">((D13/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$46)*100</f>
         <v>20.9706461048468</v>
       </c>
       <c r="G13" s="20" t="n">
@@ -2478,22 +2495,22 @@
         <v>-0.00407722858800952</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="22" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="22" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="22" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -2525,12 +2542,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2538,24 +2555,24 @@
         <v>2</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>4</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="4" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -2565,10 +2582,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D7" s="13"/>
       <c r="E7" s="23" t="n">
@@ -2579,15 +2596,15 @@
         <v>19</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D8" s="13" t="n">
         <f aca="false">MAX(0.45,'3 ขนาดบ่อ'!$E$7/0.4)+'1 ข้อมูล'!$C$14</f>
@@ -2601,15 +2618,15 @@
         <v>19</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D9" s="13" t="n">
         <f aca="false">MAX(0.9,'3 ขนาดบ่อ'!$E$7/0.2)</f>
@@ -2623,15 +2640,15 @@
         <v>19</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D10" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$7+'1 ข้อมูล'!$C$15</f>
@@ -2645,15 +2662,15 @@
         <v>19</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D11" s="13"/>
       <c r="E11" s="23" t="n">
@@ -2664,15 +2681,15 @@
         <v>19</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D12" s="13" t="n">
         <f aca="false">10*'3 ขนาดบ่อ'!$E$7</f>
@@ -2686,15 +2703,15 @@
         <v>19</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="6" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D13" s="13" t="n">
         <f aca="false">4.5*'3 ขนาดบ่อ'!$E$7</f>
@@ -2708,15 +2725,15 @@
         <v>19</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="6" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D14" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$7/'3 ขนาดบ่อ'!$E$8</f>
@@ -2731,10 +2748,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="6" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D15" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$7/'3 ขนาดบ่อ'!$E$9</f>
@@ -2749,10 +2766,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D16" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$13/'3 ขนาดบ่อ'!$E$7</f>
@@ -2767,10 +2784,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D17" s="13" t="n">
         <f aca="false">'2 เวียร์'!$E$10/100</f>
@@ -2782,12 +2799,12 @@
       </c>
       <c r="F17" s="6"/>
       <c r="G17" s="6" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="4" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5"/>
@@ -2797,14 +2814,14 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="6" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D20" s="13"/>
       <c r="E20" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$30/2+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$47*PI()*'1 ข้อมูล'!$C$30^2/4))^2/(2*'1 ข้อมูล'!$C$41)</f>
+        <f aca="false">'1 ข้อมูล'!$C$31/2+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$48*PI()*'1 ข้อมูล'!$C$31^2/4))^2/(2*'1 ข้อมูล'!$C$42)</f>
         <v>0.210686269183871</v>
       </c>
       <c r="F20" s="6" t="s">
@@ -2814,10 +2831,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="6" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D21" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8-'3 ขนาดบ่อ'!$E$20</f>
@@ -2829,34 +2846,34 @@
       </c>
       <c r="F21" s="6"/>
       <c r="G21" s="6" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="6" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D22" s="13"/>
       <c r="E22" s="23" t="n">
-        <f aca="false">SQRT(2*'1 ข้อมูล'!$C$41*'3 ขนาดบ่อ'!$E$7)</f>
+        <f aca="false">SQRT(2*'1 ข้อมูล'!$C$42*'3 ขนาดบ่อ'!$E$7)</f>
         <v>2.02821123493634</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>34</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="6" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D23" s="13"/>
       <c r="E23" s="23" t="n">
@@ -2870,32 +2887,32 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="6" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D24" s="13"/>
       <c r="E24" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$22*SQRT(2*'3 ขนาดบ่อ'!$E$23/'1 ข้อมูล'!$C$41)</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$22*SQRT(2*'3 ขนาดบ่อ'!$E$23/'1 ข้อมูล'!$C$42)</f>
         <v>0.708760700266562</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="6" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D25" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$24+'1 ข้อมูล'!$C$29</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$24+'1 ข้อมูล'!$C$30</f>
         <v>0.908760700266562</v>
       </c>
       <c r="E25" s="23" t="n">
@@ -2909,7 +2926,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="4" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C27" s="5"/>
       <c r="D27" s="5"/>
@@ -2919,10 +2936,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="6" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D28" s="13"/>
       <c r="E28" s="23" t="n">
@@ -2936,10 +2953,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="6" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D29" s="13"/>
       <c r="E29" s="23" t="n">
@@ -2953,14 +2970,14 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="6" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D30" s="13"/>
       <c r="E30" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$28/'1 ข้อมูล'!$C$27*'3 ขนาดบ่อ'!$E$29</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$28/'1 ข้อมูล'!$C$28*'3 ขนาดบ่อ'!$E$29</f>
         <v>0.264550264550265</v>
       </c>
       <c r="F30" s="6" t="s">
@@ -2970,13 +2987,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="6" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D31" s="13" t="n">
-        <f aca="false">MAX('1 ข้อมูล'!$C$28,'3 ขนาดบ่อ'!$E$30)</f>
+        <f aca="false">MAX('1 ข้อมูล'!$C$29,'3 ขนาดบ่อ'!$E$30)</f>
         <v>0.5</v>
       </c>
       <c r="E31" s="23" t="n">
@@ -2987,15 +3004,15 @@
         <v>19</v>
       </c>
       <c r="G31" s="6" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="6" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="D32" s="13" t="n">
         <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$9*'1 ข้อมูล'!$C$20)</f>
@@ -3009,15 +3026,15 @@
         <v>19</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D33" s="13"/>
       <c r="E33" s="23" t="n">
@@ -3031,10 +3048,10 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="6" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D34" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$32+'1 ข้อมูล'!$C$26</f>
@@ -3048,15 +3065,15 @@
         <v>19</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="6" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D35" s="13"/>
       <c r="E35" s="23" t="n">
@@ -3070,7 +3087,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="6" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C36" s="6"/>
       <c r="D36" s="13" t="n">
@@ -3086,10 +3103,10 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D37" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8+'2 เวียร์'!$E$10/100-'3 ขนาดบ่อ'!$E$34</f>
@@ -3101,12 +3118,12 @@
       </c>
       <c r="F37" s="6"/>
       <c r="G37" s="6" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="4" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C39" s="5"/>
       <c r="D39" s="5"/>
@@ -3116,29 +3133,29 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="6" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D40" s="13"/>
       <c r="E40" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$17+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$46*'3 ขนาดบ่อ'!$E$9))^(2/3)</f>
+        <f aca="false">'1 ข้อมูล'!$C$17+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$47*'3 ขนาดบ่อ'!$E$9))^(2/3)</f>
         <v>0.0791280538460372</v>
       </c>
       <c r="F40" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D41" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$28+'1 ข้อมูล'!$C$16-'1 ข้อมูล'!$C$17</f>
@@ -3157,10 +3174,10 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="6" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D42" s="13" t="n">
         <f aca="false">10*'3 ขนาดบ่อ'!$E$40</f>
@@ -3174,15 +3191,15 @@
         <v>19</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="6" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D43" s="13"/>
       <c r="E43" s="23" t="n">
@@ -3196,7 +3213,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="6" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C44" s="6"/>
       <c r="D44" s="13" t="n">
@@ -3212,7 +3229,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="4" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C46" s="5"/>
       <c r="D46" s="5"/>
@@ -3222,10 +3239,10 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="6" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="D47" s="13" t="n">
         <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$9*'1 ข้อมูล'!$C$20)</f>
@@ -3242,10 +3259,10 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="6" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D48" s="13" t="n">
         <f aca="false">'1 ข้อมูล'!$C$21+2*'1 ข้อมูล'!$C$22</f>
@@ -3262,10 +3279,10 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="6" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D49" s="13"/>
       <c r="E49" s="23" t="n">
@@ -3279,10 +3296,10 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="6" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D50" s="13" t="n">
         <f aca="false">'1 ข้อมูล'!$C$24+2*'1 ข้อมูล'!$C$25</f>
@@ -3299,10 +3316,10 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="6" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D51" s="13"/>
       <c r="E51" s="23" t="n">
@@ -3316,10 +3333,10 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="6" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D52" s="13"/>
       <c r="E52" s="23" t="n">
@@ -3333,26 +3350,26 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="6" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D53" s="13"/>
       <c r="E53" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$41+'3 ขนาดบ่อ'!$E$40+1.5*'3 ขนาดบ่อ'!$E$52^2/(2*'1 ข้อมูล'!$C$41)</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$41+'3 ขนาดบ่อ'!$E$40+1.5*'3 ขนาดบ่อ'!$E$52^2/(2*'1 ข้อมูล'!$C$42)</f>
         <v>0.987673754729172</v>
       </c>
       <c r="F53" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G53" s="6" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="4" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C55" s="5"/>
       <c r="D55" s="5"/>
@@ -3362,10 +3379,10 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="6" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="D56" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$53+'1 ข้อมูล'!$C$19</f>
@@ -3379,12 +3396,12 @@
         <v>19</v>
       </c>
       <c r="G56" s="6" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="4" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C58" s="5"/>
       <c r="D58" s="5"/>
@@ -3394,33 +3411,33 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="6" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="D59" s="13"/>
       <c r="E59" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$8-'1 ข้อมูล'!$C$31</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$8-'1 ข้อมูล'!$C$32</f>
         <v>0.5</v>
       </c>
       <c r="F59" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G59" s="6" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="6" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D60" s="13"/>
       <c r="E60" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$9+2*'1 ข้อมูล'!$C$34</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$9+2*'1 ข้อมูล'!$C$35</f>
         <v>1.25</v>
       </c>
       <c r="F60" s="6" t="s">
@@ -3430,33 +3447,33 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="6" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D61" s="13"/>
       <c r="E61" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$59-'1 ข้อมูล'!$C$32</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$59-'1 ข้อมูล'!$C$33</f>
         <v>0.4</v>
       </c>
       <c r="F61" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G61" s="6" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="6" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="D62" s="13"/>
       <c r="E62" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$10+'1 ข้อมูล'!$C$33</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$10+'1 ข้อมูล'!$C$34</f>
         <v>1</v>
       </c>
       <c r="F62" s="6" t="s">
@@ -3466,10 +3483,10 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="6" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D63" s="13"/>
       <c r="E63" s="23" t="n">
@@ -3483,10 +3500,10 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B64" s="6" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="D64" s="13"/>
       <c r="E64" s="23" t="n">
@@ -3500,63 +3517,63 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="6" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="D65" s="13"/>
       <c r="E65" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$42*'3 ขนาดบ่อ'!$E$64^3/6</f>
+        <f aca="false">'1 ข้อมูล'!$C$43*'3 ขนาดบ่อ'!$E$64^3/6</f>
         <v>0.0485508704265308</v>
       </c>
       <c r="F65" s="6" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="G65" s="6" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="6" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D66" s="13"/>
       <c r="E66" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$65/('1 ข้อมูล'!$C$35^2/6)/1000</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$65/('1 ข้อมูล'!$C$36^2/6)/1000</f>
         <v>8.09181173775513</v>
       </c>
       <c r="F66" s="6" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G66" s="6"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="6" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="D67" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$66</f>
         <v>8.09181173775513</v>
       </c>
       <c r="E67" s="17" t="str">
-        <f aca="false">IF(D67&lt;=0.6*'1 ข้อมูล'!$C$48,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <f aca="false">IF(D67&lt;=0.6*'1 ข้อมูล'!$C$49,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
       <c r="F67" s="6"/>
       <c r="G67" s="6" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B69" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C69" s="5"/>
       <c r="D69" s="5"/>
@@ -3566,101 +3583,101 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B70" s="6" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="D70" s="13"/>
       <c r="E70" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$42*'3 ขนาดบ่อ'!$E$56^3/6</f>
+        <f aca="false">'1 ข้อมูล'!$C$43*'3 ขนาดบ่อ'!$E$56^3/6</f>
         <v>2.82528</v>
       </c>
       <c r="F70" s="6" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="G70" s="6" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B71" s="6" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="D71" s="13"/>
       <c r="E71" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$50*'3 ขนาดบ่อ'!$E$70</f>
+        <f aca="false">'1 ข้อมูล'!$C$51*'3 ขนาดบ่อ'!$E$70</f>
         <v>4.802976</v>
       </c>
       <c r="F71" s="6" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="G71" s="6"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B72" s="6" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D72" s="13"/>
       <c r="E72" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$36-'1 ข้อมูล'!$C$38-0.006</f>
+        <f aca="false">'1 ข้อมูล'!$C$37-'1 ข้อมูล'!$C$39-0.006</f>
         <v>0.144</v>
       </c>
       <c r="F72" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G72" s="6" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B73" s="6" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="D73" s="13"/>
       <c r="E73" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$71/(0.9*'1 ข้อมูล'!$C$49*1000*0.9*'3 ขนาดบ่อ'!$E$72)*1000000</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$71/(0.9*'1 ข้อมูล'!$C$50*1000*0.9*'3 ขนาดบ่อ'!$E$72)*1000000</f>
         <v>102.944444444444</v>
       </c>
       <c r="F73" s="6" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="G73" s="6"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B74" s="6" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="D74" s="13"/>
       <c r="E74" s="23" t="n">
-        <f aca="false">0.003*1000*'1 ข้อมูล'!$C$36*1000</f>
+        <f aca="false">0.003*1000*'1 ข้อมูล'!$C$37*1000</f>
         <v>600</v>
       </c>
       <c r="F74" s="6" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="G74" s="6" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B75" s="6" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="D75" s="13"/>
       <c r="E75" s="23" t="n">
@@ -3668,13 +3685,13 @@
         <v>175</v>
       </c>
       <c r="F75" s="6" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="G75" s="6"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B76" s="6" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C76" s="6"/>
       <c r="D76" s="13" t="n">
@@ -3687,12 +3704,12 @@
       </c>
       <c r="F76" s="6"/>
       <c r="G76" s="6" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B78" s="4" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C78" s="5"/>
       <c r="D78" s="5"/>
@@ -3702,34 +3719,32 @@
     </row>
     <row r="79" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B79" s="6" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D79" s="13"/>
       <c r="E79" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$31+'3 ขนาดบ่อ'!$E$33+'3 ขนาดบ่อ'!$E$12+'1 ข้อมูล'!$C$36+'3 ขนาดบ่อ'!$E$25</f>
-        <v>4.05</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$31+'1 ข้อมูล'!$C$27+'3 ขนาดบ่อ'!$E$33+'1 ข้อมูล'!$C$27+'3 ขนาดบ่อ'!$E$12+'1 ข้อมูล'!$C$37+'3 ขนาดบ่อ'!$E$25</f>
+        <v>4.25</v>
       </c>
       <c r="F79" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G79" s="6" t="s">
-        <v>276</v>
-      </c>
+      <c r="G79" s="6"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B80" s="6" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D80" s="13"/>
       <c r="E80" s="23" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$51+'3 ขนาดบ่อ'!$E$43+'3 ขนาดบ่อ'!$E$79</f>
-        <v>6.65</v>
+        <v>6.85</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>19</v>
@@ -3738,10 +3753,10 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B81" s="6" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C81" s="6" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D81" s="13"/>
       <c r="E81" s="23" t="n">
@@ -3755,10 +3770,10 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B82" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C82" s="6" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D82" s="13"/>
       <c r="E82" s="23" t="n">
@@ -3772,15 +3787,15 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B83" s="6" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C83" s="6" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D83" s="13"/>
       <c r="E83" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$80+2*'1 ข้อมูล'!$C$36</f>
-        <v>7.05</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$80+2*'1 ข้อมูล'!$C$37</f>
+        <v>7.25</v>
       </c>
       <c r="F83" s="6" t="s">
         <v>19</v>
@@ -3789,14 +3804,14 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B84" s="6" t="s">
+        <v>286</v>
+      </c>
+      <c r="C84" s="6" t="s">
         <v>285</v>
-      </c>
-      <c r="C84" s="6" t="s">
-        <v>284</v>
       </c>
       <c r="D84" s="13"/>
       <c r="E84" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$81+2*'1 ข้อมูล'!$C$36</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$81+2*'1 ข้อมูล'!$C$37</f>
         <v>1.45</v>
       </c>
       <c r="F84" s="6" t="s">
@@ -3806,14 +3821,14 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B85" s="6" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C85" s="6" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D85" s="13"/>
       <c r="E85" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$82+'1 ข้อมูล'!$C$37</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$82+'1 ข้อมูล'!$C$38</f>
         <v>1.4</v>
       </c>
       <c r="F85" s="6" t="s">
@@ -3853,43 +3868,43 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C5" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$7-'1 ข้อมูล'!$C$9</f>
@@ -3900,7 +3915,7 @@
         <v>0.0111111111111111</v>
       </c>
       <c r="E5" s="9" t="n">
-        <f aca="false">(D5/('1 ข้อมูล'!$C$46*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
+        <f aca="false">(D5/('1 ข้อมูล'!$C$47*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
         <v>3.20996461989311</v>
       </c>
       <c r="F5" s="19" t="n">
@@ -3912,7 +3927,7 @@
         <v>0.203110987387621</v>
       </c>
       <c r="H5" s="12" t="n">
-        <f aca="false">G5/SQRT('1 ข้อมูล'!$C$41*F5/100)</f>
+        <f aca="false">G5/SQRT('1 ข้อมูล'!$C$42*F5/100)</f>
         <v>0.284106733367315</v>
       </c>
       <c r="I5" s="17" t="str">
@@ -3922,7 +3937,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C6" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$10-'1 ข้อมูล'!$C$9</f>
@@ -3933,7 +3948,7 @@
         <v>0.0146643518518519</v>
       </c>
       <c r="E6" s="9" t="n">
-        <f aca="false">(D6/('1 ข้อมูล'!$C$46*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
+        <f aca="false">(D6/('1 ข้อมูล'!$C$47*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
         <v>3.86222140891387</v>
       </c>
       <c r="F6" s="19" t="n">
@@ -3945,7 +3960,7 @@
         <v>0.23823817642711</v>
       </c>
       <c r="H6" s="12" t="n">
-        <f aca="false">G6/SQRT('1 ข้อมูล'!$C$41*F6/100)</f>
+        <f aca="false">G6/SQRT('1 ข้อมูล'!$C$42*F6/100)</f>
         <v>0.314156278671783</v>
       </c>
       <c r="I6" s="17" t="str">
@@ -3955,7 +3970,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C7" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8-'1 ข้อมูล'!$C$9</f>
@@ -3966,7 +3981,7 @@
         <v>0.025</v>
       </c>
       <c r="E7" s="9" t="n">
-        <f aca="false">(D7/('1 ข้อมูล'!$C$46*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
+        <f aca="false">(D7/('1 ข้อมูล'!$C$47*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
         <v>5.5117383277259</v>
       </c>
       <c r="F7" s="19" t="n">
@@ -3978,7 +3993,7 @@
         <v>0.316964233453695</v>
       </c>
       <c r="H7" s="12" t="n">
-        <f aca="false">G7/SQRT('1 ข้อมูล'!$C$41*F7/100)</f>
+        <f aca="false">G7/SQRT('1 ข้อมูล'!$C$42*F7/100)</f>
         <v>0.369237268621783</v>
       </c>
       <c r="I7" s="17" t="str">
@@ -3988,7 +4003,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C8" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8</f>
@@ -3999,7 +4014,7 @@
         <v>0.0277777777777778</v>
       </c>
       <c r="E8" s="9" t="n">
-        <f aca="false">(D8/('1 ข้อมูล'!$C$46*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
+        <f aca="false">(D8/('1 ข้อมูล'!$C$47*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
         <v>5.91280538460372</v>
       </c>
       <c r="F8" s="19" t="n">
@@ -4011,7 +4026,7 @@
         <v>0.334331822522782</v>
       </c>
       <c r="H8" s="12" t="n">
-        <f aca="false">G8/SQRT('1 ข้อมูล'!$C$41*F8/100)</f>
+        <f aca="false">G8/SQRT('1 ข้อมูล'!$C$42*F8/100)</f>
         <v>0.379470456623503</v>
       </c>
       <c r="I8" s="17" t="str">
@@ -4021,17 +4036,17 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="22" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="22" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="22" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
   </sheetData>
@@ -4061,172 +4076,172 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>19</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="6" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C5" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$56</f>
         <v>1.2</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C6" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$53</f>
         <v>0.987673754729172</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C7" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$41+'1 ข้อมูล'!$C$17</f>
         <v>0.92</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C8" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$41</f>
         <v>0.9</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="6" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C9" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$62</f>
         <v>1</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C10" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$10</f>
         <v>0.9</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C11" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$28</f>
         <v>0.809665688762588</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C12" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8</f>
         <v>0.6</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C13" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$59</f>
         <v>0.5</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="6" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C14" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$61</f>
         <v>0.4</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="6" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C15" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$47</f>
         <v>0.3</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C16" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$20</f>
         <v>0.210686269183871</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C17" s="24" t="n">
         <f aca="false">0</f>
@@ -4262,32 +4277,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4299,7 +4314,7 @@
         <v>2.77719642805474</v>
       </c>
       <c r="D5" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B5/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B5/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
         <v>2.86619650300861</v>
       </c>
       <c r="E5" s="25" t="n">
@@ -4324,7 +4339,7 @@
         <v>4.38086341517286</v>
       </c>
       <c r="D6" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B6/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B6/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
         <v>4.48983131905459</v>
       </c>
       <c r="E6" s="25" t="n">
@@ -4349,7 +4364,7 @@
         <v>6.44060533155076</v>
       </c>
       <c r="D7" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B7/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B7/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
         <v>6.56792530595593</v>
       </c>
       <c r="E7" s="25" t="n">
@@ -4374,7 +4389,7 @@
         <v>8.99304061167301</v>
       </c>
       <c r="D8" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B8/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B8/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
         <v>9.13647413844802</v>
       </c>
       <c r="E8" s="25" t="n">
@@ -4399,7 +4414,7 @@
         <v>12.07224</v>
       </c>
       <c r="D9" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B9/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B9/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
         <v>12.2289986697729</v>
       </c>
       <c r="E9" s="25" t="n">
@@ -4424,7 +4439,7 @@
         <v>15.7101954157165</v>
       </c>
       <c r="D10" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B10/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B10/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
         <v>15.8769956216084</v>
       </c>
       <c r="E10" s="25" t="n">
@@ -4449,7 +4464,7 @@
         <v>19.9371602697676</v>
       </c>
       <c r="D11" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B11/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B11/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
         <v>20.1102658699656</v>
       </c>
       <c r="E11" s="25" t="n">
@@ -4474,7 +4489,7 @@
         <v>24.7819058265663</v>
       </c>
       <c r="D12" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B12/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B12/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
         <v>24.9571624264048</v>
       </c>
       <c r="E12" s="25" t="n">
@@ -4499,7 +4514,7 @@
         <v>30.2719200646936</v>
       </c>
       <c r="D13" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B13/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B13/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
         <v>30.4447832233961</v>
       </c>
       <c r="E13" s="25" t="n">
@@ -4524,7 +4539,7 @@
         <v>36.4335656390862</v>
       </c>
       <c r="D14" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B14/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B14/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
         <v>36.599124528368</v>
       </c>
       <c r="E14" s="25" t="n">
@@ -4549,7 +4564,7 @@
         <v>43.2922078439065</v>
       </c>
       <c r="D15" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B15/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B15/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
         <v>43.4452054104805</v>
       </c>
       <c r="E15" s="25" t="n">
@@ -4574,7 +4589,7 @@
         <v>50.87232</v>
       </c>
       <c r="D16" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B16/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B16/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
         <v>51.0071703805085</v>
       </c>
       <c r="E16" s="25" t="n">
@@ -4599,7 +4614,7 @@
         <v>59.1975714819181</v>
       </c>
       <c r="D17" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B17/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B17/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
         <v>59.3083752175669</v>
       </c>
       <c r="E17" s="25" t="n">
@@ -4624,7 +4639,7 @@
         <v>68.2909021448919</v>
       </c>
       <c r="D18" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B18/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B18/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
         <v>68.3714596053392</v>
       </c>
       <c r="E18" s="25" t="n">
@@ -4649,7 +4664,7 @@
         <v>78.1745859249513</v>
       </c>
       <c r="D19" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B19/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B19/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
         <v>78.2184092541632</v>
       </c>
       <c r="E19" s="25" t="n">
@@ -4674,7 +4689,7 @@
         <v>88.8702856977516</v>
       </c>
       <c r="D20" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B20/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B20/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
         <v>88.8706095248216</v>
       </c>
       <c r="E20" s="25" t="n">
@@ -4699,7 +4714,7 @@
         <v>100.399100991704</v>
       </c>
       <c r="D21" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B21/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B21/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
         <v>100.348892098404</v>
       </c>
       <c r="E21" s="25" t="n">
@@ -4724,7 +4739,7 @@
         <v>112.781609794846</v>
       </c>
       <c r="D22" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B22/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B22/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
         <v>112.673575893332</v>
       </c>
       <c r="E22" s="25" t="n">
@@ -4749,7 +4764,7 @@
         <v>126.037905431355</v>
       </c>
       <c r="D23" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B23/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B23/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
         <v>125.864503176292</v>
       </c>
       <c r="E23" s="25" t="n">
@@ -4774,7 +4789,7 @@
         <v>140.187629285531</v>
       </c>
       <c r="D24" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B24/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B24/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
         <v>139.941071622383</v>
       </c>
       <c r="E24" s="25" t="n">
@@ -4799,7 +4814,7 @@
         <v>155.25</v>
       </c>
       <c r="D25" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B25/100+'1 ข้อมูล'!$C$45)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B25/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
         <v>154.922262933655</v>
       </c>
       <c r="E25" s="25" t="n">

</xml_diff>

<commit_message>
Remove compartment 3 baffle and sill (tank back to 6.75 m)
Falling sheet from compartment 2 has little energy; the 0.50 m plunge
zone and 2.10 m straight approach settle the flow. V-notch stays SS304.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXLmoKkgGBxM2QbbegGKn7
</commit_message>
<xml_diff>
--- a/weir_design.xlsx
+++ b/weir_design.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="316">
   <si>
     <t xml:space="preserve">1) ข้อมูลออกแบบ — บ่อ 3 ช่อง: ปั๊มจุ่ม | โชว์น้ำใส | V-notch 90°</t>
   </si>
@@ -163,18 +163,6 @@
   </si>
   <si>
     <t xml:space="preserve">ไม่ให้เกิดกระแสวน / ยกปั๊มขึ้นซ่อมได้</t>
-  </si>
-  <si>
-    <t xml:space="preserve">สันล้นช่อง 3 สูงกว่าช่องลอดใต้</t>
-  </si>
-  <si>
-    <t xml:space="preserve">บังคับให้น้ำที่ลอดใต้ต้องยกตัวขึ้น</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ความหนาผนังลอดใต้ / สันล้น ช่อง 3 (คสล.)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">หล่อพร้อมบ่อ</t>
   </si>
   <si>
     <t xml:space="preserve">ความเร็วลอยตัวฟองอากาศ</t>
@@ -564,7 +552,7 @@
     <t xml:space="preserve">ม่านน้ำพุ่งไกล + เผื่อ 0.20</t>
   </si>
   <si>
-    <t xml:space="preserve">ค. โซนรับน้ำตก + ผนังลอดใต้ + สันล้น ช่อง 3 (ทำให้น้ำนิ่งก่อนเข้าช่วงตรง)</t>
+    <t xml:space="preserve">ค. โซนรับน้ำตก ช่อง 3 (ให้ฟองลอยขึ้นและคลื่นสลายก่อนเข้าช่วงตรง)</t>
   </si>
   <si>
     <t xml:space="preserve">ความลึกน้ำช่อง 3 สูงสุด</t>
@@ -591,93 +579,54 @@
     <t xml:space="preserve">MAX(ระยะทำงาน 0.50, ระยะฟอง)</t>
   </si>
   <si>
-    <t xml:space="preserve">ฟองลอยหมดก่อนถึงผนังลอดใต้</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ช่องลอดใต้ผนัง ช่อง 3</t>
+    <t xml:space="preserve">ฟองลอยขึ้นผิวน้ำก่อนเข้าช่วงตรง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ง. ช่อง 2 โชว์น้ำใส</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ชั้นน้ำบนพื้นยก (สูงสุด)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">สันปลาย + (Q ÷ (1.84 B))^(2/3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">รายละเอียดทุกกรณีในชีต 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ระดับผิวพื้นยก</t>
+  </si>
+  <si>
+    <t xml:space="preserve">น้ำช่อง 3 + 0.10 − สันปลาย</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ความยาวช่อง 2 ขั้นต่ำ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 × ชั้นน้ำ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ให้ผิวน้ำเรียบหลังขึ้นขั้น</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ความยาวช่อง 2 ที่ใช้</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ค่าที่เลือก (ชีต 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ตรวจ: ความยาวช่อง 2 ≥ ขั้นต่ำ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">จ. ช่อง 1 รับน้ำ + ปั๊มจุ่ม</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ช่องลอดใต้ผนังกั้น</t>
   </si>
   <si>
     <t xml:space="preserve">Q ÷ (B × v ไม่เกิน 0.10)</t>
   </si>
   <si>
-    <t xml:space="preserve">ผนังลอดใต้ คสล. ขอบบนเสมอสันกำแพง ผูกเหล็กเข้าผนังบ่อ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ระยะผนังลอดใต้ ถึง สันล้น (ผิวถึงผิว)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">เท่าช่องลอด (น้ำเลี้ยวขึ้นเรียบ)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ความสูงสันล้น</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ช่องลอด + 0.10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">สันล้น คสล. หล่อพร้อมพื้น</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ความเร็วน้ำข้ามสันล้น (สูงสุด)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Q ÷ (B × (น้ำช่อง 3 − สันล้น))</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ตรวจ: ความเร็วข้ามสันล้น ≤ 0.10 m/s</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ตรวจ: น้ำเหนือสันล้น ที่น้ำต่ำสุด (m)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">≥ 0.10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">น้ำ 50 m³/h ยังข้ามสันได้สบาย</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ง. ช่อง 2 โชว์น้ำใส</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ชั้นน้ำบนพื้นยก (สูงสุด)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">สันปลาย + (Q ÷ (1.84 B))^(2/3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">รายละเอียดทุกกรณีในชีต 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ระดับผิวพื้นยก</t>
-  </si>
-  <si>
-    <t xml:space="preserve">น้ำช่อง 3 + 0.10 − สันปลาย</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ความยาวช่อง 2 ขั้นต่ำ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10 × ชั้นน้ำ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ให้ผิวน้ำเรียบหลังขึ้นขั้น</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ความยาวช่อง 2 ที่ใช้</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ค่าที่เลือก (ชีต 1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ตรวจ: ความยาวช่อง 2 ≥ ขั้นต่ำ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">จ. ช่อง 1 รับน้ำ + ปั๊มจุ่ม</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ช่องลอดใต้ผนังกั้น</t>
-  </si>
-  <si>
     <t xml:space="preserve">โซนน้ำเข้า</t>
   </si>
   <si>
@@ -867,7 +816,7 @@
     <t xml:space="preserve">ความยาวช่อง 3</t>
   </si>
   <si>
-    <t xml:space="preserve">รับน้ำตก + ผนัง + ระยะห่าง + สันล้น + ช่วงตรง + กำแพงเวียร์ + ท้ายเวียร์</t>
+    <t xml:space="preserve">รับน้ำตก + ช่วงตรง + กำแพงเวียร์ + ท้ายเวียร์</t>
   </si>
   <si>
     <t xml:space="preserve">ความยาวภายใน</t>
@@ -1597,7 +1546,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:E56"/>
+  <dimension ref="B1:E54"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -1908,7 +1857,7 @@
         <v>0.1</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>47</v>
@@ -1919,7 +1868,7 @@
         <v>48</v>
       </c>
       <c r="C27" s="10" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>19</v>
@@ -1933,10 +1882,10 @@
         <v>50</v>
       </c>
       <c r="C28" s="10" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>51</v>
@@ -1947,35 +1896,33 @@
         <v>52</v>
       </c>
       <c r="C29" s="10" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E29" s="6" t="s">
-        <v>53</v>
-      </c>
+      <c r="E29" s="6"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C30" s="10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E30" s="6" t="s">
         <v>54</v>
-      </c>
-      <c r="C30" s="10" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D30" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E30" s="6" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C31" s="10" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="D31" s="6" t="s">
         <v>19</v>
@@ -1984,7 +1931,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C32" s="10" t="n">
         <v>0.1</v>
@@ -1993,12 +1940,12 @@
         <v>19</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C33" s="10" t="n">
         <v>0.1</v>
@@ -2006,42 +1953,42 @@
       <c r="D33" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E33" s="6"/>
+      <c r="E33" s="6" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="C34" s="10" t="n">
-        <v>0.1</v>
+      <c r="C34" s="11" t="n">
+        <v>0.006</v>
       </c>
       <c r="D34" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E34" s="6" t="s">
-        <v>61</v>
-      </c>
+      <c r="E34" s="6"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C35" s="10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E35" s="6" t="s">
         <v>62</v>
-      </c>
-      <c r="C35" s="10" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D35" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E35" s="6" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="C36" s="11" t="n">
-        <v>0.006</v>
+        <v>63</v>
+      </c>
+      <c r="C36" s="10" t="n">
+        <v>0.2</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>19</v>
@@ -2050,224 +1997,198 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C37" s="10" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E37" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="C37" s="10" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D37" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E37" s="6" t="s">
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B39" s="4" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="6" t="s">
+      <c r="C39" s="5"/>
+      <c r="D39" s="5"/>
+      <c r="E39" s="5"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B40" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="C38" s="10" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D38" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E38" s="6"/>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="6" t="s">
+      <c r="C40" s="12" t="n">
+        <v>9.81</v>
+      </c>
+      <c r="D40" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="C39" s="10" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="D39" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E39" s="6" t="s">
+      <c r="E40" s="6"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B41" s="6" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="4" t="s">
+      <c r="C41" s="12" t="n">
+        <v>9.81</v>
+      </c>
+      <c r="D41" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="C41" s="5"/>
-      <c r="D41" s="5"/>
-      <c r="E41" s="5"/>
+      <c r="E41" s="6"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="C42" s="12" t="n">
-        <v>9.81</v>
+      <c r="C42" s="13" t="n">
+        <v>1.38</v>
       </c>
       <c r="D42" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="E42" s="6"/>
+      <c r="E42" s="6" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="C43" s="12" t="n">
-        <v>9.81</v>
+        <v>74</v>
+      </c>
+      <c r="C43" s="13" t="n">
+        <v>0.578</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="E43" s="6"/>
+        <v>72</v>
+      </c>
+      <c r="E43" s="6" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C44" s="14" t="n">
+        <v>0.00085</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E44" s="6" t="s">
         <v>75</v>
-      </c>
-      <c r="C44" s="13" t="n">
-        <v>1.38</v>
-      </c>
-      <c r="D44" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C45" s="12" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="E45" s="6" t="s">
         <v>78</v>
-      </c>
-      <c r="C45" s="13" t="n">
-        <v>0.578</v>
-      </c>
-      <c r="D45" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="E45" s="6" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="C46" s="12" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D46" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="E46" s="6" t="s">
         <v>80</v>
-      </c>
-      <c r="C46" s="14" t="n">
-        <v>0.00085</v>
-      </c>
-      <c r="D46" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="C47" s="12" t="n">
-        <v>1.84</v>
+      <c r="C47" s="15" t="n">
+        <v>205</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="E47" s="6" t="s">
         <v>82</v>
       </c>
+      <c r="E47" s="6"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="C48" s="12" t="n">
-        <v>0.6</v>
+      <c r="C48" s="15" t="n">
+        <v>400</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="E48" s="6" t="s">
-        <v>84</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="E48" s="6"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C49" s="9" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="D49" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="E49" s="6"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B51" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="C49" s="15" t="n">
-        <v>205</v>
-      </c>
-      <c r="D49" s="6" t="s">
+      <c r="C51" s="5"/>
+      <c r="D51" s="5"/>
+      <c r="E51" s="5"/>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B52" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="E49" s="6"/>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B50" s="6" t="s">
+      <c r="C52" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="C50" s="15" t="n">
-        <v>400</v>
-      </c>
-      <c r="D50" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="E50" s="6"/>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="6" t="s">
+      <c r="D52" s="6"/>
+      <c r="E52" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="C51" s="9" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="D51" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="E51" s="6"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="4" t="s">
+      <c r="B53" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="C53" s="5"/>
-      <c r="D53" s="5"/>
-      <c r="E53" s="5"/>
+      <c r="C53" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="D53" s="6"/>
+      <c r="E53" s="6" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="C54" s="16" t="s">
-        <v>91</v>
+        <v>92</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>93</v>
       </c>
       <c r="D54" s="6"/>
       <c r="E54" s="6" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B55" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="C55" s="17" t="s">
         <v>94</v>
-      </c>
-      <c r="D55" s="6"/>
-      <c r="E55" s="6" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B56" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="D56" s="6"/>
-      <c r="E56" s="6" t="s">
-        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -2301,17 +2222,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="4" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="5"/>
@@ -2322,17 +2243,17 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="6" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C5" s="13" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$44</f>
+        <f aca="false">'1 ข้อมูล'!$C$42</f>
         <v>1.38</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
@@ -2340,17 +2261,17 @@
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C6" s="18" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$45*(8/15)*SQRT(2*'1 ข้อมูล'!$C$42)</f>
+        <f aca="false">'1 ข้อมูล'!$C$43*(8/15)*SQRT(2*'1 ข้อมูล'!$C$40)</f>
         <v>1.36545083661038</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
@@ -2358,7 +2279,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="4" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
@@ -2369,30 +2290,30 @@
     </row>
     <row r="9" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="G9" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="H9" s="3" t="s">
         <v>109</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C10" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$7-'1 ข้อมูล'!$C$9</f>
@@ -2407,7 +2328,7 @@
         <v>14.532869095236</v>
       </c>
       <c r="F10" s="9" t="n">
-        <f aca="false">((D10/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$46)*100</f>
+        <f aca="false">((D10/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$44)*100</f>
         <v>14.5096125168743</v>
       </c>
       <c r="G10" s="20" t="n">
@@ -2418,7 +2339,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="C11" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$10-'1 ข้อมูล'!$C$9</f>
@@ -2433,7 +2354,7 @@
         <v>16.2387843483091</v>
       </c>
       <c r="F11" s="9" t="n">
-        <f aca="false">((D11/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$46)*100</f>
+        <f aca="false">((D11/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$44)*100</f>
         <v>16.2227754127948</v>
       </c>
       <c r="G11" s="20" t="n">
@@ -2441,12 +2362,12 @@
         <v>0.0160089355143072</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C12" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8-'1 ข้อมูล'!$C$9</f>
@@ -2461,7 +2382,7 @@
         <v>20.1013103538681</v>
       </c>
       <c r="F12" s="9" t="n">
-        <f aca="false">((D12/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$46)*100</f>
+        <f aca="false">((D12/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$44)*100</f>
         <v>20.1017115002301</v>
       </c>
       <c r="G12" s="20" t="n">
@@ -2472,7 +2393,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="21" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C13" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8</f>
@@ -2487,7 +2408,7 @@
         <v>20.9665688762588</v>
       </c>
       <c r="F13" s="9" t="n">
-        <f aca="false">((D13/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$46)*100</f>
+        <f aca="false">((D13/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$44)*100</f>
         <v>20.9706461048468</v>
       </c>
       <c r="G13" s="20" t="n">
@@ -2495,22 +2416,22 @@
         <v>-0.00407722858800952</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="22" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="22" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="22" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>
@@ -2529,7 +2450,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:G85"/>
+  <dimension ref="B1:G79"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -2542,12 +2463,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2555,24 +2476,24 @@
         <v>2</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>4</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="4" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -2582,10 +2503,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="D7" s="13"/>
       <c r="E7" s="23" t="n">
@@ -2596,15 +2517,15 @@
         <v>19</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="D8" s="13" t="n">
         <f aca="false">MAX(0.45,'3 ขนาดบ่อ'!$E$7/0.4)+'1 ข้อมูล'!$C$14</f>
@@ -2618,15 +2539,15 @@
         <v>19</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="6" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="D9" s="13" t="n">
         <f aca="false">MAX(0.9,'3 ขนาดบ่อ'!$E$7/0.2)</f>
@@ -2640,15 +2561,15 @@
         <v>19</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="D10" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$7+'1 ข้อมูล'!$C$15</f>
@@ -2662,15 +2583,15 @@
         <v>19</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D11" s="13"/>
       <c r="E11" s="23" t="n">
@@ -2681,15 +2602,15 @@
         <v>19</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="D12" s="13" t="n">
         <f aca="false">10*'3 ขนาดบ่อ'!$E$7</f>
@@ -2703,15 +2624,15 @@
         <v>19</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="6" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="D13" s="13" t="n">
         <f aca="false">4.5*'3 ขนาดบ่อ'!$E$7</f>
@@ -2725,15 +2646,15 @@
         <v>19</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="6" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="D14" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$7/'3 ขนาดบ่อ'!$E$8</f>
@@ -2748,10 +2669,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="6" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="D15" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$7/'3 ขนาดบ่อ'!$E$9</f>
@@ -2766,10 +2687,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="D16" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$13/'3 ขนาดบ่อ'!$E$7</f>
@@ -2784,10 +2705,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="D17" s="13" t="n">
         <f aca="false">'2 เวียร์'!$E$10/100</f>
@@ -2799,12 +2720,12 @@
       </c>
       <c r="F17" s="6"/>
       <c r="G17" s="6" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="4" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5"/>
@@ -2814,14 +2735,14 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="6" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="D20" s="13"/>
       <c r="E20" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$31/2+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$48*PI()*'1 ข้อมูล'!$C$31^2/4))^2/(2*'1 ข้อมูล'!$C$42)</f>
+        <f aca="false">'1 ข้อมูล'!$C$29/2+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$46*PI()*'1 ข้อมูล'!$C$29^2/4))^2/(2*'1 ข้อมูล'!$C$40)</f>
         <v>0.210686269183871</v>
       </c>
       <c r="F20" s="6" t="s">
@@ -2831,10 +2752,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="6" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="D21" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8-'3 ขนาดบ่อ'!$E$20</f>
@@ -2846,34 +2767,34 @@
       </c>
       <c r="F21" s="6"/>
       <c r="G21" s="6" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="6" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="D22" s="13"/>
       <c r="E22" s="23" t="n">
-        <f aca="false">SQRT(2*'1 ข้อมูล'!$C$42*'3 ขนาดบ่อ'!$E$7)</f>
+        <f aca="false">SQRT(2*'1 ข้อมูล'!$C$40*'3 ขนาดบ่อ'!$E$7)</f>
         <v>2.02821123493634</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>34</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="6" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="D23" s="13"/>
       <c r="E23" s="23" t="n">
@@ -2887,32 +2808,32 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="6" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="D24" s="13"/>
       <c r="E24" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$22*SQRT(2*'3 ขนาดบ่อ'!$E$23/'1 ข้อมูล'!$C$42)</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$22*SQRT(2*'3 ขนาดบ่อ'!$E$23/'1 ข้อมูล'!$C$40)</f>
         <v>0.708760700266562</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="6" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D25" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$24+'1 ข้อมูล'!$C$30</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$24+'1 ข้อมูล'!$C$28</f>
         <v>0.908760700266562</v>
       </c>
       <c r="E25" s="23" t="n">
@@ -2926,7 +2847,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="4" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="C27" s="5"/>
       <c r="D27" s="5"/>
@@ -2936,10 +2857,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="6" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D28" s="13"/>
       <c r="E28" s="23" t="n">
@@ -2953,10 +2874,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="6" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="D29" s="13"/>
       <c r="E29" s="23" t="n">
@@ -2970,14 +2891,14 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="6" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D30" s="13"/>
       <c r="E30" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$28/'1 ข้อมูล'!$C$28*'3 ขนาดบ่อ'!$E$29</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$28/'1 ข้อมูล'!$C$26*'3 ขนาดบ่อ'!$E$29</f>
         <v>0.264550264550265</v>
       </c>
       <c r="F30" s="6" t="s">
@@ -2987,13 +2908,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="6" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="D31" s="13" t="n">
-        <f aca="false">MAX('1 ข้อมูล'!$C$29,'3 ขนาดบ่อ'!$E$30)</f>
+        <f aca="false">MAX('1 ข้อมูล'!$C$27,'3 ขนาดบ่อ'!$E$30)</f>
         <v>0.5</v>
       </c>
       <c r="E31" s="23" t="n">
@@ -3004,207 +2925,176 @@
         <v>19</v>
       </c>
       <c r="G31" s="6" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="C33" s="5"/>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
+      <c r="G33" s="5"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="D34" s="13"/>
+      <c r="E34" s="23" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$17+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$45*'3 ขนาดบ่อ'!$E$9))^(2/3)</f>
+        <v>0.0791280538460372</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G34" s="6" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="6" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B35" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="C35" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="D32" s="13" t="n">
+      <c r="D35" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$28+'1 ข้อมูล'!$C$16-'1 ข้อมูล'!$C$17</f>
+        <v>0.889665688762588</v>
+      </c>
+      <c r="E35" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D35,4),'1 ข้อมูล'!$C$13)</f>
+        <v>0.9</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G35" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B36" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="D36" s="13" t="n">
+        <f aca="false">10*'3 ขนาดบ่อ'!$E$34</f>
+        <v>0.791280538460372</v>
+      </c>
+      <c r="E36" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D36,4),'1 ข้อมูล'!$C$13)</f>
+        <v>0.8</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G36" s="6" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B37" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="D37" s="13"/>
+      <c r="E37" s="23" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$18</f>
+        <v>1</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G37" s="6"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B38" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="C38" s="6"/>
+      <c r="D38" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$37-'3 ขนาดบ่อ'!$E$36</f>
+        <v>0.2</v>
+      </c>
+      <c r="E38" s="17" t="str">
+        <f aca="false">IF(D38&gt;=0,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F38" s="6"/>
+      <c r="G38" s="6"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B40" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="C40" s="5"/>
+      <c r="D40" s="5"/>
+      <c r="E40" s="5"/>
+      <c r="F40" s="5"/>
+      <c r="G40" s="5"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B41" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="D41" s="13" t="n">
         <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$9*'1 ข้อมูล'!$C$20)</f>
         <v>0.264550264550265</v>
       </c>
-      <c r="E32" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D32,4),'1 ข้อมูล'!$C$13)</f>
-        <v>0.3</v>
-      </c>
-      <c r="F32" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G32" s="6" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="6" t="s">
-        <v>189</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>190</v>
-      </c>
-      <c r="D33" s="13"/>
-      <c r="E33" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$32</f>
-        <v>0.3</v>
-      </c>
-      <c r="F33" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G33" s="6"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="6" t="s">
-        <v>191</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>192</v>
-      </c>
-      <c r="D34" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$32+'1 ข้อมูล'!$C$26</f>
-        <v>0.4</v>
-      </c>
-      <c r="E34" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D34,4),'1 ข้อมูล'!$C$13)</f>
-        <v>0.4</v>
-      </c>
-      <c r="F34" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G34" s="6" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="C35" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="D35" s="13"/>
-      <c r="E35" s="23" t="n">
-        <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$9*('3 ขนาดบ่อ'!$E$28-'3 ขนาดบ่อ'!$E$34))</f>
-        <v>0.0645771105091445</v>
-      </c>
-      <c r="F35" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="G35" s="6"/>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="C36" s="6"/>
-      <c r="D36" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$35</f>
-        <v>0.0645771105091445</v>
-      </c>
-      <c r="E36" s="17" t="str">
-        <f aca="false">IF(D36&lt;=0.1,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
-        <v>ผ่าน ✔</v>
-      </c>
-      <c r="F36" s="6"/>
-      <c r="G36" s="6"/>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="D37" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$8+'2 เวียร์'!$E$10/100-'3 ขนาดบ่อ'!$E$34</f>
-        <v>0.34532869095236</v>
-      </c>
-      <c r="E37" s="17" t="str">
-        <f aca="false">IF(D37&gt;=0.1,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
-        <v>ผ่าน ✔</v>
-      </c>
-      <c r="F37" s="6"/>
-      <c r="G37" s="6" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="C39" s="5"/>
-      <c r="D39" s="5"/>
-      <c r="E39" s="5"/>
-      <c r="F39" s="5"/>
-      <c r="G39" s="5"/>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="6" t="s">
-        <v>201</v>
-      </c>
-      <c r="C40" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="D40" s="13"/>
-      <c r="E40" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$17+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$47*'3 ขนาดบ่อ'!$E$9))^(2/3)</f>
-        <v>0.0791280538460372</v>
-      </c>
-      <c r="F40" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G40" s="6" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="C41" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="D41" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$28+'1 ข้อมูล'!$C$16-'1 ข้อมูล'!$C$17</f>
-        <v>0.889665688762588</v>
-      </c>
       <c r="E41" s="23" t="n">
         <f aca="false">CEILING(ROUND(D41,4),'1 ข้อมูล'!$C$13)</f>
-        <v>0.9</v>
+        <v>0.3</v>
       </c>
       <c r="F41" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G41" s="6" t="s">
-        <v>26</v>
-      </c>
+      <c r="G41" s="6"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="6" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="D42" s="13" t="n">
-        <f aca="false">10*'3 ขนาดบ่อ'!$E$40</f>
-        <v>0.791280538460372</v>
+        <f aca="false">'1 ข้อมูล'!$C$21+2*'1 ข้อมูล'!$C$22</f>
+        <v>0.468</v>
       </c>
       <c r="E42" s="23" t="n">
         <f aca="false">CEILING(ROUND(D42,4),'1 ข้อมูล'!$C$13)</f>
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="F42" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G42" s="6" t="s">
-        <v>208</v>
-      </c>
+      <c r="G42" s="6"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="6" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="D43" s="13"/>
       <c r="E43" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$18</f>
-        <v>1</v>
+        <f aca="false">'1 ข้อมูล'!$C$23</f>
+        <v>0.1</v>
       </c>
       <c r="F43" s="6" t="s">
         <v>19</v>
@@ -3213,628 +3103,545 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="C44" s="6"/>
+        <v>201</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>202</v>
+      </c>
       <c r="D44" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$43-'3 ขนาดบ่อ'!$E$42</f>
-        <v>0.2</v>
-      </c>
-      <c r="E44" s="17" t="str">
-        <f aca="false">IF(D44&gt;=0,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
-        <v>ผ่าน ✔</v>
-      </c>
-      <c r="F44" s="6"/>
+        <f aca="false">'1 ข้อมูล'!$C$24+2*'1 ข้อมูล'!$C$25</f>
+        <v>1</v>
+      </c>
+      <c r="E44" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D44,4),'1 ข้อมูล'!$C$13)</f>
+        <v>1</v>
+      </c>
+      <c r="F44" s="6" t="s">
+        <v>19</v>
+      </c>
       <c r="G44" s="6"/>
     </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B45" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="D45" s="13"/>
+      <c r="E45" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$42+'3 ขนาดบ่อ'!$E$43+'3 ขนาดบ่อ'!$E$44</f>
+        <v>1.6</v>
+      </c>
+      <c r="F45" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G45" s="6"/>
+    </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="C46" s="5"/>
-      <c r="D46" s="5"/>
-      <c r="E46" s="5"/>
-      <c r="F46" s="5"/>
-      <c r="G46" s="5"/>
+      <c r="B46" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="D46" s="13"/>
+      <c r="E46" s="23" t="n">
+        <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$9*'3 ขนาดบ่อ'!$E$34)</f>
+        <v>0.334331822522782</v>
+      </c>
+      <c r="F46" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="G46" s="6"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="6" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="D47" s="13" t="n">
-        <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$9*'1 ข้อมูล'!$C$20)</f>
-        <v>0.264550264550265</v>
-      </c>
+        <v>208</v>
+      </c>
+      <c r="D47" s="13"/>
       <c r="E47" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D47,4),'1 ข้อมูล'!$C$13)</f>
-        <v>0.3</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$35+'3 ขนาดบ่อ'!$E$34+1.5*'3 ขนาดบ่อ'!$E$46^2/(2*'1 ข้อมูล'!$C$40)</f>
+        <v>0.987673754729172</v>
       </c>
       <c r="F47" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G47" s="6"/>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B48" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C48" s="6" t="s">
-        <v>215</v>
-      </c>
-      <c r="D48" s="13" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$21+2*'1 ข้อมูล'!$C$22</f>
-        <v>0.468</v>
-      </c>
-      <c r="E48" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D48,4),'1 ข้อมูล'!$C$13)</f>
-        <v>0.5</v>
-      </c>
-      <c r="F48" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G48" s="6"/>
+      <c r="G47" s="6" t="s">
+        <v>209</v>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B49" s="6" t="s">
-        <v>216</v>
-      </c>
-      <c r="C49" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="D49" s="13"/>
-      <c r="E49" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$23</f>
-        <v>0.1</v>
-      </c>
-      <c r="F49" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G49" s="6"/>
+      <c r="B49" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="C49" s="5"/>
+      <c r="D49" s="5"/>
+      <c r="E49" s="5"/>
+      <c r="F49" s="5"/>
+      <c r="G49" s="5"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="6" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="D50" s="13" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$24+2*'1 ข้อมูล'!$C$25</f>
-        <v>1</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$47+'1 ข้อมูล'!$C$19</f>
+        <v>1.18767375472917</v>
       </c>
       <c r="E50" s="23" t="n">
         <f aca="false">CEILING(ROUND(D50,4),'1 ข้อมูล'!$C$13)</f>
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="F50" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G50" s="6"/>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="6" t="s">
-        <v>220</v>
-      </c>
-      <c r="C51" s="6" t="s">
-        <v>221</v>
-      </c>
-      <c r="D51" s="13"/>
-      <c r="E51" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$48+'3 ขนาดบ่อ'!$E$49+'3 ขนาดบ่อ'!$E$50</f>
-        <v>1.6</v>
-      </c>
-      <c r="F51" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G51" s="6"/>
+      <c r="G50" s="6" t="s">
+        <v>213</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B52" s="6" t="s">
-        <v>222</v>
-      </c>
-      <c r="C52" s="6" t="s">
-        <v>223</v>
-      </c>
-      <c r="D52" s="13"/>
-      <c r="E52" s="23" t="n">
-        <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$9*'3 ขนาดบ่อ'!$E$40)</f>
-        <v>0.334331822522782</v>
-      </c>
-      <c r="F52" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="G52" s="6"/>
+      <c r="B52" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="C52" s="5"/>
+      <c r="D52" s="5"/>
+      <c r="E52" s="5"/>
+      <c r="F52" s="5"/>
+      <c r="G52" s="5"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="6" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="D53" s="13"/>
       <c r="E53" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$41+'3 ขนาดบ่อ'!$E$40+1.5*'3 ขนาดบ่อ'!$E$52^2/(2*'1 ข้อมูล'!$C$42)</f>
-        <v>0.987673754729172</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$8-'1 ข้อมูล'!$C$30</f>
+        <v>0.5</v>
       </c>
       <c r="F53" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G53" s="6" t="s">
-        <v>226</v>
-      </c>
+        <v>217</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B54" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="D54" s="13"/>
+      <c r="E54" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$9+2*'1 ข้อมูล'!$C$33</f>
+        <v>1.25</v>
+      </c>
+      <c r="F54" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G54" s="6"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B55" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="C55" s="5"/>
-      <c r="D55" s="5"/>
-      <c r="E55" s="5"/>
-      <c r="F55" s="5"/>
-      <c r="G55" s="5"/>
+      <c r="B55" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="D55" s="13"/>
+      <c r="E55" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$53-'1 ข้อมูล'!$C$31</f>
+        <v>0.4</v>
+      </c>
+      <c r="F55" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G55" s="6" t="s">
+        <v>222</v>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>224</v>
+      </c>
+      <c r="D56" s="13"/>
+      <c r="E56" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$10+'1 ข้อมูล'!$C$32</f>
+        <v>1</v>
+      </c>
+      <c r="F56" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G56" s="6"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B57" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="D57" s="13"/>
+      <c r="E57" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$56-'3 ขนาดบ่อ'!$E$55</f>
+        <v>0.6</v>
+      </c>
+      <c r="F57" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G57" s="6"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B58" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="C58" s="6" t="s">
         <v>228</v>
       </c>
-      <c r="C56" s="6" t="s">
-        <v>229</v>
-      </c>
-      <c r="D56" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$53+'1 ข้อมูล'!$C$19</f>
-        <v>1.18767375472917</v>
-      </c>
-      <c r="E56" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D56,4),'1 ข้อมูล'!$C$13)</f>
-        <v>1.2</v>
-      </c>
-      <c r="F56" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G56" s="6" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B58" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="C58" s="5"/>
-      <c r="D58" s="5"/>
-      <c r="E58" s="5"/>
-      <c r="F58" s="5"/>
-      <c r="G58" s="5"/>
+      <c r="D58" s="13"/>
+      <c r="E58" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$28-'3 ขนาดบ่อ'!$E$53</f>
+        <v>0.309665688762588</v>
+      </c>
+      <c r="F58" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G58" s="6"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="6" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D59" s="13"/>
       <c r="E59" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$8-'1 ข้อมูล'!$C$32</f>
-        <v>0.5</v>
+        <f aca="false">'1 ข้อมูล'!$C$41*'3 ขนาดบ่อ'!$E$58^3/6</f>
+        <v>0.0485508704265308</v>
       </c>
       <c r="F59" s="6" t="s">
-        <v>19</v>
+        <v>231</v>
       </c>
       <c r="G59" s="6" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="6" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="D60" s="13"/>
       <c r="E60" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$9+2*'1 ข้อมูล'!$C$35</f>
-        <v>1.25</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$59/('1 ข้อมูล'!$C$34^2/6)/1000</f>
+        <v>8.09181173775513</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>19</v>
+        <v>82</v>
       </c>
       <c r="G60" s="6"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="D61" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$60</f>
+        <v>8.09181173775513</v>
+      </c>
+      <c r="E61" s="17" t="str">
+        <f aca="false">IF(D61&lt;=0.6*'1 ข้อมูล'!$C$47,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F61" s="6"/>
+      <c r="G61" s="6" t="s">
         <v>237</v>
       </c>
-      <c r="C61" s="6" t="s">
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B63" s="4" t="s">
         <v>238</v>
       </c>
-      <c r="D61" s="13"/>
-      <c r="E61" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$59-'1 ข้อมูล'!$C$33</f>
-        <v>0.4</v>
-      </c>
-      <c r="F61" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G61" s="6" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B62" s="6" t="s">
-        <v>240</v>
-      </c>
-      <c r="C62" s="6" t="s">
-        <v>241</v>
-      </c>
-      <c r="D62" s="13"/>
-      <c r="E62" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$10+'1 ข้อมูล'!$C$34</f>
-        <v>1</v>
-      </c>
-      <c r="F62" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G62" s="6"/>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B63" s="6" t="s">
-        <v>242</v>
-      </c>
-      <c r="C63" s="6" t="s">
-        <v>243</v>
-      </c>
-      <c r="D63" s="13"/>
-      <c r="E63" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$62-'3 ขนาดบ่อ'!$E$61</f>
-        <v>0.6</v>
-      </c>
-      <c r="F63" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G63" s="6"/>
+      <c r="C63" s="5"/>
+      <c r="D63" s="5"/>
+      <c r="E63" s="5"/>
+      <c r="F63" s="5"/>
+      <c r="G63" s="5"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B64" s="6" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="D64" s="13"/>
       <c r="E64" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$28-'3 ขนาดบ่อ'!$E$59</f>
-        <v>0.309665688762588</v>
+        <f aca="false">'1 ข้อมูล'!$C$41*'3 ขนาดบ่อ'!$E$50^3/6</f>
+        <v>2.82528</v>
       </c>
       <c r="F64" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G64" s="6"/>
+        <v>231</v>
+      </c>
+      <c r="G64" s="6" t="s">
+        <v>241</v>
+      </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="6" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="D65" s="13"/>
       <c r="E65" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$43*'3 ขนาดบ่อ'!$E$64^3/6</f>
-        <v>0.0485508704265308</v>
+        <f aca="false">'1 ข้อมูล'!$C$49*'3 ขนาดบ่อ'!$E$64</f>
+        <v>4.802976</v>
       </c>
       <c r="F65" s="6" t="s">
-        <v>248</v>
-      </c>
-      <c r="G65" s="6" t="s">
-        <v>249</v>
-      </c>
+        <v>231</v>
+      </c>
+      <c r="G65" s="6"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="6" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="D66" s="13"/>
       <c r="E66" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$65/('1 ข้อมูล'!$C$36^2/6)/1000</f>
-        <v>8.09181173775513</v>
+        <f aca="false">'1 ข้อมูล'!$C$35-'1 ข้อมูล'!$C$37-0.006</f>
+        <v>0.144</v>
       </c>
       <c r="F66" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="G66" s="6"/>
+        <v>19</v>
+      </c>
+      <c r="G66" s="6" t="s">
+        <v>246</v>
+      </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="D67" s="13"/>
+      <c r="E67" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$65/(0.9*'1 ข้อมูล'!$C$48*1000*0.9*'3 ขนาดบ่อ'!$E$66)*1000000</f>
+        <v>102.944444444444</v>
+      </c>
+      <c r="F67" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="G67" s="6"/>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B68" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="D68" s="13"/>
+      <c r="E68" s="23" t="n">
+        <f aca="false">0.003*1000*'1 ข้อมูล'!$C$35*1000</f>
+        <v>600</v>
+      </c>
+      <c r="F68" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="G68" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="C67" s="6" t="s">
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B69" s="6" t="s">
         <v>253</v>
       </c>
-      <c r="D67" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$66</f>
-        <v>8.09181173775513</v>
-      </c>
-      <c r="E67" s="17" t="str">
-        <f aca="false">IF(D67&lt;=0.6*'1 ข้อมูล'!$C$49,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
-        <v>ผ่าน ✔</v>
-      </c>
-      <c r="F67" s="6"/>
-      <c r="G67" s="6" t="s">
+      <c r="C69" s="6" t="s">
         <v>254</v>
       </c>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B69" s="4" t="s">
+      <c r="D69" s="13"/>
+      <c r="E69" s="23" t="n">
+        <f aca="false">FLOOR(113/MAX('3 ขนาดบ่อ'!$E$67,'3 ขนาดบ่อ'!$E$68)*1000,25)</f>
+        <v>175</v>
+      </c>
+      <c r="F69" s="6" t="s">
         <v>255</v>
       </c>
-      <c r="C69" s="5"/>
-      <c r="D69" s="5"/>
-      <c r="E69" s="5"/>
-      <c r="F69" s="5"/>
-      <c r="G69" s="5"/>
+      <c r="G69" s="6"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B70" s="6" t="s">
         <v>256</v>
       </c>
-      <c r="C70" s="6" t="s">
+      <c r="C70" s="6"/>
+      <c r="D70" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$69</f>
+        <v>175</v>
+      </c>
+      <c r="E70" s="17" t="str">
+        <f aca="false">IF(D70&gt;=100,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F70" s="6"/>
+      <c r="G70" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="D70" s="13"/>
-      <c r="E70" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$43*'3 ขนาดบ่อ'!$E$56^3/6</f>
-        <v>2.82528</v>
-      </c>
-      <c r="F70" s="6" t="s">
-        <v>248</v>
-      </c>
-      <c r="G70" s="6" t="s">
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B72" s="4" t="s">
         <v>258</v>
       </c>
-    </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B71" s="6" t="s">
-        <v>259</v>
-      </c>
-      <c r="C71" s="6" t="s">
-        <v>260</v>
-      </c>
-      <c r="D71" s="13"/>
-      <c r="E71" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$51*'3 ขนาดบ่อ'!$E$70</f>
-        <v>4.802976</v>
-      </c>
-      <c r="F71" s="6" t="s">
-        <v>248</v>
-      </c>
-      <c r="G71" s="6"/>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B72" s="6" t="s">
-        <v>261</v>
-      </c>
-      <c r="C72" s="6" t="s">
-        <v>262</v>
-      </c>
-      <c r="D72" s="13"/>
-      <c r="E72" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$37-'1 ข้อมูล'!$C$39-0.006</f>
-        <v>0.144</v>
-      </c>
-      <c r="F72" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G72" s="6" t="s">
-        <v>263</v>
-      </c>
+      <c r="C72" s="5"/>
+      <c r="D72" s="5"/>
+      <c r="E72" s="5"/>
+      <c r="F72" s="5"/>
+      <c r="G72" s="5"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B73" s="6" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="D73" s="13"/>
       <c r="E73" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$71/(0.9*'1 ข้อมูล'!$C$50*1000*0.9*'3 ขนาดบ่อ'!$E$72)*1000000</f>
-        <v>102.944444444444</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$31+'3 ขนาดบ่อ'!$E$12+'1 ข้อมูล'!$C$35+'3 ขนาดบ่อ'!$E$25</f>
+        <v>3.75</v>
       </c>
       <c r="F73" s="6" t="s">
-        <v>266</v>
+        <v>19</v>
       </c>
       <c r="G73" s="6"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B74" s="6" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="D74" s="13"/>
       <c r="E74" s="23" t="n">
-        <f aca="false">0.003*1000*'1 ข้อมูล'!$C$37*1000</f>
-        <v>600</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$45+'3 ขนาดบ่อ'!$E$37+'3 ขนาดบ่อ'!$E$73</f>
+        <v>6.35</v>
       </c>
       <c r="F74" s="6" t="s">
-        <v>266</v>
-      </c>
-      <c r="G74" s="6" t="s">
-        <v>269</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="G74" s="6"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B75" s="6" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="D75" s="13"/>
       <c r="E75" s="23" t="n">
-        <f aca="false">FLOOR(113/MAX('3 ขนาดบ่อ'!$E$73,'3 ขนาดบ่อ'!$E$74)*1000,25)</f>
-        <v>175</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$9</f>
+        <v>1.05</v>
       </c>
       <c r="F75" s="6" t="s">
-        <v>272</v>
+        <v>19</v>
       </c>
       <c r="G75" s="6"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B76" s="6" t="s">
-        <v>273</v>
-      </c>
-      <c r="C76" s="6"/>
-      <c r="D76" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$75</f>
-        <v>175</v>
-      </c>
-      <c r="E76" s="17" t="str">
-        <f aca="false">IF(D76&gt;=100,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
-        <v>ผ่าน ✔</v>
-      </c>
-      <c r="F76" s="6"/>
-      <c r="G76" s="6" t="s">
-        <v>274</v>
-      </c>
+        <v>265</v>
+      </c>
+      <c r="C76" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="D76" s="13"/>
+      <c r="E76" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$50</f>
+        <v>1.2</v>
+      </c>
+      <c r="F76" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G76" s="6"/>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B77" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="D77" s="13"/>
+      <c r="E77" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$74+2*'1 ข้อมูล'!$C$35</f>
+        <v>6.75</v>
+      </c>
+      <c r="F77" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G77" s="6"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B78" s="4" t="s">
-        <v>275</v>
-      </c>
-      <c r="C78" s="5"/>
-      <c r="D78" s="5"/>
-      <c r="E78" s="5"/>
-      <c r="F78" s="5"/>
-      <c r="G78" s="5"/>
-    </row>
-    <row r="79" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B78" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="C78" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="D78" s="13"/>
+      <c r="E78" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$75+2*'1 ข้อมูล'!$C$35</f>
+        <v>1.45</v>
+      </c>
+      <c r="F78" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G78" s="6"/>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B79" s="6" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="D79" s="13"/>
       <c r="E79" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$31+'1 ข้อมูล'!$C$27+'3 ขนาดบ่อ'!$E$33+'1 ข้อมูล'!$C$27+'3 ขนาดบ่อ'!$E$12+'1 ข้อมูล'!$C$37+'3 ขนาดบ่อ'!$E$25</f>
-        <v>4.25</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$76+'1 ข้อมูล'!$C$36</f>
+        <v>1.4</v>
       </c>
       <c r="F79" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G79" s="6"/>
-    </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B80" s="6" t="s">
-        <v>278</v>
-      </c>
-      <c r="C80" s="6" t="s">
-        <v>279</v>
-      </c>
-      <c r="D80" s="13"/>
-      <c r="E80" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$51+'3 ขนาดบ่อ'!$E$43+'3 ขนาดบ่อ'!$E$79</f>
-        <v>6.85</v>
-      </c>
-      <c r="F80" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G80" s="6"/>
-    </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B81" s="6" t="s">
-        <v>280</v>
-      </c>
-      <c r="C81" s="6" t="s">
-        <v>281</v>
-      </c>
-      <c r="D81" s="13"/>
-      <c r="E81" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$9</f>
-        <v>1.05</v>
-      </c>
-      <c r="F81" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G81" s="6"/>
-    </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B82" s="6" t="s">
-        <v>282</v>
-      </c>
-      <c r="C82" s="6" t="s">
-        <v>283</v>
-      </c>
-      <c r="D82" s="13"/>
-      <c r="E82" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$56</f>
-        <v>1.2</v>
-      </c>
-      <c r="F82" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G82" s="6"/>
-    </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B83" s="6" t="s">
-        <v>284</v>
-      </c>
-      <c r="C83" s="6" t="s">
-        <v>285</v>
-      </c>
-      <c r="D83" s="13"/>
-      <c r="E83" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$80+2*'1 ข้อมูล'!$C$37</f>
-        <v>7.25</v>
-      </c>
-      <c r="F83" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G83" s="6"/>
-    </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B84" s="6" t="s">
-        <v>286</v>
-      </c>
-      <c r="C84" s="6" t="s">
-        <v>285</v>
-      </c>
-      <c r="D84" s="13"/>
-      <c r="E84" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$81+2*'1 ข้อมูล'!$C$37</f>
-        <v>1.45</v>
-      </c>
-      <c r="F84" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G84" s="6"/>
-    </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B85" s="6" t="s">
-        <v>287</v>
-      </c>
-      <c r="C85" s="6" t="s">
-        <v>288</v>
-      </c>
-      <c r="D85" s="13"/>
-      <c r="E85" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$82+'1 ข้อมูล'!$C$38</f>
-        <v>1.4</v>
-      </c>
-      <c r="F85" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G85" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -3868,43 +3675,43 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>289</v>
+        <v>272</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>290</v>
+        <v>273</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>291</v>
+        <v>274</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>292</v>
+        <v>275</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>293</v>
+        <v>276</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>294</v>
+        <v>277</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>295</v>
+        <v>278</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>296</v>
+        <v>279</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>297</v>
+        <v>280</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="6" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C5" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$7-'1 ข้อมูล'!$C$9</f>
@@ -3915,7 +3722,7 @@
         <v>0.0111111111111111</v>
       </c>
       <c r="E5" s="9" t="n">
-        <f aca="false">(D5/('1 ข้อมูล'!$C$47*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
+        <f aca="false">(D5/('1 ข้อมูล'!$C$45*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
         <v>3.20996461989311</v>
       </c>
       <c r="F5" s="19" t="n">
@@ -3927,7 +3734,7 @@
         <v>0.203110987387621</v>
       </c>
       <c r="H5" s="12" t="n">
-        <f aca="false">G5/SQRT('1 ข้อมูล'!$C$42*F5/100)</f>
+        <f aca="false">G5/SQRT('1 ข้อมูล'!$C$40*F5/100)</f>
         <v>0.284106733367315</v>
       </c>
       <c r="I5" s="17" t="str">
@@ -3937,7 +3744,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="C6" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$10-'1 ข้อมูล'!$C$9</f>
@@ -3948,7 +3755,7 @@
         <v>0.0146643518518519</v>
       </c>
       <c r="E6" s="9" t="n">
-        <f aca="false">(D6/('1 ข้อมูล'!$C$47*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
+        <f aca="false">(D6/('1 ข้อมูล'!$C$45*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
         <v>3.86222140891387</v>
       </c>
       <c r="F6" s="19" t="n">
@@ -3960,7 +3767,7 @@
         <v>0.23823817642711</v>
       </c>
       <c r="H6" s="12" t="n">
-        <f aca="false">G6/SQRT('1 ข้อมูล'!$C$42*F6/100)</f>
+        <f aca="false">G6/SQRT('1 ข้อมูล'!$C$40*F6/100)</f>
         <v>0.314156278671783</v>
       </c>
       <c r="I6" s="17" t="str">
@@ -3970,7 +3777,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C7" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8-'1 ข้อมูล'!$C$9</f>
@@ -3981,7 +3788,7 @@
         <v>0.025</v>
       </c>
       <c r="E7" s="9" t="n">
-        <f aca="false">(D7/('1 ข้อมูล'!$C$47*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
+        <f aca="false">(D7/('1 ข้อมูล'!$C$45*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
         <v>5.5117383277259</v>
       </c>
       <c r="F7" s="19" t="n">
@@ -3993,7 +3800,7 @@
         <v>0.316964233453695</v>
       </c>
       <c r="H7" s="12" t="n">
-        <f aca="false">G7/SQRT('1 ข้อมูล'!$C$42*F7/100)</f>
+        <f aca="false">G7/SQRT('1 ข้อมูล'!$C$40*F7/100)</f>
         <v>0.369237268621783</v>
       </c>
       <c r="I7" s="17" t="str">
@@ -4003,7 +3810,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C8" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8</f>
@@ -4014,7 +3821,7 @@
         <v>0.0277777777777778</v>
       </c>
       <c r="E8" s="9" t="n">
-        <f aca="false">(D8/('1 ข้อมูล'!$C$47*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
+        <f aca="false">(D8/('1 ข้อมูล'!$C$45*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
         <v>5.91280538460372</v>
       </c>
       <c r="F8" s="19" t="n">
@@ -4026,7 +3833,7 @@
         <v>0.334331822522782</v>
       </c>
       <c r="H8" s="12" t="n">
-        <f aca="false">G8/SQRT('1 ข้อมูล'!$C$42*F8/100)</f>
+        <f aca="false">G8/SQRT('1 ข้อมูล'!$C$40*F8/100)</f>
         <v>0.379470456623503</v>
       </c>
       <c r="I8" s="17" t="str">
@@ -4036,17 +3843,17 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="22" t="s">
-        <v>298</v>
+        <v>281</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="22" t="s">
-        <v>299</v>
+        <v>282</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="22" t="s">
-        <v>300</v>
+        <v>283</v>
       </c>
     </row>
   </sheetData>
@@ -4076,172 +3883,172 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>301</v>
+        <v>284</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>302</v>
+        <v>285</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>303</v>
+        <v>286</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>19</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>304</v>
+        <v>287</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="6" t="s">
-        <v>283</v>
+        <v>266</v>
       </c>
       <c r="C5" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$56</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$50</f>
         <v>1.2</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>229</v>
+        <v>212</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>305</v>
+        <v>288</v>
       </c>
       <c r="C6" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$53</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$47</f>
         <v>0.987673754729172</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>306</v>
+        <v>289</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>307</v>
+        <v>290</v>
       </c>
       <c r="C7" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$41+'1 ข้อมูล'!$C$17</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$35+'1 ข้อมูล'!$C$17</f>
         <v>0.92</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>308</v>
+        <v>291</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>309</v>
+        <v>292</v>
       </c>
       <c r="C8" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$41</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$35</f>
         <v>0.9</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>205</v>
+        <v>187</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="6" t="s">
-        <v>310</v>
+        <v>293</v>
       </c>
       <c r="C9" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$62</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$56</f>
         <v>1</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>241</v>
+        <v>224</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>311</v>
+        <v>294</v>
       </c>
       <c r="C10" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$10</f>
         <v>0.9</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>312</v>
+        <v>295</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
-        <v>313</v>
+        <v>296</v>
       </c>
       <c r="C11" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$28</f>
         <v>0.809665688762588</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>314</v>
+        <v>297</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>315</v>
+        <v>298</v>
       </c>
       <c r="C12" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8</f>
         <v>0.6</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>316</v>
+        <v>299</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="6" t="s">
-        <v>317</v>
+        <v>300</v>
       </c>
       <c r="C13" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$59</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$53</f>
         <v>0.5</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>233</v>
+        <v>216</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="6" t="s">
-        <v>318</v>
+        <v>301</v>
       </c>
       <c r="C14" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$61</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$55</f>
         <v>0.4</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>319</v>
+        <v>302</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="6" t="s">
-        <v>320</v>
+        <v>303</v>
       </c>
       <c r="C15" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$47</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$41</f>
         <v>0.3</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>321</v>
+        <v>304</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="s">
-        <v>322</v>
+        <v>305</v>
       </c>
       <c r="C16" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$20</f>
         <v>0.210686269183871</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>323</v>
+        <v>306</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="s">
-        <v>324</v>
+        <v>307</v>
       </c>
       <c r="C17" s="24" t="n">
         <f aca="false">0</f>
@@ -4277,32 +4084,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>325</v>
+        <v>308</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>326</v>
+        <v>309</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>327</v>
+        <v>310</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>328</v>
+        <v>311</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>329</v>
+        <v>312</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>330</v>
+        <v>313</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>331</v>
+        <v>314</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>332</v>
+        <v>315</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4314,7 +4121,7 @@
         <v>2.77719642805474</v>
       </c>
       <c r="D5" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B5/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B5/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
         <v>2.86619650300861</v>
       </c>
       <c r="E5" s="25" t="n">
@@ -4339,7 +4146,7 @@
         <v>4.38086341517286</v>
       </c>
       <c r="D6" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B6/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B6/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
         <v>4.48983131905459</v>
       </c>
       <c r="E6" s="25" t="n">
@@ -4364,7 +4171,7 @@
         <v>6.44060533155076</v>
       </c>
       <c r="D7" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B7/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B7/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
         <v>6.56792530595593</v>
       </c>
       <c r="E7" s="25" t="n">
@@ -4389,7 +4196,7 @@
         <v>8.99304061167301</v>
       </c>
       <c r="D8" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B8/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B8/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
         <v>9.13647413844802</v>
       </c>
       <c r="E8" s="25" t="n">
@@ -4414,7 +4221,7 @@
         <v>12.07224</v>
       </c>
       <c r="D9" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B9/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B9/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
         <v>12.2289986697729</v>
       </c>
       <c r="E9" s="25" t="n">
@@ -4439,7 +4246,7 @@
         <v>15.7101954157165</v>
       </c>
       <c r="D10" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B10/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B10/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
         <v>15.8769956216084</v>
       </c>
       <c r="E10" s="25" t="n">
@@ -4464,7 +4271,7 @@
         <v>19.9371602697676</v>
       </c>
       <c r="D11" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B11/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B11/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
         <v>20.1102658699656</v>
       </c>
       <c r="E11" s="25" t="n">
@@ -4489,7 +4296,7 @@
         <v>24.7819058265663</v>
       </c>
       <c r="D12" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B12/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B12/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
         <v>24.9571624264048</v>
       </c>
       <c r="E12" s="25" t="n">
@@ -4514,7 +4321,7 @@
         <v>30.2719200646936</v>
       </c>
       <c r="D13" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B13/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B13/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
         <v>30.4447832233961</v>
       </c>
       <c r="E13" s="25" t="n">
@@ -4539,7 +4346,7 @@
         <v>36.4335656390862</v>
       </c>
       <c r="D14" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B14/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B14/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
         <v>36.599124528368</v>
       </c>
       <c r="E14" s="25" t="n">
@@ -4564,7 +4371,7 @@
         <v>43.2922078439065</v>
       </c>
       <c r="D15" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B15/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B15/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
         <v>43.4452054104805</v>
       </c>
       <c r="E15" s="25" t="n">
@@ -4589,7 +4396,7 @@
         <v>50.87232</v>
       </c>
       <c r="D16" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B16/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B16/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
         <v>51.0071703805085</v>
       </c>
       <c r="E16" s="25" t="n">
@@ -4614,7 +4421,7 @@
         <v>59.1975714819181</v>
       </c>
       <c r="D17" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B17/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B17/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
         <v>59.3083752175669</v>
       </c>
       <c r="E17" s="25" t="n">
@@ -4639,7 +4446,7 @@
         <v>68.2909021448919</v>
       </c>
       <c r="D18" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B18/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B18/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
         <v>68.3714596053392</v>
       </c>
       <c r="E18" s="25" t="n">
@@ -4664,7 +4471,7 @@
         <v>78.1745859249513</v>
       </c>
       <c r="D19" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B19/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B19/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
         <v>78.2184092541632</v>
       </c>
       <c r="E19" s="25" t="n">
@@ -4689,7 +4496,7 @@
         <v>88.8702856977516</v>
       </c>
       <c r="D20" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B20/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B20/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
         <v>88.8706095248216</v>
       </c>
       <c r="E20" s="25" t="n">
@@ -4714,7 +4521,7 @@
         <v>100.399100991704</v>
       </c>
       <c r="D21" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B21/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B21/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
         <v>100.348892098404</v>
       </c>
       <c r="E21" s="25" t="n">
@@ -4739,7 +4546,7 @@
         <v>112.781609794846</v>
       </c>
       <c r="D22" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B22/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B22/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
         <v>112.673575893332</v>
       </c>
       <c r="E22" s="25" t="n">
@@ -4764,7 +4571,7 @@
         <v>126.037905431355</v>
       </c>
       <c r="D23" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B23/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B23/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
         <v>125.864503176292</v>
       </c>
       <c r="E23" s="25" t="n">
@@ -4789,7 +4596,7 @@
         <v>140.187629285531</v>
       </c>
       <c r="D24" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B24/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B24/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
         <v>139.941071622383</v>
       </c>
       <c r="E24" s="25" t="n">
@@ -4814,7 +4621,7 @@
         <v>155.25</v>
       </c>
       <c r="D25" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B25/100+'1 ข้อมูล'!$C$46)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B25/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
         <v>154.922262933655</v>
       </c>
       <c r="E25" s="25" t="n">

</xml_diff>

<commit_message>
Place BOD probe and DL10 level sensor in compartment 3
Excel computes probe tip level (+0.30, always >= 0.30 m submerged since
compartment 3 holds water at the V vertex) and DL10 mounting (+1.10,
0.29-0.50 m to water, within 0.05-1.25 m range). Drawings, dimension
sheet and animation show both sensors.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXLmoKkgGBxM2QbbegGKn7
</commit_message>
<xml_diff>
--- a/weir_design.xlsx
+++ b/weir_design.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="351">
   <si>
     <t xml:space="preserve">1) ข้อมูลออกแบบ — บ่อ 3 ช่อง: ปั๊มจุ่ม | โชว์น้ำใส | V-notch 90°</t>
   </si>
@@ -208,6 +208,45 @@
   </si>
   <si>
     <t xml:space="preserve">ความหนาแผ่นเวียร์ SS304</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BOD probe: ระยะจากต้นช่วงตรง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ช่วงต้นของช่วงตรง พ้นโซนฟอง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BOD probe: ระยะจากผนังข้าง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ชิดผนัง ไม่ขวางกลางร่องน้ำ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BOD probe: จมน้ำขั้นต่ำ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ยืนยันกับผู้ขาย WTW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BOD probe: สูงจากพื้นขั้นต่ำ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">พ้นตะกอนที่พื้น</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DL10: ระดับหน้าเซนเซอร์</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ติดคานพาดขวางเหนือจุดวัด H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DL10: ระยะวัดต่ำสุด (blanking)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Badger DL10: 50–1,250 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DL10: ระยะวัดสูงสุด</t>
   </si>
   <si>
     <t xml:space="preserve">ความหนาผนัง คสล.</t>
@@ -810,7 +849,73 @@
     <t xml:space="preserve">ผนัง 0.20 m เพียงพอ — ควบคุมด้วยเหล็กขั้นต่ำ</t>
   </si>
   <si>
-    <t xml:space="preserve">ฌ. สรุปขนาดบ่อ</t>
+    <t xml:space="preserve">ฌ. ตำแหน่งเซนเซอร์ (ช่อง 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BOD probe: ระดับปลาย probe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">กลางระหว่าง (พื้น + 0.20) กับ (ยอด V − จมขั้นต่ำ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ปัดเป็นทวีคูณ 0.05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ตรวจ: probe จมน้ำเมื่อน้ำหยุดไหล (ยอด V − ปลาย)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≥ จมขั้นต่ำ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">น้ำในช่อง 3 ค้างที่ยอด V เสมอ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ตรวจ: probe สูงจากพื้น</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≥ 0.20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BOD probe: ระยะถึงแผ่นเวียร์</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ช่วงตรง − ระยะจากต้นช่วงตรง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ตรวจ: probe อยู่เหนือน้ำของจุดวัด H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ห่างจุดวัด ≥ 0.5 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ไม่รบกวนผิวน้ำที่จุดวัด</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DL10: ระยะถึงผิวน้ำ ตอนน้ำสูงสุด</t>
+  </si>
+  <si>
+    <t xml:space="preserve">หน้าเซนเซอร์ − (P + Hmax)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DL10: ระยะถึงผิวน้ำ ตอนน้ำหยุดไหล</t>
+  </si>
+  <si>
+    <t xml:space="preserve">หน้าเซนเซอร์ − P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ตรวจ: DL10 อยู่ในช่วงวัด</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.05–1.25 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ตรวจ: หน้าเซนเซอร์ต่ำกว่าสันกำแพง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ติดคานบนสันกำแพงได้</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ญ. สรุปขนาดบ่อ</t>
   </si>
   <si>
     <t xml:space="preserve">ความยาวช่อง 3</t>
@@ -1546,7 +1651,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:E54"/>
+  <dimension ref="B1:E61"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -1974,7 +2079,7 @@
         <v>61</v>
       </c>
       <c r="C35" s="10" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>19</v>
@@ -1988,150 +2093,152 @@
         <v>63</v>
       </c>
       <c r="C36" s="10" t="n">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E36" s="6"/>
+      <c r="E36" s="6" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C37" s="10" t="n">
-        <v>0.05</v>
+        <v>0.25</v>
       </c>
       <c r="D37" s="6" t="s">
         <v>19</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B38" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C38" s="10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E38" s="6" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="C39" s="5"/>
-      <c r="D39" s="5"/>
-      <c r="E39" s="5"/>
+      <c r="B39" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C39" s="10" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="C40" s="12" t="n">
-        <v>9.81</v>
+        <v>71</v>
+      </c>
+      <c r="C40" s="10" t="n">
+        <v>0.05</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="E40" s="6"/>
+        <v>19</v>
+      </c>
+      <c r="E40" s="6" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="C41" s="12" t="n">
-        <v>9.81</v>
+        <v>73</v>
+      </c>
+      <c r="C41" s="10" t="n">
+        <v>1.25</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>70</v>
+        <v>19</v>
       </c>
       <c r="E41" s="6"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="C42" s="13" t="n">
-        <v>1.38</v>
+        <v>74</v>
+      </c>
+      <c r="C42" s="10" t="n">
+        <v>0.2</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>72</v>
+        <v>19</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="C43" s="13" t="n">
-        <v>0.578</v>
+        <v>76</v>
+      </c>
+      <c r="C43" s="10" t="n">
+        <v>0.2</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>75</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="E43" s="6"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C44" s="14" t="n">
-        <v>0.00085</v>
+        <v>77</v>
+      </c>
+      <c r="C44" s="10" t="n">
+        <v>0.05</v>
       </c>
       <c r="D44" s="6" t="s">
         <v>19</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="C45" s="12" t="n">
-        <v>1.84</v>
-      </c>
-      <c r="D45" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="E45" s="6" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="6" t="s">
+      <c r="B46" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C46" s="12" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="D46" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>80</v>
-      </c>
+      <c r="C46" s="5"/>
+      <c r="D46" s="5"/>
+      <c r="E46" s="5"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C47" s="12" t="n">
+        <v>9.81</v>
+      </c>
+      <c r="D47" s="6" t="s">
         <v>81</v>
-      </c>
-      <c r="C47" s="15" t="n">
-        <v>205</v>
-      </c>
-      <c r="D47" s="6" t="s">
-        <v>82</v>
       </c>
       <c r="E47" s="6"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C48" s="12" t="n">
+        <v>9.81</v>
+      </c>
+      <c r="D48" s="6" t="s">
         <v>83</v>
-      </c>
-      <c r="C48" s="15" t="n">
-        <v>400</v>
-      </c>
-      <c r="D48" s="6" t="s">
-        <v>82</v>
       </c>
       <c r="E48" s="6"/>
     </row>
@@ -2139,56 +2246,150 @@
       <c r="B49" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="C49" s="9" t="n">
-        <v>1.7</v>
+      <c r="C49" s="13" t="n">
+        <v>1.38</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="E49" s="6"/>
+        <v>85</v>
+      </c>
+      <c r="E49" s="6" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B50" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="C50" s="13" t="n">
+        <v>0.578</v>
+      </c>
+      <c r="D50" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="E50" s="6" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="C51" s="5"/>
-      <c r="D51" s="5"/>
-      <c r="E51" s="5"/>
+      <c r="B51" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="C51" s="14" t="n">
+        <v>0.00085</v>
+      </c>
+      <c r="D51" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E51" s="6" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="C52" s="16" t="s">
-        <v>87</v>
-      </c>
-      <c r="D52" s="6"/>
+        <v>90</v>
+      </c>
+      <c r="C52" s="12" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="D52" s="6" t="s">
+        <v>85</v>
+      </c>
       <c r="E52" s="6" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="C53" s="17" t="s">
-        <v>90</v>
-      </c>
-      <c r="D53" s="6"/>
+        <v>92</v>
+      </c>
+      <c r="C53" s="12" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D53" s="6" t="s">
+        <v>85</v>
+      </c>
       <c r="E53" s="6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="C54" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="D54" s="6"/>
-      <c r="E54" s="6" t="s">
         <v>94</v>
+      </c>
+      <c r="C54" s="15" t="n">
+        <v>205</v>
+      </c>
+      <c r="D54" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="E54" s="6"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B55" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C55" s="15" t="n">
+        <v>400</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="E55" s="6"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B56" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C56" s="9" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="D56" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="E56" s="6"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B58" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C58" s="5"/>
+      <c r="D58" s="5"/>
+      <c r="E58" s="5"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B59" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C59" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="D59" s="6"/>
+      <c r="E59" s="6" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B60" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C60" s="17" t="s">
+        <v>103</v>
+      </c>
+      <c r="D60" s="6"/>
+      <c r="E60" s="6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B61" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D61" s="6"/>
+      <c r="E61" s="6" t="s">
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -2222,17 +2423,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="4" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="5"/>
@@ -2243,17 +2444,17 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="6" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="C5" s="13" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$42</f>
+        <f aca="false">'1 ข้อมูล'!$C$49</f>
         <v>1.38</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
@@ -2261,17 +2462,17 @@
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="C6" s="18" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$43*(8/15)*SQRT(2*'1 ข้อมูล'!$C$40)</f>
+        <f aca="false">'1 ข้อมูล'!$C$50*(8/15)*SQRT(2*'1 ข้อมูล'!$C$47)</f>
         <v>1.36545083661038</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>101</v>
+        <v>114</v>
       </c>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
@@ -2279,7 +2480,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="4" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
@@ -2290,30 +2491,30 @@
     </row>
     <row r="9" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="3" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="C10" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$7-'1 ข้อมูล'!$C$9</f>
@@ -2328,7 +2529,7 @@
         <v>14.532869095236</v>
       </c>
       <c r="F10" s="9" t="n">
-        <f aca="false">((D10/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$44)*100</f>
+        <f aca="false">((D10/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$51)*100</f>
         <v>14.5096125168743</v>
       </c>
       <c r="G10" s="20" t="n">
@@ -2339,7 +2540,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
       <c r="C11" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$10-'1 ข้อมูล'!$C$9</f>
@@ -2354,7 +2555,7 @@
         <v>16.2387843483091</v>
       </c>
       <c r="F11" s="9" t="n">
-        <f aca="false">((D11/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$44)*100</f>
+        <f aca="false">((D11/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$51)*100</f>
         <v>16.2227754127948</v>
       </c>
       <c r="G11" s="20" t="n">
@@ -2362,12 +2563,12 @@
         <v>0.0160089355143072</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>112</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="C12" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8-'1 ข้อมูล'!$C$9</f>
@@ -2382,7 +2583,7 @@
         <v>20.1013103538681</v>
       </c>
       <c r="F12" s="9" t="n">
-        <f aca="false">((D12/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$44)*100</f>
+        <f aca="false">((D12/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$51)*100</f>
         <v>20.1017115002301</v>
       </c>
       <c r="G12" s="20" t="n">
@@ -2393,7 +2594,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="21" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="C13" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8</f>
@@ -2408,7 +2609,7 @@
         <v>20.9665688762588</v>
       </c>
       <c r="F13" s="9" t="n">
-        <f aca="false">((D13/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$44)*100</f>
+        <f aca="false">((D13/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$51)*100</f>
         <v>20.9706461048468</v>
       </c>
       <c r="G13" s="20" t="n">
@@ -2416,22 +2617,22 @@
         <v>-0.00407722858800952</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>115</v>
+        <v>128</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="22" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="22" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="22" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -2450,7 +2651,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:G79"/>
+  <dimension ref="B1:G90"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -2463,12 +2664,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2476,24 +2677,24 @@
         <v>2</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>122</v>
+        <v>135</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>4</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>124</v>
+        <v>137</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="4" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -2503,10 +2704,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="D7" s="13"/>
       <c r="E7" s="23" t="n">
@@ -2517,15 +2718,15 @@
         <v>19</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>129</v>
+        <v>142</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>130</v>
+        <v>143</v>
       </c>
       <c r="D8" s="13" t="n">
         <f aca="false">MAX(0.45,'3 ขนาดบ่อ'!$E$7/0.4)+'1 ข้อมูล'!$C$14</f>
@@ -2539,15 +2740,15 @@
         <v>19</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>131</v>
+        <v>144</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="6" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="D9" s="13" t="n">
         <f aca="false">MAX(0.9,'3 ขนาดบ่อ'!$E$7/0.2)</f>
@@ -2561,15 +2762,15 @@
         <v>19</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>135</v>
+        <v>148</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>136</v>
+        <v>149</v>
       </c>
       <c r="D10" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$7+'1 ข้อมูล'!$C$15</f>
@@ -2583,15 +2784,15 @@
         <v>19</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>137</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>139</v>
+        <v>152</v>
       </c>
       <c r="D11" s="13"/>
       <c r="E11" s="23" t="n">
@@ -2602,15 +2803,15 @@
         <v>19</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>142</v>
+        <v>155</v>
       </c>
       <c r="D12" s="13" t="n">
         <f aca="false">10*'3 ขนาดบ่อ'!$E$7</f>
@@ -2624,15 +2825,15 @@
         <v>19</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>143</v>
+        <v>156</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="6" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>145</v>
+        <v>158</v>
       </c>
       <c r="D13" s="13" t="n">
         <f aca="false">4.5*'3 ขนาดบ่อ'!$E$7</f>
@@ -2646,15 +2847,15 @@
         <v>19</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>146</v>
+        <v>159</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="6" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="D14" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$7/'3 ขนาดบ่อ'!$E$8</f>
@@ -2669,10 +2870,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="6" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="D15" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$7/'3 ขนาดบ่อ'!$E$9</f>
@@ -2687,10 +2888,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="s">
-        <v>151</v>
+        <v>164</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="D16" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$13/'3 ขนาดบ่อ'!$E$7</f>
@@ -2705,10 +2906,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="s">
-        <v>153</v>
+        <v>166</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>154</v>
+        <v>167</v>
       </c>
       <c r="D17" s="13" t="n">
         <f aca="false">'2 เวียร์'!$E$10/100</f>
@@ -2720,12 +2921,12 @@
       </c>
       <c r="F17" s="6"/>
       <c r="G17" s="6" t="s">
-        <v>155</v>
+        <v>168</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="4" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5"/>
@@ -2735,14 +2936,14 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="6" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>158</v>
+        <v>171</v>
       </c>
       <c r="D20" s="13"/>
       <c r="E20" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$29/2+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$46*PI()*'1 ข้อมูล'!$C$29^2/4))^2/(2*'1 ข้อมูล'!$C$40)</f>
+        <f aca="false">'1 ข้อมูล'!$C$29/2+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$53*PI()*'1 ข้อมูล'!$C$29^2/4))^2/(2*'1 ข้อมูล'!$C$47)</f>
         <v>0.210686269183871</v>
       </c>
       <c r="F20" s="6" t="s">
@@ -2752,10 +2953,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="6" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="D21" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8-'3 ขนาดบ่อ'!$E$20</f>
@@ -2767,34 +2968,34 @@
       </c>
       <c r="F21" s="6"/>
       <c r="G21" s="6" t="s">
-        <v>161</v>
+        <v>174</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="6" t="s">
-        <v>162</v>
+        <v>175</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>163</v>
+        <v>176</v>
       </c>
       <c r="D22" s="13"/>
       <c r="E22" s="23" t="n">
-        <f aca="false">SQRT(2*'1 ข้อมูล'!$C$40*'3 ขนาดบ่อ'!$E$7)</f>
+        <f aca="false">SQRT(2*'1 ข้อมูล'!$C$47*'3 ขนาดบ่อ'!$E$7)</f>
         <v>2.02821123493634</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>34</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>164</v>
+        <v>177</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="6" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>166</v>
+        <v>179</v>
       </c>
       <c r="D23" s="13"/>
       <c r="E23" s="23" t="n">
@@ -2808,29 +3009,29 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="6" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>168</v>
+        <v>181</v>
       </c>
       <c r="D24" s="13"/>
       <c r="E24" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$22*SQRT(2*'3 ขนาดบ่อ'!$E$23/'1 ข้อมูล'!$C$40)</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$22*SQRT(2*'3 ขนาดบ่อ'!$E$23/'1 ข้อมูล'!$C$47)</f>
         <v>0.708760700266562</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>169</v>
+        <v>182</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="6" t="s">
-        <v>170</v>
+        <v>183</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>171</v>
+        <v>184</v>
       </c>
       <c r="D25" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$24+'1 ข้อมูล'!$C$28</f>
@@ -2847,7 +3048,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="4" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="C27" s="5"/>
       <c r="D27" s="5"/>
@@ -2857,10 +3058,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="6" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
       <c r="D28" s="13"/>
       <c r="E28" s="23" t="n">
@@ -2874,10 +3075,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="6" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="D29" s="13"/>
       <c r="E29" s="23" t="n">
@@ -2891,10 +3092,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="6" t="s">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
       <c r="D30" s="13"/>
       <c r="E30" s="23" t="n">
@@ -2908,10 +3109,10 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="6" t="s">
-        <v>179</v>
+        <v>192</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
       <c r="D31" s="13" t="n">
         <f aca="false">MAX('1 ข้อมูล'!$C$27,'3 ขนาดบ่อ'!$E$30)</f>
@@ -2925,12 +3126,12 @@
         <v>19</v>
       </c>
       <c r="G31" s="6" t="s">
-        <v>181</v>
+        <v>194</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="4" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="C33" s="5"/>
       <c r="D33" s="5"/>
@@ -2940,29 +3141,29 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="6" t="s">
-        <v>183</v>
+        <v>196</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>184</v>
+        <v>197</v>
       </c>
       <c r="D34" s="13"/>
       <c r="E34" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$17+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$45*'3 ขนาดบ่อ'!$E$9))^(2/3)</f>
+        <f aca="false">'1 ข้อมูล'!$C$17+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$52*'3 ขนาดบ่อ'!$E$9))^(2/3)</f>
         <v>0.0791280538460372</v>
       </c>
       <c r="F34" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>185</v>
+        <v>198</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="6" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="D35" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$28+'1 ข้อมูล'!$C$16-'1 ข้อมูล'!$C$17</f>
@@ -2981,10 +3182,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="6" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="D36" s="13" t="n">
         <f aca="false">10*'3 ขนาดบ่อ'!$E$34</f>
@@ -2998,15 +3199,15 @@
         <v>19</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="6" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="D37" s="13"/>
       <c r="E37" s="23" t="n">
@@ -3020,7 +3221,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="6" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="C38" s="6"/>
       <c r="D38" s="13" t="n">
@@ -3036,7 +3237,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="4" t="s">
-        <v>194</v>
+        <v>207</v>
       </c>
       <c r="C40" s="5"/>
       <c r="D40" s="5"/>
@@ -3046,10 +3247,10 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="6" t="s">
-        <v>195</v>
+        <v>208</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="D41" s="13" t="n">
         <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$9*'1 ข้อมูล'!$C$20)</f>
@@ -3066,10 +3267,10 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="6" t="s">
-        <v>197</v>
+        <v>210</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>198</v>
+        <v>211</v>
       </c>
       <c r="D42" s="13" t="n">
         <f aca="false">'1 ข้อมูล'!$C$21+2*'1 ข้อมูล'!$C$22</f>
@@ -3086,10 +3287,10 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="6" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>200</v>
+        <v>213</v>
       </c>
       <c r="D43" s="13"/>
       <c r="E43" s="23" t="n">
@@ -3103,10 +3304,10 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="6" t="s">
-        <v>201</v>
+        <v>214</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>202</v>
+        <v>215</v>
       </c>
       <c r="D44" s="13" t="n">
         <f aca="false">'1 ข้อมูล'!$C$24+2*'1 ข้อมูล'!$C$25</f>
@@ -3123,10 +3324,10 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="6" t="s">
-        <v>203</v>
+        <v>216</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>204</v>
+        <v>217</v>
       </c>
       <c r="D45" s="13"/>
       <c r="E45" s="23" t="n">
@@ -3140,10 +3341,10 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="6" t="s">
-        <v>205</v>
+        <v>218</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>206</v>
+        <v>219</v>
       </c>
       <c r="D46" s="13"/>
       <c r="E46" s="23" t="n">
@@ -3157,26 +3358,26 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="6" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>208</v>
+        <v>221</v>
       </c>
       <c r="D47" s="13"/>
       <c r="E47" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$35+'3 ขนาดบ่อ'!$E$34+1.5*'3 ขนาดบ่อ'!$E$46^2/(2*'1 ข้อมูล'!$C$40)</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$35+'3 ขนาดบ่อ'!$E$34+1.5*'3 ขนาดบ่อ'!$E$46^2/(2*'1 ข้อมูล'!$C$47)</f>
         <v>0.987673754729172</v>
       </c>
       <c r="F47" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G47" s="6" t="s">
-        <v>209</v>
+        <v>222</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="4" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
       <c r="C49" s="5"/>
       <c r="D49" s="5"/>
@@ -3186,10 +3387,10 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="6" t="s">
-        <v>211</v>
+        <v>224</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>212</v>
+        <v>225</v>
       </c>
       <c r="D50" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$47+'1 ข้อมูล'!$C$19</f>
@@ -3203,12 +3404,12 @@
         <v>19</v>
       </c>
       <c r="G50" s="6" t="s">
-        <v>213</v>
+        <v>226</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="4" t="s">
-        <v>214</v>
+        <v>227</v>
       </c>
       <c r="C52" s="5"/>
       <c r="D52" s="5"/>
@@ -3218,10 +3419,10 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="6" t="s">
-        <v>215</v>
+        <v>228</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>216</v>
+        <v>229</v>
       </c>
       <c r="D53" s="13"/>
       <c r="E53" s="23" t="n">
@@ -3232,15 +3433,15 @@
         <v>19</v>
       </c>
       <c r="G53" s="6" t="s">
-        <v>217</v>
+        <v>230</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="6" t="s">
-        <v>218</v>
+        <v>231</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>219</v>
+        <v>232</v>
       </c>
       <c r="D54" s="13"/>
       <c r="E54" s="23" t="n">
@@ -3254,10 +3455,10 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="6" t="s">
-        <v>220</v>
+        <v>233</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>221</v>
+        <v>234</v>
       </c>
       <c r="D55" s="13"/>
       <c r="E55" s="23" t="n">
@@ -3268,15 +3469,15 @@
         <v>19</v>
       </c>
       <c r="G55" s="6" t="s">
-        <v>222</v>
+        <v>235</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="6" t="s">
-        <v>223</v>
+        <v>236</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
       <c r="D56" s="13"/>
       <c r="E56" s="23" t="n">
@@ -3290,10 +3491,10 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="6" t="s">
-        <v>225</v>
+        <v>238</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="D57" s="13"/>
       <c r="E57" s="23" t="n">
@@ -3307,10 +3508,10 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="6" t="s">
-        <v>227</v>
+        <v>240</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>228</v>
+        <v>241</v>
       </c>
       <c r="D58" s="13"/>
       <c r="E58" s="23" t="n">
@@ -3324,29 +3525,29 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="6" t="s">
-        <v>229</v>
+        <v>242</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>230</v>
+        <v>243</v>
       </c>
       <c r="D59" s="13"/>
       <c r="E59" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$41*'3 ขนาดบ่อ'!$E$58^3/6</f>
+        <f aca="false">'1 ข้อมูล'!$C$48*'3 ขนาดบ่อ'!$E$58^3/6</f>
         <v>0.0485508704265308</v>
       </c>
       <c r="F59" s="6" t="s">
-        <v>231</v>
+        <v>244</v>
       </c>
       <c r="G59" s="6" t="s">
-        <v>232</v>
+        <v>245</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="6" t="s">
-        <v>233</v>
+        <v>246</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="D60" s="13"/>
       <c r="E60" s="23" t="n">
@@ -3354,33 +3555,33 @@
         <v>8.09181173775513</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="G60" s="6"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="6" t="s">
-        <v>235</v>
+        <v>248</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>236</v>
+        <v>249</v>
       </c>
       <c r="D61" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$60</f>
         <v>8.09181173775513</v>
       </c>
       <c r="E61" s="17" t="str">
-        <f aca="false">IF(D61&lt;=0.6*'1 ข้อมูล'!$C$47,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <f aca="false">IF(D61&lt;=0.6*'1 ข้อมูล'!$C$54,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
       <c r="F61" s="6"/>
       <c r="G61" s="6" t="s">
-        <v>237</v>
+        <v>250</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="4" t="s">
-        <v>238</v>
+        <v>251</v>
       </c>
       <c r="C63" s="5"/>
       <c r="D63" s="5"/>
@@ -3390,101 +3591,101 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B64" s="6" t="s">
-        <v>239</v>
+        <v>252</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>240</v>
+        <v>253</v>
       </c>
       <c r="D64" s="13"/>
       <c r="E64" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$41*'3 ขนาดบ่อ'!$E$50^3/6</f>
+        <f aca="false">'1 ข้อมูล'!$C$48*'3 ขนาดบ่อ'!$E$50^3/6</f>
         <v>2.82528</v>
       </c>
       <c r="F64" s="6" t="s">
-        <v>231</v>
+        <v>244</v>
       </c>
       <c r="G64" s="6" t="s">
-        <v>241</v>
+        <v>254</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="6" t="s">
-        <v>242</v>
+        <v>255</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>243</v>
+        <v>256</v>
       </c>
       <c r="D65" s="13"/>
       <c r="E65" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$49*'3 ขนาดบ่อ'!$E$64</f>
+        <f aca="false">'1 ข้อมูล'!$C$56*'3 ขนาดบ่อ'!$E$64</f>
         <v>4.802976</v>
       </c>
       <c r="F65" s="6" t="s">
-        <v>231</v>
+        <v>244</v>
       </c>
       <c r="G65" s="6"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="6" t="s">
-        <v>244</v>
+        <v>257</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>245</v>
+        <v>258</v>
       </c>
       <c r="D66" s="13"/>
       <c r="E66" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$35-'1 ข้อมูล'!$C$37-0.006</f>
+        <f aca="false">'1 ข้อมูล'!$C$42-'1 ข้อมูล'!$C$44-0.006</f>
         <v>0.144</v>
       </c>
       <c r="F66" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G66" s="6" t="s">
-        <v>246</v>
+        <v>259</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="6" t="s">
-        <v>247</v>
+        <v>260</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>248</v>
+        <v>261</v>
       </c>
       <c r="D67" s="13"/>
       <c r="E67" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$65/(0.9*'1 ข้อมูล'!$C$48*1000*0.9*'3 ขนาดบ่อ'!$E$66)*1000000</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$65/(0.9*'1 ข้อมูล'!$C$55*1000*0.9*'3 ขนาดบ่อ'!$E$66)*1000000</f>
         <v>102.944444444444</v>
       </c>
       <c r="F67" s="6" t="s">
-        <v>249</v>
+        <v>262</v>
       </c>
       <c r="G67" s="6"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B68" s="6" t="s">
-        <v>250</v>
+        <v>263</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>251</v>
+        <v>264</v>
       </c>
       <c r="D68" s="13"/>
       <c r="E68" s="23" t="n">
-        <f aca="false">0.003*1000*'1 ข้อมูล'!$C$35*1000</f>
+        <f aca="false">0.003*1000*'1 ข้อมูล'!$C$42*1000</f>
         <v>600</v>
       </c>
       <c r="F68" s="6" t="s">
-        <v>249</v>
+        <v>262</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>252</v>
+        <v>265</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B69" s="6" t="s">
-        <v>253</v>
+        <v>266</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>254</v>
+        <v>267</v>
       </c>
       <c r="D69" s="13"/>
       <c r="E69" s="23" t="n">
@@ -3492,13 +3693,13 @@
         <v>175</v>
       </c>
       <c r="F69" s="6" t="s">
-        <v>255</v>
+        <v>268</v>
       </c>
       <c r="G69" s="6"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B70" s="6" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="13" t="n">
@@ -3511,12 +3712,12 @@
       </c>
       <c r="F70" s="6"/>
       <c r="G70" s="6" t="s">
-        <v>257</v>
+        <v>270</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B72" s="4" t="s">
-        <v>258</v>
+        <v>271</v>
       </c>
       <c r="C72" s="5"/>
       <c r="D72" s="5"/>
@@ -3526,122 +3727,296 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B73" s="6" t="s">
-        <v>259</v>
+        <v>272</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>260</v>
+        <v>273</v>
       </c>
       <c r="D73" s="13"/>
       <c r="E73" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$31+'3 ขนาดบ่อ'!$E$12+'1 ข้อมูล'!$C$35+'3 ขนาดบ่อ'!$E$25</f>
-        <v>3.75</v>
+        <f aca="false">('1 ข้อมูล'!$C$38+'3 ขนาดบ่อ'!$E$8-'1 ข้อมูล'!$C$37)/2+0.025</f>
+        <v>0.3</v>
       </c>
       <c r="F73" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G73" s="6"/>
-    </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G73" s="6" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B74" s="6" t="s">
-        <v>261</v>
+        <v>275</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>262</v>
-      </c>
-      <c r="D74" s="13"/>
-      <c r="E74" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$45+'3 ขนาดบ่อ'!$E$37+'3 ขนาดบ่อ'!$E$73</f>
-        <v>6.35</v>
-      </c>
-      <c r="F74" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G74" s="6"/>
+        <v>276</v>
+      </c>
+      <c r="D74" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$8-'3 ขนาดบ่อ'!$E$73</f>
+        <v>0.3</v>
+      </c>
+      <c r="E74" s="17" t="str">
+        <f aca="false">IF(D74&gt;='1 ข้อมูล'!$C$37-0.0001,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F74" s="6"/>
+      <c r="G74" s="6" t="s">
+        <v>277</v>
+      </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B75" s="6" t="s">
-        <v>263</v>
+        <v>278</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>264</v>
-      </c>
-      <c r="D75" s="13"/>
-      <c r="E75" s="23" t="n">
+        <v>279</v>
+      </c>
+      <c r="D75" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$73</f>
+        <v>0.3</v>
+      </c>
+      <c r="E75" s="17" t="str">
+        <f aca="false">IF(D75&gt;='1 ข้อมูล'!$C$38-0.0001,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F75" s="6"/>
+      <c r="G75" s="6"/>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B76" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="C76" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="D76" s="13"/>
+      <c r="E76" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$12-'1 ข้อมูล'!$C$35</f>
+        <v>1.8</v>
+      </c>
+      <c r="F76" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G76" s="6"/>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B77" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="D77" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$76-'3 ขนาดบ่อ'!$E$13</f>
+        <v>0.85</v>
+      </c>
+      <c r="E77" s="17" t="str">
+        <f aca="false">IF(D77&gt;=0.5,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F77" s="6"/>
+      <c r="G77" s="6" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B78" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="C78" s="6" t="s">
+        <v>286</v>
+      </c>
+      <c r="D78" s="13"/>
+      <c r="E78" s="23" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$39-'3 ขนาดบ่อ'!$E$28</f>
+        <v>0.290334311237412</v>
+      </c>
+      <c r="F78" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G78" s="6"/>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B79" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="C79" s="6" t="s">
+        <v>288</v>
+      </c>
+      <c r="D79" s="13"/>
+      <c r="E79" s="23" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$39-'3 ขนาดบ่อ'!$E$8</f>
+        <v>0.5</v>
+      </c>
+      <c r="F79" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G79" s="6"/>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B80" s="6" t="s">
+        <v>289</v>
+      </c>
+      <c r="C80" s="6" t="s">
+        <v>290</v>
+      </c>
+      <c r="D80" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$78</f>
+        <v>0.290334311237412</v>
+      </c>
+      <c r="E80" s="17" t="str">
+        <f aca="false">IF(AND(D80&gt;='1 ข้อมูล'!$C$40,'3 ขนาดบ่อ'!$E$79&lt;='1 ข้อมูล'!$C$41),"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F80" s="6"/>
+      <c r="G80" s="6"/>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B81" s="6" t="s">
+        <v>291</v>
+      </c>
+      <c r="C81" s="6"/>
+      <c r="D81" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$50-'1 ข้อมูล'!$C$39</f>
+        <v>0.1</v>
+      </c>
+      <c r="E81" s="17" t="str">
+        <f aca="false">IF(D81&gt;=0,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F81" s="6"/>
+      <c r="G81" s="6" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B83" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="C83" s="5"/>
+      <c r="D83" s="5"/>
+      <c r="E83" s="5"/>
+      <c r="F83" s="5"/>
+      <c r="G83" s="5"/>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B84" s="6" t="s">
+        <v>294</v>
+      </c>
+      <c r="C84" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="D84" s="13"/>
+      <c r="E84" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$31+'3 ขนาดบ่อ'!$E$12+'1 ข้อมูล'!$C$42+'3 ขนาดบ่อ'!$E$25</f>
+        <v>3.75</v>
+      </c>
+      <c r="F84" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G84" s="6"/>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B85" s="6" t="s">
+        <v>296</v>
+      </c>
+      <c r="C85" s="6" t="s">
+        <v>297</v>
+      </c>
+      <c r="D85" s="13"/>
+      <c r="E85" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$45+'3 ขนาดบ่อ'!$E$37+'3 ขนาดบ่อ'!$E$84</f>
+        <v>6.35</v>
+      </c>
+      <c r="F85" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G85" s="6"/>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B86" s="6" t="s">
+        <v>298</v>
+      </c>
+      <c r="C86" s="6" t="s">
+        <v>299</v>
+      </c>
+      <c r="D86" s="13"/>
+      <c r="E86" s="23" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$9</f>
         <v>1.05</v>
       </c>
-      <c r="F75" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G75" s="6"/>
-    </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B76" s="6" t="s">
-        <v>265</v>
-      </c>
-      <c r="C76" s="6" t="s">
-        <v>266</v>
-      </c>
-      <c r="D76" s="13"/>
-      <c r="E76" s="23" t="n">
+      <c r="F86" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G86" s="6"/>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B87" s="6" t="s">
+        <v>300</v>
+      </c>
+      <c r="C87" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="D87" s="13"/>
+      <c r="E87" s="23" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$50</f>
         <v>1.2</v>
       </c>
-      <c r="F76" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G76" s="6"/>
-    </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B77" s="6" t="s">
-        <v>267</v>
-      </c>
-      <c r="C77" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="D77" s="13"/>
-      <c r="E77" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$74+2*'1 ข้อมูล'!$C$35</f>
+      <c r="F87" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G87" s="6"/>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B88" s="6" t="s">
+        <v>302</v>
+      </c>
+      <c r="C88" s="6" t="s">
+        <v>303</v>
+      </c>
+      <c r="D88" s="13"/>
+      <c r="E88" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$85+2*'1 ข้อมูล'!$C$42</f>
         <v>6.75</v>
       </c>
-      <c r="F77" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G77" s="6"/>
-    </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B78" s="6" t="s">
-        <v>269</v>
-      </c>
-      <c r="C78" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="D78" s="13"/>
-      <c r="E78" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$75+2*'1 ข้อมูล'!$C$35</f>
+      <c r="F88" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G88" s="6"/>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B89" s="6" t="s">
+        <v>304</v>
+      </c>
+      <c r="C89" s="6" t="s">
+        <v>303</v>
+      </c>
+      <c r="D89" s="13"/>
+      <c r="E89" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$86+2*'1 ข้อมูล'!$C$42</f>
         <v>1.45</v>
       </c>
-      <c r="F78" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G78" s="6"/>
-    </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B79" s="6" t="s">
-        <v>270</v>
-      </c>
-      <c r="C79" s="6" t="s">
-        <v>271</v>
-      </c>
-      <c r="D79" s="13"/>
-      <c r="E79" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$76+'1 ข้อมูล'!$C$36</f>
+      <c r="F89" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G89" s="6"/>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B90" s="6" t="s">
+        <v>305</v>
+      </c>
+      <c r="C90" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="D90" s="13"/>
+      <c r="E90" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$87+'1 ข้อมูล'!$C$43</f>
         <v>1.4</v>
       </c>
-      <c r="F79" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G79" s="6"/>
+      <c r="F90" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G90" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -3675,43 +4050,43 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>272</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>273</v>
+        <v>308</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>274</v>
+        <v>309</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>275</v>
+        <v>310</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>276</v>
+        <v>311</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>277</v>
+        <v>312</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>278</v>
+        <v>313</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>279</v>
+        <v>314</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>280</v>
+        <v>315</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="6" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="C5" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$7-'1 ข้อมูล'!$C$9</f>
@@ -3722,7 +4097,7 @@
         <v>0.0111111111111111</v>
       </c>
       <c r="E5" s="9" t="n">
-        <f aca="false">(D5/('1 ข้อมูล'!$C$45*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
+        <f aca="false">(D5/('1 ข้อมูล'!$C$52*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
         <v>3.20996461989311</v>
       </c>
       <c r="F5" s="19" t="n">
@@ -3734,7 +4109,7 @@
         <v>0.203110987387621</v>
       </c>
       <c r="H5" s="12" t="n">
-        <f aca="false">G5/SQRT('1 ข้อมูล'!$C$40*F5/100)</f>
+        <f aca="false">G5/SQRT('1 ข้อมูล'!$C$47*F5/100)</f>
         <v>0.284106733367315</v>
       </c>
       <c r="I5" s="17" t="str">
@@ -3744,7 +4119,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
       <c r="C6" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$10-'1 ข้อมูล'!$C$9</f>
@@ -3755,7 +4130,7 @@
         <v>0.0146643518518519</v>
       </c>
       <c r="E6" s="9" t="n">
-        <f aca="false">(D6/('1 ข้อมูล'!$C$45*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
+        <f aca="false">(D6/('1 ข้อมูล'!$C$52*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
         <v>3.86222140891387</v>
       </c>
       <c r="F6" s="19" t="n">
@@ -3767,7 +4142,7 @@
         <v>0.23823817642711</v>
       </c>
       <c r="H6" s="12" t="n">
-        <f aca="false">G6/SQRT('1 ข้อมูล'!$C$40*F6/100)</f>
+        <f aca="false">G6/SQRT('1 ข้อมูล'!$C$47*F6/100)</f>
         <v>0.314156278671783</v>
       </c>
       <c r="I6" s="17" t="str">
@@ -3777,7 +4152,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="C7" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8-'1 ข้อมูล'!$C$9</f>
@@ -3788,7 +4163,7 @@
         <v>0.025</v>
       </c>
       <c r="E7" s="9" t="n">
-        <f aca="false">(D7/('1 ข้อมูล'!$C$45*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
+        <f aca="false">(D7/('1 ข้อมูล'!$C$52*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
         <v>5.5117383277259</v>
       </c>
       <c r="F7" s="19" t="n">
@@ -3800,7 +4175,7 @@
         <v>0.316964233453695</v>
       </c>
       <c r="H7" s="12" t="n">
-        <f aca="false">G7/SQRT('1 ข้อมูล'!$C$40*F7/100)</f>
+        <f aca="false">G7/SQRT('1 ข้อมูล'!$C$47*F7/100)</f>
         <v>0.369237268621783</v>
       </c>
       <c r="I7" s="17" t="str">
@@ -3810,7 +4185,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="C8" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8</f>
@@ -3821,7 +4196,7 @@
         <v>0.0277777777777778</v>
       </c>
       <c r="E8" s="9" t="n">
-        <f aca="false">(D8/('1 ข้อมูล'!$C$45*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
+        <f aca="false">(D8/('1 ข้อมูล'!$C$52*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
         <v>5.91280538460372</v>
       </c>
       <c r="F8" s="19" t="n">
@@ -3833,7 +4208,7 @@
         <v>0.334331822522782</v>
       </c>
       <c r="H8" s="12" t="n">
-        <f aca="false">G8/SQRT('1 ข้อมูล'!$C$40*F8/100)</f>
+        <f aca="false">G8/SQRT('1 ข้อมูล'!$C$47*F8/100)</f>
         <v>0.379470456623503</v>
       </c>
       <c r="I8" s="17" t="str">
@@ -3843,17 +4218,17 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="22" t="s">
-        <v>281</v>
+        <v>316</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="22" t="s">
-        <v>282</v>
+        <v>317</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="22" t="s">
-        <v>283</v>
+        <v>318</v>
       </c>
     </row>
   </sheetData>
@@ -3883,172 +4258,172 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>284</v>
+        <v>319</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>285</v>
+        <v>320</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>286</v>
+        <v>321</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>19</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>287</v>
+        <v>322</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="6" t="s">
-        <v>266</v>
+        <v>301</v>
       </c>
       <c r="C5" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$50</f>
         <v>1.2</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>212</v>
+        <v>225</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>288</v>
+        <v>323</v>
       </c>
       <c r="C6" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$47</f>
         <v>0.987673754729172</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>289</v>
+        <v>324</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>290</v>
+        <v>325</v>
       </c>
       <c r="C7" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$35+'1 ข้อมูล'!$C$17</f>
         <v>0.92</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>291</v>
+        <v>326</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>292</v>
+        <v>327</v>
       </c>
       <c r="C8" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$35</f>
         <v>0.9</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="6" t="s">
-        <v>293</v>
+        <v>328</v>
       </c>
       <c r="C9" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$56</f>
         <v>1</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>294</v>
+        <v>329</v>
       </c>
       <c r="C10" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$10</f>
         <v>0.9</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>295</v>
+        <v>330</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
-        <v>296</v>
+        <v>331</v>
       </c>
       <c r="C11" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$28</f>
         <v>0.809665688762588</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>297</v>
+        <v>332</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>298</v>
+        <v>333</v>
       </c>
       <c r="C12" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8</f>
         <v>0.6</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>299</v>
+        <v>334</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="6" t="s">
-        <v>300</v>
+        <v>335</v>
       </c>
       <c r="C13" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$53</f>
         <v>0.5</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>216</v>
+        <v>229</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="6" t="s">
-        <v>301</v>
+        <v>336</v>
       </c>
       <c r="C14" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$55</f>
         <v>0.4</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>302</v>
+        <v>337</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="6" t="s">
-        <v>303</v>
+        <v>338</v>
       </c>
       <c r="C15" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$41</f>
         <v>0.3</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>304</v>
+        <v>339</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="s">
-        <v>305</v>
+        <v>340</v>
       </c>
       <c r="C16" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$20</f>
         <v>0.210686269183871</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>306</v>
+        <v>341</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="s">
-        <v>307</v>
+        <v>342</v>
       </c>
       <c r="C17" s="24" t="n">
         <f aca="false">0</f>
@@ -4084,32 +4459,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>308</v>
+        <v>343</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>309</v>
+        <v>344</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>310</v>
+        <v>345</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>311</v>
+        <v>346</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>312</v>
+        <v>347</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>313</v>
+        <v>348</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>314</v>
+        <v>349</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>315</v>
+        <v>350</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4121,7 +4496,7 @@
         <v>2.77719642805474</v>
       </c>
       <c r="D5" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B5/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B5/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
         <v>2.86619650300861</v>
       </c>
       <c r="E5" s="25" t="n">
@@ -4146,7 +4521,7 @@
         <v>4.38086341517286</v>
       </c>
       <c r="D6" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B6/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B6/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
         <v>4.48983131905459</v>
       </c>
       <c r="E6" s="25" t="n">
@@ -4171,7 +4546,7 @@
         <v>6.44060533155076</v>
       </c>
       <c r="D7" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B7/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B7/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
         <v>6.56792530595593</v>
       </c>
       <c r="E7" s="25" t="n">
@@ -4196,7 +4571,7 @@
         <v>8.99304061167301</v>
       </c>
       <c r="D8" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B8/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B8/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
         <v>9.13647413844802</v>
       </c>
       <c r="E8" s="25" t="n">
@@ -4221,7 +4596,7 @@
         <v>12.07224</v>
       </c>
       <c r="D9" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B9/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B9/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
         <v>12.2289986697729</v>
       </c>
       <c r="E9" s="25" t="n">
@@ -4246,7 +4621,7 @@
         <v>15.7101954157165</v>
       </c>
       <c r="D10" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B10/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B10/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
         <v>15.8769956216084</v>
       </c>
       <c r="E10" s="25" t="n">
@@ -4271,7 +4646,7 @@
         <v>19.9371602697676</v>
       </c>
       <c r="D11" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B11/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B11/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
         <v>20.1102658699656</v>
       </c>
       <c r="E11" s="25" t="n">
@@ -4296,7 +4671,7 @@
         <v>24.7819058265663</v>
       </c>
       <c r="D12" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B12/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B12/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
         <v>24.9571624264048</v>
       </c>
       <c r="E12" s="25" t="n">
@@ -4321,7 +4696,7 @@
         <v>30.2719200646936</v>
       </c>
       <c r="D13" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B13/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B13/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
         <v>30.4447832233961</v>
       </c>
       <c r="E13" s="25" t="n">
@@ -4346,7 +4721,7 @@
         <v>36.4335656390862</v>
       </c>
       <c r="D14" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B14/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B14/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
         <v>36.599124528368</v>
       </c>
       <c r="E14" s="25" t="n">
@@ -4371,7 +4746,7 @@
         <v>43.2922078439065</v>
       </c>
       <c r="D15" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B15/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B15/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
         <v>43.4452054104805</v>
       </c>
       <c r="E15" s="25" t="n">
@@ -4396,7 +4771,7 @@
         <v>50.87232</v>
       </c>
       <c r="D16" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B16/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B16/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
         <v>51.0071703805085</v>
       </c>
       <c r="E16" s="25" t="n">
@@ -4421,7 +4796,7 @@
         <v>59.1975714819181</v>
       </c>
       <c r="D17" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B17/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B17/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
         <v>59.3083752175669</v>
       </c>
       <c r="E17" s="25" t="n">
@@ -4446,7 +4821,7 @@
         <v>68.2909021448919</v>
       </c>
       <c r="D18" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B18/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B18/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
         <v>68.3714596053392</v>
       </c>
       <c r="E18" s="25" t="n">
@@ -4471,7 +4846,7 @@
         <v>78.1745859249513</v>
       </c>
       <c r="D19" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B19/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B19/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
         <v>78.2184092541632</v>
       </c>
       <c r="E19" s="25" t="n">
@@ -4496,7 +4871,7 @@
         <v>88.8702856977516</v>
       </c>
       <c r="D20" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B20/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B20/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
         <v>88.8706095248216</v>
       </c>
       <c r="E20" s="25" t="n">
@@ -4521,7 +4896,7 @@
         <v>100.399100991704</v>
       </c>
       <c r="D21" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B21/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B21/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
         <v>100.348892098404</v>
       </c>
       <c r="E21" s="25" t="n">
@@ -4546,7 +4921,7 @@
         <v>112.781609794846</v>
       </c>
       <c r="D22" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B22/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B22/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
         <v>112.673575893332</v>
       </c>
       <c r="E22" s="25" t="n">
@@ -4571,7 +4946,7 @@
         <v>126.037905431355</v>
       </c>
       <c r="D23" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B23/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B23/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
         <v>125.864503176292</v>
       </c>
       <c r="E23" s="25" t="n">
@@ -4596,7 +4971,7 @@
         <v>140.187629285531</v>
       </c>
       <c r="D24" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B24/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B24/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
         <v>139.941071622383</v>
       </c>
       <c r="E24" s="25" t="n">
@@ -4621,7 +4996,7 @@
         <v>155.25</v>
       </c>
       <c r="D25" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B25/100+'1 ข้อมูล'!$C$44)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B25/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
         <v>154.922262933655</v>
       </c>
       <c r="E25" s="25" t="n">

</xml_diff>

<commit_message>
Label the level sensor as the Flow meter (quotation item 1.3)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXLmoKkgGBxM2QbbegGKn7
</commit_message>
<xml_diff>
--- a/weir_design.xlsx
+++ b/weir_design.xlsx
@@ -234,19 +234,19 @@
     <t xml:space="preserve">พ้นตะกอนที่พื้น</t>
   </si>
   <si>
-    <t xml:space="preserve">DL10: ระดับหน้าเซนเซอร์</t>
+    <t xml:space="preserve">Flow meter (DL10): ระดับหน้าเซนเซอร์</t>
   </si>
   <si>
     <t xml:space="preserve">ติดคานพาดขวางเหนือจุดวัด H</t>
   </si>
   <si>
-    <t xml:space="preserve">DL10: ระยะวัดต่ำสุด (blanking)</t>
+    <t xml:space="preserve">Flow meter (DL10): ระยะวัดต่ำสุด (blanking)</t>
   </si>
   <si>
     <t xml:space="preserve">Badger DL10: 50–1,250 mm</t>
   </si>
   <si>
-    <t xml:space="preserve">DL10: ระยะวัดสูงสุด</t>
+    <t xml:space="preserve">Flow meter (DL10): ระยะวัดสูงสุด</t>
   </si>
   <si>
     <t xml:space="preserve">ความหนาผนัง คสล.</t>
@@ -891,19 +891,19 @@
     <t xml:space="preserve">ไม่รบกวนผิวน้ำที่จุดวัด</t>
   </si>
   <si>
-    <t xml:space="preserve">DL10: ระยะถึงผิวน้ำ ตอนน้ำสูงสุด</t>
+    <t xml:space="preserve">Flow meter (DL10): ระยะถึงผิวน้ำ ตอนน้ำสูงสุด</t>
   </si>
   <si>
     <t xml:space="preserve">หน้าเซนเซอร์ − (P + Hmax)</t>
   </si>
   <si>
-    <t xml:space="preserve">DL10: ระยะถึงผิวน้ำ ตอนน้ำหยุดไหล</t>
+    <t xml:space="preserve">Flow meter (DL10): ระยะถึงผิวน้ำ ตอนน้ำหยุดไหล</t>
   </si>
   <si>
     <t xml:space="preserve">หน้าเซนเซอร์ − P</t>
   </si>
   <si>
-    <t xml:space="preserve">ตรวจ: DL10 อยู่ในช่วงวัด</t>
+    <t xml:space="preserve">ตรวจ: Flow meter อยู่ในช่วงวัด</t>
   </si>
   <si>
     <t xml:space="preserve">0.05–1.25 m</t>
@@ -3734,7 +3734,7 @@
       </c>
       <c r="D73" s="13"/>
       <c r="E73" s="23" t="n">
-        <f aca="false">('1 ข้อมูล'!$C$38+'3 ขนาดบ่อ'!$E$8-'1 ข้อมูล'!$C$37)/2+0.025</f>
+        <f aca="false">ROUND(('1 ข้อมูล'!$C$38+'3 ขนาดบ่อ'!$E$8-'1 ข้อมูล'!$C$37)/2/0.05,0)*0.05</f>
         <v>0.3</v>
       </c>
       <c r="F73" s="6" t="s">
@@ -3819,7 +3819,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B78" s="6" t="s">
         <v>285</v>
       </c>
@@ -3836,7 +3836,7 @@
       </c>
       <c r="G78" s="6"/>
     </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B79" s="6" t="s">
         <v>287</v>
       </c>

</xml_diff>

<commit_message>
Add folded (U/L) layout comparison sheet to workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXLmoKkgGBxM2QbbegGKn7
</commit_message>
<xml_diff>
--- a/weir_design.xlsx
+++ b/weir_design.xlsx
@@ -14,6 +14,7 @@
     <sheet name="4 ช่องโชว์น้ำ" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="5 ระดับ" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="6 ตาราง H-Q" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="7 แบบพับ" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="351">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="401">
   <si>
     <t xml:space="preserve">1) ข้อมูลออกแบบ — บ่อ 3 ช่อง: ปั๊มจุ่ม | โชว์น้ำใส | V-notch 90°</t>
   </si>
@@ -1099,13 +1100,163 @@
   <si>
     <t xml:space="preserve">Q กรมฯ
 (m³/วัน)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7) แบบพับบ่อเป็น 2 แถว (U / L) เทียบกับแบบตรง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">แถว 1: ช่อง 1 → ช่อง 2 (พื้นยก)  |  น้ำล้นข้ามสันด้านข้างลงแถว 2  |  แถว 2: รับน้ำตก → ช่วงตรง → เวียร์ → ท่อออก (ไหลย้อนกลับ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ก. ความยาวแต่ละแถว (ใช้ขนาดจากชีต 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">แถว 1: ช่อง 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">โซนน้ำเข้า + ผนังกั้น + โซนปั๊ม</t>
+  </si>
+  <si>
+    <t xml:space="preserve">แถว 1: ช่อง 2 (พื้นยก)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ความยาวช่อง 2 = ความยาวสันข้าง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">น้ำไหลขวางบ่อ แล้วล้นสันลงแถว 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">แถว 1: รวม</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ช่อง 1 + ช่อง 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">แถว 2: โซนรับน้ำตก</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAX(ความยาวสัน, โซนรับน้ำตกขั้นต่ำ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ม่านน้ำตกตลอดความยาวสัน</t>
+  </si>
+  <si>
+    <t xml:space="preserve">แถว 2: รวม</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ความยาวภายในบ่อ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAX(แถว 1, แถว 2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">พื้นที่ว่างท้ายแถว 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ความยาวภายใน − แถว 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">แบบ L: ตัดส่วนนี้ทิ้ง / แบบ U: ใช้เป็นที่ตั้งตู้คอนโทรล</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B + ผนังกลาง + B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ข. เทียบ 3 แบบ (ขนาดภายนอก)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">แบบตรง (ปัจจุบัน)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">แบบ U (สี่เหลี่ยม)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">แบบ L (ตัดมุมว่าง)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ยาว (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">กว้าง (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">พื้นที่ฐาน (m²)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ผนังรอบนอก (m³)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ผนังกลาง (m³)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">พื้น (m³)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">คอนกรีตรวม (m³) โดยประมาณ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ไม่รวมพื้นยก กำแพงเวียร์ ผนังกั้น (เท่ากันทุกแบบ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ยาวลดลงจากแบบตรง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ค. ได้อะไร / เสียอะไร</t>
+  </si>
+  <si>
+    <t xml:space="preserve">✔ สั้นลง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">บ่อยาวลดลงประมาณ 30% วางในพื้นที่จำกัดได้ง่าย</t>
+  </si>
+  <si>
+    <t xml:space="preserve">✔ ท่อเข้า–ออกอยู่ด้านเดียวกัน</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ท่อเข้า 6" (แถว 1) และท่อออก 8" (แถว 2) อยู่ฝั่งเดียวกัน เดินท่อสั้นลง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">✔ จุดโชว์รวมกัน</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ช่อง 2 (น้ำใส) อยู่ติด BOD probe และ Flow meter ยืนดูจุดเดียวเห็นครบ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">✔ คอนกรีตแบบ L ใกล้เคียงแบบตรง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">แบบ U ใช้คอนกรีตมากกว่า เพราะมีมุมว่าง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">✘ น้ำต้องเลี้ยว 2 ครั้ง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">บนพื้นยก (เลี้ยว 90°) และตอนตกลงแถว 2 (ไหลจากด้านข้างแล้วเลี้ยวไปตามแถว)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">✘ ผิวน้ำช่อง 2 อาจไม่เรียบเท่าแบบตรง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">น้ำขึ้นพื้นยกจากด้านหนึ่ง แล้วไหลออกอีกด้าน มุมพื้นยกจะมีน้ำนิ่งหรือวน</t>
+  </si>
+  <si>
+    <t xml:space="preserve">✘ ความเสี่ยงค่า Flow แกว่ง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">น้ำเข้าแถว 2 จากด้านข้าง กระแสช่วงต้นไม่สม่ำเสมอ ช่วงตรง 2.10 m ช่วยได้ ถ้ายังแกว่งให้ใส่ผนังลอดใต้ต้นช่วงตรง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">✘ แบบหล่อซับซ้อนขึ้น</t>
+  </si>
+  <si>
+    <t xml:space="preserve">มีผนังกลางและมุมเพิ่ม ค่าแรงไม้แบบเพิ่ม</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="11">
+  <numFmts count="12">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="0"/>
@@ -1117,8 +1268,9 @@
     <numFmt numFmtId="172" formatCode="\+0.00;\-0.00;0.00"/>
     <numFmt numFmtId="173" formatCode="\+0.000;\-0.000;\±0.000"/>
     <numFmt numFmtId="174" formatCode="\+0.0%;\-0.0%;0.0%"/>
+    <numFmt numFmtId="175" formatCode="0%"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1208,6 +1360,22 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF2F8F4E"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FFC2410C"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -1290,7 +1458,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="32">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1399,6 +1567,26 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="168" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="175" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1459,10 +1647,10 @@
       <rgbColor rgb="FF595959"/>
       <rgbColor rgb="FFA6A6A6"/>
       <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF2F8F4E"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FFC2410C"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF1F4E78"/>
       <rgbColor rgb="FF333333"/>
@@ -5021,4 +5209,464 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="B1:F36"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="40"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B1" s="1" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="4" t="s">
+        <v>353</v>
+      </c>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>355</v>
+      </c>
+      <c r="D7" s="12" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$45</f>
+        <v>1.6</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" s="6"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="6" t="s">
+        <v>356</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="D8" s="12" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$37</f>
+        <v>1</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="D9" s="27" t="n">
+        <f aca="false">'7 แบบพับ'!$D$7+'7 แบบพับ'!$D$8</f>
+        <v>2.6</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9" s="6"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="D10" s="12" t="n">
+        <f aca="false">MAX('7 แบบพับ'!$D$8,'3 ขนาดบ่อ'!$E$31)</f>
+        <v>1</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="D11" s="27" t="n">
+        <f aca="false">'7 แบบพับ'!$D$10+'3 ขนาดบ่อ'!$E$12+'1 ข้อมูล'!$C$42+'3 ขนาดบ่อ'!$E$25</f>
+        <v>4.25</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" s="6"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>366</v>
+      </c>
+      <c r="D12" s="27" t="n">
+        <f aca="false">MAX('7 แบบพับ'!$D$9,'7 แบบพับ'!$D$11)</f>
+        <v>4.25</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" s="6"/>
+    </row>
+    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>368</v>
+      </c>
+      <c r="D13" s="12" t="n">
+        <f aca="false">'7 แบบพับ'!$D$12-'7 แบบพับ'!$D$9</f>
+        <v>1.65</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="6" t="s">
+        <v>298</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="D14" s="12" t="n">
+        <f aca="false">2*'3 ขนาดบ่อ'!$E$9+'1 ข้อมูล'!$C$42</f>
+        <v>2.3</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F14" s="6"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="28"/>
+      <c r="C17" s="28" t="s">
+        <v>372</v>
+      </c>
+      <c r="D17" s="28" t="s">
+        <v>373</v>
+      </c>
+      <c r="E17" s="28" t="s">
+        <v>374</v>
+      </c>
+      <c r="F17" s="28"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="6" t="s">
+        <v>375</v>
+      </c>
+      <c r="C18" s="12" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$88</f>
+        <v>6.75</v>
+      </c>
+      <c r="D18" s="12" t="n">
+        <f aca="false">'7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$42</f>
+        <v>4.65</v>
+      </c>
+      <c r="E18" s="12" t="n">
+        <f aca="false">'7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$42</f>
+        <v>4.65</v>
+      </c>
+      <c r="F18" s="6"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="6" t="s">
+        <v>376</v>
+      </c>
+      <c r="C19" s="12" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$89</f>
+        <v>1.45</v>
+      </c>
+      <c r="D19" s="12" t="n">
+        <f aca="false">'7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$42</f>
+        <v>2.7</v>
+      </c>
+      <c r="E19" s="12" t="n">
+        <f aca="false">'7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$42</f>
+        <v>2.7</v>
+      </c>
+      <c r="F19" s="6"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="6" t="s">
+        <v>377</v>
+      </c>
+      <c r="C20" s="12" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$88*'3 ขนาดบ่อ'!$E$89</f>
+        <v>9.7875</v>
+      </c>
+      <c r="D20" s="12" t="n">
+        <f aca="false">('7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$42)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$42)</f>
+        <v>12.555</v>
+      </c>
+      <c r="E20" s="12" t="n">
+        <f aca="false">('7 แบบพับ'!$D$9+2*'1 ข้อมูล'!$C$42)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$42)+('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$9)*('3 ขนาดบ่อ'!$E$9+2*'1 ข้อมูล'!$C$42)</f>
+        <v>10.4925</v>
+      </c>
+      <c r="F20" s="6"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="6" t="s">
+        <v>378</v>
+      </c>
+      <c r="C21" s="12" t="n">
+        <f aca="false">2*('3 ขนาดบ่อ'!$E$85+'1 ข้อมูล'!$C$42+'3 ขนาดบ่อ'!$E$86+'1 ข้อมูล'!$C$42)*'1 ข้อมูล'!$C$42*'3 ขนาดบ่อ'!$E$50</f>
+        <v>3.744</v>
+      </c>
+      <c r="D21" s="12" t="n">
+        <f aca="false">2*('7 แบบพับ'!$D$12+'1 ข้อมูล'!$C$42+'7 แบบพับ'!$D$14+'1 ข้อมูล'!$C$42)*'1 ข้อมูล'!$C$42*'3 ขนาดบ่อ'!$E$50</f>
+        <v>3.336</v>
+      </c>
+      <c r="E21" s="12" t="n">
+        <f aca="false">2*('7 แบบพับ'!$D$12+'1 ข้อมูล'!$C$42+'7 แบบพับ'!$D$14+'1 ข้อมูล'!$C$42)*'1 ข้อมูล'!$C$42*'3 ขนาดบ่อ'!$E$50</f>
+        <v>3.336</v>
+      </c>
+      <c r="F21" s="6"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="6" t="s">
+        <v>379</v>
+      </c>
+      <c r="C22" s="12" t="n">
+        <f aca="false">0</f>
+        <v>0</v>
+      </c>
+      <c r="D22" s="12" t="n">
+        <f aca="false">('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$8)*'1 ข้อมูล'!$C$42*'3 ขนาดบ่อ'!$E$50</f>
+        <v>0.78</v>
+      </c>
+      <c r="E22" s="12" t="n">
+        <f aca="false">'7 แบบพับ'!$D$7*'1 ข้อมูล'!$C$42*'3 ขนาดบ่อ'!$E$50</f>
+        <v>0.384</v>
+      </c>
+      <c r="F22" s="6"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="6" t="s">
+        <v>380</v>
+      </c>
+      <c r="C23" s="12" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$88*'3 ขนาดบ่อ'!$E$89*'1 ข้อมูล'!$C$43</f>
+        <v>1.9575</v>
+      </c>
+      <c r="D23" s="12" t="n">
+        <f aca="false">('7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$42)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$42)*'1 ข้อมูล'!$C$43</f>
+        <v>2.511</v>
+      </c>
+      <c r="E23" s="12" t="n">
+        <f aca="false">(('7 แบบพับ'!$D$9+2*'1 ข้อมูล'!$C$42)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$42)+('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$9)*('3 ขนาดบ่อ'!$E$9+2*'1 ข้อมูล'!$C$42))*'1 ข้อมูล'!$C$43</f>
+        <v>2.0985</v>
+      </c>
+      <c r="F23" s="6"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="6" t="s">
+        <v>381</v>
+      </c>
+      <c r="C24" s="27" t="n">
+        <f aca="false">SUM(C21:C23)</f>
+        <v>5.7015</v>
+      </c>
+      <c r="D24" s="27" t="n">
+        <f aca="false">SUM(D21:D23)</f>
+        <v>6.627</v>
+      </c>
+      <c r="E24" s="27" t="n">
+        <f aca="false">SUM(E21:E23)</f>
+        <v>5.8185</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="6" t="s">
+        <v>383</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="D25" s="29" t="n">
+        <f aca="false">1-D18/C18</f>
+        <v>0.311111111111111</v>
+      </c>
+      <c r="E25" s="29" t="n">
+        <f aca="false">1-E18/C18</f>
+        <v>0.311111111111111</v>
+      </c>
+      <c r="F25" s="6"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="C28" s="5"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="5"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="30" t="s">
+        <v>385</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>386</v>
+      </c>
+      <c r="D29" s="6"/>
+      <c r="E29" s="6"/>
+      <c r="F29" s="6"/>
+    </row>
+    <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="30" t="s">
+        <v>387</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>388</v>
+      </c>
+      <c r="D30" s="6"/>
+      <c r="E30" s="6"/>
+      <c r="F30" s="6"/>
+    </row>
+    <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="30" t="s">
+        <v>389</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="D31" s="6"/>
+      <c r="E31" s="6"/>
+      <c r="F31" s="6"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="30" t="s">
+        <v>391</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>392</v>
+      </c>
+      <c r="D32" s="6"/>
+      <c r="E32" s="6"/>
+      <c r="F32" s="6"/>
+    </row>
+    <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="31" t="s">
+        <v>393</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>394</v>
+      </c>
+      <c r="D33" s="6"/>
+      <c r="E33" s="6"/>
+      <c r="F33" s="6"/>
+    </row>
+    <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="31" t="s">
+        <v>395</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>396</v>
+      </c>
+      <c r="D34" s="6"/>
+      <c r="E34" s="6"/>
+      <c r="F34" s="6"/>
+    </row>
+    <row r="35" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B35" s="31" t="s">
+        <v>397</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>398</v>
+      </c>
+      <c r="D35" s="6"/>
+      <c r="E35" s="6"/>
+      <c r="F35" s="6"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B36" s="31" t="s">
+        <v>399</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>400</v>
+      </c>
+      <c r="D36" s="6"/>
+      <c r="E36" s="6"/>
+      <c r="F36" s="6"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add sheet comparing design with KKU EN614102 V-notch method
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXLmoKkgGBxM2QbbegGKn7
</commit_message>
<xml_diff>
--- a/weir_design.xlsx
+++ b/weir_design.xlsx
@@ -15,6 +15,7 @@
     <sheet name="5 ระดับ" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="6 ตาราง H-Q" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="7 แบบพับ" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="8 เทียบวิธี มข." sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="401">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="456">
   <si>
     <t xml:space="preserve">1) ข้อมูลออกแบบ — บ่อ 3 ช่อง: ปั๊มจุ่ม | โชว์น้ำใส | V-notch 90°</t>
   </si>
@@ -1250,6 +1251,171 @@
   </si>
   <si>
     <t xml:space="preserve">มีผนังกลางและมุมเพิ่ม ค่าแรงไม้แบบเพิ่ม</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8) ออกแบบตามวิธีในเอกสาร มข. (EN614102 Ex 3.9) เทียบกับแบบของเรา</t>
+  </si>
+  <si>
+    <t xml:space="preserve">สมการ USBR: Q = 1.36 H^2.48  |  เกณฑ์: P ≥ 2Hmax, b ≥ 2Hmax (b = ระยะจากขอบบนร่อง V ถึงผนัง), จุดวัด 3–5 Hmax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parameters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Symbol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value (วิธี มข.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remark (ตามเอกสาร)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">แบบของเรา (ชีต 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">แบบเราผ่านเกณฑ์ มข.?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Average flow rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qavg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">m³/s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,507 m³/วัน ÷ 24 ÷ 3600</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peak flow rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qpeak</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*Calculated from 1.5 of average</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peak flow (ใบเสนอราคา)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qmax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100 m³/h ตามใบเสนอราคา</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number of Weir Channel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*Design</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flow rate at Hmax of each weir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QHmax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*MAX(Qpeak, ใบเสนอราคา) / n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*Calculate from Hmax*2*1.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*Calculate from Hmax*2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hmax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*Calculated from Q=1.36Hmax^2.48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">เราใช้สูตรกรมฯ 1.38H^2.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P/2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b/2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Point of measurement H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*Calculate from Hmax*3 (เอกสารยอมให้ 3–5 Hmax)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H of V-Notch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*Calculate from Hmax*1.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*Calculate from b*2+[2*H of V Notch]/tan45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• สไลด์ตัวอย่าง (Q = 0.75 m³/s) ได้ B = 4.63 เพราะ Excel ใช้ TAN(45) ซึ่งตีความ 45 เป็นเรเดียน (tan = 1.62) — ค่าที่ถูกคือ TAN(RADIANS(45)) = 1 → B = 5.34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• b ในเอกสาร = ระยะจากขอบบนร่อง V ถึงผนังข้างละด้าน (เกณฑ์ USBR: ≥ 2Hmax) — แบบของเราใช้เกณฑ์ ISO 1438 (B ≥ 5Hmax) จึงแคบกว่า</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• สูตร USBR 1.36H^2.48 ให้ Q สูงกว่าสูตรกรมฯ 1.38H^2.5 ประมาณ 2% ในช่วง H 0.15–0.21 m</t>
   </si>
 </sst>
 </file>
@@ -1458,7 +1624,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1585,6 +1751,10 @@
     </xf>
     <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -5669,4 +5839,415 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="B1:I22"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="22"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B1" s="1" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B4" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>409</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="32" t="s">
+        <v>411</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="F5" s="23" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$10/3600</f>
+        <v>0.0174421296296296</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="H5" s="12"/>
+      <c r="I5" s="17"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="32" t="s">
+        <v>416</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>418</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="F6" s="23" t="n">
+        <f aca="false">1.5*F5</f>
+        <v>0.0261631944444444</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>419</v>
+      </c>
+      <c r="H6" s="12"/>
+      <c r="I6" s="17"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="32" t="s">
+        <v>420</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>421</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>422</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="F7" s="23" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$8/3600</f>
+        <v>0.0277777777777778</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>423</v>
+      </c>
+      <c r="H7" s="12"/>
+      <c r="I7" s="17"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="32" t="s">
+        <v>424</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>425</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="E8" s="6"/>
+      <c r="F8" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>411</v>
+      </c>
+      <c r="I8" s="17"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="32" t="s">
+        <v>428</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>430</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="F9" s="23" t="n">
+        <f aca="false">MAX(F6,F7)/F8</f>
+        <v>0.0277777777777778</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>431</v>
+      </c>
+      <c r="H9" s="12" t="n">
+        <f aca="false">'2 เวียร์'!$D$13</f>
+        <v>0.0277777777777778</v>
+      </c>
+      <c r="I9" s="17"/>
+    </row>
+    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="32" t="s">
+        <v>432</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>433</v>
+      </c>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" s="27" t="n">
+        <f aca="false">F12*2*1.1</f>
+        <v>0.458178826795053</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="H10" s="12" t="n">
+        <f aca="false">('3 ขนาดบ่อ'!$E$9-'3 ขนาดบ่อ'!$E$11)/2</f>
+        <v>0.225</v>
+      </c>
+      <c r="I10" s="17" t="str">
+        <f aca="false">IF(H10&gt;=2*F12,"ผ่าน ✔","ไม่ผ่าน ✘ (ต้อง ≥ 2Hmax)")</f>
+        <v>ไม่ผ่าน ✘ (ต้อง ≥ 2Hmax)</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="32" t="s">
+        <v>435</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>334</v>
+      </c>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" s="27" t="n">
+        <f aca="false">F12*2</f>
+        <v>0.416526206177321</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>436</v>
+      </c>
+      <c r="H11" s="12" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$8</f>
+        <v>0.6</v>
+      </c>
+      <c r="I11" s="17" t="str">
+        <f aca="false">IF(H11&gt;=2*F12,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="32" t="s">
+        <v>437</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>438</v>
+      </c>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" s="27" t="n">
+        <f aca="false">(F9/1.36)^(1/2.48)</f>
+        <v>0.208263103088661</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>439</v>
+      </c>
+      <c r="H12" s="12" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$7</f>
+        <v>0.209665688762588</v>
+      </c>
+      <c r="I12" s="17" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="32" t="s">
+        <v>441</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>442</v>
+      </c>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="27" t="n">
+        <f aca="false">F11/2</f>
+        <v>0.208263103088661</v>
+      </c>
+      <c r="G13" s="6" t="str">
+        <f aca="false">"Check P/2 ≥ Hmax: "&amp;IF(F13&gt;=F12,"✔","✘")</f>
+        <v>Check P/2 ≥ Hmax: ✔</v>
+      </c>
+      <c r="H13" s="12"/>
+      <c r="I13" s="17"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="32" t="s">
+        <v>443</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>444</v>
+      </c>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="27" t="n">
+        <f aca="false">F10/2</f>
+        <v>0.229089413397527</v>
+      </c>
+      <c r="G14" s="6" t="str">
+        <f aca="false">"Check b/2 ≥ Hmax: "&amp;IF(F14&gt;=F12,"✔","✘")</f>
+        <v>Check b/2 ≥ Hmax: ✔</v>
+      </c>
+      <c r="H14" s="12"/>
+      <c r="I14" s="17"/>
+    </row>
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="32" t="s">
+        <v>445</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>446</v>
+      </c>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F15" s="27" t="n">
+        <f aca="false">F12*3</f>
+        <v>0.624789309265982</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>447</v>
+      </c>
+      <c r="H15" s="12" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$13</f>
+        <v>0.95</v>
+      </c>
+      <c r="I15" s="17" t="str">
+        <f aca="false">IF(AND(H15&gt;=3*F12,H15&lt;=5*F12),"ผ่าน ✔ (อยู่ใน 3–5 Hmax)","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔ (อยู่ใน 3–5 Hmax)</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="32" t="s">
+        <v>448</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>449</v>
+      </c>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F16" s="27" t="n">
+        <f aca="false">F12*1.2</f>
+        <v>0.249915723706393</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>450</v>
+      </c>
+      <c r="H16" s="12" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$10</f>
+        <v>0.3</v>
+      </c>
+      <c r="I16" s="17" t="str">
+        <f aca="false">IF(H16&gt;=1.2*F12,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="32" t="s">
+        <v>451</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>299</v>
+      </c>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F17" s="27" t="n">
+        <f aca="false">F10*2+2*F16/TAN(RADIANS(45))</f>
+        <v>1.41618910100289</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>452</v>
+      </c>
+      <c r="H17" s="12" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$9</f>
+        <v>1.05</v>
+      </c>
+      <c r="I17" s="17" t="str">
+        <f aca="false">IF(H17&gt;=F17,"ผ่าน ✔","แคบกว่า ✘")</f>
+        <v>แคบกว่า ✘</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+      <c r="I19" s="5"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="22" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="22" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="22" t="s">
+        <v>455</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Widen tank to B = 1.45 m to meet USBR/KKU side clearance (b >= 2Hmax)
B now governed by max of ISO (H/B <= 0.2) and USBR (b >= 2Hmax each
side). External 6.75 x 1.85 m, weir plate 1.65 x 0.60 m, show-section
layer 4.6-6.8 cm. Workbook, drawings and animation updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXLmoKkgGBxM2QbbegGKn7
</commit_message>
<xml_diff>
--- a/weir_design.xlsx
+++ b/weir_design.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="456">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="462">
   <si>
     <t xml:space="preserve">1) ข้อมูลออกแบบ — บ่อ 3 ช่อง: ปั๊มจุ่ม | โชว์น้ำใส | V-notch 90°</t>
   </si>
@@ -473,31 +473,40 @@
     <t xml:space="preserve">เกณฑ์ ISO: P ≥ 0.45 m และ H/P ≤ 0.4</t>
   </si>
   <si>
+    <t xml:space="preserve">ความลึกร่อง V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H + 0.08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">น้ำไม่ล้นขอบร่อง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ความกว้างปากร่อง V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 × ความลึก × tan45°</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ร่อง 90° กว้าง = 2 เท่าของลึก</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b ระยะขอบร่อง V ถึงผนัง (ข้างละ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≥ 2 × H (เกณฑ์ USBR / เอกสาร มข.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">น้ำเข้าร่องไม่ถูกผนังข้างบีบ</t>
+  </si>
+  <si>
     <t xml:space="preserve">B ความกว้างภายในบ่อ</t>
   </si>
   <si>
-    <t xml:space="preserve">MAX(0.90, H ÷ 0.2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">เกณฑ์ ISO: B ≥ 0.90 m และ H/B ≤ 0.2 (fully contracted)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ความลึกร่อง V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">H + 0.08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">น้ำไม่ล้นขอบร่อง</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ความกว้างปากร่อง V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 × ความลึก × tan45°</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ร่อง 90° กว้าง = 2 เท่าของลึก</t>
+    <t xml:space="preserve">MAX(0.90, H ÷ 0.2, ปากร่อง + 2b)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISO: B ≥ 0.90 และ H/B ≤ 0.2 / USBR–มข.: b ≥ 2H ข้างละ (ใช้ค่าที่มากกว่า)</t>
   </si>
   <si>
     <t xml:space="preserve">ช่วงตรงหน้าเวียร์</t>
@@ -528,6 +537,15 @@
   </si>
   <si>
     <t xml:space="preserve">≤ 0.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ตรวจ: b จริง = (B − ปากร่อง) ÷ 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≥ 2H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">เกณฑ์ USBR / เอกสาร มข.</t>
   </si>
   <si>
     <t xml:space="preserve">ตรวจ: จุดวัด ÷ H</t>
@@ -3009,7 +3027,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:G90"/>
+  <dimension ref="B1:G92"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -3101,7 +3119,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="6" t="s">
         <v>145</v>
       </c>
@@ -3109,12 +3127,12 @@
         <v>146</v>
       </c>
       <c r="D9" s="13" t="n">
-        <f aca="false">MAX(0.9,'3 ขนาดบ่อ'!$E$7/0.2)</f>
-        <v>1.04832844381294</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$7+'1 ข้อมูล'!$C$15</f>
+        <v>0.289665688762588</v>
       </c>
       <c r="E9" s="23" t="n">
         <f aca="false">CEILING(ROUND(D9,4),'1 ข้อมูล'!$C$13)</f>
-        <v>1.05</v>
+        <v>0.3</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>19</v>
@@ -3130,13 +3148,10 @@
       <c r="C10" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="D10" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$7+'1 ข้อมูล'!$C$15</f>
-        <v>0.289665688762588</v>
-      </c>
+      <c r="D10" s="13"/>
       <c r="E10" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D10,4),'1 ข้อมูล'!$C$13)</f>
-        <v>0.3</v>
+        <f aca="false">2*'3 ขนาดบ่อ'!$E$9</f>
+        <v>0.6</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>19</v>
@@ -3154,8 +3169,8 @@
       </c>
       <c r="D11" s="13"/>
       <c r="E11" s="23" t="n">
-        <f aca="false">2*'3 ขนาดบ่อ'!$E$10</f>
-        <v>0.6</v>
+        <f aca="false">2*'3 ขนาดบ่อ'!$E$7</f>
+        <v>0.419331377525176</v>
       </c>
       <c r="F11" s="6" t="s">
         <v>19</v>
@@ -3164,7 +3179,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
         <v>154</v>
       </c>
@@ -3172,12 +3187,12 @@
         <v>155</v>
       </c>
       <c r="D12" s="13" t="n">
-        <f aca="false">10*'3 ขนาดบ่อ'!$E$7</f>
-        <v>2.09665688762588</v>
+        <f aca="false">MAX(0.9,'3 ขนาดบ่อ'!$E$7/0.2,'3 ขนาดบ่อ'!$E$10+2*'3 ขนาดบ่อ'!$E$11)</f>
+        <v>1.43866275505035</v>
       </c>
       <c r="E12" s="23" t="n">
         <f aca="false">CEILING(ROUND(D12,4),'1 ข้อมูล'!$C$13)</f>
-        <v>2.1</v>
+        <v>1.45</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>19</v>
@@ -3194,12 +3209,12 @@
         <v>158</v>
       </c>
       <c r="D13" s="13" t="n">
-        <f aca="false">4.5*'3 ขนาดบ่อ'!$E$7</f>
-        <v>0.943495599431645</v>
+        <f aca="false">10*'3 ขนาดบ่อ'!$E$7</f>
+        <v>2.09665688762588</v>
       </c>
       <c r="E13" s="23" t="n">
-        <f aca="false">ROUND(D13/'1 ข้อมูล'!$C$13,0)*'1 ข้อมูล'!$C$13</f>
-        <v>0.95</v>
+        <f aca="false">CEILING(ROUND(D13,4),'1 ข้อมูล'!$C$13)</f>
+        <v>2.1</v>
       </c>
       <c r="F13" s="6" t="s">
         <v>19</v>
@@ -3216,29 +3231,33 @@
         <v>161</v>
       </c>
       <c r="D14" s="13" t="n">
+        <f aca="false">4.5*'3 ขนาดบ่อ'!$E$7</f>
+        <v>0.943495599431645</v>
+      </c>
+      <c r="E14" s="23" t="n">
+        <f aca="false">ROUND(D14/'1 ข้อมูล'!$C$13,0)*'1 ข้อมูล'!$C$13</f>
+        <v>0.95</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="D15" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$7/'3 ขนาดบ่อ'!$E$8</f>
         <v>0.349442814604313</v>
       </c>
-      <c r="E14" s="17" t="str">
-        <f aca="false">IF(D14&lt;=0.4,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
-        <v>ผ่าน ✔</v>
-      </c>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="D15" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$7/'3 ขนาดบ่อ'!$E$9</f>
-        <v>0.199681608345322</v>
-      </c>
       <c r="E15" s="17" t="str">
-        <f aca="false">IF(D15&lt;=0.2,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <f aca="false">IF(D15&lt;=0.4,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
       <c r="F15" s="6"/>
@@ -3246,17 +3265,17 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D16" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$13/'3 ขนาดบ่อ'!$E$7</f>
-        <v>4.5310227229202</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$7/'3 ขนาดบ่อ'!$E$12</f>
+        <v>0.144597026732819</v>
       </c>
       <c r="E16" s="17" t="str">
-        <f aca="false">IF(AND(D16&gt;=4,D16&lt;=5),"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <f aca="false">IF(D16&lt;=0.2,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
       <c r="F16" s="6"/>
@@ -3264,89 +3283,88 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D17" s="13" t="n">
+        <f aca="false">('3 ขนาดบ่อ'!$E$12-'3 ขนาดบ่อ'!$E$10)/2</f>
+        <v>0.425</v>
+      </c>
+      <c r="E17" s="17" t="str">
+        <f aca="false">IF(D17&gt;=2*'3 ขนาดบ่อ'!$E$7,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="D18" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$14/'3 ขนาดบ่อ'!$E$7</f>
+        <v>4.5310227229202</v>
+      </c>
+      <c r="E18" s="17" t="str">
+        <f aca="false">IF(AND(D18&gt;=4,D18&lt;=5),"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F18" s="6"/>
+      <c r="G18" s="6"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="D19" s="13" t="n">
         <f aca="false">'2 เวียร์'!$E$10/100</f>
         <v>0.14532869095236</v>
       </c>
-      <c r="E17" s="17" t="str">
-        <f aca="false">IF(D17&gt;=0.05,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+      <c r="E19" s="17" t="str">
+        <f aca="false">IF(D19&gt;=0.05,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="D20" s="13"/>
-      <c r="E20" s="23" t="n">
+      <c r="F19" s="6"/>
+      <c r="G19" s="6" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="D22" s="13"/>
+      <c r="E22" s="23" t="n">
         <f aca="false">'1 ข้อมูล'!$C$29/2+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$53*PI()*'1 ข้อมูล'!$C$29^2/4))^2/(2*'1 ข้อมูล'!$C$47)</f>
         <v>0.210686269183871</v>
       </c>
-      <c r="F20" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G20" s="6"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="D21" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$8-'3 ขนาดบ่อ'!$E$20</f>
-        <v>0.389313730816129</v>
-      </c>
-      <c r="E21" s="17" t="str">
-        <f aca="false">IF(D21&gt;=0.06,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
-        <v>ผ่าน ✔</v>
-      </c>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="D22" s="13"/>
-      <c r="E22" s="23" t="n">
-        <f aca="false">SQRT(2*'1 ข้อมูล'!$C$47*'3 ขนาดบ่อ'!$E$7)</f>
-        <v>2.02821123493634</v>
-      </c>
       <c r="F22" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="G22" s="6" t="s">
-        <v>177</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="G22" s="6"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="6" t="s">
@@ -3355,111 +3373,116 @@
       <c r="C23" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="D23" s="13"/>
-      <c r="E23" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$7-'3 ขนาดบ่อ'!$E$20</f>
-        <v>0.598979419578717</v>
-      </c>
-      <c r="F23" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G23" s="6"/>
+      <c r="D23" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$8-'3 ขนาดบ่อ'!$E$22</f>
+        <v>0.389313730816129</v>
+      </c>
+      <c r="E23" s="17" t="str">
+        <f aca="false">IF(D23&gt;=0.06,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6" t="s">
+        <v>180</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D24" s="13"/>
       <c r="E24" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$22*SQRT(2*'3 ขนาดบ่อ'!$E$23/'1 ข้อมูล'!$C$47)</f>
-        <v>0.708760700266562</v>
+        <f aca="false">SQRT(2*'1 ข้อมูล'!$C$47*'3 ขนาดบ่อ'!$E$7)</f>
+        <v>2.02821123493634</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="6" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="D25" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$24+'1 ข้อมูล'!$C$28</f>
+        <v>185</v>
+      </c>
+      <c r="D25" s="13"/>
+      <c r="E25" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$7-'3 ขนาดบ่อ'!$E$22</f>
+        <v>0.598979419578717</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G25" s="6"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="D26" s="13"/>
+      <c r="E26" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$24*SQRT(2*'3 ขนาดบ่อ'!$E$25/'1 ข้อมูล'!$C$47)</f>
+        <v>0.708760700266562</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="D27" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$26+'1 ข้อมูล'!$C$28</f>
         <v>0.908760700266562</v>
       </c>
-      <c r="E25" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D25,4),'1 ข้อมูล'!$C$13)</f>
+      <c r="E27" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D27,4),'1 ข้อมูล'!$C$13)</f>
         <v>0.95</v>
       </c>
-      <c r="F25" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G25" s="6"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="C27" s="5"/>
-      <c r="D27" s="5"/>
-      <c r="E27" s="5"/>
-      <c r="F27" s="5"/>
-      <c r="G27" s="5"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="6" t="s">
-        <v>186</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="D28" s="13"/>
-      <c r="E28" s="23" t="n">
+      <c r="F27" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G27" s="6"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="C29" s="5"/>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
+      <c r="G29" s="5"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="D30" s="13"/>
+      <c r="E30" s="23" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$7</f>
         <v>0.809665688762588</v>
       </c>
-      <c r="F28" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G28" s="6"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="6" t="s">
-        <v>188</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>189</v>
-      </c>
-      <c r="D29" s="13"/>
-      <c r="E29" s="23" t="n">
-        <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$9*'3 ขนาดบ่อ'!$E$28)</f>
-        <v>0.0326740120301475</v>
-      </c>
-      <c r="F29" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="G29" s="6"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="6" t="s">
-        <v>190</v>
-      </c>
-      <c r="C30" s="6" t="s">
-        <v>191</v>
-      </c>
-      <c r="D30" s="13"/>
-      <c r="E30" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$28/'1 ข้อมูล'!$C$26*'3 ขนาดบ่อ'!$E$29</f>
-        <v>0.264550264550265</v>
-      </c>
       <c r="F30" s="6" t="s">
         <v>19</v>
       </c>
@@ -3467,380 +3490,378 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="6" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="D31" s="13" t="n">
-        <f aca="false">MAX('1 ข้อมูล'!$C$27,'3 ขนาดบ่อ'!$E$30)</f>
+        <v>195</v>
+      </c>
+      <c r="D31" s="13"/>
+      <c r="E31" s="23" t="n">
+        <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$12*'3 ขนาดบ่อ'!$E$30)</f>
+        <v>0.0236604914701068</v>
+      </c>
+      <c r="F31" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="G31" s="6"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="D32" s="13"/>
+      <c r="E32" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$30/'1 ข้อมูล'!$C$26*'3 ขนาดบ่อ'!$E$31</f>
+        <v>0.191570881226054</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G32" s="6"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="D33" s="13" t="n">
+        <f aca="false">MAX('1 ข้อมูล'!$C$27,'3 ขนาดบ่อ'!$E$32)</f>
         <v>0.5</v>
       </c>
-      <c r="E31" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D31,4),'1 ข้อมูล'!$C$13)</f>
+      <c r="E33" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D33,4),'1 ข้อมูล'!$C$13)</f>
         <v>0.5</v>
       </c>
-      <c r="F31" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G31" s="6" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="C33" s="5"/>
-      <c r="D33" s="5"/>
-      <c r="E33" s="5"/>
-      <c r="F33" s="5"/>
-      <c r="G33" s="5"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="D34" s="13"/>
-      <c r="E34" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$17+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$52*'3 ขนาดบ่อ'!$E$9))^(2/3)</f>
-        <v>0.0791280538460372</v>
-      </c>
-      <c r="F34" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G34" s="6" t="s">
-        <v>198</v>
+      <c r="F33" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G33" s="6" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="C35" s="6" t="s">
-        <v>200</v>
-      </c>
-      <c r="D35" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$28+'1 ข้อมูล'!$C$16-'1 ข้อมูล'!$C$17</f>
-        <v>0.889665688762588</v>
-      </c>
-      <c r="E35" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D35,4),'1 ข้อมูล'!$C$13)</f>
-        <v>0.9</v>
-      </c>
-      <c r="F35" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G35" s="6" t="s">
-        <v>26</v>
-      </c>
+      <c r="B35" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="C35" s="5"/>
+      <c r="D35" s="5"/>
+      <c r="E35" s="5"/>
+      <c r="F35" s="5"/>
+      <c r="G35" s="5"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="D36" s="13" t="n">
-        <f aca="false">10*'3 ขนาดบ่อ'!$E$34</f>
-        <v>0.791280538460372</v>
-      </c>
+        <v>203</v>
+      </c>
+      <c r="D36" s="13"/>
       <c r="E36" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D36,4),'1 ข้อมูล'!$C$13)</f>
-        <v>0.8</v>
+        <f aca="false">'1 ข้อมูล'!$C$17+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$52*'3 ขนาดบ่อ'!$E$12))^(2/3)</f>
+        <v>0.067680534585692</v>
       </c>
       <c r="F36" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="6" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="D37" s="13"/>
+        <v>206</v>
+      </c>
+      <c r="D37" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$30+'1 ข้อมูล'!$C$16-'1 ข้อมูล'!$C$17</f>
+        <v>0.889665688762588</v>
+      </c>
       <c r="E37" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D37,4),'1 ข้อมูล'!$C$13)</f>
+        <v>0.9</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G37" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B38" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="D38" s="13" t="n">
+        <f aca="false">10*'3 ขนาดบ่อ'!$E$36</f>
+        <v>0.67680534585692</v>
+      </c>
+      <c r="E38" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D38,4),'1 ข้อมูล'!$C$13)</f>
+        <v>0.7</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G38" s="6" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B39" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="D39" s="13"/>
+      <c r="E39" s="23" t="n">
         <f aca="false">'1 ข้อมูล'!$C$18</f>
         <v>1</v>
       </c>
-      <c r="F37" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G37" s="6"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="6" t="s">
-        <v>206</v>
-      </c>
-      <c r="C38" s="6"/>
-      <c r="D38" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$37-'3 ขนาดบ่อ'!$E$36</f>
+      <c r="F39" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G39" s="6"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B40" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="C40" s="6"/>
+      <c r="D40" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$39-'3 ขนาดบ่อ'!$E$38</f>
+        <v>0.3</v>
+      </c>
+      <c r="E40" s="17" t="str">
+        <f aca="false">IF(D40&gt;=0,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F40" s="6"/>
+      <c r="G40" s="6"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B42" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="C42" s="5"/>
+      <c r="D42" s="5"/>
+      <c r="E42" s="5"/>
+      <c r="F42" s="5"/>
+      <c r="G42" s="5"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B43" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="D43" s="13" t="n">
+        <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$12*'1 ข้อมูล'!$C$20)</f>
+        <v>0.191570881226054</v>
+      </c>
+      <c r="E43" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D43,4),'1 ข้อมูล'!$C$13)</f>
         <v>0.2</v>
       </c>
-      <c r="E38" s="17" t="str">
-        <f aca="false">IF(D38&gt;=0,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
-        <v>ผ่าน ✔</v>
-      </c>
-      <c r="F38" s="6"/>
-      <c r="G38" s="6"/>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="C40" s="5"/>
-      <c r="D40" s="5"/>
-      <c r="E40" s="5"/>
-      <c r="F40" s="5"/>
-      <c r="G40" s="5"/>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="6" t="s">
-        <v>208</v>
-      </c>
-      <c r="C41" s="6" t="s">
-        <v>209</v>
-      </c>
-      <c r="D41" s="13" t="n">
-        <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$9*'1 ข้อมูล'!$C$20)</f>
-        <v>0.264550264550265</v>
-      </c>
-      <c r="E41" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D41,4),'1 ข้อมูล'!$C$13)</f>
-        <v>0.3</v>
-      </c>
-      <c r="F41" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G41" s="6"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="6" t="s">
-        <v>210</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="D42" s="13" t="n">
+      <c r="F43" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G43" s="6"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B44" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="D44" s="13" t="n">
         <f aca="false">'1 ข้อมูล'!$C$21+2*'1 ข้อมูล'!$C$22</f>
         <v>0.468</v>
       </c>
-      <c r="E42" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D42,4),'1 ข้อมูล'!$C$13)</f>
+      <c r="E44" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D44,4),'1 ข้อมูล'!$C$13)</f>
         <v>0.5</v>
       </c>
-      <c r="F42" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G42" s="6"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="6" t="s">
-        <v>212</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>213</v>
-      </c>
-      <c r="D43" s="13"/>
-      <c r="E43" s="23" t="n">
+      <c r="F44" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G44" s="6"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B45" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="D45" s="13"/>
+      <c r="E45" s="23" t="n">
         <f aca="false">'1 ข้อมูล'!$C$23</f>
         <v>0.1</v>
       </c>
-      <c r="F43" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G43" s="6"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C44" s="6" t="s">
-        <v>215</v>
-      </c>
-      <c r="D44" s="13" t="n">
+      <c r="F45" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G45" s="6"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B46" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="D46" s="13" t="n">
         <f aca="false">'1 ข้อมูล'!$C$24+2*'1 ข้อมูล'!$C$25</f>
         <v>1</v>
       </c>
-      <c r="E44" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D44,4),'1 ข้อมูล'!$C$13)</f>
+      <c r="E46" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D46,4),'1 ข้อมูล'!$C$13)</f>
         <v>1</v>
       </c>
-      <c r="F44" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G44" s="6"/>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="6" t="s">
-        <v>216</v>
-      </c>
-      <c r="C45" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="D45" s="13"/>
-      <c r="E45" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$42+'3 ขนาดบ่อ'!$E$43+'3 ขนาดบ่อ'!$E$44</f>
-        <v>1.6</v>
-      </c>
-      <c r="F45" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G45" s="6"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="6" t="s">
-        <v>218</v>
-      </c>
-      <c r="C46" s="6" t="s">
-        <v>219</v>
-      </c>
-      <c r="D46" s="13"/>
-      <c r="E46" s="23" t="n">
-        <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$9*'3 ขนาดบ่อ'!$E$34)</f>
-        <v>0.334331822522782</v>
-      </c>
       <c r="F46" s="6" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="G46" s="6"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="6" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D47" s="13"/>
       <c r="E47" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$35+'3 ขนาดบ่อ'!$E$34+1.5*'3 ขนาดบ่อ'!$E$46^2/(2*'1 ข้อมูล'!$C$47)</f>
-        <v>0.987673754729172</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$44+'3 ขนาดบ่อ'!$E$45+'3 ขนาดบ่อ'!$E$46</f>
+        <v>1.6</v>
       </c>
       <c r="F47" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G47" s="6" t="s">
-        <v>222</v>
-      </c>
+      <c r="G47" s="6"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B48" s="6" t="s">
+        <v>224</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="D48" s="13"/>
+      <c r="E48" s="23" t="n">
+        <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$12*'3 ขนาดบ่อ'!$E$36)</f>
+        <v>0.283051666773555</v>
+      </c>
+      <c r="F48" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="G48" s="6"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B49" s="4" t="s">
-        <v>223</v>
-      </c>
-      <c r="C49" s="5"/>
-      <c r="D49" s="5"/>
-      <c r="E49" s="5"/>
-      <c r="F49" s="5"/>
-      <c r="G49" s="5"/>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B50" s="6" t="s">
-        <v>224</v>
-      </c>
-      <c r="C50" s="6" t="s">
-        <v>225</v>
-      </c>
-      <c r="D50" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$47+'1 ข้อมูล'!$C$19</f>
-        <v>1.18767375472917</v>
-      </c>
-      <c r="E50" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D50,4),'1 ข้อมูล'!$C$13)</f>
+      <c r="B49" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="D49" s="13"/>
+      <c r="E49" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$37+'3 ขนาดบ่อ'!$E$36+1.5*'3 ขนาดบ่อ'!$E$48^2/(2*'1 ข้อมูล'!$C$47)</f>
+        <v>0.973805782755668</v>
+      </c>
+      <c r="F49" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G49" s="6" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B51" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="C51" s="5"/>
+      <c r="D51" s="5"/>
+      <c r="E51" s="5"/>
+      <c r="F51" s="5"/>
+      <c r="G51" s="5"/>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B52" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="C52" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="D52" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$49+'1 ข้อมูล'!$C$19</f>
+        <v>1.17380578275567</v>
+      </c>
+      <c r="E52" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D52,4),'1 ข้อมูล'!$C$13)</f>
         <v>1.2</v>
       </c>
-      <c r="F50" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G50" s="6" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B52" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="C52" s="5"/>
-      <c r="D52" s="5"/>
-      <c r="E52" s="5"/>
-      <c r="F52" s="5"/>
-      <c r="G52" s="5"/>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="6" t="s">
-        <v>228</v>
-      </c>
-      <c r="C53" s="6" t="s">
-        <v>229</v>
-      </c>
-      <c r="D53" s="13"/>
-      <c r="E53" s="23" t="n">
+      <c r="F52" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G52" s="6" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B54" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="C54" s="5"/>
+      <c r="D54" s="5"/>
+      <c r="E54" s="5"/>
+      <c r="F54" s="5"/>
+      <c r="G54" s="5"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B55" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="D55" s="13"/>
+      <c r="E55" s="23" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8-'1 ข้อมูล'!$C$30</f>
         <v>0.5</v>
       </c>
-      <c r="F53" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G53" s="6" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B54" s="6" t="s">
-        <v>231</v>
-      </c>
-      <c r="C54" s="6" t="s">
-        <v>232</v>
-      </c>
-      <c r="D54" s="13"/>
-      <c r="E54" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$9+2*'1 ข้อมูล'!$C$33</f>
-        <v>1.25</v>
-      </c>
-      <c r="F54" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G54" s="6"/>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B55" s="6" t="s">
-        <v>233</v>
-      </c>
-      <c r="C55" s="6" t="s">
-        <v>234</v>
-      </c>
-      <c r="D55" s="13"/>
-      <c r="E55" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$53-'1 ข้อมูล'!$C$31</f>
-        <v>0.4</v>
-      </c>
       <c r="F55" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G55" s="6" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="6" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D56" s="13"/>
       <c r="E56" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$10+'1 ข้อมูล'!$C$32</f>
-        <v>1</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$12+2*'1 ข้อมูล'!$C$33</f>
+        <v>1.65</v>
       </c>
       <c r="F56" s="6" t="s">
         <v>19</v>
@@ -3849,32 +3870,34 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="6" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D57" s="13"/>
       <c r="E57" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$56-'3 ขนาดบ่อ'!$E$55</f>
-        <v>0.6</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$55-'1 ข้อมูล'!$C$31</f>
+        <v>0.4</v>
       </c>
       <c r="F57" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G57" s="6"/>
+      <c r="G57" s="6" t="s">
+        <v>241</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="6" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D58" s="13"/>
       <c r="E58" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$28-'3 ขนาดบ่อ'!$E$53</f>
-        <v>0.309665688762588</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$9+'1 ข้อมูล'!$C$32</f>
+        <v>1</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>19</v>
@@ -3883,22 +3906,20 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="6" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="D59" s="13"/>
       <c r="E59" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$48*'3 ขนาดบ่อ'!$E$58^3/6</f>
-        <v>0.0485508704265308</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$58-'3 ขนาดบ่อ'!$E$57</f>
+        <v>0.6</v>
       </c>
       <c r="F59" s="6" t="s">
-        <v>244</v>
-      </c>
-      <c r="G59" s="6" t="s">
-        <v>245</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="G59" s="6"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="6" t="s">
@@ -3909,11 +3930,11 @@
       </c>
       <c r="D60" s="13"/>
       <c r="E60" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$59/('1 ข้อมูล'!$C$34^2/6)/1000</f>
-        <v>8.09181173775513</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$30-'3 ขนาดบ่อ'!$E$55</f>
+        <v>0.309665688762588</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>95</v>
+        <v>19</v>
       </c>
       <c r="G60" s="6"/>
     </row>
@@ -3924,98 +3945,98 @@
       <c r="C61" s="6" t="s">
         <v>249</v>
       </c>
-      <c r="D61" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$60</f>
+      <c r="D61" s="13"/>
+      <c r="E61" s="23" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$48*'3 ขนาดบ่อ'!$E$60^3/6</f>
+        <v>0.0485508704265308</v>
+      </c>
+      <c r="F61" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="G61" s="6" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B62" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="D62" s="13"/>
+      <c r="E62" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$61/('1 ข้อมูล'!$C$34^2/6)/1000</f>
         <v>8.09181173775513</v>
       </c>
-      <c r="E61" s="17" t="str">
-        <f aca="false">IF(D61&lt;=0.6*'1 ข้อมูล'!$C$54,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+      <c r="F62" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="G62" s="6"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B63" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="D63" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$62</f>
+        <v>8.09181173775513</v>
+      </c>
+      <c r="E63" s="17" t="str">
+        <f aca="false">IF(D63&lt;=0.6*'1 ข้อมูล'!$C$54,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
-      <c r="F61" s="6"/>
-      <c r="G61" s="6" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B63" s="4" t="s">
-        <v>251</v>
-      </c>
-      <c r="C63" s="5"/>
-      <c r="D63" s="5"/>
-      <c r="E63" s="5"/>
-      <c r="F63" s="5"/>
-      <c r="G63" s="5"/>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B64" s="6" t="s">
-        <v>252</v>
-      </c>
-      <c r="C64" s="6" t="s">
-        <v>253</v>
-      </c>
-      <c r="D64" s="13"/>
-      <c r="E64" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$48*'3 ขนาดบ่อ'!$E$50^3/6</f>
-        <v>2.82528</v>
-      </c>
-      <c r="F64" s="6" t="s">
-        <v>244</v>
-      </c>
-      <c r="G64" s="6" t="s">
-        <v>254</v>
+      <c r="F63" s="6"/>
+      <c r="G63" s="6" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B65" s="6" t="s">
-        <v>255</v>
-      </c>
-      <c r="C65" s="6" t="s">
-        <v>256</v>
-      </c>
-      <c r="D65" s="13"/>
-      <c r="E65" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$56*'3 ขนาดบ่อ'!$E$64</f>
-        <v>4.802976</v>
-      </c>
-      <c r="F65" s="6" t="s">
-        <v>244</v>
-      </c>
-      <c r="G65" s="6"/>
+      <c r="B65" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="C65" s="5"/>
+      <c r="D65" s="5"/>
+      <c r="E65" s="5"/>
+      <c r="F65" s="5"/>
+      <c r="G65" s="5"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="6" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D66" s="13"/>
       <c r="E66" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$42-'1 ข้อมูล'!$C$44-0.006</f>
-        <v>0.144</v>
+        <f aca="false">'1 ข้อมูล'!$C$48*'3 ขนาดบ่อ'!$E$52^3/6</f>
+        <v>2.82528</v>
       </c>
       <c r="F66" s="6" t="s">
-        <v>19</v>
+        <v>250</v>
       </c>
       <c r="G66" s="6" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="6" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D67" s="13"/>
       <c r="E67" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$65/(0.9*'1 ข้อมูล'!$C$55*1000*0.9*'3 ขนาดบ่อ'!$E$66)*1000000</f>
-        <v>102.944444444444</v>
+        <f aca="false">'1 ข้อมูล'!$C$56*'3 ขนาดบ่อ'!$E$66</f>
+        <v>4.802976</v>
       </c>
       <c r="F67" s="6" t="s">
-        <v>262</v>
+        <v>250</v>
       </c>
       <c r="G67" s="6"/>
     </row>
@@ -4028,11 +4049,11 @@
       </c>
       <c r="D68" s="13"/>
       <c r="E68" s="23" t="n">
-        <f aca="false">0.003*1000*'1 ข้อมูล'!$C$42*1000</f>
-        <v>600</v>
+        <f aca="false">'1 ข้อมูล'!$C$42-'1 ข้อมูล'!$C$44-0.006</f>
+        <v>0.144</v>
       </c>
       <c r="F68" s="6" t="s">
-        <v>262</v>
+        <v>19</v>
       </c>
       <c r="G68" s="6" t="s">
         <v>265</v>
@@ -4047,8 +4068,8 @@
       </c>
       <c r="D69" s="13"/>
       <c r="E69" s="23" t="n">
-        <f aca="false">FLOOR(113/MAX('3 ขนาดบ่อ'!$E$67,'3 ขนาดบ่อ'!$E$68)*1000,25)</f>
-        <v>175</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$67/(0.9*'1 ข้อมูล'!$C$55*1000*0.9*'3 ขนาดบ่อ'!$E$68)*1000000</f>
+        <v>102.944444444444</v>
       </c>
       <c r="F69" s="6" t="s">
         <v>268</v>
@@ -4059,68 +4080,65 @@
       <c r="B70" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="C70" s="6"/>
-      <c r="D70" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$69</f>
+      <c r="C70" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="D70" s="13"/>
+      <c r="E70" s="23" t="n">
+        <f aca="false">0.003*1000*'1 ข้อมูล'!$C$42*1000</f>
+        <v>600</v>
+      </c>
+      <c r="F70" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="G70" s="6" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B71" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="D71" s="13"/>
+      <c r="E71" s="23" t="n">
+        <f aca="false">FLOOR(113/MAX('3 ขนาดบ่อ'!$E$69,'3 ขนาดบ่อ'!$E$70)*1000,25)</f>
         <v>175</v>
       </c>
-      <c r="E70" s="17" t="str">
-        <f aca="false">IF(D70&gt;=100,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+      <c r="F71" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="G71" s="6"/>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B72" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="C72" s="6"/>
+      <c r="D72" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$71</f>
+        <v>175</v>
+      </c>
+      <c r="E72" s="17" t="str">
+        <f aca="false">IF(D72&gt;=100,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
-      <c r="F70" s="6"/>
-      <c r="G70" s="6" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B72" s="4" t="s">
-        <v>271</v>
-      </c>
-      <c r="C72" s="5"/>
-      <c r="D72" s="5"/>
-      <c r="E72" s="5"/>
-      <c r="F72" s="5"/>
-      <c r="G72" s="5"/>
-    </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B73" s="6" t="s">
-        <v>272</v>
-      </c>
-      <c r="C73" s="6" t="s">
-        <v>273</v>
-      </c>
-      <c r="D73" s="13"/>
-      <c r="E73" s="23" t="n">
-        <f aca="false">ROUND(('1 ข้อมูล'!$C$38+'3 ขนาดบ่อ'!$E$8-'1 ข้อมูล'!$C$37)/2/0.05,0)*0.05</f>
-        <v>0.3</v>
-      </c>
-      <c r="F73" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G73" s="6" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="74" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B74" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="C74" s="6" t="s">
+      <c r="F72" s="6"/>
+      <c r="G72" s="6" t="s">
         <v>276</v>
       </c>
-      <c r="D74" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$8-'3 ขนาดบ่อ'!$E$73</f>
-        <v>0.3</v>
-      </c>
-      <c r="E74" s="17" t="str">
-        <f aca="false">IF(D74&gt;='1 ข้อมูล'!$C$37-0.0001,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
-        <v>ผ่าน ✔</v>
-      </c>
-      <c r="F74" s="6"/>
-      <c r="G74" s="6" t="s">
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B74" s="4" t="s">
         <v>277</v>
       </c>
+      <c r="C74" s="5"/>
+      <c r="D74" s="5"/>
+      <c r="E74" s="5"/>
+      <c r="F74" s="5"/>
+      <c r="G74" s="5"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B75" s="6" t="s">
@@ -4129,179 +4147,184 @@
       <c r="C75" s="6" t="s">
         <v>279</v>
       </c>
-      <c r="D75" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$73</f>
+      <c r="D75" s="13"/>
+      <c r="E75" s="23" t="n">
+        <f aca="false">ROUND(('1 ข้อมูล'!$C$38+'3 ขนาดบ่อ'!$E$8-'1 ข้อมูล'!$C$37)/2/0.05,0)*0.05</f>
         <v>0.3</v>
       </c>
-      <c r="E75" s="17" t="str">
-        <f aca="false">IF(D75&gt;='1 ข้อมูล'!$C$38-0.0001,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+      <c r="F75" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G75" s="6" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B76" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="C76" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="D76" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$8-'3 ขนาดบ่อ'!$E$75</f>
+        <v>0.3</v>
+      </c>
+      <c r="E76" s="17" t="str">
+        <f aca="false">IF(D76&gt;='1 ข้อมูล'!$C$37-0.0001,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
-      <c r="F75" s="6"/>
-      <c r="G75" s="6"/>
-    </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B76" s="6" t="s">
-        <v>280</v>
-      </c>
-      <c r="C76" s="6" t="s">
-        <v>281</v>
-      </c>
-      <c r="D76" s="13"/>
-      <c r="E76" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$12-'1 ข้อมูล'!$C$35</f>
-        <v>1.8</v>
-      </c>
-      <c r="F76" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G76" s="6"/>
+      <c r="F76" s="6"/>
+      <c r="G76" s="6" t="s">
+        <v>283</v>
+      </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B77" s="6" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="D77" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$76-'3 ขนาดบ่อ'!$E$13</f>
-        <v>0.85</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$75</f>
+        <v>0.3</v>
       </c>
       <c r="E77" s="17" t="str">
-        <f aca="false">IF(D77&gt;=0.5,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <f aca="false">IF(D77&gt;='1 ข้อมูล'!$C$38-0.0001,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
       <c r="F77" s="6"/>
-      <c r="G77" s="6" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="78" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G77" s="6"/>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B78" s="6" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C78" s="6" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D78" s="13"/>
       <c r="E78" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$39-'3 ขนาดบ่อ'!$E$28</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$13-'1 ข้อมูล'!$C$35</f>
+        <v>1.8</v>
+      </c>
+      <c r="F78" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G78" s="6"/>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B79" s="6" t="s">
+        <v>288</v>
+      </c>
+      <c r="C79" s="6" t="s">
+        <v>289</v>
+      </c>
+      <c r="D79" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$78-'3 ขนาดบ่อ'!$E$14</f>
+        <v>0.85</v>
+      </c>
+      <c r="E79" s="17" t="str">
+        <f aca="false">IF(D79&gt;=0.5,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F79" s="6"/>
+      <c r="G79" s="6" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B80" s="6" t="s">
+        <v>291</v>
+      </c>
+      <c r="C80" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="D80" s="13"/>
+      <c r="E80" s="23" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$39-'3 ขนาดบ่อ'!$E$30</f>
         <v>0.290334311237412</v>
       </c>
-      <c r="F78" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G78" s="6"/>
-    </row>
-    <row r="79" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B79" s="6" t="s">
-        <v>287</v>
-      </c>
-      <c r="C79" s="6" t="s">
-        <v>288</v>
-      </c>
-      <c r="D79" s="13"/>
-      <c r="E79" s="23" t="n">
+      <c r="F80" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G80" s="6"/>
+    </row>
+    <row r="81" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B81" s="6" t="s">
+        <v>293</v>
+      </c>
+      <c r="C81" s="6" t="s">
+        <v>294</v>
+      </c>
+      <c r="D81" s="13"/>
+      <c r="E81" s="23" t="n">
         <f aca="false">'1 ข้อมูล'!$C$39-'3 ขนาดบ่อ'!$E$8</f>
         <v>0.5</v>
       </c>
-      <c r="F79" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G79" s="6"/>
-    </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B80" s="6" t="s">
-        <v>289</v>
-      </c>
-      <c r="C80" s="6" t="s">
-        <v>290</v>
-      </c>
-      <c r="D80" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$78</f>
+      <c r="F81" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G81" s="6"/>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B82" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="C82" s="6" t="s">
+        <v>296</v>
+      </c>
+      <c r="D82" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$80</f>
         <v>0.290334311237412</v>
       </c>
-      <c r="E80" s="17" t="str">
-        <f aca="false">IF(AND(D80&gt;='1 ข้อมูล'!$C$40,'3 ขนาดบ่อ'!$E$79&lt;='1 ข้อมูล'!$C$41),"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+      <c r="E82" s="17" t="str">
+        <f aca="false">IF(AND(D82&gt;='1 ข้อมูล'!$C$40,'3 ขนาดบ่อ'!$E$81&lt;='1 ข้อมูล'!$C$41),"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
-      <c r="F80" s="6"/>
-      <c r="G80" s="6"/>
-    </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B81" s="6" t="s">
-        <v>291</v>
-      </c>
-      <c r="C81" s="6"/>
-      <c r="D81" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$50-'1 ข้อมูล'!$C$39</f>
+      <c r="F82" s="6"/>
+      <c r="G82" s="6"/>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B83" s="6" t="s">
+        <v>297</v>
+      </c>
+      <c r="C83" s="6"/>
+      <c r="D83" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$52-'1 ข้อมูล'!$C$39</f>
         <v>0.1</v>
       </c>
-      <c r="E81" s="17" t="str">
-        <f aca="false">IF(D81&gt;=0,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+      <c r="E83" s="17" t="str">
+        <f aca="false">IF(D83&gt;=0,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
-      <c r="F81" s="6"/>
-      <c r="G81" s="6" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B83" s="4" t="s">
-        <v>293</v>
-      </c>
-      <c r="C83" s="5"/>
-      <c r="D83" s="5"/>
-      <c r="E83" s="5"/>
-      <c r="F83" s="5"/>
-      <c r="G83" s="5"/>
-    </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B84" s="6" t="s">
-        <v>294</v>
-      </c>
-      <c r="C84" s="6" t="s">
-        <v>295</v>
-      </c>
-      <c r="D84" s="13"/>
-      <c r="E84" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$31+'3 ขนาดบ่อ'!$E$12+'1 ข้อมูล'!$C$42+'3 ขนาดบ่อ'!$E$25</f>
-        <v>3.75</v>
-      </c>
-      <c r="F84" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G84" s="6"/>
+      <c r="F83" s="6"/>
+      <c r="G83" s="6" t="s">
+        <v>298</v>
+      </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B85" s="6" t="s">
-        <v>296</v>
-      </c>
-      <c r="C85" s="6" t="s">
-        <v>297</v>
-      </c>
-      <c r="D85" s="13"/>
-      <c r="E85" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$45+'3 ขนาดบ่อ'!$E$37+'3 ขนาดบ่อ'!$E$84</f>
-        <v>6.35</v>
-      </c>
-      <c r="F85" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G85" s="6"/>
+      <c r="B85" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="C85" s="5"/>
+      <c r="D85" s="5"/>
+      <c r="E85" s="5"/>
+      <c r="F85" s="5"/>
+      <c r="G85" s="5"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B86" s="6" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="C86" s="6" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="D86" s="13"/>
       <c r="E86" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$9</f>
-        <v>1.05</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$33+'3 ขนาดบ่อ'!$E$13+'1 ข้อมูล'!$C$42+'3 ขนาดบ่อ'!$E$27</f>
+        <v>3.75</v>
       </c>
       <c r="F86" s="6" t="s">
         <v>19</v>
@@ -4310,15 +4333,15 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B87" s="6" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="C87" s="6" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="D87" s="13"/>
       <c r="E87" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$50</f>
-        <v>1.2</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$47+'3 ขนาดบ่อ'!$E$39+'3 ขนาดบ่อ'!$E$86</f>
+        <v>6.35</v>
       </c>
       <c r="F87" s="6" t="s">
         <v>19</v>
@@ -4327,15 +4350,15 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B88" s="6" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C88" s="6" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="D88" s="13"/>
       <c r="E88" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$85+2*'1 ข้อมูล'!$C$42</f>
-        <v>6.75</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$12</f>
+        <v>1.45</v>
       </c>
       <c r="F88" s="6" t="s">
         <v>19</v>
@@ -4344,15 +4367,15 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B89" s="6" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="C89" s="6" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="D89" s="13"/>
       <c r="E89" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$86+2*'1 ข้อมูล'!$C$42</f>
-        <v>1.45</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$52</f>
+        <v>1.2</v>
       </c>
       <c r="F89" s="6" t="s">
         <v>19</v>
@@ -4361,20 +4384,54 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B90" s="6" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="C90" s="6" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="D90" s="13"/>
       <c r="E90" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$87+'1 ข้อมูล'!$C$43</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$87+2*'1 ข้อมูล'!$C$42</f>
+        <v>6.75</v>
+      </c>
+      <c r="F90" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G90" s="6"/>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B91" s="6" t="s">
+        <v>310</v>
+      </c>
+      <c r="C91" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="D91" s="13"/>
+      <c r="E91" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$88+2*'1 ข้อมูล'!$C$42</f>
+        <v>1.85</v>
+      </c>
+      <c r="F91" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G91" s="6"/>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B92" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="C92" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="D92" s="13"/>
+      <c r="E92" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$89+'1 ข้อมูล'!$C$43</f>
         <v>1.4</v>
       </c>
-      <c r="F90" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G90" s="6"/>
+      <c r="F92" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G92" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -4408,12 +4465,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4421,25 +4478,25 @@
         <v>116</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>314</v>
+        <v>320</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4455,20 +4512,20 @@
         <v>0.0111111111111111</v>
       </c>
       <c r="E5" s="9" t="n">
-        <f aca="false">(D5/('1 ข้อมูล'!$C$52*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
-        <v>3.20996461989311</v>
+        <f aca="false">(D5/('1 ข้อมูล'!$C$52*'3 ขนาดบ่อ'!$E$12))^(2/3)*100</f>
+        <v>2.5884976609613</v>
       </c>
       <c r="F5" s="19" t="n">
         <f aca="false">'1 ข้อมูล'!$C$17*100+E5</f>
-        <v>5.20996461989311</v>
+        <v>4.5884976609613</v>
       </c>
       <c r="G5" s="12" t="n">
-        <f aca="false">D5/('3 ขนาดบ่อ'!$E$9*F5/100)</f>
-        <v>0.203110987387621</v>
+        <f aca="false">D5/('3 ขนาดบ่อ'!$E$12*F5/100)</f>
+        <v>0.167000962302698</v>
       </c>
       <c r="H5" s="12" t="n">
         <f aca="false">G5/SQRT('1 ข้อมูล'!$C$47*F5/100)</f>
-        <v>0.284106733367315</v>
+        <v>0.248913936242837</v>
       </c>
       <c r="I5" s="17" t="str">
         <f aca="false">IF(H5&lt;0.5,"เรียบ ✔",IF(H5&lt;0.7,"พอใช้","เป็นระลอก ✘"))</f>
@@ -4488,20 +4545,20 @@
         <v>0.0146643518518519</v>
       </c>
       <c r="E6" s="9" t="n">
-        <f aca="false">(D6/('1 ข้อมูล'!$C$52*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
-        <v>3.86222140891387</v>
+        <f aca="false">(D6/('1 ข้อมูล'!$C$52*'3 ขนาดบ่อ'!$E$12))^(2/3)*100</f>
+        <v>3.11447391698078</v>
       </c>
       <c r="F6" s="19" t="n">
         <f aca="false">'1 ข้อมูล'!$C$17*100+E6</f>
-        <v>5.86222140891387</v>
+        <v>5.11447391698078</v>
       </c>
       <c r="G6" s="12" t="n">
-        <f aca="false">D6/('3 ขนาดบ่อ'!$E$9*F6/100)</f>
-        <v>0.23823817642711</v>
+        <f aca="false">D6/('3 ขนาดบ่อ'!$E$12*F6/100)</f>
+        <v>0.197739714169774</v>
       </c>
       <c r="H6" s="12" t="n">
         <f aca="false">G6/SQRT('1 ข้อมูล'!$C$47*F6/100)</f>
-        <v>0.314156278671783</v>
+        <v>0.279163679771048</v>
       </c>
       <c r="I6" s="17" t="str">
         <f aca="false">IF(H6&lt;0.5,"เรียบ ✔",IF(H6&lt;0.7,"พอใช้","เป็นระลอก ✘"))</f>
@@ -4521,20 +4578,20 @@
         <v>0.025</v>
       </c>
       <c r="E7" s="9" t="n">
-        <f aca="false">(D7/('1 ข้อมูล'!$C$52*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
-        <v>5.5117383277259</v>
+        <f aca="false">(D7/('1 ข้อมูล'!$C$52*'3 ขนาดบ่อ'!$E$12))^(2/3)*100</f>
+        <v>4.44463520897758</v>
       </c>
       <c r="F7" s="19" t="n">
         <f aca="false">'1 ข้อมูล'!$C$17*100+E7</f>
-        <v>7.5117383277259</v>
+        <v>6.44463520897758</v>
       </c>
       <c r="G7" s="12" t="n">
-        <f aca="false">D7/('3 ขนาดบ่อ'!$E$9*F7/100)</f>
-        <v>0.316964233453695</v>
+        <f aca="false">D7/('3 ขนาดบ่อ'!$E$12*F7/100)</f>
+        <v>0.267530725188713</v>
       </c>
       <c r="H7" s="12" t="n">
         <f aca="false">G7/SQRT('1 ข้อมูล'!$C$47*F7/100)</f>
-        <v>0.369237268621783</v>
+        <v>0.336465076577215</v>
       </c>
       <c r="I7" s="17" t="str">
         <f aca="false">IF(H7&lt;0.5,"เรียบ ✔",IF(H7&lt;0.7,"พอใช้","เป็นระลอก ✘"))</f>
@@ -4554,20 +4611,20 @@
         <v>0.0277777777777778</v>
       </c>
       <c r="E8" s="9" t="n">
-        <f aca="false">(D8/('1 ข้อมูล'!$C$52*'3 ขนาดบ่อ'!$E$9))^(2/3)*100</f>
-        <v>5.91280538460372</v>
+        <f aca="false">(D8/('1 ข้อมูล'!$C$52*'3 ขนาดบ่อ'!$E$12))^(2/3)*100</f>
+        <v>4.7680534585692</v>
       </c>
       <c r="F8" s="19" t="n">
         <f aca="false">'1 ข้อมูล'!$C$17*100+E8</f>
-        <v>7.91280538460372</v>
+        <v>6.7680534585692</v>
       </c>
       <c r="G8" s="12" t="n">
-        <f aca="false">D8/('3 ขนาดบ่อ'!$E$9*F8/100)</f>
-        <v>0.334331822522782</v>
+        <f aca="false">D8/('3 ขนาดบ่อ'!$E$12*F8/100)</f>
+        <v>0.283051666773555</v>
       </c>
       <c r="H8" s="12" t="n">
         <f aca="false">G8/SQRT('1 ข้อมูล'!$C$47*F8/100)</f>
-        <v>0.379470456623503</v>
+        <v>0.347375610243974</v>
       </c>
       <c r="I8" s="17" t="str">
         <f aca="false">IF(H8&lt;0.5,"เรียบ ✔",IF(H8&lt;0.7,"พอใช้","เป็นระลอก ✘"))</f>
@@ -4576,17 +4633,17 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="22" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="22" t="s">
-        <v>317</v>
+        <v>323</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="22" t="s">
-        <v>318</v>
+        <v>324</v>
       </c>
     </row>
   </sheetData>
@@ -4616,172 +4673,172 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>319</v>
+        <v>325</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>320</v>
+        <v>326</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>321</v>
+        <v>327</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>19</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="6" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="C5" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$50</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$52</f>
         <v>1.2</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="C6" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$47</f>
-        <v>0.987673754729172</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$49</f>
+        <v>0.973805782755668</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="C7" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$35+'1 ข้อมูล'!$C$17</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$37+'1 ข้อมูล'!$C$17</f>
         <v>0.92</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>326</v>
+        <v>332</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>327</v>
+        <v>333</v>
       </c>
       <c r="C8" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$35</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$37</f>
         <v>0.9</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="6" t="s">
-        <v>328</v>
+        <v>334</v>
       </c>
       <c r="C9" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$56</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$58</f>
         <v>1</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>329</v>
+        <v>335</v>
       </c>
       <c r="C10" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$10</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$9</f>
         <v>0.9</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="C11" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$28</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$30</f>
         <v>0.809665688762588</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="C12" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8</f>
         <v>0.6</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="6" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="C13" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$53</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$55</f>
         <v>0.5</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="6" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="C14" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$55</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$57</f>
         <v>0.4</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="6" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="C15" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$41</f>
-        <v>0.3</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$43</f>
+        <v>0.2</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>339</v>
+        <v>345</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="C16" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$20</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$22</f>
         <v>0.210686269183871</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="C17" s="24" t="n">
         <f aca="false">0</f>
@@ -4817,32 +4874,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>348</v>
+        <v>354</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>349</v>
+        <v>355</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5398,12 +5455,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>352</v>
+        <v>358</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5425,7 +5482,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="4" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -5434,13 +5491,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
       <c r="D7" s="12" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$45</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$47</f>
         <v>1.6</v>
       </c>
       <c r="E7" s="6" t="s">
@@ -5450,28 +5507,28 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="D8" s="12" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$37</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$39</f>
         <v>1</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>19</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="6" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="D9" s="27" t="n">
         <f aca="false">'7 แบบพับ'!$D$7+'7 แบบพับ'!$D$8</f>
@@ -5484,31 +5541,31 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
       <c r="D10" s="12" t="n">
-        <f aca="false">MAX('7 แบบพับ'!$D$8,'3 ขนาดบ่อ'!$E$31)</f>
+        <f aca="false">MAX('7 แบบพับ'!$D$8,'3 ขนาดบ่อ'!$E$33)</f>
         <v>1</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>19</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
       <c r="D11" s="27" t="n">
-        <f aca="false">'7 แบบพับ'!$D$10+'3 ขนาดบ่อ'!$E$12+'1 ข้อมูล'!$C$42+'3 ขนาดบ่อ'!$E$25</f>
+        <f aca="false">'7 แบบพับ'!$D$10+'3 ขนาดบ่อ'!$E$13+'1 ข้อมูล'!$C$42+'3 ขนาดบ่อ'!$E$27</f>
         <v>4.25</v>
       </c>
       <c r="E11" s="6" t="s">
@@ -5518,10 +5575,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="D12" s="27" t="n">
         <f aca="false">MAX('7 แบบพับ'!$D$9,'7 แบบพับ'!$D$11)</f>
@@ -5534,10 +5591,10 @@
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="6" t="s">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>368</v>
+        <v>374</v>
       </c>
       <c r="D13" s="12" t="n">
         <f aca="false">'7 แบบพับ'!$D$12-'7 แบบพับ'!$D$9</f>
@@ -5547,19 +5604,19 @@
         <v>19</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="6" t="s">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="D14" s="12" t="n">
-        <f aca="false">2*'3 ขนาดบ่อ'!$E$9+'1 ข้อมูล'!$C$42</f>
-        <v>2.3</v>
+        <f aca="false">2*'3 ขนาดบ่อ'!$E$12+'1 ข้อมูล'!$C$42</f>
+        <v>3.1</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>19</v>
@@ -5568,7 +5625,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="4" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
@@ -5578,22 +5635,22 @@
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="28"/>
       <c r="C17" s="28" t="s">
-        <v>372</v>
+        <v>378</v>
       </c>
       <c r="D17" s="28" t="s">
-        <v>373</v>
+        <v>379</v>
       </c>
       <c r="E17" s="28" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="F17" s="28"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="6" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="C18" s="12" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$88</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$90</f>
         <v>6.75</v>
       </c>
       <c r="D18" s="12" t="n">
@@ -5608,117 +5665,117 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="6" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="C19" s="12" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$89</f>
-        <v>1.45</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$91</f>
+        <v>1.85</v>
       </c>
       <c r="D19" s="12" t="n">
         <f aca="false">'7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$42</f>
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="E19" s="12" t="n">
         <f aca="false">'7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$42</f>
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="F19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="6" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="C20" s="12" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$88*'3 ขนาดบ่อ'!$E$89</f>
-        <v>9.7875</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$90*'3 ขนาดบ่อ'!$E$91</f>
+        <v>12.4875</v>
       </c>
       <c r="D20" s="12" t="n">
         <f aca="false">('7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$42)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$42)</f>
-        <v>12.555</v>
+        <v>16.275</v>
       </c>
       <c r="E20" s="12" t="n">
-        <f aca="false">('7 แบบพับ'!$D$9+2*'1 ข้อมูล'!$C$42)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$42)+('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$9)*('3 ขนาดบ่อ'!$E$9+2*'1 ข้อมูล'!$C$42)</f>
-        <v>10.4925</v>
+        <f aca="false">('7 แบบพับ'!$D$9+2*'1 ข้อมูล'!$C$42)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$42)+('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$9)*('3 ขนาดบ่อ'!$E$12+2*'1 ข้อมูล'!$C$42)</f>
+        <v>13.5525</v>
       </c>
       <c r="F20" s="6"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="6" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
       <c r="C21" s="12" t="n">
-        <f aca="false">2*('3 ขนาดบ่อ'!$E$85+'1 ข้อมูล'!$C$42+'3 ขนาดบ่อ'!$E$86+'1 ข้อมูล'!$C$42)*'1 ข้อมูล'!$C$42*'3 ขนาดบ่อ'!$E$50</f>
-        <v>3.744</v>
+        <f aca="false">2*('3 ขนาดบ่อ'!$E$87+'1 ข้อมูล'!$C$42+'3 ขนาดบ่อ'!$E$88+'1 ข้อมูล'!$C$42)*'1 ข้อมูล'!$C$42*'3 ขนาดบ่อ'!$E$52</f>
+        <v>3.936</v>
       </c>
       <c r="D21" s="12" t="n">
-        <f aca="false">2*('7 แบบพับ'!$D$12+'1 ข้อมูล'!$C$42+'7 แบบพับ'!$D$14+'1 ข้อมูล'!$C$42)*'1 ข้อมูล'!$C$42*'3 ขนาดบ่อ'!$E$50</f>
-        <v>3.336</v>
+        <f aca="false">2*('7 แบบพับ'!$D$12+'1 ข้อมูล'!$C$42+'7 แบบพับ'!$D$14+'1 ข้อมูล'!$C$42)*'1 ข้อมูล'!$C$42*'3 ขนาดบ่อ'!$E$52</f>
+        <v>3.72</v>
       </c>
       <c r="E21" s="12" t="n">
-        <f aca="false">2*('7 แบบพับ'!$D$12+'1 ข้อมูล'!$C$42+'7 แบบพับ'!$D$14+'1 ข้อมูล'!$C$42)*'1 ข้อมูล'!$C$42*'3 ขนาดบ่อ'!$E$50</f>
-        <v>3.336</v>
+        <f aca="false">2*('7 แบบพับ'!$D$12+'1 ข้อมูล'!$C$42+'7 แบบพับ'!$D$14+'1 ข้อมูล'!$C$42)*'1 ข้อมูล'!$C$42*'3 ขนาดบ่อ'!$E$52</f>
+        <v>3.72</v>
       </c>
       <c r="F21" s="6"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="6" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="C22" s="12" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
       <c r="D22" s="12" t="n">
-        <f aca="false">('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$8)*'1 ข้อมูล'!$C$42*'3 ขนาดบ่อ'!$E$50</f>
+        <f aca="false">('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$8)*'1 ข้อมูล'!$C$42*'3 ขนาดบ่อ'!$E$52</f>
         <v>0.78</v>
       </c>
       <c r="E22" s="12" t="n">
-        <f aca="false">'7 แบบพับ'!$D$7*'1 ข้อมูล'!$C$42*'3 ขนาดบ่อ'!$E$50</f>
+        <f aca="false">'7 แบบพับ'!$D$7*'1 ข้อมูล'!$C$42*'3 ขนาดบ่อ'!$E$52</f>
         <v>0.384</v>
       </c>
       <c r="F22" s="6"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="6" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
       <c r="C23" s="12" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$88*'3 ขนาดบ่อ'!$E$89*'1 ข้อมูล'!$C$43</f>
-        <v>1.9575</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$90*'3 ขนาดบ่อ'!$E$91*'1 ข้อมูล'!$C$43</f>
+        <v>2.4975</v>
       </c>
       <c r="D23" s="12" t="n">
         <f aca="false">('7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$42)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$42)*'1 ข้อมูล'!$C$43</f>
-        <v>2.511</v>
+        <v>3.255</v>
       </c>
       <c r="E23" s="12" t="n">
-        <f aca="false">(('7 แบบพับ'!$D$9+2*'1 ข้อมูล'!$C$42)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$42)+('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$9)*('3 ขนาดบ่อ'!$E$9+2*'1 ข้อมูล'!$C$42))*'1 ข้อมูล'!$C$43</f>
-        <v>2.0985</v>
+        <f aca="false">(('7 แบบพับ'!$D$9+2*'1 ข้อมูล'!$C$42)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$42)+('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$9)*('3 ขนาดบ่อ'!$E$12+2*'1 ข้อมูล'!$C$42))*'1 ข้อมูล'!$C$43</f>
+        <v>2.7105</v>
       </c>
       <c r="F23" s="6"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="6" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="C24" s="27" t="n">
         <f aca="false">SUM(C21:C23)</f>
-        <v>5.7015</v>
+        <v>6.4335</v>
       </c>
       <c r="D24" s="27" t="n">
         <f aca="false">SUM(D21:D23)</f>
-        <v>6.627</v>
+        <v>7.755</v>
       </c>
       <c r="E24" s="27" t="n">
         <f aca="false">SUM(E21:E23)</f>
-        <v>5.8185</v>
+        <v>6.8145</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>382</v>
+        <v>388</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="6" t="s">
-        <v>383</v>
+        <v>389</v>
       </c>
       <c r="C25" s="6" t="s">
         <v>85</v>
@@ -5735,7 +5792,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="4" t="s">
-        <v>384</v>
+        <v>390</v>
       </c>
       <c r="C28" s="5"/>
       <c r="D28" s="5"/>
@@ -5744,10 +5801,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="30" t="s">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>386</v>
+        <v>392</v>
       </c>
       <c r="D29" s="6"/>
       <c r="E29" s="6"/>
@@ -5755,10 +5812,10 @@
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="30" t="s">
-        <v>387</v>
+        <v>393</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>388</v>
+        <v>394</v>
       </c>
       <c r="D30" s="6"/>
       <c r="E30" s="6"/>
@@ -5766,10 +5823,10 @@
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="30" t="s">
-        <v>389</v>
+        <v>395</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>390</v>
+        <v>396</v>
       </c>
       <c r="D31" s="6"/>
       <c r="E31" s="6"/>
@@ -5777,10 +5834,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="30" t="s">
-        <v>391</v>
+        <v>397</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="D32" s="6"/>
       <c r="E32" s="6"/>
@@ -5788,10 +5845,10 @@
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="31" t="s">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
       <c r="D33" s="6"/>
       <c r="E33" s="6"/>
@@ -5799,10 +5856,10 @@
     </row>
     <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="31" t="s">
-        <v>395</v>
+        <v>401</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
       <c r="D34" s="6"/>
       <c r="E34" s="6"/>
@@ -5810,10 +5867,10 @@
     </row>
     <row r="35" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="31" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>398</v>
+        <v>404</v>
       </c>
       <c r="D35" s="6"/>
       <c r="E35" s="6"/>
@@ -5821,10 +5878,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="31" t="s">
-        <v>399</v>
+        <v>405</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>400</v>
+        <v>406</v>
       </c>
       <c r="D36" s="6"/>
       <c r="E36" s="6"/>
@@ -5862,150 +5919,150 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>401</v>
+        <v>407</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>402</v>
+        <v>408</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>403</v>
+        <v>409</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>404</v>
+        <v>410</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>405</v>
+        <v>411</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>406</v>
+        <v>412</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>407</v>
+        <v>413</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>408</v>
+        <v>414</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>409</v>
+        <v>415</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>410</v>
+        <v>416</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="32" t="s">
-        <v>411</v>
+        <v>417</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>412</v>
+        <v>418</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>413</v>
+        <v>419</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>414</v>
+        <v>420</v>
       </c>
       <c r="F5" s="23" t="n">
         <f aca="false">'1 ข้อมูล'!$C$10/3600</f>
         <v>0.0174421296296296</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>415</v>
+        <v>421</v>
       </c>
       <c r="H5" s="12"/>
       <c r="I5" s="17"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="32" t="s">
-        <v>416</v>
+        <v>422</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>417</v>
+        <v>423</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>418</v>
+        <v>424</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>414</v>
+        <v>420</v>
       </c>
       <c r="F6" s="23" t="n">
         <f aca="false">1.5*F5</f>
         <v>0.0261631944444444</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>419</v>
+        <v>425</v>
       </c>
       <c r="H6" s="12"/>
       <c r="I6" s="17"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="32" t="s">
+        <v>426</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>428</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>420</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>421</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>422</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>414</v>
       </c>
       <c r="F7" s="23" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8/3600</f>
         <v>0.0277777777777778</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>423</v>
+        <v>429</v>
       </c>
       <c r="H7" s="12"/>
       <c r="I7" s="17"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="32" t="s">
-        <v>424</v>
+        <v>430</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>425</v>
+        <v>431</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>426</v>
+        <v>432</v>
       </c>
       <c r="E8" s="6"/>
       <c r="F8" s="23" t="n">
         <v>1</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>427</v>
+        <v>433</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>411</v>
+        <v>417</v>
       </c>
       <c r="I8" s="17"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="32" t="s">
-        <v>428</v>
+        <v>434</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>429</v>
+        <v>435</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>430</v>
+        <v>436</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>414</v>
+        <v>420</v>
       </c>
       <c r="F9" s="23" t="n">
         <f aca="false">MAX(F6,F7)/F8</f>
         <v>0.0277777777777778</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
       <c r="H9" s="12" t="n">
         <f aca="false">'2 เวียร์'!$D$13</f>
@@ -6013,12 +6070,12 @@
       </c>
       <c r="I9" s="17"/>
     </row>
-    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="32" t="s">
-        <v>432</v>
+        <v>438</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>433</v>
+        <v>439</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="6" t="s">
@@ -6029,23 +6086,23 @@
         <v>0.458178826795053</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>434</v>
+        <v>440</v>
       </c>
       <c r="H10" s="12" t="n">
-        <f aca="false">('3 ขนาดบ่อ'!$E$9-'3 ขนาดบ่อ'!$E$11)/2</f>
-        <v>0.225</v>
+        <f aca="false">('3 ขนาดบ่อ'!$E$12-'3 ขนาดบ่อ'!$E$10)/2</f>
+        <v>0.425</v>
       </c>
       <c r="I10" s="17" t="str">
         <f aca="false">IF(H10&gt;=2*F12,"ผ่าน ✔","ไม่ผ่าน ✘ (ต้อง ≥ 2Hmax)")</f>
-        <v>ไม่ผ่าน ✘ (ต้อง ≥ 2Hmax)</v>
+        <v>ผ่าน ✔</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="32" t="s">
-        <v>435</v>
+        <v>441</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="D11" s="6"/>
       <c r="E11" s="6" t="s">
@@ -6056,7 +6113,7 @@
         <v>0.416526206177321</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>436</v>
+        <v>442</v>
       </c>
       <c r="H11" s="12" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8</f>
@@ -6069,10 +6126,10 @@
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="32" t="s">
-        <v>437</v>
+        <v>443</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>438</v>
+        <v>444</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6" t="s">
@@ -6083,22 +6140,22 @@
         <v>0.208263103088661</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>439</v>
+        <v>445</v>
       </c>
       <c r="H12" s="12" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$7</f>
         <v>0.209665688762588</v>
       </c>
       <c r="I12" s="17" t="s">
-        <v>440</v>
+        <v>446</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="32" t="s">
-        <v>441</v>
+        <v>447</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>442</v>
+        <v>448</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="6"/>
@@ -6115,10 +6172,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="32" t="s">
-        <v>443</v>
+        <v>449</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>444</v>
+        <v>450</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
@@ -6135,10 +6192,10 @@
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="32" t="s">
-        <v>445</v>
+        <v>451</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>446</v>
+        <v>452</v>
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="6" t="s">
@@ -6149,10 +6206,10 @@
         <v>0.624789309265982</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
       <c r="H15" s="12" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$13</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$14</f>
         <v>0.95</v>
       </c>
       <c r="I15" s="17" t="str">
@@ -6162,10 +6219,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="32" t="s">
-        <v>448</v>
+        <v>454</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>449</v>
+        <v>455</v>
       </c>
       <c r="D16" s="6"/>
       <c r="E16" s="6" t="s">
@@ -6176,10 +6233,10 @@
         <v>0.249915723706393</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
       <c r="H16" s="12" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$10</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$9</f>
         <v>0.3</v>
       </c>
       <c r="I16" s="17" t="str">
@@ -6189,10 +6246,10 @@
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="32" t="s">
-        <v>451</v>
+        <v>457</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="D17" s="6"/>
       <c r="E17" s="6" t="s">
@@ -6203,15 +6260,15 @@
         <v>1.41618910100289</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>452</v>
+        <v>458</v>
       </c>
       <c r="H17" s="12" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$9</f>
-        <v>1.05</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$12</f>
+        <v>1.45</v>
       </c>
       <c r="I17" s="17" t="str">
         <f aca="false">IF(H17&gt;=F17,"ผ่าน ✔","แคบกว่า ✘")</f>
-        <v>แคบกว่า ✘</v>
+        <v>ผ่าน ✔</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6228,17 +6285,17 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="22" t="s">
-        <v>453</v>
+        <v>459</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="22" t="s">
-        <v>454</v>
+        <v>460</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="22" t="s">
-        <v>455</v>
+        <v>461</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Widen tank to B = 1.50 m for margin on b >= 2Hmax
b = 0.45 m; side-clearance criterion holds up to ~119 m3/h. External
6.75 x 1.90 m, weir plate 1.70 x 0.60 m.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXLmoKkgGBxM2QbbegGKn7
</commit_message>
<xml_diff>
--- a/weir_design.xlsx
+++ b/weir_design.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="462">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="612" uniqueCount="470">
   <si>
     <t xml:space="preserve">1) ข้อมูลออกแบบ — บ่อ 3 ช่อง: ปั๊มจุ่ม | โชว์น้ำใส | V-notch 90°</t>
   </si>
@@ -120,6 +120,12 @@
   </si>
   <si>
     <t xml:space="preserve">เลือกตามความสวยงาม (ต้อง ≥ ค่าขั้นต่ำในชีต 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ความกว้างบ่อขั้นต่ำที่เลือก</t>
+  </si>
+  <si>
+    <t xml:space="preserve">เผื่อ b ≥ 2Hmax ไว้ถึงน้ำเข้า ~125 m³/h (ค่าตามเกณฑ์ 1.44)</t>
   </si>
   <si>
     <t xml:space="preserve">ระยะเผื่อขอบบ่อ (freeboard)</t>
@@ -500,13 +506,22 @@
     <t xml:space="preserve">น้ำเข้าร่องไม่ถูกผนังข้างบีบ</t>
   </si>
   <si>
-    <t xml:space="preserve">B ความกว้างภายในบ่อ</t>
+    <t xml:space="preserve">B ตามเกณฑ์</t>
   </si>
   <si>
     <t xml:space="preserve">MAX(0.90, H ÷ 0.2, ปากร่อง + 2b)</t>
   </si>
   <si>
-    <t xml:space="preserve">ISO: B ≥ 0.90 และ H/B ≤ 0.2 / USBR–มข.: b ≥ 2H ข้างละ (ใช้ค่าที่มากกว่า)</t>
+    <t xml:space="preserve">ISO: B ≥ 0.90 และ H/B ≤ 0.2 / USBR–มข.: b ≥ 2H ข้างละ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B ความกว้างภายในบ่อ (ใช้)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAX(ตามเกณฑ์, ค่าที่เลือก)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">เลือก 1.50 เพื่อมีระยะเผื่อ</t>
   </si>
   <si>
     <t xml:space="preserve">ช่วงตรงหน้าเวียร์</t>
@@ -546,6 +561,15 @@
   </si>
   <si>
     <t xml:space="preserve">เกณฑ์ USBR / เอกสาร มข.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">น้ำเข้าสูงสุดที่ b ยังผ่าน</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.38 × (b ÷ 2)^2.5 × 3600</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ระยะเผื่อเทียบกับ 100 m³/h</t>
   </si>
   <si>
     <t xml:space="preserve">ตรวจ: จุดวัด ÷ H</t>
@@ -2027,7 +2051,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:E61"/>
+  <dimension ref="B1:E62"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -2237,7 +2261,7 @@
         <v>31</v>
       </c>
       <c r="C19" s="10" t="n">
-        <v>0.2</v>
+        <v>1.5</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>19</v>
@@ -2251,24 +2275,24 @@
         <v>33</v>
       </c>
       <c r="C20" s="10" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="D20" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E20" s="6" t="s">
         <v>34</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C21" s="10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D21" s="6" t="s">
         <v>36</v>
-      </c>
-      <c r="C21" s="11" t="n">
-        <v>0.168</v>
-      </c>
-      <c r="D21" s="6" t="s">
-        <v>19</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>37</v>
@@ -2278,8 +2302,8 @@
       <c r="B22" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C22" s="10" t="n">
-        <v>0.15</v>
+      <c r="C22" s="11" t="n">
+        <v>0.168</v>
       </c>
       <c r="D22" s="6" t="s">
         <v>19</v>
@@ -2293,7 +2317,7 @@
         <v>40</v>
       </c>
       <c r="C23" s="10" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>19</v>
@@ -2307,7 +2331,7 @@
         <v>42</v>
       </c>
       <c r="C24" s="10" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>19</v>
@@ -2321,7 +2345,7 @@
         <v>44</v>
       </c>
       <c r="C25" s="10" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>19</v>
@@ -2335,10 +2359,10 @@
         <v>46</v>
       </c>
       <c r="C26" s="10" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>47</v>
@@ -2349,10 +2373,10 @@
         <v>48</v>
       </c>
       <c r="C27" s="10" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="E27" s="6" t="s">
         <v>49</v>
@@ -2363,7 +2387,7 @@
         <v>50</v>
       </c>
       <c r="C28" s="10" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="D28" s="6" t="s">
         <v>19</v>
@@ -2382,21 +2406,21 @@
       <c r="D29" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E29" s="6"/>
+      <c r="E29" s="6" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C30" s="10" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="D30" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E30" s="6" t="s">
-        <v>54</v>
-      </c>
+      <c r="E30" s="6"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="6" t="s">
@@ -2408,11 +2432,13 @@
       <c r="D31" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E31" s="6"/>
+      <c r="E31" s="6" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C32" s="10" t="n">
         <v>0.1</v>
@@ -2420,9 +2446,7 @@
       <c r="D32" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E32" s="6" t="s">
-        <v>57</v>
-      </c>
+      <c r="E32" s="6"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="6" t="s">
@@ -2442,34 +2466,34 @@
       <c r="B34" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="C34" s="11" t="n">
-        <v>0.006</v>
+      <c r="C34" s="10" t="n">
+        <v>0.1</v>
       </c>
       <c r="D34" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E34" s="6"/>
+      <c r="E34" s="6" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="C35" s="10" t="n">
-        <v>0.3</v>
+        <v>62</v>
+      </c>
+      <c r="C35" s="11" t="n">
+        <v>0.006</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E35" s="6" t="s">
-        <v>62</v>
-      </c>
+      <c r="E35" s="6"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="6" t="s">
         <v>63</v>
       </c>
       <c r="C36" s="10" t="n">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>19</v>
@@ -2483,7 +2507,7 @@
         <v>65</v>
       </c>
       <c r="C37" s="10" t="n">
-        <v>0.25</v>
+        <v>0.15</v>
       </c>
       <c r="D37" s="6" t="s">
         <v>19</v>
@@ -2497,7 +2521,7 @@
         <v>67</v>
       </c>
       <c r="C38" s="10" t="n">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="D38" s="6" t="s">
         <v>19</v>
@@ -2511,7 +2535,7 @@
         <v>69</v>
       </c>
       <c r="C39" s="10" t="n">
-        <v>1.1</v>
+        <v>0.2</v>
       </c>
       <c r="D39" s="6" t="s">
         <v>19</v>
@@ -2525,7 +2549,7 @@
         <v>71</v>
       </c>
       <c r="C40" s="10" t="n">
-        <v>0.05</v>
+        <v>1.1</v>
       </c>
       <c r="D40" s="6" t="s">
         <v>19</v>
@@ -2539,26 +2563,26 @@
         <v>73</v>
       </c>
       <c r="C41" s="10" t="n">
-        <v>1.25</v>
+        <v>0.05</v>
       </c>
       <c r="D41" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E41" s="6"/>
+      <c r="E41" s="6" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C42" s="10" t="n">
-        <v>0.2</v>
+        <v>1.25</v>
       </c>
       <c r="D42" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E42" s="6" t="s">
-        <v>75</v>
-      </c>
+      <c r="E42" s="6"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="6" t="s">
@@ -2570,41 +2594,43 @@
       <c r="D43" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E43" s="6"/>
+      <c r="E43" s="6" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C44" s="10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E44" s="6"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B45" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="C45" s="10" t="n">
         <v>0.05</v>
       </c>
-      <c r="D44" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="C46" s="5"/>
-      <c r="D46" s="5"/>
-      <c r="E46" s="5"/>
+      <c r="D45" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E45" s="6" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="C47" s="12" t="n">
-        <v>9.81</v>
-      </c>
-      <c r="D47" s="6" t="s">
+      <c r="B47" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="E47" s="6"/>
+      <c r="C47" s="5"/>
+      <c r="D47" s="5"/>
+      <c r="E47" s="5"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="6" t="s">
@@ -2622,25 +2648,23 @@
       <c r="B49" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="C49" s="13" t="n">
-        <v>1.38</v>
+      <c r="C49" s="12" t="n">
+        <v>9.81</v>
       </c>
       <c r="D49" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="E49" s="6" t="s">
-        <v>86</v>
-      </c>
+      <c r="E49" s="6"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C50" s="13" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="D50" s="6" t="s">
         <v>87</v>
-      </c>
-      <c r="C50" s="13" t="n">
-        <v>0.578</v>
-      </c>
-      <c r="D50" s="6" t="s">
-        <v>85</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>88</v>
@@ -2650,28 +2674,28 @@
       <c r="B51" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="C51" s="14" t="n">
-        <v>0.00085</v>
+      <c r="C51" s="13" t="n">
+        <v>0.578</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>19</v>
+        <v>87</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="C52" s="14" t="n">
+        <v>0.00085</v>
+      </c>
+      <c r="D52" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E52" s="6" t="s">
         <v>90</v>
-      </c>
-      <c r="C52" s="12" t="n">
-        <v>1.84</v>
-      </c>
-      <c r="D52" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="E52" s="6" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2679,10 +2703,10 @@
         <v>92</v>
       </c>
       <c r="C53" s="12" t="n">
-        <v>0.6</v>
+        <v>1.84</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E53" s="6" t="s">
         <v>93</v>
@@ -2692,80 +2716,94 @@
       <c r="B54" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="C54" s="15" t="n">
-        <v>205</v>
+      <c r="C54" s="12" t="n">
+        <v>0.6</v>
       </c>
       <c r="D54" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="E54" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="E54" s="6"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="6" t="s">
         <v>96</v>
       </c>
       <c r="C55" s="15" t="n">
-        <v>400</v>
+        <v>205</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E55" s="6"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="C56" s="15" t="n">
+        <v>400</v>
+      </c>
+      <c r="D56" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="C56" s="9" t="n">
+      <c r="E56" s="6"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B57" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C57" s="9" t="n">
         <v>1.7</v>
       </c>
-      <c r="D56" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="E56" s="6"/>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B58" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="C58" s="5"/>
-      <c r="D58" s="5"/>
-      <c r="E58" s="5"/>
+      <c r="D57" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="E57" s="6"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B59" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C59" s="16" t="s">
+      <c r="B59" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="D59" s="6"/>
-      <c r="E59" s="6" t="s">
-        <v>101</v>
-      </c>
+      <c r="C59" s="5"/>
+      <c r="D59" s="5"/>
+      <c r="E59" s="5"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C60" s="16" t="s">
         <v>102</v>
-      </c>
-      <c r="C60" s="17" t="s">
-        <v>103</v>
       </c>
       <c r="D60" s="6"/>
       <c r="E60" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C61" s="17" t="s">
         <v>105</v>
-      </c>
-      <c r="C61" s="6" t="s">
-        <v>106</v>
       </c>
       <c r="D61" s="6"/>
       <c r="E61" s="6" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B62" s="6" t="s">
         <v>107</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="D62" s="6"/>
+      <c r="E62" s="6" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -2799,17 +2837,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="4" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="5"/>
@@ -2820,17 +2858,17 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C5" s="13" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$49</f>
+        <f aca="false">'1 ข้อมูล'!$C$50</f>
         <v>1.38</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
@@ -2838,17 +2876,17 @@
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C6" s="18" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$50*(8/15)*SQRT(2*'1 ข้อมูล'!$C$47)</f>
+        <f aca="false">'1 ข้อมูล'!$C$51*(8/15)*SQRT(2*'1 ข้อมูล'!$C$48)</f>
         <v>1.36545083661038</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
@@ -2856,7 +2894,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="4" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
@@ -2867,30 +2905,30 @@
     </row>
     <row r="9" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="3" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C10" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$7-'1 ข้อมูล'!$C$9</f>
@@ -2905,7 +2943,7 @@
         <v>14.532869095236</v>
       </c>
       <c r="F10" s="9" t="n">
-        <f aca="false">((D10/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$51)*100</f>
+        <f aca="false">((D10/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$52)*100</f>
         <v>14.5096125168743</v>
       </c>
       <c r="G10" s="20" t="n">
@@ -2916,7 +2954,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C11" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$10-'1 ข้อมูล'!$C$9</f>
@@ -2931,7 +2969,7 @@
         <v>16.2387843483091</v>
       </c>
       <c r="F11" s="9" t="n">
-        <f aca="false">((D11/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$51)*100</f>
+        <f aca="false">((D11/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$52)*100</f>
         <v>16.2227754127948</v>
       </c>
       <c r="G11" s="20" t="n">
@@ -2939,12 +2977,12 @@
         <v>0.0160089355143072</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C12" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8-'1 ข้อมูล'!$C$9</f>
@@ -2959,7 +2997,7 @@
         <v>20.1013103538681</v>
       </c>
       <c r="F12" s="9" t="n">
-        <f aca="false">((D12/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$51)*100</f>
+        <f aca="false">((D12/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$52)*100</f>
         <v>20.1017115002301</v>
       </c>
       <c r="G12" s="20" t="n">
@@ -2970,7 +3008,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="21" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C13" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8</f>
@@ -2985,7 +3023,7 @@
         <v>20.9665688762588</v>
       </c>
       <c r="F13" s="9" t="n">
-        <f aca="false">((D13/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$51)*100</f>
+        <f aca="false">((D13/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$52)*100</f>
         <v>20.9706461048468</v>
       </c>
       <c r="G13" s="20" t="n">
@@ -2993,22 +3031,22 @@
         <v>-0.00407722858800952</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="22" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="22" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="22" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -3027,7 +3065,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:G92"/>
+  <dimension ref="B1:G94"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -3040,12 +3078,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3053,24 +3091,24 @@
         <v>2</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>4</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="4" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -3080,10 +3118,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D7" s="13"/>
       <c r="E7" s="23" t="n">
@@ -3094,15 +3132,15 @@
         <v>19</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D8" s="13" t="n">
         <f aca="false">MAX(0.45,'3 ขนาดบ่อ'!$E$7/0.4)+'1 ข้อมูล'!$C$14</f>
@@ -3116,15 +3154,15 @@
         <v>19</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="6" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D9" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$7+'1 ข้อมูล'!$C$15</f>
@@ -3138,15 +3176,15 @@
         <v>19</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D10" s="13"/>
       <c r="E10" s="23" t="n">
@@ -3157,15 +3195,15 @@
         <v>19</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D11" s="13"/>
       <c r="E11" s="23" t="n">
@@ -3176,106 +3214,107 @@
         <v>19</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="D12" s="13" t="n">
+        <v>157</v>
+      </c>
+      <c r="D12" s="13"/>
+      <c r="E12" s="23" t="n">
         <f aca="false">MAX(0.9,'3 ขนาดบ่อ'!$E$7/0.2,'3 ขนาดบ่อ'!$E$10+2*'3 ขนาดบ่อ'!$E$11)</f>
         <v>1.43866275505035</v>
       </c>
-      <c r="E12" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D12,4),'1 ข้อมูล'!$C$13)</f>
-        <v>1.45</v>
-      </c>
       <c r="F12" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="6" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D13" s="13" t="n">
+        <f aca="false">MAX('3 ขนาดบ่อ'!$E$12,'1 ข้อมูล'!$C$19)</f>
+        <v>1.5</v>
+      </c>
+      <c r="E13" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D13,4),'1 ข้อมูล'!$C$13)</f>
+        <v>1.5</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="D14" s="13" t="n">
         <f aca="false">10*'3 ขนาดบ่อ'!$E$7</f>
         <v>2.09665688762588</v>
       </c>
-      <c r="E13" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D13,4),'1 ข้อมูล'!$C$13)</f>
+      <c r="E14" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D14,4),'1 ข้อมูล'!$C$13)</f>
         <v>2.1</v>
       </c>
-      <c r="F13" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G13" s="6" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="D14" s="13" t="n">
+      <c r="F14" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="D15" s="13" t="n">
         <f aca="false">4.5*'3 ขนาดบ่อ'!$E$7</f>
         <v>0.943495599431645</v>
       </c>
-      <c r="E14" s="23" t="n">
-        <f aca="false">ROUND(D14/'1 ข้อมูล'!$C$13,0)*'1 ข้อมูล'!$C$13</f>
+      <c r="E15" s="23" t="n">
+        <f aca="false">ROUND(D15/'1 ข้อมูล'!$C$13,0)*'1 ข้อมูล'!$C$13</f>
         <v>0.95</v>
       </c>
-      <c r="F14" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G14" s="6" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>164</v>
-      </c>
-      <c r="D15" s="13" t="n">
+      <c r="F15" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="D16" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$7/'3 ขนาดบ่อ'!$E$8</f>
         <v>0.349442814604313</v>
       </c>
-      <c r="E15" s="17" t="str">
-        <f aca="false">IF(D15&lt;=0.4,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
-        <v>ผ่าน ✔</v>
-      </c>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="D16" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$7/'3 ขนาดบ่อ'!$E$12</f>
-        <v>0.144597026732819</v>
-      </c>
       <c r="E16" s="17" t="str">
-        <f aca="false">IF(D16&lt;=0.2,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <f aca="false">IF(D16&lt;=0.4,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
       <c r="F16" s="6"/>
@@ -3283,240 +3322,243 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="D17" s="13" t="n">
-        <f aca="false">('3 ขนาดบ่อ'!$E$12-'3 ขนาดบ่อ'!$E$10)/2</f>
-        <v>0.425</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$7/'3 ขนาดบ่อ'!$E$13</f>
+        <v>0.139777125841725</v>
       </c>
       <c r="E17" s="17" t="str">
-        <f aca="false">IF(D17&gt;=2*'3 ขนาดบ่อ'!$E$7,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <f aca="false">IF(D17&lt;=0.2,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
       <c r="F17" s="6"/>
-      <c r="G17" s="6" t="s">
-        <v>169</v>
-      </c>
+      <c r="G17" s="6"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="6" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D18" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$14/'3 ขนาดบ่อ'!$E$7</f>
-        <v>4.5310227229202</v>
+        <f aca="false">('3 ขนาดบ่อ'!$E$13-'3 ขนาดบ่อ'!$E$10)/2</f>
+        <v>0.45</v>
       </c>
       <c r="E18" s="17" t="str">
-        <f aca="false">IF(AND(D18&gt;=4,D18&lt;=5),"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <f aca="false">IF(D18&gt;=2*'3 ขนาดบ่อ'!$E$7,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
       <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
+      <c r="G18" s="6" t="s">
+        <v>174</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="6" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="D19" s="13" t="n">
+        <v>176</v>
+      </c>
+      <c r="D19" s="9"/>
+      <c r="E19" s="19" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$50*(('3 ขนาดบ่อ'!$E$13-'3 ขนาดบ่อ'!$E$10)/4)^2.5*3600</f>
+        <v>119.299296438097</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="D20" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$15/'3 ขนาดบ่อ'!$E$7</f>
+        <v>4.5310227229202</v>
+      </c>
+      <c r="E20" s="17" t="str">
+        <f aca="false">IF(AND(D20&gt;=4,D20&lt;=5),"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F20" s="6"/>
+      <c r="G20" s="6"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="D21" s="13" t="n">
         <f aca="false">'2 เวียร์'!$E$10/100</f>
         <v>0.14532869095236</v>
       </c>
-      <c r="E19" s="17" t="str">
-        <f aca="false">IF(D19&gt;=0.05,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+      <c r="E21" s="17" t="str">
+        <f aca="false">IF(D21&gt;=0.05,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="D22" s="13"/>
-      <c r="E22" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$29/2+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$53*PI()*'1 ข้อมูล'!$C$29^2/4))^2/(2*'1 ข้อมูล'!$C$47)</f>
-        <v>0.210686269183871</v>
-      </c>
-      <c r="F22" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G22" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="6" t="s">
+        <v>182</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="D23" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$8-'3 ขนาดบ่อ'!$E$22</f>
-        <v>0.389313730816129</v>
-      </c>
-      <c r="E23" s="17" t="str">
-        <f aca="false">IF(D23&gt;=0.06,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
-        <v>ผ่าน ✔</v>
-      </c>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6" t="s">
-        <v>180</v>
-      </c>
+      <c r="B23" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="6" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="D24" s="13"/>
       <c r="E24" s="23" t="n">
-        <f aca="false">SQRT(2*'1 ข้อมูล'!$C$47*'3 ขนาดบ่อ'!$E$7)</f>
-        <v>2.02821123493634</v>
+        <f aca="false">'1 ข้อมูล'!$C$30/2+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$54*PI()*'1 ข้อมูล'!$C$30^2/4))^2/(2*'1 ข้อมูล'!$C$48)</f>
+        <v>0.210686269183871</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="G24" s="6" t="s">
-        <v>183</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="G24" s="6"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="6" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="D25" s="13"/>
-      <c r="E25" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$7-'3 ขนาดบ่อ'!$E$22</f>
-        <v>0.598979419578717</v>
-      </c>
-      <c r="F25" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G25" s="6"/>
+        <v>187</v>
+      </c>
+      <c r="D25" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$8-'3 ขนาดบ่อ'!$E$24</f>
+        <v>0.389313730816129</v>
+      </c>
+      <c r="E25" s="17" t="str">
+        <f aca="false">IF(D25&gt;=0.06,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F25" s="6"/>
+      <c r="G25" s="6" t="s">
+        <v>188</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="6" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="D26" s="13"/>
       <c r="E26" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$24*SQRT(2*'3 ขนาดบ่อ'!$E$25/'1 ข้อมูล'!$C$47)</f>
-        <v>0.708760700266562</v>
+        <f aca="false">SQRT(2*'1 ข้อมูล'!$C$48*'3 ขนาดบ่อ'!$E$7)</f>
+        <v>2.02821123493634</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="6" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>190</v>
-      </c>
-      <c r="D27" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$26+'1 ข้อมูล'!$C$28</f>
+        <v>193</v>
+      </c>
+      <c r="D27" s="13"/>
+      <c r="E27" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$7-'3 ขนาดบ่อ'!$E$24</f>
+        <v>0.598979419578717</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G27" s="6"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="D28" s="13"/>
+      <c r="E28" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$26*SQRT(2*'3 ขนาดบ่อ'!$E$27/'1 ข้อมูล'!$C$48)</f>
+        <v>0.708760700266562</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="D29" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$28+'1 ข้อมูล'!$C$29</f>
         <v>0.908760700266562</v>
       </c>
-      <c r="E27" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D27,4),'1 ข้อมูล'!$C$13)</f>
+      <c r="E29" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D29,4),'1 ข้อมูล'!$C$13)</f>
         <v>0.95</v>
       </c>
-      <c r="F27" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G27" s="6"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="C29" s="5"/>
-      <c r="D29" s="5"/>
-      <c r="E29" s="5"/>
-      <c r="F29" s="5"/>
-      <c r="G29" s="5"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="6" t="s">
-        <v>192</v>
-      </c>
-      <c r="C30" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="D30" s="13"/>
-      <c r="E30" s="23" t="n">
+      <c r="F29" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G29" s="6"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="C31" s="5"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
+      <c r="G31" s="5"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="D32" s="13"/>
+      <c r="E32" s="23" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$7</f>
         <v>0.809665688762588</v>
       </c>
-      <c r="F30" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G30" s="6"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="D31" s="13"/>
-      <c r="E31" s="23" t="n">
-        <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$12*'3 ขนาดบ่อ'!$E$30)</f>
-        <v>0.0236604914701068</v>
-      </c>
-      <c r="F31" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="G31" s="6"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="C32" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="D32" s="13"/>
-      <c r="E32" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$30/'1 ข้อมูล'!$C$26*'3 ขนาดบ่อ'!$E$31</f>
-        <v>0.191570881226054</v>
-      </c>
       <c r="F32" s="6" t="s">
         <v>19</v>
       </c>
@@ -3524,193 +3566,190 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="6" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="D33" s="13" t="n">
-        <f aca="false">MAX('1 ข้อมูล'!$C$27,'3 ขนาดบ่อ'!$E$32)</f>
+        <v>203</v>
+      </c>
+      <c r="D33" s="13"/>
+      <c r="E33" s="23" t="n">
+        <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$13*'3 ขนาดบ่อ'!$E$32)</f>
+        <v>0.0228718084211032</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="G33" s="6"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="D34" s="13"/>
+      <c r="E34" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$32/'1 ข้อมูล'!$C$27*'3 ขนาดบ่อ'!$E$33</f>
+        <v>0.185185185185185</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G34" s="6"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B35" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="D35" s="13" t="n">
+        <f aca="false">MAX('1 ข้อมูล'!$C$28,'3 ขนาดบ่อ'!$E$34)</f>
         <v>0.5</v>
       </c>
-      <c r="E33" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D33,4),'1 ข้อมูล'!$C$13)</f>
+      <c r="E35" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D35,4),'1 ข้อมูล'!$C$13)</f>
         <v>0.5</v>
       </c>
-      <c r="F33" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G33" s="6" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="C35" s="5"/>
-      <c r="D35" s="5"/>
-      <c r="E35" s="5"/>
-      <c r="F35" s="5"/>
-      <c r="G35" s="5"/>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="C36" s="6" t="s">
-        <v>203</v>
-      </c>
-      <c r="D36" s="13"/>
-      <c r="E36" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$17+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$52*'3 ขนาดบ่อ'!$E$12))^(2/3)</f>
-        <v>0.067680534585692</v>
-      </c>
-      <c r="F36" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G36" s="6" t="s">
-        <v>204</v>
+      <c r="F35" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G35" s="6" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>206</v>
-      </c>
-      <c r="D37" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$30+'1 ข้อมูล'!$C$16-'1 ข้อมูล'!$C$17</f>
-        <v>0.889665688762588</v>
-      </c>
-      <c r="E37" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D37,4),'1 ข้อมูล'!$C$13)</f>
-        <v>0.9</v>
-      </c>
-      <c r="F37" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G37" s="6" t="s">
-        <v>26</v>
-      </c>
+      <c r="B37" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="C37" s="5"/>
+      <c r="D37" s="5"/>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
+      <c r="G37" s="5"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="6" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>208</v>
-      </c>
-      <c r="D38" s="13" t="n">
-        <f aca="false">10*'3 ขนาดบ่อ'!$E$36</f>
-        <v>0.67680534585692</v>
-      </c>
+        <v>211</v>
+      </c>
+      <c r="D38" s="13"/>
       <c r="E38" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D38,4),'1 ข้อมูล'!$C$13)</f>
-        <v>0.7</v>
+        <f aca="false">'1 ข้อมูล'!$C$17+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$53*'3 ขนาดบ่อ'!$E$13))^(2/3)</f>
+        <v>0.0666149917231983</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="6" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="D39" s="13"/>
+        <v>214</v>
+      </c>
+      <c r="D39" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$32+'1 ข้อมูล'!$C$16-'1 ข้อมูล'!$C$17</f>
+        <v>0.889665688762588</v>
+      </c>
       <c r="E39" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D39,4),'1 ข้อมูล'!$C$13)</f>
+        <v>0.9</v>
+      </c>
+      <c r="F39" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G39" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B40" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="D40" s="13" t="n">
+        <f aca="false">10*'3 ขนาดบ่อ'!$E$38</f>
+        <v>0.666149917231983</v>
+      </c>
+      <c r="E40" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D40,4),'1 ข้อมูล'!$C$13)</f>
+        <v>0.7</v>
+      </c>
+      <c r="F40" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G40" s="6" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B41" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="D41" s="13"/>
+      <c r="E41" s="23" t="n">
         <f aca="false">'1 ข้อมูล'!$C$18</f>
         <v>1</v>
       </c>
-      <c r="F39" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G39" s="6"/>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="6" t="s">
-        <v>212</v>
-      </c>
-      <c r="C40" s="6"/>
-      <c r="D40" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$39-'3 ขนาดบ่อ'!$E$38</f>
+      <c r="F41" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G41" s="6"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B42" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C42" s="6"/>
+      <c r="D42" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$41-'3 ขนาดบ่อ'!$E$40</f>
         <v>0.3</v>
       </c>
-      <c r="E40" s="17" t="str">
-        <f aca="false">IF(D40&gt;=0,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+      <c r="E42" s="17" t="str">
+        <f aca="false">IF(D42&gt;=0,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
-      <c r="F40" s="6"/>
-      <c r="G40" s="6"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="C42" s="5"/>
-      <c r="D42" s="5"/>
-      <c r="E42" s="5"/>
-      <c r="F42" s="5"/>
-      <c r="G42" s="5"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>215</v>
-      </c>
-      <c r="D43" s="13" t="n">
-        <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$12*'1 ข้อมูล'!$C$20)</f>
-        <v>0.191570881226054</v>
-      </c>
-      <c r="E43" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D43,4),'1 ข้อมูล'!$C$13)</f>
-        <v>0.2</v>
-      </c>
-      <c r="F43" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G43" s="6"/>
+      <c r="F42" s="6"/>
+      <c r="G42" s="6"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="6" t="s">
-        <v>216</v>
-      </c>
-      <c r="C44" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="D44" s="13" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$21+2*'1 ข้อมูล'!$C$22</f>
-        <v>0.468</v>
-      </c>
-      <c r="E44" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D44,4),'1 ข้อมูล'!$C$13)</f>
-        <v>0.5</v>
-      </c>
-      <c r="F44" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G44" s="6"/>
+      <c r="B44" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="C44" s="5"/>
+      <c r="D44" s="5"/>
+      <c r="E44" s="5"/>
+      <c r="F44" s="5"/>
+      <c r="G44" s="5"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="6" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>219</v>
-      </c>
-      <c r="D45" s="13"/>
+        <v>223</v>
+      </c>
+      <c r="D45" s="13" t="n">
+        <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$13*'1 ข้อมูล'!$C$21)</f>
+        <v>0.185185185185185</v>
+      </c>
       <c r="E45" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$23</f>
-        <v>0.1</v>
+        <f aca="false">CEILING(ROUND(D45,4),'1 ข้อมูล'!$C$13)</f>
+        <v>0.2</v>
       </c>
       <c r="F45" s="6" t="s">
         <v>19</v>
@@ -3719,18 +3758,18 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="6" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="D46" s="13" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$24+2*'1 ข้อมูล'!$C$25</f>
-        <v>1</v>
+        <f aca="false">'1 ข้อมูล'!$C$22+2*'1 ข้อมูล'!$C$23</f>
+        <v>0.468</v>
       </c>
       <c r="E46" s="23" t="n">
         <f aca="false">CEILING(ROUND(D46,4),'1 ข้อมูล'!$C$13)</f>
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>19</v>
@@ -3739,15 +3778,15 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="6" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="D47" s="13"/>
       <c r="E47" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$44+'3 ขนาดบ่อ'!$E$45+'3 ขนาดบ่อ'!$E$46</f>
-        <v>1.6</v>
+        <f aca="false">'1 ข้อมูล'!$C$24</f>
+        <v>0.1</v>
       </c>
       <c r="F47" s="6" t="s">
         <v>19</v>
@@ -3756,148 +3795,149 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="6" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>225</v>
-      </c>
-      <c r="D48" s="13"/>
+        <v>229</v>
+      </c>
+      <c r="D48" s="13" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$25+2*'1 ข้อมูล'!$C$26</f>
+        <v>1</v>
+      </c>
       <c r="E48" s="23" t="n">
-        <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$12*'3 ขนาดบ่อ'!$E$36)</f>
-        <v>0.283051666773555</v>
+        <f aca="false">CEILING(ROUND(D48,4),'1 ข้อมูล'!$C$13)</f>
+        <v>1</v>
       </c>
       <c r="F48" s="6" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="G48" s="6"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="6" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="D49" s="13"/>
       <c r="E49" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$37+'3 ขนาดบ่อ'!$E$36+1.5*'3 ขนาดบ่อ'!$E$48^2/(2*'1 ข้อมูล'!$C$47)</f>
-        <v>0.973805782755668</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$46+'3 ขนาดบ่อ'!$E$47+'3 ขนาดบ่อ'!$E$48</f>
+        <v>1.6</v>
       </c>
       <c r="F49" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G49" s="6" t="s">
-        <v>228</v>
-      </c>
+      <c r="G49" s="6"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B50" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="D50" s="13"/>
+      <c r="E50" s="23" t="n">
+        <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$13*'3 ขนาดบ่อ'!$E$38)</f>
+        <v>0.277993257065429</v>
+      </c>
+      <c r="F50" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="G50" s="6"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="4" t="s">
-        <v>229</v>
-      </c>
-      <c r="C51" s="5"/>
-      <c r="D51" s="5"/>
-      <c r="E51" s="5"/>
-      <c r="F51" s="5"/>
-      <c r="G51" s="5"/>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B52" s="6" t="s">
-        <v>230</v>
-      </c>
-      <c r="C52" s="6" t="s">
-        <v>231</v>
-      </c>
-      <c r="D52" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$49+'1 ข้อมูล'!$C$19</f>
-        <v>1.17380578275567</v>
-      </c>
-      <c r="E52" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D52,4),'1 ข้อมูล'!$C$13)</f>
+      <c r="B51" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="D51" s="13"/>
+      <c r="E51" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$39+'3 ขนาดบ่อ'!$E$38+1.5*'3 ขนาดบ่อ'!$E$50^2/(2*'1 ข้อมูล'!$C$48)</f>
+        <v>0.972523267791535</v>
+      </c>
+      <c r="F51" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G51" s="6" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B53" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="C53" s="5"/>
+      <c r="D53" s="5"/>
+      <c r="E53" s="5"/>
+      <c r="F53" s="5"/>
+      <c r="G53" s="5"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B54" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="D54" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$51+'1 ข้อมูล'!$C$20</f>
+        <v>1.17252326779154</v>
+      </c>
+      <c r="E54" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D54,4),'1 ข้อมูล'!$C$13)</f>
         <v>1.2</v>
       </c>
-      <c r="F52" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G52" s="6" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B54" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="C54" s="5"/>
-      <c r="D54" s="5"/>
-      <c r="E54" s="5"/>
-      <c r="F54" s="5"/>
-      <c r="G54" s="5"/>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B55" s="6" t="s">
-        <v>234</v>
-      </c>
-      <c r="C55" s="6" t="s">
-        <v>235</v>
-      </c>
-      <c r="D55" s="13"/>
-      <c r="E55" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$8-'1 ข้อมูล'!$C$30</f>
-        <v>0.5</v>
-      </c>
-      <c r="F55" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G55" s="6" t="s">
-        <v>236</v>
+      <c r="F54" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G54" s="6" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B56" s="6" t="s">
-        <v>237</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="D56" s="13"/>
-      <c r="E56" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$12+2*'1 ข้อมูล'!$C$33</f>
-        <v>1.65</v>
-      </c>
-      <c r="F56" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G56" s="6"/>
+      <c r="B56" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="C56" s="5"/>
+      <c r="D56" s="5"/>
+      <c r="E56" s="5"/>
+      <c r="F56" s="5"/>
+      <c r="G56" s="5"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="6" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="D57" s="13"/>
       <c r="E57" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$55-'1 ข้อมูล'!$C$31</f>
-        <v>0.4</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$8-'1 ข้อมูล'!$C$31</f>
+        <v>0.5</v>
       </c>
       <c r="F57" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G57" s="6" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="6" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="D58" s="13"/>
       <c r="E58" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$9+'1 ข้อมูล'!$C$32</f>
-        <v>1</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$13+2*'1 ข้อมูล'!$C$34</f>
+        <v>1.7</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>19</v>
@@ -3906,32 +3946,34 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="6" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="D59" s="13"/>
       <c r="E59" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$58-'3 ขนาดบ่อ'!$E$57</f>
-        <v>0.6</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$57-'1 ข้อมูล'!$C$32</f>
+        <v>0.4</v>
       </c>
       <c r="F59" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G59" s="6"/>
+      <c r="G59" s="6" t="s">
+        <v>249</v>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="6" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="D60" s="13"/>
       <c r="E60" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$30-'3 ขนาดบ่อ'!$E$55</f>
-        <v>0.309665688762588</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$9+'1 ข้อมูล'!$C$33</f>
+        <v>1</v>
       </c>
       <c r="F60" s="6" t="s">
         <v>19</v>
@@ -3940,425 +3982,425 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="6" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="D61" s="13"/>
       <c r="E61" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$48*'3 ขนาดบ่อ'!$E$60^3/6</f>
-        <v>0.0485508704265308</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$60-'3 ขนาดบ่อ'!$E$59</f>
+        <v>0.6</v>
       </c>
       <c r="F61" s="6" t="s">
-        <v>250</v>
-      </c>
-      <c r="G61" s="6" t="s">
-        <v>251</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="G61" s="6"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="6" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="D62" s="13"/>
       <c r="E62" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$61/('1 ข้อมูล'!$C$34^2/6)/1000</f>
-        <v>8.09181173775513</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$32-'3 ขนาดบ่อ'!$E$57</f>
+        <v>0.309665688762588</v>
       </c>
       <c r="F62" s="6" t="s">
-        <v>95</v>
+        <v>19</v>
       </c>
       <c r="G62" s="6"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="6" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>255</v>
-      </c>
-      <c r="D63" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$62</f>
+        <v>257</v>
+      </c>
+      <c r="D63" s="13"/>
+      <c r="E63" s="23" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$49*'3 ขนาดบ่อ'!$E$62^3/6</f>
+        <v>0.0485508704265308</v>
+      </c>
+      <c r="F63" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="G63" s="6" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B64" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="D64" s="13"/>
+      <c r="E64" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$63/('1 ข้อมูล'!$C$35^2/6)/1000</f>
         <v>8.09181173775513</v>
       </c>
-      <c r="E63" s="17" t="str">
-        <f aca="false">IF(D63&lt;=0.6*'1 ข้อมูล'!$C$54,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+      <c r="F64" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="G64" s="6"/>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B65" s="6" t="s">
+        <v>262</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="D65" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$64</f>
+        <v>8.09181173775513</v>
+      </c>
+      <c r="E65" s="17" t="str">
+        <f aca="false">IF(D65&lt;=0.6*'1 ข้อมูล'!$C$55,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
-      <c r="F63" s="6"/>
-      <c r="G63" s="6" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B65" s="4" t="s">
-        <v>257</v>
-      </c>
-      <c r="C65" s="5"/>
-      <c r="D65" s="5"/>
-      <c r="E65" s="5"/>
-      <c r="F65" s="5"/>
-      <c r="G65" s="5"/>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B66" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="C66" s="6" t="s">
-        <v>259</v>
-      </c>
-      <c r="D66" s="13"/>
-      <c r="E66" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$48*'3 ขนาดบ่อ'!$E$52^3/6</f>
-        <v>2.82528</v>
-      </c>
-      <c r="F66" s="6" t="s">
-        <v>250</v>
-      </c>
-      <c r="G66" s="6" t="s">
-        <v>260</v>
+      <c r="F65" s="6"/>
+      <c r="G65" s="6" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B67" s="6" t="s">
-        <v>261</v>
-      </c>
-      <c r="C67" s="6" t="s">
-        <v>262</v>
-      </c>
-      <c r="D67" s="13"/>
-      <c r="E67" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$56*'3 ขนาดบ่อ'!$E$66</f>
-        <v>4.802976</v>
-      </c>
-      <c r="F67" s="6" t="s">
-        <v>250</v>
-      </c>
-      <c r="G67" s="6"/>
+      <c r="B67" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="C67" s="5"/>
+      <c r="D67" s="5"/>
+      <c r="E67" s="5"/>
+      <c r="F67" s="5"/>
+      <c r="G67" s="5"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B68" s="6" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="D68" s="13"/>
       <c r="E68" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$42-'1 ข้อมูล'!$C$44-0.006</f>
-        <v>0.144</v>
+        <f aca="false">'1 ข้อมูล'!$C$49*'3 ขนาดบ่อ'!$E$54^3/6</f>
+        <v>2.82528</v>
       </c>
       <c r="F68" s="6" t="s">
-        <v>19</v>
+        <v>258</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B69" s="6" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="D69" s="13"/>
       <c r="E69" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$67/(0.9*'1 ข้อมูล'!$C$55*1000*0.9*'3 ขนาดบ่อ'!$E$68)*1000000</f>
-        <v>102.944444444444</v>
+        <f aca="false">'1 ข้อมูล'!$C$57*'3 ขนาดบ่อ'!$E$68</f>
+        <v>4.802976</v>
       </c>
       <c r="F69" s="6" t="s">
-        <v>268</v>
+        <v>258</v>
       </c>
       <c r="G69" s="6"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B70" s="6" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="D70" s="13"/>
       <c r="E70" s="23" t="n">
-        <f aca="false">0.003*1000*'1 ข้อมูล'!$C$42*1000</f>
-        <v>600</v>
+        <f aca="false">'1 ข้อมูล'!$C$43-'1 ข้อมูล'!$C$45-0.006</f>
+        <v>0.144</v>
       </c>
       <c r="F70" s="6" t="s">
-        <v>268</v>
+        <v>19</v>
       </c>
       <c r="G70" s="6" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B71" s="6" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D71" s="13"/>
       <c r="E71" s="23" t="n">
-        <f aca="false">FLOOR(113/MAX('3 ขนาดบ่อ'!$E$69,'3 ขนาดบ่อ'!$E$70)*1000,25)</f>
-        <v>175</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$69/(0.9*'1 ข้อมูล'!$C$56*1000*0.9*'3 ขนาดบ่อ'!$E$70)*1000000</f>
+        <v>102.944444444444</v>
       </c>
       <c r="F71" s="6" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="G71" s="6"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B72" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="C72" s="6"/>
-      <c r="D72" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$71</f>
+        <v>277</v>
+      </c>
+      <c r="C72" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="D72" s="13"/>
+      <c r="E72" s="23" t="n">
+        <f aca="false">0.003*1000*'1 ข้อมูล'!$C$43*1000</f>
+        <v>600</v>
+      </c>
+      <c r="F72" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="G72" s="6" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B73" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="D73" s="13"/>
+      <c r="E73" s="23" t="n">
+        <f aca="false">FLOOR(113/MAX('3 ขนาดบ่อ'!$E$71,'3 ขนาดบ่อ'!$E$72)*1000,25)</f>
         <v>175</v>
       </c>
-      <c r="E72" s="17" t="str">
-        <f aca="false">IF(D72&gt;=100,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+      <c r="F73" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="G73" s="6"/>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B74" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="C74" s="6"/>
+      <c r="D74" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$73</f>
+        <v>175</v>
+      </c>
+      <c r="E74" s="17" t="str">
+        <f aca="false">IF(D74&gt;=100,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
-      <c r="F72" s="6"/>
-      <c r="G72" s="6" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B74" s="4" t="s">
-        <v>277</v>
-      </c>
-      <c r="C74" s="5"/>
-      <c r="D74" s="5"/>
-      <c r="E74" s="5"/>
-      <c r="F74" s="5"/>
-      <c r="G74" s="5"/>
-    </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B75" s="6" t="s">
-        <v>278</v>
-      </c>
-      <c r="C75" s="6" t="s">
-        <v>279</v>
-      </c>
-      <c r="D75" s="13"/>
-      <c r="E75" s="23" t="n">
-        <f aca="false">ROUND(('1 ข้อมูล'!$C$38+'3 ขนาดบ่อ'!$E$8-'1 ข้อมูล'!$C$37)/2/0.05,0)*0.05</f>
-        <v>0.3</v>
-      </c>
-      <c r="F75" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G75" s="6" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="76" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B76" s="6" t="s">
-        <v>281</v>
-      </c>
-      <c r="C76" s="6" t="s">
-        <v>282</v>
-      </c>
-      <c r="D76" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$8-'3 ขนาดบ่อ'!$E$75</f>
-        <v>0.3</v>
-      </c>
-      <c r="E76" s="17" t="str">
-        <f aca="false">IF(D76&gt;='1 ข้อมูล'!$C$37-0.0001,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
-        <v>ผ่าน ✔</v>
-      </c>
-      <c r="F76" s="6"/>
-      <c r="G76" s="6" t="s">
-        <v>283</v>
-      </c>
+      <c r="F74" s="6"/>
+      <c r="G74" s="6" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B76" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="C76" s="5"/>
+      <c r="D76" s="5"/>
+      <c r="E76" s="5"/>
+      <c r="F76" s="5"/>
+      <c r="G76" s="5"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B77" s="6" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>285</v>
-      </c>
-      <c r="D77" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$75</f>
+        <v>287</v>
+      </c>
+      <c r="D77" s="13"/>
+      <c r="E77" s="23" t="n">
+        <f aca="false">ROUND(('1 ข้อมูล'!$C$39+'3 ขนาดบ่อ'!$E$8-'1 ข้อมูล'!$C$38)/2/0.05,0)*0.05</f>
         <v>0.3</v>
       </c>
-      <c r="E77" s="17" t="str">
-        <f aca="false">IF(D77&gt;='1 ข้อมูล'!$C$38-0.0001,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+      <c r="F77" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G77" s="6" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B78" s="6" t="s">
+        <v>289</v>
+      </c>
+      <c r="C78" s="6" t="s">
+        <v>290</v>
+      </c>
+      <c r="D78" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$8-'3 ขนาดบ่อ'!$E$77</f>
+        <v>0.3</v>
+      </c>
+      <c r="E78" s="17" t="str">
+        <f aca="false">IF(D78&gt;='1 ข้อมูล'!$C$38-0.0001,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
-      <c r="F77" s="6"/>
-      <c r="G77" s="6"/>
-    </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B78" s="6" t="s">
-        <v>286</v>
-      </c>
-      <c r="C78" s="6" t="s">
-        <v>287</v>
-      </c>
-      <c r="D78" s="13"/>
-      <c r="E78" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$13-'1 ข้อมูล'!$C$35</f>
-        <v>1.8</v>
-      </c>
-      <c r="F78" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G78" s="6"/>
+      <c r="F78" s="6"/>
+      <c r="G78" s="6" t="s">
+        <v>291</v>
+      </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B79" s="6" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="D79" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$78-'3 ขนาดบ่อ'!$E$14</f>
-        <v>0.85</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$77</f>
+        <v>0.3</v>
       </c>
       <c r="E79" s="17" t="str">
-        <f aca="false">IF(D79&gt;=0.5,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <f aca="false">IF(D79&gt;='1 ข้อมูล'!$C$39-0.0001,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
       <c r="F79" s="6"/>
-      <c r="G79" s="6" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G79" s="6"/>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B80" s="6" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="D80" s="13"/>
       <c r="E80" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$39-'3 ขนาดบ่อ'!$E$30</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$14-'1 ข้อมูล'!$C$36</f>
+        <v>1.8</v>
+      </c>
+      <c r="F80" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G80" s="6"/>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B81" s="6" t="s">
+        <v>296</v>
+      </c>
+      <c r="C81" s="6" t="s">
+        <v>297</v>
+      </c>
+      <c r="D81" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$80-'3 ขนาดบ่อ'!$E$15</f>
+        <v>0.85</v>
+      </c>
+      <c r="E81" s="17" t="str">
+        <f aca="false">IF(D81&gt;=0.5,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F81" s="6"/>
+      <c r="G81" s="6" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B82" s="6" t="s">
+        <v>299</v>
+      </c>
+      <c r="C82" s="6" t="s">
+        <v>300</v>
+      </c>
+      <c r="D82" s="13"/>
+      <c r="E82" s="23" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$40-'3 ขนาดบ่อ'!$E$32</f>
         <v>0.290334311237412</v>
       </c>
-      <c r="F80" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G80" s="6"/>
-    </row>
-    <row r="81" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B81" s="6" t="s">
-        <v>293</v>
-      </c>
-      <c r="C81" s="6" t="s">
-        <v>294</v>
-      </c>
-      <c r="D81" s="13"/>
-      <c r="E81" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$39-'3 ขนาดบ่อ'!$E$8</f>
+      <c r="F82" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G82" s="6"/>
+    </row>
+    <row r="83" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B83" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="C83" s="6" t="s">
+        <v>302</v>
+      </c>
+      <c r="D83" s="13"/>
+      <c r="E83" s="23" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$40-'3 ขนาดบ่อ'!$E$8</f>
         <v>0.5</v>
       </c>
-      <c r="F81" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G81" s="6"/>
-    </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B82" s="6" t="s">
-        <v>295</v>
-      </c>
-      <c r="C82" s="6" t="s">
-        <v>296</v>
-      </c>
-      <c r="D82" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$80</f>
+      <c r="F83" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G83" s="6"/>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B84" s="6" t="s">
+        <v>303</v>
+      </c>
+      <c r="C84" s="6" t="s">
+        <v>304</v>
+      </c>
+      <c r="D84" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$82</f>
         <v>0.290334311237412</v>
       </c>
-      <c r="E82" s="17" t="str">
-        <f aca="false">IF(AND(D82&gt;='1 ข้อมูล'!$C$40,'3 ขนาดบ่อ'!$E$81&lt;='1 ข้อมูล'!$C$41),"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+      <c r="E84" s="17" t="str">
+        <f aca="false">IF(AND(D84&gt;='1 ข้อมูล'!$C$41,'3 ขนาดบ่อ'!$E$83&lt;='1 ข้อมูล'!$C$42),"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
-      <c r="F82" s="6"/>
-      <c r="G82" s="6"/>
-    </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B83" s="6" t="s">
-        <v>297</v>
-      </c>
-      <c r="C83" s="6"/>
-      <c r="D83" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$52-'1 ข้อมูล'!$C$39</f>
+      <c r="F84" s="6"/>
+      <c r="G84" s="6"/>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B85" s="6" t="s">
+        <v>305</v>
+      </c>
+      <c r="C85" s="6"/>
+      <c r="D85" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$54-'1 ข้อมูล'!$C$40</f>
         <v>0.1</v>
       </c>
-      <c r="E83" s="17" t="str">
-        <f aca="false">IF(D83&gt;=0,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+      <c r="E85" s="17" t="str">
+        <f aca="false">IF(D85&gt;=0,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
-      <c r="F83" s="6"/>
-      <c r="G83" s="6" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B85" s="4" t="s">
-        <v>299</v>
-      </c>
-      <c r="C85" s="5"/>
-      <c r="D85" s="5"/>
-      <c r="E85" s="5"/>
-      <c r="F85" s="5"/>
-      <c r="G85" s="5"/>
-    </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B86" s="6" t="s">
-        <v>300</v>
-      </c>
-      <c r="C86" s="6" t="s">
-        <v>301</v>
-      </c>
-      <c r="D86" s="13"/>
-      <c r="E86" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$33+'3 ขนาดบ่อ'!$E$13+'1 ข้อมูล'!$C$42+'3 ขนาดบ่อ'!$E$27</f>
-        <v>3.75</v>
-      </c>
-      <c r="F86" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G86" s="6"/>
+      <c r="F85" s="6"/>
+      <c r="G85" s="6" t="s">
+        <v>306</v>
+      </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B87" s="6" t="s">
-        <v>302</v>
-      </c>
-      <c r="C87" s="6" t="s">
-        <v>303</v>
-      </c>
-      <c r="D87" s="13"/>
-      <c r="E87" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$47+'3 ขนาดบ่อ'!$E$39+'3 ขนาดบ่อ'!$E$86</f>
-        <v>6.35</v>
-      </c>
-      <c r="F87" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G87" s="6"/>
+      <c r="B87" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="C87" s="5"/>
+      <c r="D87" s="5"/>
+      <c r="E87" s="5"/>
+      <c r="F87" s="5"/>
+      <c r="G87" s="5"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B88" s="6" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="C88" s="6" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="D88" s="13"/>
       <c r="E88" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$12</f>
-        <v>1.45</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$35+'3 ขนาดบ่อ'!$E$14+'1 ข้อมูล'!$C$43+'3 ขนาดบ่อ'!$E$29</f>
+        <v>3.75</v>
       </c>
       <c r="F88" s="6" t="s">
         <v>19</v>
@@ -4367,15 +4409,15 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B89" s="6" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="C89" s="6" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="D89" s="13"/>
       <c r="E89" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$52</f>
-        <v>1.2</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$49+'3 ขนาดบ่อ'!$E$41+'3 ขนาดบ่อ'!$E$88</f>
+        <v>6.35</v>
       </c>
       <c r="F89" s="6" t="s">
         <v>19</v>
@@ -4384,15 +4426,15 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B90" s="6" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="C90" s="6" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="D90" s="13"/>
       <c r="E90" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$87+2*'1 ข้อมูล'!$C$42</f>
-        <v>6.75</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$13</f>
+        <v>1.5</v>
       </c>
       <c r="F90" s="6" t="s">
         <v>19</v>
@@ -4401,15 +4443,15 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B91" s="6" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="C91" s="6" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="D91" s="13"/>
       <c r="E91" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$88+2*'1 ข้อมูล'!$C$42</f>
-        <v>1.85</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$54</f>
+        <v>1.2</v>
       </c>
       <c r="F91" s="6" t="s">
         <v>19</v>
@@ -4418,20 +4460,54 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B92" s="6" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="C92" s="6" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="D92" s="13"/>
       <c r="E92" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$89+'1 ข้อมูล'!$C$43</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$89+2*'1 ข้อมูล'!$C$43</f>
+        <v>6.75</v>
+      </c>
+      <c r="F92" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G92" s="6"/>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B93" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="C93" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="D93" s="13"/>
+      <c r="E93" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$90+2*'1 ข้อมูล'!$C$43</f>
+        <v>1.9</v>
+      </c>
+      <c r="F93" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G93" s="6"/>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B94" s="6" t="s">
+        <v>319</v>
+      </c>
+      <c r="C94" s="6" t="s">
+        <v>320</v>
+      </c>
+      <c r="D94" s="13"/>
+      <c r="E94" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$91+'1 ข้อมูล'!$C$44</f>
         <v>1.4</v>
       </c>
-      <c r="F92" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G92" s="6"/>
+      <c r="F94" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G94" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -4465,43 +4541,43 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>313</v>
+        <v>321</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>315</v>
+        <v>323</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>316</v>
+        <v>324</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>317</v>
+        <v>325</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>318</v>
+        <v>326</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>319</v>
+        <v>327</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>321</v>
+        <v>329</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C5" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$7-'1 ข้อมูล'!$C$9</f>
@@ -4512,20 +4588,20 @@
         <v>0.0111111111111111</v>
       </c>
       <c r="E5" s="9" t="n">
-        <f aca="false">(D5/('1 ข้อมูล'!$C$52*'3 ขนาดบ่อ'!$E$12))^(2/3)*100</f>
-        <v>2.5884976609613</v>
+        <f aca="false">(D5/('1 ข้อมูล'!$C$53*'3 ขนาดบ่อ'!$E$13))^(2/3)*100</f>
+        <v>2.53065109461751</v>
       </c>
       <c r="F5" s="19" t="n">
         <f aca="false">'1 ข้อมูล'!$C$17*100+E5</f>
-        <v>4.5884976609613</v>
+        <v>4.53065109461751</v>
       </c>
       <c r="G5" s="12" t="n">
-        <f aca="false">D5/('3 ขนาดบ่อ'!$E$12*F5/100)</f>
-        <v>0.167000962302698</v>
+        <f aca="false">D5/('3 ขนาดบ่อ'!$E$13*F5/100)</f>
+        <v>0.163495428200321</v>
       </c>
       <c r="H5" s="12" t="n">
-        <f aca="false">G5/SQRT('1 ข้อมูล'!$C$47*F5/100)</f>
-        <v>0.248913936242837</v>
+        <f aca="false">G5/SQRT('1 ข้อมูล'!$C$48*F5/100)</f>
+        <v>0.24523971352263</v>
       </c>
       <c r="I5" s="17" t="str">
         <f aca="false">IF(H5&lt;0.5,"เรียบ ✔",IF(H5&lt;0.7,"พอใช้","เป็นระลอก ✘"))</f>
@@ -4534,7 +4610,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C6" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$10-'1 ข้อมูล'!$C$9</f>
@@ -4545,20 +4621,20 @@
         <v>0.0146643518518519</v>
       </c>
       <c r="E6" s="9" t="n">
-        <f aca="false">(D6/('1 ข้อมูล'!$C$52*'3 ขนาดบ่อ'!$E$12))^(2/3)*100</f>
-        <v>3.11447391698078</v>
+        <f aca="false">(D6/('1 ข้อมูล'!$C$53*'3 ขนาดบ่อ'!$E$13))^(2/3)*100</f>
+        <v>3.04487307291521</v>
       </c>
       <c r="F6" s="19" t="n">
         <f aca="false">'1 ข้อมูล'!$C$17*100+E6</f>
-        <v>5.11447391698078</v>
+        <v>5.04487307291521</v>
       </c>
       <c r="G6" s="12" t="n">
-        <f aca="false">D6/('3 ขนาดบ่อ'!$E$12*F6/100)</f>
-        <v>0.197739714169774</v>
+        <f aca="false">D6/('3 ขนาดบ่อ'!$E$13*F6/100)</f>
+        <v>0.193785540817422</v>
       </c>
       <c r="H6" s="12" t="n">
-        <f aca="false">G6/SQRT('1 ข้อมูล'!$C$47*F6/100)</f>
-        <v>0.279163679771048</v>
+        <f aca="false">G6/SQRT('1 ข้อมูล'!$C$48*F6/100)</f>
+        <v>0.275462029969398</v>
       </c>
       <c r="I6" s="17" t="str">
         <f aca="false">IF(H6&lt;0.5,"เรียบ ✔",IF(H6&lt;0.7,"พอใช้","เป็นระลอก ✘"))</f>
@@ -4567,7 +4643,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C7" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8-'1 ข้อมูล'!$C$9</f>
@@ -4578,20 +4654,20 @@
         <v>0.025</v>
       </c>
       <c r="E7" s="9" t="n">
-        <f aca="false">(D7/('1 ข้อมูล'!$C$52*'3 ขนาดบ่อ'!$E$12))^(2/3)*100</f>
-        <v>4.44463520897758</v>
+        <f aca="false">(D7/('1 ข้อมูล'!$C$53*'3 ขนาดบ่อ'!$E$13))^(2/3)*100</f>
+        <v>4.34530852641276</v>
       </c>
       <c r="F7" s="19" t="n">
         <f aca="false">'1 ข้อมูล'!$C$17*100+E7</f>
-        <v>6.44463520897758</v>
+        <v>6.34530852641276</v>
       </c>
       <c r="G7" s="12" t="n">
-        <f aca="false">D7/('3 ขนาดบ่อ'!$E$12*F7/100)</f>
-        <v>0.267530725188713</v>
+        <f aca="false">D7/('3 ขนาดบ่อ'!$E$13*F7/100)</f>
+        <v>0.262661249603397</v>
       </c>
       <c r="H7" s="12" t="n">
-        <f aca="false">G7/SQRT('1 ข้อมูล'!$C$47*F7/100)</f>
-        <v>0.336465076577215</v>
+        <f aca="false">G7/SQRT('1 ข้อมูล'!$C$48*F7/100)</f>
+        <v>0.332916354683497</v>
       </c>
       <c r="I7" s="17" t="str">
         <f aca="false">IF(H7&lt;0.5,"เรียบ ✔",IF(H7&lt;0.7,"พอใช้","เป็นระลอก ✘"))</f>
@@ -4600,7 +4676,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C8" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8</f>
@@ -4611,20 +4687,20 @@
         <v>0.0277777777777778</v>
       </c>
       <c r="E8" s="9" t="n">
-        <f aca="false">(D8/('1 ข้อมูล'!$C$52*'3 ขนาดบ่อ'!$E$12))^(2/3)*100</f>
-        <v>4.7680534585692</v>
+        <f aca="false">(D8/('1 ข้อมูล'!$C$53*'3 ขนาดบ่อ'!$E$13))^(2/3)*100</f>
+        <v>4.66149917231983</v>
       </c>
       <c r="F8" s="19" t="n">
         <f aca="false">'1 ข้อมูล'!$C$17*100+E8</f>
-        <v>6.7680534585692</v>
+        <v>6.66149917231983</v>
       </c>
       <c r="G8" s="12" t="n">
-        <f aca="false">D8/('3 ขนาดบ่อ'!$E$12*F8/100)</f>
-        <v>0.283051666773555</v>
+        <f aca="false">D8/('3 ขนาดบ่อ'!$E$13*F8/100)</f>
+        <v>0.277993257065429</v>
       </c>
       <c r="H8" s="12" t="n">
-        <f aca="false">G8/SQRT('1 ข้อมูล'!$C$47*F8/100)</f>
-        <v>0.347375610243974</v>
+        <f aca="false">G8/SQRT('1 ข้อมูล'!$C$48*F8/100)</f>
+        <v>0.343885424767124</v>
       </c>
       <c r="I8" s="17" t="str">
         <f aca="false">IF(H8&lt;0.5,"เรียบ ✔",IF(H8&lt;0.7,"พอใช้","เป็นระลอก ✘"))</f>
@@ -4633,17 +4709,17 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="22" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="22" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="22" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
     </row>
   </sheetData>
@@ -4673,172 +4749,172 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>325</v>
+        <v>333</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>326</v>
+        <v>334</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>327</v>
+        <v>335</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>19</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>328</v>
+        <v>336</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="6" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="C5" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$52</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$54</f>
         <v>1.2</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>329</v>
+        <v>337</v>
       </c>
       <c r="C6" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$49</f>
-        <v>0.973805782755668</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$51</f>
+        <v>0.972523267791535</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>331</v>
+        <v>339</v>
       </c>
       <c r="C7" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$37+'1 ข้อมูล'!$C$17</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$39+'1 ข้อมูล'!$C$17</f>
         <v>0.92</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>332</v>
+        <v>340</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="C8" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$37</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$39</f>
         <v>0.9</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="6" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="C9" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$58</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$60</f>
         <v>1</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
       <c r="C10" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$9</f>
         <v>0.9</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>336</v>
+        <v>344</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
-        <v>337</v>
+        <v>345</v>
       </c>
       <c r="C11" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$30</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$32</f>
         <v>0.809665688762588</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>338</v>
+        <v>346</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>339</v>
+        <v>347</v>
       </c>
       <c r="C12" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8</f>
         <v>0.6</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="6" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C13" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$55</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$57</f>
         <v>0.5</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="6" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="C14" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$57</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$59</f>
         <v>0.4</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="6" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="C15" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$43</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$45</f>
         <v>0.2</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="C16" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$22</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$24</f>
         <v>0.210686269183871</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>347</v>
+        <v>355</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="s">
-        <v>348</v>
+        <v>356</v>
       </c>
       <c r="C17" s="24" t="n">
         <f aca="false">0</f>
@@ -4874,32 +4950,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>352</v>
+        <v>360</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>353</v>
+        <v>361</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4911,7 +4987,7 @@
         <v>2.77719642805474</v>
       </c>
       <c r="D5" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B5/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B5/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
         <v>2.86619650300861</v>
       </c>
       <c r="E5" s="25" t="n">
@@ -4936,7 +5012,7 @@
         <v>4.38086341517286</v>
       </c>
       <c r="D6" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B6/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B6/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
         <v>4.48983131905459</v>
       </c>
       <c r="E6" s="25" t="n">
@@ -4961,7 +5037,7 @@
         <v>6.44060533155076</v>
       </c>
       <c r="D7" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B7/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B7/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
         <v>6.56792530595593</v>
       </c>
       <c r="E7" s="25" t="n">
@@ -4986,7 +5062,7 @@
         <v>8.99304061167301</v>
       </c>
       <c r="D8" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B8/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B8/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
         <v>9.13647413844802</v>
       </c>
       <c r="E8" s="25" t="n">
@@ -5011,7 +5087,7 @@
         <v>12.07224</v>
       </c>
       <c r="D9" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B9/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B9/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
         <v>12.2289986697729</v>
       </c>
       <c r="E9" s="25" t="n">
@@ -5036,7 +5112,7 @@
         <v>15.7101954157165</v>
       </c>
       <c r="D10" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B10/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B10/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
         <v>15.8769956216084</v>
       </c>
       <c r="E10" s="25" t="n">
@@ -5061,7 +5137,7 @@
         <v>19.9371602697676</v>
       </c>
       <c r="D11" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B11/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B11/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
         <v>20.1102658699656</v>
       </c>
       <c r="E11" s="25" t="n">
@@ -5086,7 +5162,7 @@
         <v>24.7819058265663</v>
       </c>
       <c r="D12" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B12/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B12/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
         <v>24.9571624264048</v>
       </c>
       <c r="E12" s="25" t="n">
@@ -5111,7 +5187,7 @@
         <v>30.2719200646936</v>
       </c>
       <c r="D13" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B13/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B13/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
         <v>30.4447832233961</v>
       </c>
       <c r="E13" s="25" t="n">
@@ -5136,7 +5212,7 @@
         <v>36.4335656390862</v>
       </c>
       <c r="D14" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B14/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B14/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
         <v>36.599124528368</v>
       </c>
       <c r="E14" s="25" t="n">
@@ -5161,7 +5237,7 @@
         <v>43.2922078439065</v>
       </c>
       <c r="D15" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B15/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B15/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
         <v>43.4452054104805</v>
       </c>
       <c r="E15" s="25" t="n">
@@ -5186,7 +5262,7 @@
         <v>50.87232</v>
       </c>
       <c r="D16" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B16/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B16/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
         <v>51.0071703805085</v>
       </c>
       <c r="E16" s="25" t="n">
@@ -5211,7 +5287,7 @@
         <v>59.1975714819181</v>
       </c>
       <c r="D17" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B17/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B17/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
         <v>59.3083752175669</v>
       </c>
       <c r="E17" s="25" t="n">
@@ -5236,7 +5312,7 @@
         <v>68.2909021448919</v>
       </c>
       <c r="D18" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B18/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B18/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
         <v>68.3714596053392</v>
       </c>
       <c r="E18" s="25" t="n">
@@ -5261,7 +5337,7 @@
         <v>78.1745859249513</v>
       </c>
       <c r="D19" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B19/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B19/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
         <v>78.2184092541632</v>
       </c>
       <c r="E19" s="25" t="n">
@@ -5286,7 +5362,7 @@
         <v>88.8702856977516</v>
       </c>
       <c r="D20" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B20/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B20/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
         <v>88.8706095248216</v>
       </c>
       <c r="E20" s="25" t="n">
@@ -5311,7 +5387,7 @@
         <v>100.399100991704</v>
       </c>
       <c r="D21" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B21/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B21/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
         <v>100.348892098404</v>
       </c>
       <c r="E21" s="25" t="n">
@@ -5336,7 +5412,7 @@
         <v>112.781609794846</v>
       </c>
       <c r="D22" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B22/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B22/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
         <v>112.673575893332</v>
       </c>
       <c r="E22" s="25" t="n">
@@ -5361,7 +5437,7 @@
         <v>126.037905431355</v>
       </c>
       <c r="D23" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B23/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B23/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
         <v>125.864503176292</v>
       </c>
       <c r="E23" s="25" t="n">
@@ -5386,7 +5462,7 @@
         <v>140.187629285531</v>
       </c>
       <c r="D24" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B24/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B24/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
         <v>139.941071622383</v>
       </c>
       <c r="E24" s="25" t="n">
@@ -5411,7 +5487,7 @@
         <v>155.25</v>
       </c>
       <c r="D25" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B25/100+'1 ข้อมูล'!$C$51)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B25/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
         <v>154.922262933655</v>
       </c>
       <c r="E25" s="25" t="n">
@@ -5455,12 +5531,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5468,7 +5544,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>3</v>
@@ -5477,12 +5553,12 @@
         <v>4</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="4" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -5491,13 +5567,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="D7" s="12" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$47</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$49</f>
         <v>1.6</v>
       </c>
       <c r="E7" s="6" t="s">
@@ -5507,28 +5583,28 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="D8" s="12" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$39</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$41</f>
         <v>1</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>19</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="6" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="D9" s="27" t="n">
         <f aca="false">'7 แบบพับ'!$D$7+'7 แบบพับ'!$D$8</f>
@@ -5541,31 +5617,31 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
       <c r="D10" s="12" t="n">
-        <f aca="false">MAX('7 แบบพับ'!$D$8,'3 ขนาดบ่อ'!$E$33)</f>
+        <f aca="false">MAX('7 แบบพับ'!$D$8,'3 ขนาดบ่อ'!$E$35)</f>
         <v>1</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>19</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="D11" s="27" t="n">
-        <f aca="false">'7 แบบพับ'!$D$10+'3 ขนาดบ่อ'!$E$13+'1 ข้อมูล'!$C$42+'3 ขนาดบ่อ'!$E$27</f>
+        <f aca="false">'7 แบบพับ'!$D$10+'3 ขนาดบ่อ'!$E$14+'1 ข้อมูล'!$C$43+'3 ขนาดบ่อ'!$E$29</f>
         <v>4.25</v>
       </c>
       <c r="E11" s="6" t="s">
@@ -5575,10 +5651,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>371</v>
+        <v>379</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="D12" s="27" t="n">
         <f aca="false">MAX('7 แบบพับ'!$D$9,'7 แบบพับ'!$D$11)</f>
@@ -5591,10 +5667,10 @@
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="6" t="s">
-        <v>373</v>
+        <v>381</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>374</v>
+        <v>382</v>
       </c>
       <c r="D13" s="12" t="n">
         <f aca="false">'7 แบบพับ'!$D$12-'7 แบบพับ'!$D$9</f>
@@ -5604,19 +5680,19 @@
         <v>19</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>375</v>
+        <v>383</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="6" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>376</v>
+        <v>384</v>
       </c>
       <c r="D14" s="12" t="n">
-        <f aca="false">2*'3 ขนาดบ่อ'!$E$12+'1 ข้อมูล'!$C$42</f>
-        <v>3.1</v>
+        <f aca="false">2*'3 ขนาดบ่อ'!$E$13+'1 ข้อมูล'!$C$43</f>
+        <v>3.2</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>19</v>
@@ -5625,7 +5701,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="4" t="s">
-        <v>377</v>
+        <v>385</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
@@ -5635,150 +5711,150 @@
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="28"/>
       <c r="C17" s="28" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="D17" s="28" t="s">
-        <v>379</v>
+        <v>387</v>
       </c>
       <c r="E17" s="28" t="s">
-        <v>380</v>
+        <v>388</v>
       </c>
       <c r="F17" s="28"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="6" t="s">
-        <v>381</v>
+        <v>389</v>
       </c>
       <c r="C18" s="12" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$90</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$92</f>
         <v>6.75</v>
       </c>
       <c r="D18" s="12" t="n">
-        <f aca="false">'7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$42</f>
+        <f aca="false">'7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$43</f>
         <v>4.65</v>
       </c>
       <c r="E18" s="12" t="n">
-        <f aca="false">'7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$42</f>
+        <f aca="false">'7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$43</f>
         <v>4.65</v>
       </c>
       <c r="F18" s="6"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="6" t="s">
-        <v>382</v>
+        <v>390</v>
       </c>
       <c r="C19" s="12" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$91</f>
-        <v>1.85</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$93</f>
+        <v>1.9</v>
       </c>
       <c r="D19" s="12" t="n">
-        <f aca="false">'7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$42</f>
-        <v>3.5</v>
+        <f aca="false">'7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$43</f>
+        <v>3.6</v>
       </c>
       <c r="E19" s="12" t="n">
-        <f aca="false">'7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$42</f>
-        <v>3.5</v>
+        <f aca="false">'7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$43</f>
+        <v>3.6</v>
       </c>
       <c r="F19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="6" t="s">
-        <v>383</v>
+        <v>391</v>
       </c>
       <c r="C20" s="12" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$90*'3 ขนาดบ่อ'!$E$91</f>
-        <v>12.4875</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$92*'3 ขนาดบ่อ'!$E$93</f>
+        <v>12.825</v>
       </c>
       <c r="D20" s="12" t="n">
-        <f aca="false">('7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$42)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$42)</f>
-        <v>16.275</v>
+        <f aca="false">('7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$43)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$43)</f>
+        <v>16.74</v>
       </c>
       <c r="E20" s="12" t="n">
-        <f aca="false">('7 แบบพับ'!$D$9+2*'1 ข้อมูล'!$C$42)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$42)+('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$9)*('3 ขนาดบ่อ'!$E$12+2*'1 ข้อมูล'!$C$42)</f>
-        <v>13.5525</v>
+        <f aca="false">('7 แบบพับ'!$D$9+2*'1 ข้อมูล'!$C$43)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$43)+('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$9)*('3 ขนาดบ่อ'!$E$13+2*'1 ข้อมูล'!$C$43)</f>
+        <v>13.935</v>
       </c>
       <c r="F20" s="6"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="6" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
       <c r="C21" s="12" t="n">
-        <f aca="false">2*('3 ขนาดบ่อ'!$E$87+'1 ข้อมูล'!$C$42+'3 ขนาดบ่อ'!$E$88+'1 ข้อมูล'!$C$42)*'1 ข้อมูล'!$C$42*'3 ขนาดบ่อ'!$E$52</f>
-        <v>3.936</v>
+        <f aca="false">2*('3 ขนาดบ่อ'!$E$89+'1 ข้อมูล'!$C$43+'3 ขนาดบ่อ'!$E$90+'1 ข้อมูล'!$C$43)*'1 ข้อมูล'!$C$43*'3 ขนาดบ่อ'!$E$54</f>
+        <v>3.96</v>
       </c>
       <c r="D21" s="12" t="n">
-        <f aca="false">2*('7 แบบพับ'!$D$12+'1 ข้อมูล'!$C$42+'7 แบบพับ'!$D$14+'1 ข้อมูล'!$C$42)*'1 ข้อมูล'!$C$42*'3 ขนาดบ่อ'!$E$52</f>
-        <v>3.72</v>
+        <f aca="false">2*('7 แบบพับ'!$D$12+'1 ข้อมูล'!$C$43+'7 แบบพับ'!$D$14+'1 ข้อมูล'!$C$43)*'1 ข้อมูล'!$C$43*'3 ขนาดบ่อ'!$E$54</f>
+        <v>3.768</v>
       </c>
       <c r="E21" s="12" t="n">
-        <f aca="false">2*('7 แบบพับ'!$D$12+'1 ข้อมูล'!$C$42+'7 แบบพับ'!$D$14+'1 ข้อมูล'!$C$42)*'1 ข้อมูล'!$C$42*'3 ขนาดบ่อ'!$E$52</f>
-        <v>3.72</v>
+        <f aca="false">2*('7 แบบพับ'!$D$12+'1 ข้อมูล'!$C$43+'7 แบบพับ'!$D$14+'1 ข้อมูล'!$C$43)*'1 ข้อมูล'!$C$43*'3 ขนาดบ่อ'!$E$54</f>
+        <v>3.768</v>
       </c>
       <c r="F21" s="6"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="6" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
       <c r="C22" s="12" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
       <c r="D22" s="12" t="n">
-        <f aca="false">('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$8)*'1 ข้อมูล'!$C$42*'3 ขนาดบ่อ'!$E$52</f>
+        <f aca="false">('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$8)*'1 ข้อมูล'!$C$43*'3 ขนาดบ่อ'!$E$54</f>
         <v>0.78</v>
       </c>
       <c r="E22" s="12" t="n">
-        <f aca="false">'7 แบบพับ'!$D$7*'1 ข้อมูล'!$C$42*'3 ขนาดบ่อ'!$E$52</f>
+        <f aca="false">'7 แบบพับ'!$D$7*'1 ข้อมูล'!$C$43*'3 ขนาดบ่อ'!$E$54</f>
         <v>0.384</v>
       </c>
       <c r="F22" s="6"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="6" t="s">
-        <v>386</v>
+        <v>394</v>
       </c>
       <c r="C23" s="12" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$90*'3 ขนาดบ่อ'!$E$91*'1 ข้อมูล'!$C$43</f>
-        <v>2.4975</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$92*'3 ขนาดบ่อ'!$E$93*'1 ข้อมูล'!$C$44</f>
+        <v>2.565</v>
       </c>
       <c r="D23" s="12" t="n">
-        <f aca="false">('7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$42)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$42)*'1 ข้อมูล'!$C$43</f>
-        <v>3.255</v>
+        <f aca="false">('7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$43)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$43)*'1 ข้อมูล'!$C$44</f>
+        <v>3.348</v>
       </c>
       <c r="E23" s="12" t="n">
-        <f aca="false">(('7 แบบพับ'!$D$9+2*'1 ข้อมูล'!$C$42)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$42)+('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$9)*('3 ขนาดบ่อ'!$E$12+2*'1 ข้อมูล'!$C$42))*'1 ข้อมูล'!$C$43</f>
-        <v>2.7105</v>
+        <f aca="false">(('7 แบบพับ'!$D$9+2*'1 ข้อมูล'!$C$43)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$43)+('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$9)*('3 ขนาดบ่อ'!$E$13+2*'1 ข้อมูล'!$C$43))*'1 ข้อมูล'!$C$44</f>
+        <v>2.787</v>
       </c>
       <c r="F23" s="6"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="6" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
       <c r="C24" s="27" t="n">
         <f aca="false">SUM(C21:C23)</f>
-        <v>6.4335</v>
+        <v>6.525</v>
       </c>
       <c r="D24" s="27" t="n">
         <f aca="false">SUM(D21:D23)</f>
-        <v>7.755</v>
+        <v>7.896</v>
       </c>
       <c r="E24" s="27" t="n">
         <f aca="false">SUM(E21:E23)</f>
-        <v>6.8145</v>
+        <v>6.939</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>388</v>
+        <v>396</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="6" t="s">
-        <v>389</v>
+        <v>397</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D25" s="29" t="n">
         <f aca="false">1-D18/C18</f>
@@ -5792,7 +5868,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="4" t="s">
-        <v>390</v>
+        <v>398</v>
       </c>
       <c r="C28" s="5"/>
       <c r="D28" s="5"/>
@@ -5801,10 +5877,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="30" t="s">
-        <v>391</v>
+        <v>399</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>392</v>
+        <v>400</v>
       </c>
       <c r="D29" s="6"/>
       <c r="E29" s="6"/>
@@ -5812,10 +5888,10 @@
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="30" t="s">
-        <v>393</v>
+        <v>401</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>394</v>
+        <v>402</v>
       </c>
       <c r="D30" s="6"/>
       <c r="E30" s="6"/>
@@ -5823,10 +5899,10 @@
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="30" t="s">
-        <v>395</v>
+        <v>403</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>396</v>
+        <v>404</v>
       </c>
       <c r="D31" s="6"/>
       <c r="E31" s="6"/>
@@ -5834,10 +5910,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="30" t="s">
-        <v>397</v>
+        <v>405</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>398</v>
+        <v>406</v>
       </c>
       <c r="D32" s="6"/>
       <c r="E32" s="6"/>
@@ -5845,10 +5921,10 @@
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="31" t="s">
-        <v>399</v>
+        <v>407</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>400</v>
+        <v>408</v>
       </c>
       <c r="D33" s="6"/>
       <c r="E33" s="6"/>
@@ -5856,10 +5932,10 @@
     </row>
     <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="31" t="s">
-        <v>401</v>
+        <v>409</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>402</v>
+        <v>410</v>
       </c>
       <c r="D34" s="6"/>
       <c r="E34" s="6"/>
@@ -5867,10 +5943,10 @@
     </row>
     <row r="35" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="31" t="s">
-        <v>403</v>
+        <v>411</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="D35" s="6"/>
       <c r="E35" s="6"/>
@@ -5878,10 +5954,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="31" t="s">
-        <v>405</v>
+        <v>413</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>406</v>
+        <v>414</v>
       </c>
       <c r="D36" s="6"/>
       <c r="E36" s="6"/>
@@ -5919,150 +5995,150 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>407</v>
+        <v>415</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>408</v>
+        <v>416</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>410</v>
+        <v>418</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>411</v>
+        <v>419</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>413</v>
+        <v>421</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>414</v>
+        <v>422</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>415</v>
+        <v>423</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>416</v>
+        <v>424</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="32" t="s">
-        <v>417</v>
+        <v>425</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>418</v>
+        <v>426</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>420</v>
+        <v>428</v>
       </c>
       <c r="F5" s="23" t="n">
         <f aca="false">'1 ข้อมูล'!$C$10/3600</f>
         <v>0.0174421296296296</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>421</v>
+        <v>429</v>
       </c>
       <c r="H5" s="12"/>
       <c r="I5" s="17"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="32" t="s">
-        <v>422</v>
+        <v>430</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>423</v>
+        <v>431</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>424</v>
+        <v>432</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>420</v>
+        <v>428</v>
       </c>
       <c r="F6" s="23" t="n">
         <f aca="false">1.5*F5</f>
         <v>0.0261631944444444</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>425</v>
+        <v>433</v>
       </c>
       <c r="H6" s="12"/>
       <c r="I6" s="17"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="32" t="s">
-        <v>426</v>
+        <v>434</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>427</v>
+        <v>435</v>
       </c>
       <c r="D7" s="6" t="s">
+        <v>436</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>428</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>420</v>
       </c>
       <c r="F7" s="23" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8/3600</f>
         <v>0.0277777777777778</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>429</v>
+        <v>437</v>
       </c>
       <c r="H7" s="12"/>
       <c r="I7" s="17"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="32" t="s">
-        <v>430</v>
+        <v>438</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>431</v>
+        <v>439</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>432</v>
+        <v>440</v>
       </c>
       <c r="E8" s="6"/>
       <c r="F8" s="23" t="n">
         <v>1</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>433</v>
+        <v>441</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>417</v>
+        <v>425</v>
       </c>
       <c r="I8" s="17"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="32" t="s">
-        <v>434</v>
+        <v>442</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>435</v>
+        <v>443</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>436</v>
+        <v>444</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>420</v>
+        <v>428</v>
       </c>
       <c r="F9" s="23" t="n">
         <f aca="false">MAX(F6,F7)/F8</f>
         <v>0.0277777777777778</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>437</v>
+        <v>445</v>
       </c>
       <c r="H9" s="12" t="n">
         <f aca="false">'2 เวียร์'!$D$13</f>
@@ -6072,10 +6148,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="32" t="s">
-        <v>438</v>
+        <v>446</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>439</v>
+        <v>447</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="6" t="s">
@@ -6086,11 +6162,11 @@
         <v>0.458178826795053</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>440</v>
+        <v>448</v>
       </c>
       <c r="H10" s="12" t="n">
-        <f aca="false">('3 ขนาดบ่อ'!$E$12-'3 ขนาดบ่อ'!$E$10)/2</f>
-        <v>0.425</v>
+        <f aca="false">('3 ขนาดบ่อ'!$E$13-'3 ขนาดบ่อ'!$E$10)/2</f>
+        <v>0.45</v>
       </c>
       <c r="I10" s="17" t="str">
         <f aca="false">IF(H10&gt;=2*F12,"ผ่าน ✔","ไม่ผ่าน ✘ (ต้อง ≥ 2Hmax)")</f>
@@ -6099,10 +6175,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="32" t="s">
-        <v>441</v>
+        <v>449</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="D11" s="6"/>
       <c r="E11" s="6" t="s">
@@ -6113,7 +6189,7 @@
         <v>0.416526206177321</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>442</v>
+        <v>450</v>
       </c>
       <c r="H11" s="12" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8</f>
@@ -6126,10 +6202,10 @@
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="32" t="s">
-        <v>443</v>
+        <v>451</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>444</v>
+        <v>452</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6" t="s">
@@ -6140,22 +6216,22 @@
         <v>0.208263103088661</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>445</v>
+        <v>453</v>
       </c>
       <c r="H12" s="12" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$7</f>
         <v>0.209665688762588</v>
       </c>
       <c r="I12" s="17" t="s">
-        <v>446</v>
+        <v>454</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="32" t="s">
-        <v>447</v>
+        <v>455</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>448</v>
+        <v>456</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="6"/>
@@ -6172,10 +6248,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="32" t="s">
-        <v>449</v>
+        <v>457</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>450</v>
+        <v>458</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
@@ -6192,10 +6268,10 @@
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="32" t="s">
-        <v>451</v>
+        <v>459</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>452</v>
+        <v>460</v>
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="6" t="s">
@@ -6206,10 +6282,10 @@
         <v>0.624789309265982</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>453</v>
+        <v>461</v>
       </c>
       <c r="H15" s="12" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$14</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$15</f>
         <v>0.95</v>
       </c>
       <c r="I15" s="17" t="str">
@@ -6219,10 +6295,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="32" t="s">
-        <v>454</v>
+        <v>462</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>455</v>
+        <v>463</v>
       </c>
       <c r="D16" s="6"/>
       <c r="E16" s="6" t="s">
@@ -6233,7 +6309,7 @@
         <v>0.249915723706393</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>456</v>
+        <v>464</v>
       </c>
       <c r="H16" s="12" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$9</f>
@@ -6246,10 +6322,10 @@
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="32" t="s">
-        <v>457</v>
+        <v>465</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>305</v>
+        <v>313</v>
       </c>
       <c r="D17" s="6"/>
       <c r="E17" s="6" t="s">
@@ -6260,11 +6336,11 @@
         <v>1.41618910100289</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>458</v>
+        <v>466</v>
       </c>
       <c r="H17" s="12" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$12</f>
-        <v>1.45</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$13</f>
+        <v>1.5</v>
       </c>
       <c r="I17" s="17" t="str">
         <f aca="false">IF(H17&gt;=F17,"ผ่าน ✔","แคบกว่า ✘")</f>
@@ -6273,7 +6349,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="4" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5"/>
@@ -6285,17 +6361,17 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="22" t="s">
-        <v>459</v>
+        <v>467</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="22" t="s">
-        <v>460</v>
+        <v>468</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="22" t="s">
-        <v>461</v>
+        <v>469</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add SS under-flow baffle and sill inside compartment 3 plunge zone
Baffle 0.30 m from the compartment-2 sill (0.20 m gap), sill 0.30 m high
0.20 m further = start of 2.10 m approach. Fits in the existing 0.50 m
zone, tank length unchanged (6.75 m). Workbook, drawings, animation.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXLmoKkgGBxM2QbbegGKn7
</commit_message>
<xml_diff>
--- a/weir_design.xlsx
+++ b/weir_design.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="612" uniqueCount="470">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="489">
   <si>
     <t xml:space="preserve">1) ข้อมูลออกแบบ — บ่อ 3 ช่อง: ปั๊มจุ่ม | โชว์น้ำใส | V-notch 90°</t>
   </si>
@@ -171,6 +171,12 @@
   </si>
   <si>
     <t xml:space="preserve">ไม่ให้เกิดกระแสวน / ยกปั๊มขึ้นซ่อมได้</t>
+  </si>
+  <si>
+    <t xml:space="preserve">สันล้นช่อง 3 สูงกว่าช่องลอดใต้</t>
+  </si>
+  <si>
+    <t xml:space="preserve">บังคับให้น้ำที่ลอดใต้ต้องยกตัวขึ้น</t>
   </si>
   <si>
     <t xml:space="preserve">ความเร็วลอยตัวฟองอากาศ</t>
@@ -635,7 +641,7 @@
     <t xml:space="preserve">ม่านน้ำพุ่งไกล + เผื่อ 0.20</t>
   </si>
   <si>
-    <t xml:space="preserve">ค. โซนรับน้ำตก ช่อง 3 (ให้ฟองลอยขึ้นและคลื่นสลายก่อนเข้าช่วงตรง)</t>
+    <t xml:space="preserve">ค. โซนรับน้ำตก + ผนังลอดใต้ + สันล้น ช่อง 3 (แผ่น SS 6 mm อยู่ในโซนรับน้ำตก ไม่ยืดบ่อ)</t>
   </si>
   <si>
     <t xml:space="preserve">ความลึกน้ำช่อง 3 สูงสุด</t>
@@ -665,6 +671,60 @@
     <t xml:space="preserve">ฟองลอยขึ้นผิวน้ำก่อนเข้าช่วงตรง</t>
   </si>
   <si>
+    <t xml:space="preserve">① ช่องลอดใต้ผนัง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q ÷ (B × v ไม่เกิน 0.10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ขอบล่างผนังลอดใต้ / ขอบบนเสมอสันกำแพง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ระยะ ① ถึง ② (สันล้น)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">เท่าช่องลอด</t>
+  </si>
+  <si>
+    <t xml:space="preserve">② ความสูงสันล้น</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ช่องลอด + 0.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">สันล้น = ต้นช่วงตรง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ระยะรับน้ำตก ก่อนถึง ①</t>
+  </si>
+  <si>
+    <t xml:space="preserve">โซนรับน้ำตก − ระยะ ①–②</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ตำแหน่ง ① วัดจากสันปลายช่อง 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ตรวจ: ระยะรับน้ำตก ≥ ระยะฟองลอย</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ฟองลอยขึ้นก่อนถึงผนังลอดใต้</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ความเร็วข้ามสันล้น (สูงสุด)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q ÷ (B × (น้ำช่อง 3 − สันล้น))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ตรวจ: ความเร็วข้ามสันล้น ≤ 0.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ตรวจ: น้ำเหนือสันล้น ที่น้ำเข้าต่ำสุด</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≥ 0.10 m</t>
+  </si>
+  <si>
     <t xml:space="preserve">ง. ช่อง 2 โชว์น้ำใส</t>
   </si>
   <si>
@@ -705,9 +765,6 @@
   </si>
   <si>
     <t xml:space="preserve">ช่องลอดใต้ผนังกั้น</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Q ÷ (B × v ไม่เกิน 0.10)</t>
   </si>
   <si>
     <t xml:space="preserve">โซนน้ำเข้า</t>
@@ -2051,7 +2108,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:E62"/>
+  <dimension ref="B1:E63"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -2376,7 +2433,7 @@
         <v>0.1</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="E27" s="6" t="s">
         <v>49</v>
@@ -2387,10 +2444,10 @@
         <v>50</v>
       </c>
       <c r="C28" s="10" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>51</v>
@@ -2401,7 +2458,7 @@
         <v>52</v>
       </c>
       <c r="C29" s="10" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>19</v>
@@ -2420,21 +2477,21 @@
       <c r="D30" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E30" s="6"/>
+      <c r="E30" s="6" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C31" s="10" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="D31" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E31" s="6" t="s">
-        <v>56</v>
-      </c>
+      <c r="E31" s="6"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="6" t="s">
@@ -2446,11 +2503,13 @@
       <c r="D32" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E32" s="6"/>
+      <c r="E32" s="6" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C33" s="10" t="n">
         <v>0.1</v>
@@ -2458,9 +2517,7 @@
       <c r="D33" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E33" s="6" t="s">
-        <v>59</v>
-      </c>
+      <c r="E33" s="6"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="6" t="s">
@@ -2480,34 +2537,34 @@
       <c r="B35" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="C35" s="11" t="n">
-        <v>0.006</v>
+      <c r="C35" s="10" t="n">
+        <v>0.1</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E35" s="6"/>
+      <c r="E35" s="6" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="C36" s="10" t="n">
-        <v>0.3</v>
+        <v>64</v>
+      </c>
+      <c r="C36" s="11" t="n">
+        <v>0.006</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E36" s="6" t="s">
-        <v>64</v>
-      </c>
+      <c r="E36" s="6"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="6" t="s">
         <v>65</v>
       </c>
       <c r="C37" s="10" t="n">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="D37" s="6" t="s">
         <v>19</v>
@@ -2521,7 +2578,7 @@
         <v>67</v>
       </c>
       <c r="C38" s="10" t="n">
-        <v>0.25</v>
+        <v>0.15</v>
       </c>
       <c r="D38" s="6" t="s">
         <v>19</v>
@@ -2535,7 +2592,7 @@
         <v>69</v>
       </c>
       <c r="C39" s="10" t="n">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="D39" s="6" t="s">
         <v>19</v>
@@ -2549,7 +2606,7 @@
         <v>71</v>
       </c>
       <c r="C40" s="10" t="n">
-        <v>1.1</v>
+        <v>0.2</v>
       </c>
       <c r="D40" s="6" t="s">
         <v>19</v>
@@ -2563,7 +2620,7 @@
         <v>73</v>
       </c>
       <c r="C41" s="10" t="n">
-        <v>0.05</v>
+        <v>1.1</v>
       </c>
       <c r="D41" s="6" t="s">
         <v>19</v>
@@ -2577,26 +2634,26 @@
         <v>75</v>
       </c>
       <c r="C42" s="10" t="n">
-        <v>1.25</v>
+        <v>0.05</v>
       </c>
       <c r="D42" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E42" s="6"/>
+      <c r="E42" s="6" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C43" s="10" t="n">
-        <v>0.2</v>
+        <v>1.25</v>
       </c>
       <c r="D43" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E43" s="6" t="s">
-        <v>77</v>
-      </c>
+      <c r="E43" s="6"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="6" t="s">
@@ -2608,41 +2665,43 @@
       <c r="D44" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E44" s="6"/>
+      <c r="E44" s="6" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C45" s="10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E45" s="6"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B46" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="C46" s="10" t="n">
         <v>0.05</v>
       </c>
-      <c r="D45" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E45" s="6" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="C47" s="5"/>
-      <c r="D47" s="5"/>
-      <c r="E47" s="5"/>
+      <c r="D46" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E46" s="6" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B48" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="C48" s="12" t="n">
-        <v>9.81</v>
-      </c>
-      <c r="D48" s="6" t="s">
+      <c r="B48" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="E48" s="6"/>
+      <c r="C48" s="5"/>
+      <c r="D48" s="5"/>
+      <c r="E48" s="5"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="6" t="s">
@@ -2660,25 +2719,23 @@
       <c r="B50" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="C50" s="13" t="n">
-        <v>1.38</v>
+      <c r="C50" s="12" t="n">
+        <v>9.81</v>
       </c>
       <c r="D50" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="E50" s="6" t="s">
-        <v>88</v>
-      </c>
+      <c r="E50" s="6"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C51" s="13" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="D51" s="6" t="s">
         <v>89</v>
-      </c>
-      <c r="C51" s="13" t="n">
-        <v>0.578</v>
-      </c>
-      <c r="D51" s="6" t="s">
-        <v>87</v>
       </c>
       <c r="E51" s="6" t="s">
         <v>90</v>
@@ -2688,28 +2745,28 @@
       <c r="B52" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="C52" s="14" t="n">
-        <v>0.00085</v>
+      <c r="C52" s="13" t="n">
+        <v>0.578</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>19</v>
+        <v>89</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C53" s="14" t="n">
+        <v>0.00085</v>
+      </c>
+      <c r="D53" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E53" s="6" t="s">
         <v>92</v>
-      </c>
-      <c r="C53" s="12" t="n">
-        <v>1.84</v>
-      </c>
-      <c r="D53" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="E53" s="6" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2717,10 +2774,10 @@
         <v>94</v>
       </c>
       <c r="C54" s="12" t="n">
-        <v>0.6</v>
+        <v>1.84</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>95</v>
@@ -2730,80 +2787,94 @@
       <c r="B55" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="C55" s="15" t="n">
-        <v>205</v>
+      <c r="C55" s="12" t="n">
+        <v>0.6</v>
       </c>
       <c r="D55" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="E55" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="E55" s="6"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="6" t="s">
         <v>98</v>
       </c>
       <c r="C56" s="15" t="n">
-        <v>400</v>
+        <v>205</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E56" s="6"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C57" s="15" t="n">
+        <v>400</v>
+      </c>
+      <c r="D57" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="C57" s="9" t="n">
+      <c r="E57" s="6"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B58" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C58" s="9" t="n">
         <v>1.7</v>
       </c>
-      <c r="D57" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="E57" s="6"/>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B59" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="C59" s="5"/>
-      <c r="D59" s="5"/>
-      <c r="E59" s="5"/>
+      <c r="D58" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="E58" s="6"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B60" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="C60" s="16" t="s">
+      <c r="B60" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="D60" s="6"/>
-      <c r="E60" s="6" t="s">
-        <v>103</v>
-      </c>
+      <c r="C60" s="5"/>
+      <c r="D60" s="5"/>
+      <c r="E60" s="5"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C61" s="16" t="s">
         <v>104</v>
-      </c>
-      <c r="C61" s="17" t="s">
-        <v>105</v>
       </c>
       <c r="D61" s="6"/>
       <c r="E61" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C62" s="17" t="s">
         <v>107</v>
-      </c>
-      <c r="C62" s="6" t="s">
-        <v>108</v>
       </c>
       <c r="D62" s="6"/>
       <c r="E62" s="6" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B63" s="6" t="s">
         <v>109</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="D63" s="6"/>
+      <c r="E63" s="6" t="s">
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -2837,17 +2908,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="4" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="5"/>
@@ -2858,17 +2929,17 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C5" s="13" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$50</f>
+        <f aca="false">'1 ข้อมูล'!$C$51</f>
         <v>1.38</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
@@ -2876,17 +2947,17 @@
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C6" s="18" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$51*(8/15)*SQRT(2*'1 ข้อมูล'!$C$48)</f>
+        <f aca="false">'1 ข้อมูล'!$C$52*(8/15)*SQRT(2*'1 ข้อมูล'!$C$49)</f>
         <v>1.36545083661038</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
@@ -2894,7 +2965,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="4" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
@@ -2905,30 +2976,30 @@
     </row>
     <row r="9" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C10" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$7-'1 ข้อมูล'!$C$9</f>
@@ -2943,7 +3014,7 @@
         <v>14.532869095236</v>
       </c>
       <c r="F10" s="9" t="n">
-        <f aca="false">((D10/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$52)*100</f>
+        <f aca="false">((D10/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$53)*100</f>
         <v>14.5096125168743</v>
       </c>
       <c r="G10" s="20" t="n">
@@ -2954,7 +3025,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C11" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$10-'1 ข้อมูล'!$C$9</f>
@@ -2969,7 +3040,7 @@
         <v>16.2387843483091</v>
       </c>
       <c r="F11" s="9" t="n">
-        <f aca="false">((D11/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$52)*100</f>
+        <f aca="false">((D11/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$53)*100</f>
         <v>16.2227754127948</v>
       </c>
       <c r="G11" s="20" t="n">
@@ -2977,12 +3048,12 @@
         <v>0.0160089355143072</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C12" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8-'1 ข้อมูล'!$C$9</f>
@@ -2997,7 +3068,7 @@
         <v>20.1013103538681</v>
       </c>
       <c r="F12" s="9" t="n">
-        <f aca="false">((D12/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$52)*100</f>
+        <f aca="false">((D12/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$53)*100</f>
         <v>20.1017115002301</v>
       </c>
       <c r="G12" s="20" t="n">
@@ -3008,7 +3079,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="21" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C13" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8</f>
@@ -3023,7 +3094,7 @@
         <v>20.9665688762588</v>
       </c>
       <c r="F13" s="9" t="n">
-        <f aca="false">((D13/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$52)*100</f>
+        <f aca="false">((D13/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$53)*100</f>
         <v>20.9706461048468</v>
       </c>
       <c r="G13" s="20" t="n">
@@ -3031,22 +3102,22 @@
         <v>-0.00407722858800952</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="22" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="22" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="22" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>
@@ -3065,7 +3136,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:G94"/>
+  <dimension ref="B1:G102"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -3078,12 +3149,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3091,24 +3162,24 @@
         <v>2</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>4</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -3118,10 +3189,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D7" s="13"/>
       <c r="E7" s="23" t="n">
@@ -3132,15 +3203,15 @@
         <v>19</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D8" s="13" t="n">
         <f aca="false">MAX(0.45,'3 ขนาดบ่อ'!$E$7/0.4)+'1 ข้อมูล'!$C$14</f>
@@ -3154,15 +3225,15 @@
         <v>19</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="6" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D9" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$7+'1 ข้อมูล'!$C$15</f>
@@ -3176,15 +3247,15 @@
         <v>19</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D10" s="13"/>
       <c r="E10" s="23" t="n">
@@ -3195,15 +3266,15 @@
         <v>19</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D11" s="13"/>
       <c r="E11" s="23" t="n">
@@ -3214,15 +3285,15 @@
         <v>19</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D12" s="13"/>
       <c r="E12" s="23" t="n">
@@ -3233,15 +3304,15 @@
         <v>19</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="6" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D13" s="13" t="n">
         <f aca="false">MAX('3 ขนาดบ่อ'!$E$12,'1 ข้อมูล'!$C$19)</f>
@@ -3255,15 +3326,15 @@
         <v>19</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="6" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D14" s="13" t="n">
         <f aca="false">10*'3 ขนาดบ่อ'!$E$7</f>
@@ -3277,15 +3348,15 @@
         <v>19</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="6" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D15" s="13" t="n">
         <f aca="false">4.5*'3 ขนาดบ่อ'!$E$7</f>
@@ -3299,15 +3370,15 @@
         <v>19</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D16" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$7/'3 ขนาดบ่อ'!$E$8</f>
@@ -3322,10 +3393,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D17" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$7/'3 ขนาดบ่อ'!$E$13</f>
@@ -3340,10 +3411,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="6" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D18" s="13" t="n">
         <f aca="false">('3 ขนาดบ่อ'!$E$13-'3 ขนาดบ่อ'!$E$10)/2</f>
@@ -3355,34 +3426,34 @@
       </c>
       <c r="F18" s="6"/>
       <c r="G18" s="6" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="6" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D19" s="9"/>
       <c r="E19" s="19" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$50*(('3 ขนาดบ่อ'!$E$13-'3 ขนาดบ่อ'!$E$10)/4)^2.5*3600</f>
+        <f aca="false">'1 ข้อมูล'!$C$51*(('3 ขนาดบ่อ'!$E$13-'3 ขนาดบ่อ'!$E$10)/4)^2.5*3600</f>
         <v>119.299296438097</v>
       </c>
       <c r="F19" s="6" t="s">
         <v>11</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="6" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D20" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$15/'3 ขนาดบ่อ'!$E$7</f>
@@ -3397,10 +3468,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="6" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="D21" s="13" t="n">
         <f aca="false">'2 เวียร์'!$E$10/100</f>
@@ -3412,12 +3483,12 @@
       </c>
       <c r="F21" s="6"/>
       <c r="G21" s="6" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="4" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="5"/>
@@ -3427,14 +3498,14 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="6" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="D24" s="13"/>
       <c r="E24" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$30/2+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$54*PI()*'1 ข้อมูล'!$C$30^2/4))^2/(2*'1 ข้อมูล'!$C$48)</f>
+        <f aca="false">'1 ข้อมูล'!$C$31/2+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$55*PI()*'1 ข้อมูล'!$C$31^2/4))^2/(2*'1 ข้อมูล'!$C$49)</f>
         <v>0.210686269183871</v>
       </c>
       <c r="F24" s="6" t="s">
@@ -3444,10 +3515,10 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="6" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D25" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8-'3 ขนาดบ่อ'!$E$24</f>
@@ -3459,34 +3530,34 @@
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="6" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D26" s="13"/>
       <c r="E26" s="23" t="n">
-        <f aca="false">SQRT(2*'1 ข้อมูล'!$C$48*'3 ขนาดบ่อ'!$E$7)</f>
+        <f aca="false">SQRT(2*'1 ข้อมูล'!$C$49*'3 ขนาดบ่อ'!$E$7)</f>
         <v>2.02821123493634</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>36</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="6" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D27" s="13"/>
       <c r="E27" s="23" t="n">
@@ -3500,32 +3571,32 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="6" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="D28" s="13"/>
       <c r="E28" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$26*SQRT(2*'3 ขนาดบ่อ'!$E$27/'1 ข้อมูล'!$C$48)</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$26*SQRT(2*'3 ขนาดบ่อ'!$E$27/'1 ข้อมูล'!$C$49)</f>
         <v>0.708760700266562</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="6" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D29" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$28+'1 ข้อมูล'!$C$29</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$28+'1 ข้อมูล'!$C$30</f>
         <v>0.908760700266562</v>
       </c>
       <c r="E29" s="23" t="n">
@@ -3539,7 +3610,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="4" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C31" s="5"/>
       <c r="D31" s="5"/>
@@ -3549,10 +3620,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="6" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D32" s="13"/>
       <c r="E32" s="23" t="n">
@@ -3566,10 +3637,10 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D33" s="13"/>
       <c r="E33" s="23" t="n">
@@ -3583,14 +3654,14 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="6" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D34" s="13"/>
       <c r="E34" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$32/'1 ข้อมูล'!$C$27*'3 ขนาดบ่อ'!$E$33</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$32/'1 ข้อมูล'!$C$28*'3 ขนาดบ่อ'!$E$33</f>
         <v>0.185185185185185</v>
       </c>
       <c r="F34" s="6" t="s">
@@ -3600,13 +3671,13 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="6" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D35" s="13" t="n">
-        <f aca="false">MAX('1 ข้อมูล'!$C$28,'3 ขนาดบ่อ'!$E$34)</f>
+        <f aca="false">MAX('1 ข้อมูล'!$C$29,'3 ขนาดบ่อ'!$E$34)</f>
         <v>0.5</v>
       </c>
       <c r="E35" s="23" t="n">
@@ -3617,790 +3688,822 @@
         <v>19</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>208</v>
+        <v>210</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B36" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="D36" s="13" t="n">
+        <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$13*'1 ข้อมูล'!$C$21)</f>
+        <v>0.185185185185185</v>
+      </c>
+      <c r="E36" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D36,4),'1 ข้อมูล'!$C$13)</f>
+        <v>0.2</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G36" s="6" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="C37" s="5"/>
-      <c r="D37" s="5"/>
-      <c r="E37" s="5"/>
-      <c r="F37" s="5"/>
-      <c r="G37" s="5"/>
+      <c r="B37" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="D37" s="13"/>
+      <c r="E37" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$36</f>
+        <v>0.2</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G37" s="6"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="6" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="D38" s="13"/>
+        <v>217</v>
+      </c>
+      <c r="D38" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$36+'1 ข้อมูล'!$C$27</f>
+        <v>0.3</v>
+      </c>
       <c r="E38" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$17+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$53*'3 ขนาดบ่อ'!$E$13))^(2/3)</f>
-        <v>0.0666149917231983</v>
+        <f aca="false">CEILING(ROUND(D38,4),'1 ข้อมูล'!$C$13)</f>
+        <v>0.3</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="6" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="D39" s="13" t="n">
+        <v>220</v>
+      </c>
+      <c r="D39" s="13"/>
+      <c r="E39" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$35-'3 ขนาดบ่อ'!$E$37</f>
+        <v>0.3</v>
+      </c>
+      <c r="F39" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G39" s="6" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B40" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="C40" s="6"/>
+      <c r="D40" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$39-'3 ขนาดบ่อ'!$E$34</f>
+        <v>0.114814814814815</v>
+      </c>
+      <c r="E40" s="17" t="str">
+        <f aca="false">IF(D40&gt;=0,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F40" s="6"/>
+      <c r="G40" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B41" s="6" t="s">
+        <v>224</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="D41" s="13"/>
+      <c r="E41" s="23" t="n">
+        <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$13*('3 ขนาดบ่อ'!$E$32-'3 ขนาดบ่อ'!$E$38))</f>
+        <v>0.0363346384244139</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="G41" s="6"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B42" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="C42" s="6"/>
+      <c r="D42" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$41</f>
+        <v>0.0363346384244139</v>
+      </c>
+      <c r="E42" s="17" t="str">
+        <f aca="false">IF(D42&lt;=0.1,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F42" s="6"/>
+      <c r="G42" s="6"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B43" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="D43" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$8+'2 เวียร์'!$E$10/100-'3 ขนาดบ่อ'!$E$38</f>
+        <v>0.44532869095236</v>
+      </c>
+      <c r="E43" s="17" t="str">
+        <f aca="false">IF(D43&gt;=0.1,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F43" s="6"/>
+      <c r="G43" s="6"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B45" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="C45" s="5"/>
+      <c r="D45" s="5"/>
+      <c r="E45" s="5"/>
+      <c r="F45" s="5"/>
+      <c r="G45" s="5"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B46" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="D46" s="13"/>
+      <c r="E46" s="23" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$17+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$54*'3 ขนาดบ่อ'!$E$13))^(2/3)</f>
+        <v>0.0666149917231983</v>
+      </c>
+      <c r="F46" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G46" s="6" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B47" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="D47" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$32+'1 ข้อมูล'!$C$16-'1 ข้อมูล'!$C$17</f>
         <v>0.889665688762588</v>
       </c>
-      <c r="E39" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D39,4),'1 ข้อมูล'!$C$13)</f>
+      <c r="E47" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D47,4),'1 ข้อมูล'!$C$13)</f>
         <v>0.9</v>
       </c>
-      <c r="F39" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G39" s="6" t="s">
+      <c r="F47" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G47" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="6" t="s">
-        <v>215</v>
-      </c>
-      <c r="C40" s="6" t="s">
-        <v>216</v>
-      </c>
-      <c r="D40" s="13" t="n">
-        <f aca="false">10*'3 ขนาดบ่อ'!$E$38</f>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B48" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="D48" s="13" t="n">
+        <f aca="false">10*'3 ขนาดบ่อ'!$E$46</f>
         <v>0.666149917231983</v>
       </c>
-      <c r="E40" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D40,4),'1 ข้อมูล'!$C$13)</f>
+      <c r="E48" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D48,4),'1 ข้อมูล'!$C$13)</f>
         <v>0.7</v>
       </c>
-      <c r="F40" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G40" s="6" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="6" t="s">
-        <v>218</v>
-      </c>
-      <c r="C41" s="6" t="s">
-        <v>219</v>
-      </c>
-      <c r="D41" s="13"/>
-      <c r="E41" s="23" t="n">
+      <c r="F48" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G48" s="6" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B49" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="D49" s="13"/>
+      <c r="E49" s="23" t="n">
         <f aca="false">'1 ข้อมูล'!$C$18</f>
         <v>1</v>
       </c>
-      <c r="F41" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G41" s="6"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="6" t="s">
-        <v>220</v>
-      </c>
-      <c r="C42" s="6"/>
-      <c r="D42" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$41-'3 ขนาดบ่อ'!$E$40</f>
+      <c r="F49" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G49" s="6"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B50" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="C50" s="6"/>
+      <c r="D50" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$49-'3 ขนาดบ่อ'!$E$48</f>
         <v>0.3</v>
       </c>
-      <c r="E42" s="17" t="str">
-        <f aca="false">IF(D42&gt;=0,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+      <c r="E50" s="17" t="str">
+        <f aca="false">IF(D50&gt;=0,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
-      <c r="F42" s="6"/>
-      <c r="G42" s="6"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="C44" s="5"/>
-      <c r="D44" s="5"/>
-      <c r="E44" s="5"/>
-      <c r="F44" s="5"/>
-      <c r="G44" s="5"/>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="6" t="s">
-        <v>222</v>
-      </c>
-      <c r="C45" s="6" t="s">
-        <v>223</v>
-      </c>
-      <c r="D45" s="13" t="n">
+      <c r="F50" s="6"/>
+      <c r="G50" s="6"/>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B52" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="C52" s="5"/>
+      <c r="D52" s="5"/>
+      <c r="E52" s="5"/>
+      <c r="F52" s="5"/>
+      <c r="G52" s="5"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B53" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="D53" s="13" t="n">
         <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$13*'1 ข้อมูล'!$C$21)</f>
         <v>0.185185185185185</v>
       </c>
-      <c r="E45" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D45,4),'1 ข้อมูล'!$C$13)</f>
+      <c r="E53" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D53,4),'1 ข้อมูล'!$C$13)</f>
         <v>0.2</v>
       </c>
-      <c r="F45" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G45" s="6"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="6" t="s">
-        <v>224</v>
-      </c>
-      <c r="C46" s="6" t="s">
-        <v>225</v>
-      </c>
-      <c r="D46" s="13" t="n">
+      <c r="F53" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G53" s="6"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B54" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="D54" s="13" t="n">
         <f aca="false">'1 ข้อมูล'!$C$22+2*'1 ข้อมูล'!$C$23</f>
         <v>0.468</v>
       </c>
-      <c r="E46" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D46,4),'1 ข้อมูล'!$C$13)</f>
+      <c r="E54" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D54,4),'1 ข้อมูล'!$C$13)</f>
         <v>0.5</v>
       </c>
-      <c r="F46" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G46" s="6"/>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="C47" s="6" t="s">
-        <v>227</v>
-      </c>
-      <c r="D47" s="13"/>
-      <c r="E47" s="23" t="n">
+      <c r="F54" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G54" s="6"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B55" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="D55" s="13"/>
+      <c r="E55" s="23" t="n">
         <f aca="false">'1 ข้อมูล'!$C$24</f>
         <v>0.1</v>
       </c>
-      <c r="F47" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G47" s="6"/>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B48" s="6" t="s">
-        <v>228</v>
-      </c>
-      <c r="C48" s="6" t="s">
-        <v>229</v>
-      </c>
-      <c r="D48" s="13" t="n">
+      <c r="F55" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G55" s="6"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B56" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="D56" s="13" t="n">
         <f aca="false">'1 ข้อมูล'!$C$25+2*'1 ข้อมูล'!$C$26</f>
         <v>1</v>
       </c>
-      <c r="E48" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D48,4),'1 ข้อมูล'!$C$13)</f>
+      <c r="E56" s="23" t="n">
+        <f aca="false">CEILING(ROUND(D56,4),'1 ข้อมูล'!$C$13)</f>
         <v>1</v>
       </c>
-      <c r="F48" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G48" s="6"/>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B49" s="6" t="s">
-        <v>230</v>
-      </c>
-      <c r="C49" s="6" t="s">
-        <v>231</v>
-      </c>
-      <c r="D49" s="13"/>
-      <c r="E49" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$46+'3 ขนาดบ่อ'!$E$47+'3 ขนาดบ่อ'!$E$48</f>
-        <v>1.6</v>
-      </c>
-      <c r="F49" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G49" s="6"/>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B50" s="6" t="s">
-        <v>232</v>
-      </c>
-      <c r="C50" s="6" t="s">
-        <v>233</v>
-      </c>
-      <c r="D50" s="13"/>
-      <c r="E50" s="23" t="n">
-        <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$13*'3 ขนาดบ่อ'!$E$38)</f>
-        <v>0.277993257065429</v>
-      </c>
-      <c r="F50" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="G50" s="6"/>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="6" t="s">
-        <v>234</v>
-      </c>
-      <c r="C51" s="6" t="s">
-        <v>235</v>
-      </c>
-      <c r="D51" s="13"/>
-      <c r="E51" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$39+'3 ขนาดบ่อ'!$E$38+1.5*'3 ขนาดบ่อ'!$E$50^2/(2*'1 ข้อมูล'!$C$48)</f>
-        <v>0.972523267791535</v>
-      </c>
-      <c r="F51" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G51" s="6" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="4" t="s">
-        <v>237</v>
-      </c>
-      <c r="C53" s="5"/>
-      <c r="D53" s="5"/>
-      <c r="E53" s="5"/>
-      <c r="F53" s="5"/>
-      <c r="G53" s="5"/>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B54" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="C54" s="6" t="s">
-        <v>239</v>
-      </c>
-      <c r="D54" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$51+'1 ข้อมูล'!$C$20</f>
-        <v>1.17252326779154</v>
-      </c>
-      <c r="E54" s="23" t="n">
-        <f aca="false">CEILING(ROUND(D54,4),'1 ข้อมูล'!$C$13)</f>
-        <v>1.2</v>
-      </c>
-      <c r="F54" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G54" s="6" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B56" s="4" t="s">
-        <v>241</v>
-      </c>
-      <c r="C56" s="5"/>
-      <c r="D56" s="5"/>
-      <c r="E56" s="5"/>
-      <c r="F56" s="5"/>
-      <c r="G56" s="5"/>
+      <c r="F56" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G56" s="6"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="6" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="D57" s="13"/>
       <c r="E57" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$8-'1 ข้อมูล'!$C$31</f>
-        <v>0.5</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$54+'3 ขนาดบ่อ'!$E$55+'3 ขนาดบ่อ'!$E$56</f>
+        <v>1.6</v>
       </c>
       <c r="F57" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G57" s="6" t="s">
-        <v>244</v>
-      </c>
+      <c r="G57" s="6"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="6" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="D58" s="13"/>
       <c r="E58" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$13+2*'1 ข้อมูล'!$C$34</f>
-        <v>1.7</v>
+        <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$13*'3 ขนาดบ่อ'!$E$46)</f>
+        <v>0.277993257065429</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="G58" s="6"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="6" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
       <c r="D59" s="13"/>
       <c r="E59" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$57-'1 ข้อมูล'!$C$32</f>
-        <v>0.4</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$47+'3 ขนาดบ่อ'!$E$46+1.5*'3 ขนาดบ่อ'!$E$58^2/(2*'1 ข้อมูล'!$C$49)</f>
+        <v>0.972523267791535</v>
       </c>
       <c r="F59" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G59" s="6" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B60" s="6" t="s">
-        <v>250</v>
-      </c>
-      <c r="C60" s="6" t="s">
-        <v>251</v>
-      </c>
-      <c r="D60" s="13"/>
-      <c r="E60" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$9+'1 ข้อมูล'!$C$33</f>
-        <v>1</v>
-      </c>
-      <c r="F60" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G60" s="6"/>
+        <v>255</v>
+      </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B61" s="6" t="s">
-        <v>252</v>
-      </c>
-      <c r="C61" s="6" t="s">
-        <v>253</v>
-      </c>
-      <c r="D61" s="13"/>
-      <c r="E61" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$60-'3 ขนาดบ่อ'!$E$59</f>
-        <v>0.6</v>
-      </c>
-      <c r="F61" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G61" s="6"/>
+      <c r="B61" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="C61" s="5"/>
+      <c r="D61" s="5"/>
+      <c r="E61" s="5"/>
+      <c r="F61" s="5"/>
+      <c r="G61" s="5"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="6" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>255</v>
-      </c>
-      <c r="D62" s="13"/>
+        <v>258</v>
+      </c>
+      <c r="D62" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$59+'1 ข้อมูล'!$C$20</f>
+        <v>1.17252326779154</v>
+      </c>
       <c r="E62" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$32-'3 ขนาดบ่อ'!$E$57</f>
-        <v>0.309665688762588</v>
+        <f aca="false">CEILING(ROUND(D62,4),'1 ข้อมูล'!$C$13)</f>
+        <v>1.2</v>
       </c>
       <c r="F62" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G62" s="6"/>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B63" s="6" t="s">
-        <v>256</v>
-      </c>
-      <c r="C63" s="6" t="s">
-        <v>257</v>
-      </c>
-      <c r="D63" s="13"/>
-      <c r="E63" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$49*'3 ขนาดบ่อ'!$E$62^3/6</f>
-        <v>0.0485508704265308</v>
-      </c>
-      <c r="F63" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="G63" s="6" t="s">
+      <c r="G62" s="6" t="s">
         <v>259</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B64" s="6" t="s">
+      <c r="B64" s="4" t="s">
         <v>260</v>
       </c>
-      <c r="C64" s="6" t="s">
-        <v>261</v>
-      </c>
-      <c r="D64" s="13"/>
-      <c r="E64" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$63/('1 ข้อมูล'!$C$35^2/6)/1000</f>
-        <v>8.09181173775513</v>
-      </c>
-      <c r="F64" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="G64" s="6"/>
+      <c r="C64" s="5"/>
+      <c r="D64" s="5"/>
+      <c r="E64" s="5"/>
+      <c r="F64" s="5"/>
+      <c r="G64" s="5"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="C65" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="C65" s="6" t="s">
+      <c r="D65" s="13"/>
+      <c r="E65" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$8-'1 ข้อมูล'!$C$32</f>
+        <v>0.5</v>
+      </c>
+      <c r="F65" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G65" s="6" t="s">
         <v>263</v>
       </c>
-      <c r="D65" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$64</f>
-        <v>8.09181173775513</v>
-      </c>
-      <c r="E65" s="17" t="str">
-        <f aca="false">IF(D65&lt;=0.6*'1 ข้อมูล'!$C$55,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
-        <v>ผ่าน ✔</v>
-      </c>
-      <c r="F65" s="6"/>
-      <c r="G65" s="6" t="s">
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B66" s="6" t="s">
         <v>264</v>
       </c>
+      <c r="C66" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="D66" s="13"/>
+      <c r="E66" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$13+2*'1 ข้อมูล'!$C$35</f>
+        <v>1.7</v>
+      </c>
+      <c r="F66" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G66" s="6"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B67" s="4" t="s">
-        <v>265</v>
-      </c>
-      <c r="C67" s="5"/>
-      <c r="D67" s="5"/>
-      <c r="E67" s="5"/>
-      <c r="F67" s="5"/>
-      <c r="G67" s="5"/>
+      <c r="B67" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="D67" s="13"/>
+      <c r="E67" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$65-'1 ข้อมูล'!$C$33</f>
+        <v>0.4</v>
+      </c>
+      <c r="F67" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G67" s="6" t="s">
+        <v>268</v>
+      </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B68" s="6" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="D68" s="13"/>
       <c r="E68" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$49*'3 ขนาดบ่อ'!$E$54^3/6</f>
-        <v>2.82528</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$9+'1 ข้อมูล'!$C$34</f>
+        <v>1</v>
       </c>
       <c r="F68" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="G68" s="6" t="s">
-        <v>268</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="G68" s="6"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B69" s="6" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="D69" s="13"/>
       <c r="E69" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$57*'3 ขนาดบ่อ'!$E$68</f>
-        <v>4.802976</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$68-'3 ขนาดบ่อ'!$E$67</f>
+        <v>0.6</v>
       </c>
       <c r="F69" s="6" t="s">
-        <v>258</v>
+        <v>19</v>
       </c>
       <c r="G69" s="6"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B70" s="6" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="D70" s="13"/>
       <c r="E70" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$43-'1 ข้อมูล'!$C$45-0.006</f>
-        <v>0.144</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$32-'3 ขนาดบ่อ'!$E$65</f>
+        <v>0.309665688762588</v>
       </c>
       <c r="F70" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G70" s="6" t="s">
-        <v>273</v>
-      </c>
+      <c r="G70" s="6"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B71" s="6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D71" s="13"/>
       <c r="E71" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$69/(0.9*'1 ข้อมูล'!$C$56*1000*0.9*'3 ขนาดบ่อ'!$E$70)*1000000</f>
-        <v>102.944444444444</v>
+        <f aca="false">'1 ข้อมูล'!$C$50*'3 ขนาดบ่อ'!$E$70^3/6</f>
+        <v>0.0485508704265308</v>
       </c>
       <c r="F71" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="G71" s="6"/>
+        <v>277</v>
+      </c>
+      <c r="G71" s="6" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B72" s="6" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="D72" s="13"/>
       <c r="E72" s="23" t="n">
-        <f aca="false">0.003*1000*'1 ข้อมูล'!$C$43*1000</f>
-        <v>600</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$71/('1 ข้อมูล'!$C$36^2/6)/1000</f>
+        <v>8.09181173775513</v>
       </c>
       <c r="F72" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="G72" s="6" t="s">
-        <v>279</v>
-      </c>
+        <v>99</v>
+      </c>
+      <c r="G72" s="6"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B73" s="6" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>281</v>
-      </c>
-      <c r="D73" s="13"/>
-      <c r="E73" s="23" t="n">
-        <f aca="false">FLOOR(113/MAX('3 ขนาดบ่อ'!$E$71,'3 ขนาดบ่อ'!$E$72)*1000,25)</f>
-        <v>175</v>
-      </c>
-      <c r="F73" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="G73" s="6"/>
-    </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B74" s="6" t="s">
+      <c r="D73" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$72</f>
+        <v>8.09181173775513</v>
+      </c>
+      <c r="E73" s="17" t="str">
+        <f aca="false">IF(D73&lt;=0.6*'1 ข้อมูล'!$C$56,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F73" s="6"/>
+      <c r="G73" s="6" t="s">
         <v>283</v>
       </c>
-      <c r="C74" s="6"/>
-      <c r="D74" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$73</f>
-        <v>175</v>
-      </c>
-      <c r="E74" s="17" t="str">
-        <f aca="false">IF(D74&gt;=100,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
-        <v>ผ่าน ✔</v>
-      </c>
-      <c r="F74" s="6"/>
-      <c r="G74" s="6" t="s">
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B75" s="4" t="s">
         <v>284</v>
       </c>
+      <c r="C75" s="5"/>
+      <c r="D75" s="5"/>
+      <c r="E75" s="5"/>
+      <c r="F75" s="5"/>
+      <c r="G75" s="5"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B76" s="4" t="s">
+      <c r="B76" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="C76" s="5"/>
-      <c r="D76" s="5"/>
-      <c r="E76" s="5"/>
-      <c r="F76" s="5"/>
-      <c r="G76" s="5"/>
+      <c r="C76" s="6" t="s">
+        <v>286</v>
+      </c>
+      <c r="D76" s="13"/>
+      <c r="E76" s="23" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$50*'3 ขนาดบ่อ'!$E$62^3/6</f>
+        <v>2.82528</v>
+      </c>
+      <c r="F76" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="G76" s="6" t="s">
+        <v>287</v>
+      </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B77" s="6" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="D77" s="13"/>
       <c r="E77" s="23" t="n">
-        <f aca="false">ROUND(('1 ข้อมูล'!$C$39+'3 ขนาดบ่อ'!$E$8-'1 ข้อมูล'!$C$38)/2/0.05,0)*0.05</f>
-        <v>0.3</v>
+        <f aca="false">'1 ข้อมูล'!$C$58*'3 ขนาดบ่อ'!$E$76</f>
+        <v>4.802976</v>
       </c>
       <c r="F77" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G77" s="6" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="78" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>277</v>
+      </c>
+      <c r="G77" s="6"/>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B78" s="6" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C78" s="6" t="s">
-        <v>290</v>
-      </c>
-      <c r="D78" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$8-'3 ขนาดบ่อ'!$E$77</f>
-        <v>0.3</v>
-      </c>
-      <c r="E78" s="17" t="str">
-        <f aca="false">IF(D78&gt;='1 ข้อมูล'!$C$38-0.0001,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
-        <v>ผ่าน ✔</v>
-      </c>
-      <c r="F78" s="6"/>
+        <v>291</v>
+      </c>
+      <c r="D78" s="13"/>
+      <c r="E78" s="23" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$44-'1 ข้อมูล'!$C$46-0.006</f>
+        <v>0.144</v>
+      </c>
+      <c r="F78" s="6" t="s">
+        <v>19</v>
+      </c>
       <c r="G78" s="6" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B79" s="6" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>293</v>
-      </c>
-      <c r="D79" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$77</f>
-        <v>0.3</v>
-      </c>
-      <c r="E79" s="17" t="str">
-        <f aca="false">IF(D79&gt;='1 ข้อมูล'!$C$39-0.0001,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
-        <v>ผ่าน ✔</v>
-      </c>
-      <c r="F79" s="6"/>
+        <v>294</v>
+      </c>
+      <c r="D79" s="13"/>
+      <c r="E79" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$77/(0.9*'1 ข้อมูล'!$C$57*1000*0.9*'3 ขนาดบ่อ'!$E$78)*1000000</f>
+        <v>102.944444444444</v>
+      </c>
+      <c r="F79" s="6" t="s">
+        <v>295</v>
+      </c>
       <c r="G79" s="6"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B80" s="6" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D80" s="13"/>
       <c r="E80" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$14-'1 ข้อมูล'!$C$36</f>
-        <v>1.8</v>
+        <f aca="false">0.003*1000*'1 ข้อมูล'!$C$44*1000</f>
+        <v>600</v>
       </c>
       <c r="F80" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G80" s="6"/>
+        <v>295</v>
+      </c>
+      <c r="G80" s="6" t="s">
+        <v>298</v>
+      </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B81" s="6" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="C81" s="6" t="s">
-        <v>297</v>
-      </c>
-      <c r="D81" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$80-'3 ขนาดบ่อ'!$E$15</f>
-        <v>0.85</v>
-      </c>
-      <c r="E81" s="17" t="str">
-        <f aca="false">IF(D81&gt;=0.5,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>300</v>
+      </c>
+      <c r="D81" s="13"/>
+      <c r="E81" s="23" t="n">
+        <f aca="false">FLOOR(113/MAX('3 ขนาดบ่อ'!$E$79,'3 ขนาดบ่อ'!$E$80)*1000,25)</f>
+        <v>175</v>
+      </c>
+      <c r="F81" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="G81" s="6"/>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B82" s="6" t="s">
+        <v>302</v>
+      </c>
+      <c r="C82" s="6"/>
+      <c r="D82" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$81</f>
+        <v>175</v>
+      </c>
+      <c r="E82" s="17" t="str">
+        <f aca="false">IF(D82&gt;=100,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
-      <c r="F81" s="6"/>
-      <c r="G81" s="6" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B82" s="6" t="s">
-        <v>299</v>
-      </c>
-      <c r="C82" s="6" t="s">
-        <v>300</v>
-      </c>
-      <c r="D82" s="13"/>
-      <c r="E82" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$40-'3 ขนาดบ่อ'!$E$32</f>
-        <v>0.290334311237412</v>
-      </c>
-      <c r="F82" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G82" s="6"/>
-    </row>
-    <row r="83" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B83" s="6" t="s">
-        <v>301</v>
-      </c>
-      <c r="C83" s="6" t="s">
-        <v>302</v>
-      </c>
-      <c r="D83" s="13"/>
-      <c r="E83" s="23" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$40-'3 ขนาดบ่อ'!$E$8</f>
-        <v>0.5</v>
-      </c>
-      <c r="F83" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G83" s="6"/>
+      <c r="F82" s="6"/>
+      <c r="G82" s="6" t="s">
+        <v>303</v>
+      </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B84" s="6" t="s">
-        <v>303</v>
-      </c>
-      <c r="C84" s="6" t="s">
+      <c r="B84" s="4" t="s">
         <v>304</v>
       </c>
-      <c r="D84" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$82</f>
-        <v>0.290334311237412</v>
-      </c>
-      <c r="E84" s="17" t="str">
-        <f aca="false">IF(AND(D84&gt;='1 ข้อมูล'!$C$41,'3 ขนาดบ่อ'!$E$83&lt;='1 ข้อมูล'!$C$42),"ผ่าน ✔","ไม่ผ่าน ✘")</f>
-        <v>ผ่าน ✔</v>
-      </c>
-      <c r="F84" s="6"/>
-      <c r="G84" s="6"/>
+      <c r="C84" s="5"/>
+      <c r="D84" s="5"/>
+      <c r="E84" s="5"/>
+      <c r="F84" s="5"/>
+      <c r="G84" s="5"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B85" s="6" t="s">
         <v>305</v>
       </c>
-      <c r="C85" s="6"/>
-      <c r="D85" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$54-'1 ข้อมูล'!$C$40</f>
-        <v>0.1</v>
-      </c>
-      <c r="E85" s="17" t="str">
-        <f aca="false">IF(D85&gt;=0,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+      <c r="C85" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="D85" s="13"/>
+      <c r="E85" s="23" t="n">
+        <f aca="false">ROUND(('1 ข้อมูล'!$C$40+'3 ขนาดบ่อ'!$E$8-'1 ข้อมูล'!$C$39)/2/0.05,0)*0.05</f>
+        <v>0.3</v>
+      </c>
+      <c r="F85" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G85" s="6" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B86" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="C86" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="D86" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$8-'3 ขนาดบ่อ'!$E$85</f>
+        <v>0.3</v>
+      </c>
+      <c r="E86" s="17" t="str">
+        <f aca="false">IF(D86&gt;='1 ข้อมูล'!$C$39-0.0001,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
-      <c r="F85" s="6"/>
-      <c r="G85" s="6" t="s">
-        <v>306</v>
+      <c r="F86" s="6"/>
+      <c r="G86" s="6" t="s">
+        <v>310</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B87" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="C87" s="5"/>
-      <c r="D87" s="5"/>
-      <c r="E87" s="5"/>
-      <c r="F87" s="5"/>
-      <c r="G87" s="5"/>
+      <c r="B87" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="C87" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="D87" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$85</f>
+        <v>0.3</v>
+      </c>
+      <c r="E87" s="17" t="str">
+        <f aca="false">IF(D87&gt;='1 ข้อมูล'!$C$40-0.0001,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F87" s="6"/>
+      <c r="G87" s="6"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B88" s="6" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="C88" s="6" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="D88" s="13"/>
       <c r="E88" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$35+'3 ขนาดบ่อ'!$E$14+'1 ข้อมูล'!$C$43+'3 ขนาดบ่อ'!$E$29</f>
-        <v>3.75</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$14-'1 ข้อมูล'!$C$37</f>
+        <v>1.8</v>
       </c>
       <c r="F88" s="6" t="s">
         <v>19</v>
@@ -4409,105 +4512,222 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B89" s="6" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="C89" s="6" t="s">
-        <v>311</v>
-      </c>
-      <c r="D89" s="13"/>
-      <c r="E89" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$49+'3 ขนาดบ่อ'!$E$41+'3 ขนาดบ่อ'!$E$88</f>
-        <v>6.35</v>
-      </c>
-      <c r="F89" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G89" s="6"/>
-    </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>316</v>
+      </c>
+      <c r="D89" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$88-'3 ขนาดบ่อ'!$E$15</f>
+        <v>0.85</v>
+      </c>
+      <c r="E89" s="17" t="str">
+        <f aca="false">IF(D89&gt;=0.5,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F89" s="6"/>
+      <c r="G89" s="6" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B90" s="6" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="C90" s="6" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
       <c r="D90" s="13"/>
       <c r="E90" s="23" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$41-'3 ขนาดบ่อ'!$E$32</f>
+        <v>0.290334311237412</v>
+      </c>
+      <c r="F90" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G90" s="6"/>
+    </row>
+    <row r="91" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B91" s="6" t="s">
+        <v>320</v>
+      </c>
+      <c r="C91" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="D91" s="13"/>
+      <c r="E91" s="23" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$41-'3 ขนาดบ่อ'!$E$8</f>
+        <v>0.5</v>
+      </c>
+      <c r="F91" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G91" s="6"/>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B92" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="C92" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="D92" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$90</f>
+        <v>0.290334311237412</v>
+      </c>
+      <c r="E92" s="17" t="str">
+        <f aca="false">IF(AND(D92&gt;='1 ข้อมูล'!$C$42,'3 ขนาดบ่อ'!$E$91&lt;='1 ข้อมูล'!$C$43),"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F92" s="6"/>
+      <c r="G92" s="6"/>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B93" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="C93" s="6"/>
+      <c r="D93" s="13" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$62-'1 ข้อมูล'!$C$41</f>
+        <v>0.1</v>
+      </c>
+      <c r="E93" s="17" t="str">
+        <f aca="false">IF(D93&gt;=0,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="F93" s="6"/>
+      <c r="G93" s="6" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B95" s="4" t="s">
+        <v>326</v>
+      </c>
+      <c r="C95" s="5"/>
+      <c r="D95" s="5"/>
+      <c r="E95" s="5"/>
+      <c r="F95" s="5"/>
+      <c r="G95" s="5"/>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B96" s="6" t="s">
+        <v>327</v>
+      </c>
+      <c r="C96" s="6" t="s">
+        <v>328</v>
+      </c>
+      <c r="D96" s="13"/>
+      <c r="E96" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$35+'3 ขนาดบ่อ'!$E$14+'1 ข้อมูล'!$C$44+'3 ขนาดบ่อ'!$E$29</f>
+        <v>3.75</v>
+      </c>
+      <c r="F96" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G96" s="6"/>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B97" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="C97" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="D97" s="13"/>
+      <c r="E97" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$57+'3 ขนาดบ่อ'!$E$49+'3 ขนาดบ่อ'!$E$96</f>
+        <v>6.35</v>
+      </c>
+      <c r="F97" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G97" s="6"/>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B98" s="6" t="s">
+        <v>331</v>
+      </c>
+      <c r="C98" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="D98" s="13"/>
+      <c r="E98" s="23" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$13</f>
         <v>1.5</v>
       </c>
-      <c r="F90" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G90" s="6"/>
-    </row>
-    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B91" s="6" t="s">
-        <v>314</v>
-      </c>
-      <c r="C91" s="6" t="s">
-        <v>315</v>
-      </c>
-      <c r="D91" s="13"/>
-      <c r="E91" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$54</f>
+      <c r="F98" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G98" s="6"/>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B99" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="C99" s="6" t="s">
+        <v>334</v>
+      </c>
+      <c r="D99" s="13"/>
+      <c r="E99" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$62</f>
         <v>1.2</v>
       </c>
-      <c r="F91" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G91" s="6"/>
-    </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B92" s="6" t="s">
-        <v>316</v>
-      </c>
-      <c r="C92" s="6" t="s">
-        <v>317</v>
-      </c>
-      <c r="D92" s="13"/>
-      <c r="E92" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$89+2*'1 ข้อมูล'!$C$43</f>
+      <c r="F99" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G99" s="6"/>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B100" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="C100" s="6" t="s">
+        <v>336</v>
+      </c>
+      <c r="D100" s="13"/>
+      <c r="E100" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$97+2*'1 ข้อมูล'!$C$44</f>
         <v>6.75</v>
       </c>
-      <c r="F92" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G92" s="6"/>
-    </row>
-    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B93" s="6" t="s">
-        <v>318</v>
-      </c>
-      <c r="C93" s="6" t="s">
-        <v>317</v>
-      </c>
-      <c r="D93" s="13"/>
-      <c r="E93" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$90+2*'1 ข้อมูล'!$C$43</f>
+      <c r="F100" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G100" s="6"/>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B101" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="C101" s="6" t="s">
+        <v>336</v>
+      </c>
+      <c r="D101" s="13"/>
+      <c r="E101" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$98+2*'1 ข้อมูล'!$C$44</f>
         <v>1.9</v>
       </c>
-      <c r="F93" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G93" s="6"/>
-    </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B94" s="6" t="s">
-        <v>319</v>
-      </c>
-      <c r="C94" s="6" t="s">
-        <v>320</v>
-      </c>
-      <c r="D94" s="13"/>
-      <c r="E94" s="23" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$91+'1 ข้อมูล'!$C$44</f>
+      <c r="F101" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G101" s="6"/>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B102" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="C102" s="6" t="s">
+        <v>339</v>
+      </c>
+      <c r="D102" s="13"/>
+      <c r="E102" s="23" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$99+'1 ข้อมูล'!$C$45</f>
         <v>1.4</v>
       </c>
-      <c r="F94" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G94" s="6"/>
+      <c r="F102" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G102" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -4541,43 +4761,43 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>321</v>
+        <v>340</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>322</v>
+        <v>341</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>323</v>
+        <v>342</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>324</v>
+        <v>343</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>325</v>
+        <v>344</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>326</v>
+        <v>345</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>327</v>
+        <v>346</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>328</v>
+        <v>347</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>329</v>
+        <v>348</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C5" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$7-'1 ข้อมูล'!$C$9</f>
@@ -4588,7 +4808,7 @@
         <v>0.0111111111111111</v>
       </c>
       <c r="E5" s="9" t="n">
-        <f aca="false">(D5/('1 ข้อมูล'!$C$53*'3 ขนาดบ่อ'!$E$13))^(2/3)*100</f>
+        <f aca="false">(D5/('1 ข้อมูล'!$C$54*'3 ขนาดบ่อ'!$E$13))^(2/3)*100</f>
         <v>2.53065109461751</v>
       </c>
       <c r="F5" s="19" t="n">
@@ -4600,7 +4820,7 @@
         <v>0.163495428200321</v>
       </c>
       <c r="H5" s="12" t="n">
-        <f aca="false">G5/SQRT('1 ข้อมูล'!$C$48*F5/100)</f>
+        <f aca="false">G5/SQRT('1 ข้อมูล'!$C$49*F5/100)</f>
         <v>0.24523971352263</v>
       </c>
       <c r="I5" s="17" t="str">
@@ -4610,7 +4830,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C6" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$10-'1 ข้อมูล'!$C$9</f>
@@ -4621,7 +4841,7 @@
         <v>0.0146643518518519</v>
       </c>
       <c r="E6" s="9" t="n">
-        <f aca="false">(D6/('1 ข้อมูล'!$C$53*'3 ขนาดบ่อ'!$E$13))^(2/3)*100</f>
+        <f aca="false">(D6/('1 ข้อมูล'!$C$54*'3 ขนาดบ่อ'!$E$13))^(2/3)*100</f>
         <v>3.04487307291521</v>
       </c>
       <c r="F6" s="19" t="n">
@@ -4633,7 +4853,7 @@
         <v>0.193785540817422</v>
       </c>
       <c r="H6" s="12" t="n">
-        <f aca="false">G6/SQRT('1 ข้อมูล'!$C$48*F6/100)</f>
+        <f aca="false">G6/SQRT('1 ข้อมูล'!$C$49*F6/100)</f>
         <v>0.275462029969398</v>
       </c>
       <c r="I6" s="17" t="str">
@@ -4643,7 +4863,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C7" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8-'1 ข้อมูล'!$C$9</f>
@@ -4654,7 +4874,7 @@
         <v>0.025</v>
       </c>
       <c r="E7" s="9" t="n">
-        <f aca="false">(D7/('1 ข้อมูล'!$C$53*'3 ขนาดบ่อ'!$E$13))^(2/3)*100</f>
+        <f aca="false">(D7/('1 ข้อมูล'!$C$54*'3 ขนาดบ่อ'!$E$13))^(2/3)*100</f>
         <v>4.34530852641276</v>
       </c>
       <c r="F7" s="19" t="n">
@@ -4666,7 +4886,7 @@
         <v>0.262661249603397</v>
       </c>
       <c r="H7" s="12" t="n">
-        <f aca="false">G7/SQRT('1 ข้อมูล'!$C$48*F7/100)</f>
+        <f aca="false">G7/SQRT('1 ข้อมูล'!$C$49*F7/100)</f>
         <v>0.332916354683497</v>
       </c>
       <c r="I7" s="17" t="str">
@@ -4676,7 +4896,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C8" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8</f>
@@ -4687,7 +4907,7 @@
         <v>0.0277777777777778</v>
       </c>
       <c r="E8" s="9" t="n">
-        <f aca="false">(D8/('1 ข้อมูล'!$C$53*'3 ขนาดบ่อ'!$E$13))^(2/3)*100</f>
+        <f aca="false">(D8/('1 ข้อมูล'!$C$54*'3 ขนาดบ่อ'!$E$13))^(2/3)*100</f>
         <v>4.66149917231983</v>
       </c>
       <c r="F8" s="19" t="n">
@@ -4699,7 +4919,7 @@
         <v>0.277993257065429</v>
       </c>
       <c r="H8" s="12" t="n">
-        <f aca="false">G8/SQRT('1 ข้อมูล'!$C$48*F8/100)</f>
+        <f aca="false">G8/SQRT('1 ข้อมูล'!$C$49*F8/100)</f>
         <v>0.343885424767124</v>
       </c>
       <c r="I8" s="17" t="str">
@@ -4709,17 +4929,17 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="22" t="s">
-        <v>330</v>
+        <v>349</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="22" t="s">
-        <v>331</v>
+        <v>350</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="22" t="s">
-        <v>332</v>
+        <v>351</v>
       </c>
     </row>
   </sheetData>
@@ -4749,172 +4969,172 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>333</v>
+        <v>352</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>334</v>
+        <v>353</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>335</v>
+        <v>354</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>19</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>336</v>
+        <v>355</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="6" t="s">
-        <v>315</v>
+        <v>334</v>
       </c>
       <c r="C5" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$54</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$62</f>
         <v>1.2</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>239</v>
+        <v>258</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>337</v>
+        <v>356</v>
       </c>
       <c r="C6" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$51</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$59</f>
         <v>0.972523267791535</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>338</v>
+        <v>357</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>339</v>
+        <v>358</v>
       </c>
       <c r="C7" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$39+'1 ข้อมูล'!$C$17</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$47+'1 ข้อมูล'!$C$17</f>
         <v>0.92</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>340</v>
+        <v>359</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>341</v>
+        <v>360</v>
       </c>
       <c r="C8" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$39</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$47</f>
         <v>0.9</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>214</v>
+        <v>234</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="6" t="s">
-        <v>342</v>
+        <v>361</v>
       </c>
       <c r="C9" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$60</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$68</f>
         <v>1</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>251</v>
+        <v>270</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>343</v>
+        <v>362</v>
       </c>
       <c r="C10" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$9</f>
         <v>0.9</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>344</v>
+        <v>363</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
-        <v>345</v>
+        <v>364</v>
       </c>
       <c r="C11" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$32</f>
         <v>0.809665688762588</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>346</v>
+        <v>365</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>347</v>
+        <v>366</v>
       </c>
       <c r="C12" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8</f>
         <v>0.6</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>348</v>
+        <v>367</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="6" t="s">
-        <v>349</v>
+        <v>368</v>
       </c>
       <c r="C13" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$57</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$65</f>
         <v>0.5</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>243</v>
+        <v>262</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="6" t="s">
-        <v>350</v>
+        <v>369</v>
       </c>
       <c r="C14" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$59</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$67</f>
         <v>0.4</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>351</v>
+        <v>370</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="6" t="s">
-        <v>352</v>
+        <v>371</v>
       </c>
       <c r="C15" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$45</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$53</f>
         <v>0.2</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>353</v>
+        <v>372</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="s">
-        <v>354</v>
+        <v>373</v>
       </c>
       <c r="C16" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$24</f>
         <v>0.210686269183871</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>355</v>
+        <v>374</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="s">
-        <v>356</v>
+        <v>375</v>
       </c>
       <c r="C17" s="24" t="n">
         <f aca="false">0</f>
@@ -4950,32 +5170,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>357</v>
+        <v>376</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>358</v>
+        <v>377</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>359</v>
+        <v>378</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>360</v>
+        <v>379</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>361</v>
+        <v>380</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>362</v>
+        <v>381</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>363</v>
+        <v>382</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>364</v>
+        <v>383</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4987,7 +5207,7 @@
         <v>2.77719642805474</v>
       </c>
       <c r="D5" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B5/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B5/100+'1 ข้อมูล'!$C$53)^2.5*3600</f>
         <v>2.86619650300861</v>
       </c>
       <c r="E5" s="25" t="n">
@@ -5012,7 +5232,7 @@
         <v>4.38086341517286</v>
       </c>
       <c r="D6" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B6/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B6/100+'1 ข้อมูล'!$C$53)^2.5*3600</f>
         <v>4.48983131905459</v>
       </c>
       <c r="E6" s="25" t="n">
@@ -5037,7 +5257,7 @@
         <v>6.44060533155076</v>
       </c>
       <c r="D7" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B7/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B7/100+'1 ข้อมูล'!$C$53)^2.5*3600</f>
         <v>6.56792530595593</v>
       </c>
       <c r="E7" s="25" t="n">
@@ -5062,7 +5282,7 @@
         <v>8.99304061167301</v>
       </c>
       <c r="D8" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B8/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B8/100+'1 ข้อมูล'!$C$53)^2.5*3600</f>
         <v>9.13647413844802</v>
       </c>
       <c r="E8" s="25" t="n">
@@ -5087,7 +5307,7 @@
         <v>12.07224</v>
       </c>
       <c r="D9" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B9/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B9/100+'1 ข้อมูล'!$C$53)^2.5*3600</f>
         <v>12.2289986697729</v>
       </c>
       <c r="E9" s="25" t="n">
@@ -5112,7 +5332,7 @@
         <v>15.7101954157165</v>
       </c>
       <c r="D10" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B10/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B10/100+'1 ข้อมูล'!$C$53)^2.5*3600</f>
         <v>15.8769956216084</v>
       </c>
       <c r="E10" s="25" t="n">
@@ -5137,7 +5357,7 @@
         <v>19.9371602697676</v>
       </c>
       <c r="D11" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B11/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B11/100+'1 ข้อมูล'!$C$53)^2.5*3600</f>
         <v>20.1102658699656</v>
       </c>
       <c r="E11" s="25" t="n">
@@ -5162,7 +5382,7 @@
         <v>24.7819058265663</v>
       </c>
       <c r="D12" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B12/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B12/100+'1 ข้อมูล'!$C$53)^2.5*3600</f>
         <v>24.9571624264048</v>
       </c>
       <c r="E12" s="25" t="n">
@@ -5187,7 +5407,7 @@
         <v>30.2719200646936</v>
       </c>
       <c r="D13" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B13/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B13/100+'1 ข้อมูล'!$C$53)^2.5*3600</f>
         <v>30.4447832233961</v>
       </c>
       <c r="E13" s="25" t="n">
@@ -5212,7 +5432,7 @@
         <v>36.4335656390862</v>
       </c>
       <c r="D14" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B14/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B14/100+'1 ข้อมูล'!$C$53)^2.5*3600</f>
         <v>36.599124528368</v>
       </c>
       <c r="E14" s="25" t="n">
@@ -5237,7 +5457,7 @@
         <v>43.2922078439065</v>
       </c>
       <c r="D15" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B15/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B15/100+'1 ข้อมูล'!$C$53)^2.5*3600</f>
         <v>43.4452054104805</v>
       </c>
       <c r="E15" s="25" t="n">
@@ -5262,7 +5482,7 @@
         <v>50.87232</v>
       </c>
       <c r="D16" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B16/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B16/100+'1 ข้อมูล'!$C$53)^2.5*3600</f>
         <v>51.0071703805085</v>
       </c>
       <c r="E16" s="25" t="n">
@@ -5287,7 +5507,7 @@
         <v>59.1975714819181</v>
       </c>
       <c r="D17" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B17/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B17/100+'1 ข้อมูล'!$C$53)^2.5*3600</f>
         <v>59.3083752175669</v>
       </c>
       <c r="E17" s="25" t="n">
@@ -5312,7 +5532,7 @@
         <v>68.2909021448919</v>
       </c>
       <c r="D18" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B18/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B18/100+'1 ข้อมูล'!$C$53)^2.5*3600</f>
         <v>68.3714596053392</v>
       </c>
       <c r="E18" s="25" t="n">
@@ -5337,7 +5557,7 @@
         <v>78.1745859249513</v>
       </c>
       <c r="D19" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B19/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B19/100+'1 ข้อมูล'!$C$53)^2.5*3600</f>
         <v>78.2184092541632</v>
       </c>
       <c r="E19" s="25" t="n">
@@ -5362,7 +5582,7 @@
         <v>88.8702856977516</v>
       </c>
       <c r="D20" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B20/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B20/100+'1 ข้อมูล'!$C$53)^2.5*3600</f>
         <v>88.8706095248216</v>
       </c>
       <c r="E20" s="25" t="n">
@@ -5387,7 +5607,7 @@
         <v>100.399100991704</v>
       </c>
       <c r="D21" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B21/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B21/100+'1 ข้อมูล'!$C$53)^2.5*3600</f>
         <v>100.348892098404</v>
       </c>
       <c r="E21" s="25" t="n">
@@ -5412,7 +5632,7 @@
         <v>112.781609794846</v>
       </c>
       <c r="D22" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B22/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B22/100+'1 ข้อมูล'!$C$53)^2.5*3600</f>
         <v>112.673575893332</v>
       </c>
       <c r="E22" s="25" t="n">
@@ -5437,7 +5657,7 @@
         <v>126.037905431355</v>
       </c>
       <c r="D23" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B23/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B23/100+'1 ข้อมูล'!$C$53)^2.5*3600</f>
         <v>125.864503176292</v>
       </c>
       <c r="E23" s="25" t="n">
@@ -5462,7 +5682,7 @@
         <v>140.187629285531</v>
       </c>
       <c r="D24" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B24/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B24/100+'1 ข้อมูล'!$C$53)^2.5*3600</f>
         <v>139.941071622383</v>
       </c>
       <c r="E24" s="25" t="n">
@@ -5487,7 +5707,7 @@
         <v>155.25</v>
       </c>
       <c r="D25" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B25/100+'1 ข้อมูล'!$C$52)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B25/100+'1 ข้อมูล'!$C$53)^2.5*3600</f>
         <v>154.922262933655</v>
       </c>
       <c r="E25" s="25" t="n">
@@ -5531,12 +5751,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>365</v>
+        <v>384</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>366</v>
+        <v>385</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5544,7 +5764,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>3</v>
@@ -5553,12 +5773,12 @@
         <v>4</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="4" t="s">
-        <v>367</v>
+        <v>386</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -5567,13 +5787,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>368</v>
+        <v>387</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>369</v>
+        <v>388</v>
       </c>
       <c r="D7" s="12" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$49</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$57</f>
         <v>1.6</v>
       </c>
       <c r="E7" s="6" t="s">
@@ -5583,28 +5803,28 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>370</v>
+        <v>389</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>371</v>
+        <v>390</v>
       </c>
       <c r="D8" s="12" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$41</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$49</f>
         <v>1</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>19</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>372</v>
+        <v>391</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="6" t="s">
-        <v>373</v>
+        <v>392</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>374</v>
+        <v>393</v>
       </c>
       <c r="D9" s="27" t="n">
         <f aca="false">'7 แบบพับ'!$D$7+'7 แบบพับ'!$D$8</f>
@@ -5617,10 +5837,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>375</v>
+        <v>394</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>376</v>
+        <v>395</v>
       </c>
       <c r="D10" s="12" t="n">
         <f aca="false">MAX('7 แบบพับ'!$D$8,'3 ขนาดบ่อ'!$E$35)</f>
@@ -5630,18 +5850,18 @@
         <v>19</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>377</v>
+        <v>396</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
-        <v>378</v>
+        <v>397</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>309</v>
+        <v>328</v>
       </c>
       <c r="D11" s="27" t="n">
-        <f aca="false">'7 แบบพับ'!$D$10+'3 ขนาดบ่อ'!$E$14+'1 ข้อมูล'!$C$43+'3 ขนาดบ่อ'!$E$29</f>
+        <f aca="false">'7 แบบพับ'!$D$10+'3 ขนาดบ่อ'!$E$14+'1 ข้อมูล'!$C$44+'3 ขนาดบ่อ'!$E$29</f>
         <v>4.25</v>
       </c>
       <c r="E11" s="6" t="s">
@@ -5651,10 +5871,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>379</v>
+        <v>398</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>380</v>
+        <v>399</v>
       </c>
       <c r="D12" s="27" t="n">
         <f aca="false">MAX('7 แบบพับ'!$D$9,'7 แบบพับ'!$D$11)</f>
@@ -5667,10 +5887,10 @@
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="6" t="s">
-        <v>381</v>
+        <v>400</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>382</v>
+        <v>401</v>
       </c>
       <c r="D13" s="12" t="n">
         <f aca="false">'7 แบบพับ'!$D$12-'7 แบบพับ'!$D$9</f>
@@ -5680,18 +5900,18 @@
         <v>19</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>383</v>
+        <v>402</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="6" t="s">
-        <v>312</v>
+        <v>331</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>384</v>
+        <v>403</v>
       </c>
       <c r="D14" s="12" t="n">
-        <f aca="false">2*'3 ขนาดบ่อ'!$E$13+'1 ข้อมูล'!$C$43</f>
+        <f aca="false">2*'3 ขนาดบ่อ'!$E$13+'1 ข้อมูล'!$C$44</f>
         <v>3.2</v>
       </c>
       <c r="E14" s="6" t="s">
@@ -5701,7 +5921,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="4" t="s">
-        <v>385</v>
+        <v>404</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
@@ -5711,127 +5931,127 @@
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="28"/>
       <c r="C17" s="28" t="s">
-        <v>386</v>
+        <v>405</v>
       </c>
       <c r="D17" s="28" t="s">
-        <v>387</v>
+        <v>406</v>
       </c>
       <c r="E17" s="28" t="s">
-        <v>388</v>
+        <v>407</v>
       </c>
       <c r="F17" s="28"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="6" t="s">
-        <v>389</v>
+        <v>408</v>
       </c>
       <c r="C18" s="12" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$92</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$100</f>
         <v>6.75</v>
       </c>
       <c r="D18" s="12" t="n">
-        <f aca="false">'7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$43</f>
+        <f aca="false">'7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$44</f>
         <v>4.65</v>
       </c>
       <c r="E18" s="12" t="n">
-        <f aca="false">'7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$43</f>
+        <f aca="false">'7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$44</f>
         <v>4.65</v>
       </c>
       <c r="F18" s="6"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="6" t="s">
-        <v>390</v>
+        <v>409</v>
       </c>
       <c r="C19" s="12" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$93</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$101</f>
         <v>1.9</v>
       </c>
       <c r="D19" s="12" t="n">
-        <f aca="false">'7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$43</f>
+        <f aca="false">'7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$44</f>
         <v>3.6</v>
       </c>
       <c r="E19" s="12" t="n">
-        <f aca="false">'7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$43</f>
+        <f aca="false">'7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$44</f>
         <v>3.6</v>
       </c>
       <c r="F19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="6" t="s">
-        <v>391</v>
+        <v>410</v>
       </c>
       <c r="C20" s="12" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$92*'3 ขนาดบ่อ'!$E$93</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$100*'3 ขนาดบ่อ'!$E$101</f>
         <v>12.825</v>
       </c>
       <c r="D20" s="12" t="n">
-        <f aca="false">('7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$43)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$43)</f>
+        <f aca="false">('7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$44)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$44)</f>
         <v>16.74</v>
       </c>
       <c r="E20" s="12" t="n">
-        <f aca="false">('7 แบบพับ'!$D$9+2*'1 ข้อมูล'!$C$43)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$43)+('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$9)*('3 ขนาดบ่อ'!$E$13+2*'1 ข้อมูล'!$C$43)</f>
+        <f aca="false">('7 แบบพับ'!$D$9+2*'1 ข้อมูล'!$C$44)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$44)+('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$9)*('3 ขนาดบ่อ'!$E$13+2*'1 ข้อมูล'!$C$44)</f>
         <v>13.935</v>
       </c>
       <c r="F20" s="6"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="6" t="s">
-        <v>392</v>
+        <v>411</v>
       </c>
       <c r="C21" s="12" t="n">
-        <f aca="false">2*('3 ขนาดบ่อ'!$E$89+'1 ข้อมูล'!$C$43+'3 ขนาดบ่อ'!$E$90+'1 ข้อมูล'!$C$43)*'1 ข้อมูล'!$C$43*'3 ขนาดบ่อ'!$E$54</f>
+        <f aca="false">2*('3 ขนาดบ่อ'!$E$97+'1 ข้อมูล'!$C$44+'3 ขนาดบ่อ'!$E$98+'1 ข้อมูล'!$C$44)*'1 ข้อมูล'!$C$44*'3 ขนาดบ่อ'!$E$62</f>
         <v>3.96</v>
       </c>
       <c r="D21" s="12" t="n">
-        <f aca="false">2*('7 แบบพับ'!$D$12+'1 ข้อมูล'!$C$43+'7 แบบพับ'!$D$14+'1 ข้อมูล'!$C$43)*'1 ข้อมูล'!$C$43*'3 ขนาดบ่อ'!$E$54</f>
+        <f aca="false">2*('7 แบบพับ'!$D$12+'1 ข้อมูล'!$C$44+'7 แบบพับ'!$D$14+'1 ข้อมูล'!$C$44)*'1 ข้อมูล'!$C$44*'3 ขนาดบ่อ'!$E$62</f>
         <v>3.768</v>
       </c>
       <c r="E21" s="12" t="n">
-        <f aca="false">2*('7 แบบพับ'!$D$12+'1 ข้อมูล'!$C$43+'7 แบบพับ'!$D$14+'1 ข้อมูล'!$C$43)*'1 ข้อมูล'!$C$43*'3 ขนาดบ่อ'!$E$54</f>
+        <f aca="false">2*('7 แบบพับ'!$D$12+'1 ข้อมูล'!$C$44+'7 แบบพับ'!$D$14+'1 ข้อมูล'!$C$44)*'1 ข้อมูล'!$C$44*'3 ขนาดบ่อ'!$E$62</f>
         <v>3.768</v>
       </c>
       <c r="F21" s="6"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="6" t="s">
-        <v>393</v>
+        <v>412</v>
       </c>
       <c r="C22" s="12" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
       <c r="D22" s="12" t="n">
-        <f aca="false">('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$8)*'1 ข้อมูล'!$C$43*'3 ขนาดบ่อ'!$E$54</f>
+        <f aca="false">('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$8)*'1 ข้อมูล'!$C$44*'3 ขนาดบ่อ'!$E$62</f>
         <v>0.78</v>
       </c>
       <c r="E22" s="12" t="n">
-        <f aca="false">'7 แบบพับ'!$D$7*'1 ข้อมูล'!$C$43*'3 ขนาดบ่อ'!$E$54</f>
+        <f aca="false">'7 แบบพับ'!$D$7*'1 ข้อมูล'!$C$44*'3 ขนาดบ่อ'!$E$62</f>
         <v>0.384</v>
       </c>
       <c r="F22" s="6"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="6" t="s">
-        <v>394</v>
+        <v>413</v>
       </c>
       <c r="C23" s="12" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$92*'3 ขนาดบ่อ'!$E$93*'1 ข้อมูล'!$C$44</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$100*'3 ขนาดบ่อ'!$E$101*'1 ข้อมูล'!$C$45</f>
         <v>2.565</v>
       </c>
       <c r="D23" s="12" t="n">
-        <f aca="false">('7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$43)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$43)*'1 ข้อมูล'!$C$44</f>
+        <f aca="false">('7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$44)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$44)*'1 ข้อมูล'!$C$45</f>
         <v>3.348</v>
       </c>
       <c r="E23" s="12" t="n">
-        <f aca="false">(('7 แบบพับ'!$D$9+2*'1 ข้อมูล'!$C$43)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$43)+('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$9)*('3 ขนาดบ่อ'!$E$13+2*'1 ข้อมูล'!$C$43))*'1 ข้อมูล'!$C$44</f>
+        <f aca="false">(('7 แบบพับ'!$D$9+2*'1 ข้อมูล'!$C$44)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$44)+('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$9)*('3 ขนาดบ่อ'!$E$13+2*'1 ข้อมูล'!$C$44))*'1 ข้อมูล'!$C$45</f>
         <v>2.787</v>
       </c>
       <c r="F23" s="6"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="6" t="s">
-        <v>395</v>
+        <v>414</v>
       </c>
       <c r="C24" s="27" t="n">
         <f aca="false">SUM(C21:C23)</f>
@@ -5846,15 +6066,15 @@
         <v>6.939</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>396</v>
+        <v>415</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="6" t="s">
-        <v>397</v>
+        <v>416</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D25" s="29" t="n">
         <f aca="false">1-D18/C18</f>
@@ -5868,7 +6088,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="4" t="s">
-        <v>398</v>
+        <v>417</v>
       </c>
       <c r="C28" s="5"/>
       <c r="D28" s="5"/>
@@ -5877,10 +6097,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="30" t="s">
-        <v>399</v>
+        <v>418</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>400</v>
+        <v>419</v>
       </c>
       <c r="D29" s="6"/>
       <c r="E29" s="6"/>
@@ -5888,10 +6108,10 @@
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="30" t="s">
-        <v>401</v>
+        <v>420</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>402</v>
+        <v>421</v>
       </c>
       <c r="D30" s="6"/>
       <c r="E30" s="6"/>
@@ -5899,10 +6119,10 @@
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="30" t="s">
-        <v>403</v>
+        <v>422</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>404</v>
+        <v>423</v>
       </c>
       <c r="D31" s="6"/>
       <c r="E31" s="6"/>
@@ -5910,10 +6130,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="30" t="s">
-        <v>405</v>
+        <v>424</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>406</v>
+        <v>425</v>
       </c>
       <c r="D32" s="6"/>
       <c r="E32" s="6"/>
@@ -5921,10 +6141,10 @@
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="31" t="s">
-        <v>407</v>
+        <v>426</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>408</v>
+        <v>427</v>
       </c>
       <c r="D33" s="6"/>
       <c r="E33" s="6"/>
@@ -5932,10 +6152,10 @@
     </row>
     <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="31" t="s">
-        <v>409</v>
+        <v>428</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>410</v>
+        <v>429</v>
       </c>
       <c r="D34" s="6"/>
       <c r="E34" s="6"/>
@@ -5943,10 +6163,10 @@
     </row>
     <row r="35" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="31" t="s">
-        <v>411</v>
+        <v>430</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>412</v>
+        <v>431</v>
       </c>
       <c r="D35" s="6"/>
       <c r="E35" s="6"/>
@@ -5954,10 +6174,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="31" t="s">
-        <v>413</v>
+        <v>432</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>414</v>
+        <v>433</v>
       </c>
       <c r="D36" s="6"/>
       <c r="E36" s="6"/>
@@ -5995,150 +6215,150 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>415</v>
+        <v>434</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>416</v>
+        <v>435</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>417</v>
+        <v>436</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>418</v>
+        <v>437</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>419</v>
+        <v>438</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>420</v>
+        <v>439</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>421</v>
+        <v>440</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>422</v>
+        <v>441</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>423</v>
+        <v>442</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>424</v>
+        <v>443</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="32" t="s">
-        <v>425</v>
+        <v>444</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>426</v>
+        <v>445</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>427</v>
+        <v>446</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>428</v>
+        <v>447</v>
       </c>
       <c r="F5" s="23" t="n">
         <f aca="false">'1 ข้อมูล'!$C$10/3600</f>
         <v>0.0174421296296296</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>429</v>
+        <v>448</v>
       </c>
       <c r="H5" s="12"/>
       <c r="I5" s="17"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="32" t="s">
-        <v>430</v>
+        <v>449</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>431</v>
+        <v>450</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>432</v>
+        <v>451</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>428</v>
+        <v>447</v>
       </c>
       <c r="F6" s="23" t="n">
         <f aca="false">1.5*F5</f>
         <v>0.0261631944444444</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>433</v>
+        <v>452</v>
       </c>
       <c r="H6" s="12"/>
       <c r="I6" s="17"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="32" t="s">
-        <v>434</v>
+        <v>453</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>435</v>
+        <v>454</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>436</v>
+        <v>455</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>428</v>
+        <v>447</v>
       </c>
       <c r="F7" s="23" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8/3600</f>
         <v>0.0277777777777778</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>437</v>
+        <v>456</v>
       </c>
       <c r="H7" s="12"/>
       <c r="I7" s="17"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="32" t="s">
-        <v>438</v>
+        <v>457</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>439</v>
+        <v>458</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>440</v>
+        <v>459</v>
       </c>
       <c r="E8" s="6"/>
       <c r="F8" s="23" t="n">
         <v>1</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>441</v>
+        <v>460</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>425</v>
+        <v>444</v>
       </c>
       <c r="I8" s="17"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="32" t="s">
-        <v>442</v>
+        <v>461</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>443</v>
+        <v>462</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>444</v>
+        <v>463</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>428</v>
+        <v>447</v>
       </c>
       <c r="F9" s="23" t="n">
         <f aca="false">MAX(F6,F7)/F8</f>
         <v>0.0277777777777778</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>445</v>
+        <v>464</v>
       </c>
       <c r="H9" s="12" t="n">
         <f aca="false">'2 เวียร์'!$D$13</f>
@@ -6148,10 +6368,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="32" t="s">
-        <v>446</v>
+        <v>465</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>447</v>
+        <v>466</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="6" t="s">
@@ -6162,7 +6382,7 @@
         <v>0.458178826795053</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>448</v>
+        <v>467</v>
       </c>
       <c r="H10" s="12" t="n">
         <f aca="false">('3 ขนาดบ่อ'!$E$13-'3 ขนาดบ่อ'!$E$10)/2</f>
@@ -6175,10 +6395,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="32" t="s">
-        <v>449</v>
+        <v>468</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>348</v>
+        <v>367</v>
       </c>
       <c r="D11" s="6"/>
       <c r="E11" s="6" t="s">
@@ -6189,7 +6409,7 @@
         <v>0.416526206177321</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>450</v>
+        <v>469</v>
       </c>
       <c r="H11" s="12" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8</f>
@@ -6202,10 +6422,10 @@
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="32" t="s">
-        <v>451</v>
+        <v>470</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>452</v>
+        <v>471</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6" t="s">
@@ -6216,22 +6436,22 @@
         <v>0.208263103088661</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>453</v>
+        <v>472</v>
       </c>
       <c r="H12" s="12" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$7</f>
         <v>0.209665688762588</v>
       </c>
       <c r="I12" s="17" t="s">
-        <v>454</v>
+        <v>473</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="32" t="s">
-        <v>455</v>
+        <v>474</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>456</v>
+        <v>475</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="6"/>
@@ -6248,10 +6468,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="32" t="s">
-        <v>457</v>
+        <v>476</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>458</v>
+        <v>477</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
@@ -6268,10 +6488,10 @@
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="32" t="s">
-        <v>459</v>
+        <v>478</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>460</v>
+        <v>479</v>
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="6" t="s">
@@ -6282,7 +6502,7 @@
         <v>0.624789309265982</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>461</v>
+        <v>480</v>
       </c>
       <c r="H15" s="12" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$15</f>
@@ -6295,10 +6515,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="32" t="s">
-        <v>462</v>
+        <v>481</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>463</v>
+        <v>482</v>
       </c>
       <c r="D16" s="6"/>
       <c r="E16" s="6" t="s">
@@ -6309,7 +6529,7 @@
         <v>0.249915723706393</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>464</v>
+        <v>483</v>
       </c>
       <c r="H16" s="12" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$9</f>
@@ -6322,10 +6542,10 @@
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="32" t="s">
-        <v>465</v>
+        <v>484</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>313</v>
+        <v>332</v>
       </c>
       <c r="D17" s="6"/>
       <c r="E17" s="6" t="s">
@@ -6336,7 +6556,7 @@
         <v>1.41618910100289</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>466</v>
+        <v>485</v>
       </c>
       <c r="H17" s="12" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$13</f>
@@ -6349,7 +6569,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="4" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5"/>
@@ -6361,17 +6581,17 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="22" t="s">
-        <v>467</v>
+        <v>486</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="22" t="s">
-        <v>468</v>
+        <v>487</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="22" t="s">
-        <v>469</v>
+        <v>488</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add compartment 1 HRT sheet with options A/B and sizing table
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXLmoKkgGBxM2QbbegGKn7
</commit_message>
<xml_diff>
--- a/weir_design.xlsx
+++ b/weir_design.xlsx
@@ -16,6 +16,7 @@
     <sheet name="6 ตาราง H-Q" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="7 แบบพับ" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="8 เทียบวิธี มข." sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="9 HRT ช่อง 1" sheetId="9" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="489">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="708" uniqueCount="537">
   <si>
     <t xml:space="preserve">1) ข้อมูลออกแบบ — บ่อ 3 ช่อง: ปั๊มจุ่ม | โชว์น้ำใส | V-notch 90°</t>
   </si>
@@ -1515,13 +1516,157 @@
   </si>
   <si>
     <t xml:space="preserve">• สูตร USBR 1.36H^2.48 ให้ Q สูงกว่าสูตรกรมฯ 1.38H^2.5 ประมาณ 2% ในช่วง H 0.15–0.21 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9) ระยะเวลากักน้ำ (HRT) ช่อง 1 — เป้าหมาย 15 นาที</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HRT = ปริมาตรน้ำช่อง 1 ÷ น้ำเข้า  |  ระดับน้ำช่อง 1 ถูกพื้นยกช่อง 2 กำหนด จึงเพิ่มปริมาตรด้วยการลดพื้นช่อง 1 และขยายขนาด</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ข้อมูล</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HRT ที่ต้องการ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">นาที</t>
+  </si>
+  <si>
+    <t xml:space="preserve">หัวหน้ากำหนด</t>
+  </si>
+  <si>
+    <t xml:space="preserve">น้ำเข้าที่ใช้คิด HRT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ค่าเฉลี่ย (แก้เป็น 100 ได้ถ้าคิดที่ค่าสูงสุด)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ปริมาตรปั๊มจุ่ม + ท่อจุ่ม (หัก)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">m³</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ปั๊ม 0.40 × 0.40 × 0.55</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ระดับน้ำช่อง 1 (ที่ Q นี้)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">พื้นยก + ชั้นน้ำ + การสูญเสีย (ที่ Qavg)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ปริมาตรน้ำที่ต้องการ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q × HRT + ส่วนที่ปั๊มกินที่</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HRT แบบเดิม (ช่อง 1 ยาว 1.60 พื้น ±0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ก่อนแก้</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ทางเลือก</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ทางเลือก A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ทางเลือก B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ระดับพื้นช่อง 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">เลือก (ช่องเหลือง)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ความกว้างช่อง 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">เลือก (B = ความกว้างบ่อ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">น้ำลึก</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ระดับน้ำ − พื้น</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ความยาวช่อง 1 ขั้นต่ำ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ปริมาตร ÷ (กว้าง × ลึก)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ความยาวช่อง 1 ที่ใช้</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ปัดขึ้นทีละ 0.05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ปริมาตรน้ำจริง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HRT ที่ได้</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ตรวจ HRT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HRT ที่น้ำเข้าสูงสุด</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ข้อมูลประกอบ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ปั๊ม recycle เดินต่อได้เมื่อน้ำเข้าหยุด</t>
+  </si>
+  <si>
+    <t xml:space="preserve">จากระดับน้ำลงถึง STOP (พื้น + 0.60)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ความสูงผนังช่อง 1 (จากพื้นช่อง 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">สันกำแพง − พื้น</t>
+  </si>
+  <si>
+    <t xml:space="preserve">บ่อยาวภายนอก</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ช่อง 1 + ช่อง 2 + ช่อง 3 + ผนัง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">กว้างภายนอก (ช่อง 1 / ช่อง 2–3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ตารางเลือกขนาด: ความยาวช่อง 1 ที่ต้องใช้ (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">พื้นช่อง 1  \  กว้าง (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">น้ำลึก (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• ระดับน้ำช่อง 1 ถูกพื้นยกช่อง 2 กำหนดไว้ (~+0.95) จึงเพิ่มปริมาตรได้ทางเดียวคือขุดพื้นช่อง 1 ให้ลึกขึ้นหรือขยายขนาด</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• HRT นานขึ้น ตะกอนจะตกที่พื้นช่อง 1 มากขึ้น — ทำพื้นลาดเข้าหาปั๊ม 1:10 และเตรียมทางดูดตะกอน</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• ผนังช่อง 1 ที่ลึกขึ้นรับแรงดันดิน/น้ำมากขึ้น — ให้วิศวกรโยธาตรวจความหนาและเหล็กเสริม</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="12">
+  <numFmts count="15">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="0"/>
@@ -1534,6 +1679,9 @@
     <numFmt numFmtId="173" formatCode="\+0.000;\-0.000;\±0.000"/>
     <numFmt numFmtId="174" formatCode="\+0.0%;\-0.0%;0.0%"/>
     <numFmt numFmtId="175" formatCode="0%"/>
+    <numFmt numFmtId="176" formatCode="\+0.000"/>
+    <numFmt numFmtId="177" formatCode="\+0.00;\-0.00"/>
+    <numFmt numFmtId="178" formatCode="\+0.00;\-0.00;\±0.00"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -1723,7 +1871,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="37">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1854,6 +2002,22 @@
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="177" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="178" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -6603,4 +6767,600 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="B1:G38"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="30"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B1" s="1" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B4" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="6" t="s">
+        <v>492</v>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>493</v>
+      </c>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="6" t="s">
+        <v>495</v>
+      </c>
+      <c r="C6" s="33" t="n">
+        <f aca="false">'1 ข้อมูล'!$C$10</f>
+        <v>62.7916666666667</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="6" t="s">
+        <v>497</v>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="6" t="s">
+        <v>500</v>
+      </c>
+      <c r="C8" s="34" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$47+'4 ช่องโชว์น้ำ'!$F$6/100+1.5*'4 ช่องโชว์น้ำ'!$G$6^2/(2*'1 ข้อมูล'!$C$49)</f>
+        <v>0.953319742642753</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="6" t="s">
+        <v>502</v>
+      </c>
+      <c r="C9" s="27" t="n">
+        <f aca="false">C6*C5/60+C7</f>
+        <v>15.7879166666667</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="6" t="s">
+        <v>504</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <f aca="false">('3 ขนาดบ่อ'!$E$57*'3 ขนาดบ่อ'!$E$13*C8-C7)/C6*60</f>
+        <v>2.10024753190004</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>493</v>
+      </c>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="4" t="s">
+        <v>506</v>
+      </c>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>507</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="6" t="s">
+        <v>509</v>
+      </c>
+      <c r="C14" s="35" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D14" s="35" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="6" t="s">
+        <v>511</v>
+      </c>
+      <c r="C15" s="10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D15" s="10" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$13</f>
+        <v>1.5</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F15" s="6"/>
+      <c r="G15" s="6" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="6" t="s">
+        <v>513</v>
+      </c>
+      <c r="C16" s="12" t="n">
+        <f aca="false">$C$8-C14</f>
+        <v>1.95331974264275</v>
+      </c>
+      <c r="D16" s="12" t="n">
+        <f aca="false">$C$8-D14</f>
+        <v>2.45331974264275</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="6" t="s">
+        <v>515</v>
+      </c>
+      <c r="C17" s="12" t="n">
+        <f aca="false">$C$9/(C15*C16)</f>
+        <v>3.23304297233106</v>
+      </c>
+      <c r="D17" s="12" t="n">
+        <f aca="false">$C$9/(D15*D16)</f>
+        <v>4.29021851283021</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="C18" s="27" t="n">
+        <f aca="false">CEILING(ROUND(C17,4),'1 ข้อมูล'!$C$13)</f>
+        <v>3.25</v>
+      </c>
+      <c r="D18" s="27" t="n">
+        <f aca="false">CEILING(ROUND(D17,4),'1 ข้อมูล'!$C$13)</f>
+        <v>4.3</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F18" s="6"/>
+      <c r="G18" s="6" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="6" t="s">
+        <v>519</v>
+      </c>
+      <c r="C19" s="9" t="n">
+        <f aca="false">C18*C15*C16-$C$7</f>
+        <v>15.7807229089724</v>
+      </c>
+      <c r="D19" s="9" t="n">
+        <f aca="false">D18*D15*D16-$C$7</f>
+        <v>15.7339123400458</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="6" t="s">
+        <v>520</v>
+      </c>
+      <c r="C20" s="19" t="n">
+        <f aca="false">C19/$C$6*60</f>
+        <v>15.079124743809</v>
+      </c>
+      <c r="D20" s="19" t="n">
+        <f aca="false">D19/$C$6*60</f>
+        <v>15.0343953348811</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>493</v>
+      </c>
+      <c r="F20" s="6"/>
+      <c r="G20" s="6"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="6" t="s">
+        <v>521</v>
+      </c>
+      <c r="C21" s="17" t="str">
+        <f aca="false">IF(C20&gt;=$C$5,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="D21" s="17" t="str">
+        <f aca="false">IF(D20&gt;=$C$5,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <v>ผ่าน ✔</v>
+      </c>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="6"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="6" t="s">
+        <v>522</v>
+      </c>
+      <c r="C22" s="9" t="n">
+        <f aca="false">C19/'1 ข้อมูล'!$C$8*60</f>
+        <v>9.46843374538342</v>
+      </c>
+      <c r="D22" s="9" t="n">
+        <f aca="false">D19/'1 ข้อมูล'!$C$8*60</f>
+        <v>9.44034740402745</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>493</v>
+      </c>
+      <c r="F22" s="6"/>
+      <c r="G22" s="6" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="C23" s="15" t="n">
+        <f aca="false">C18*C15*($C$8-(C14+0.6))/'1 ข้อมูล'!$C$9*60</f>
+        <v>65.9743374538342</v>
+      </c>
+      <c r="D23" s="15" t="n">
+        <f aca="false">D18*D15*($C$8-(D14+0.6))/'1 ข้อมูล'!$C$9*60</f>
+        <v>71.7234740402745</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>493</v>
+      </c>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="6" t="s">
+        <v>526</v>
+      </c>
+      <c r="C24" s="12" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$62-C14</f>
+        <v>2.2</v>
+      </c>
+      <c r="D24" s="12" t="n">
+        <f aca="false">'3 ขนาดบ่อ'!$E$62-D14</f>
+        <v>2.7</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F24" s="6"/>
+      <c r="G24" s="6" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="6" t="s">
+        <v>528</v>
+      </c>
+      <c r="C25" s="27" t="n">
+        <f aca="false">C18+'3 ขนาดบ่อ'!$E$49+'3 ขนาดบ่อ'!$E$96+2*'1 ข้อมูล'!$C$44</f>
+        <v>8.4</v>
+      </c>
+      <c r="D25" s="27" t="n">
+        <f aca="false">D18+'3 ขนาดบ่อ'!$E$49+'3 ขนาดบ่อ'!$E$96+2*'1 ข้อมูล'!$C$44</f>
+        <v>9.45</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F25" s="6"/>
+      <c r="G25" s="6" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="6" t="s">
+        <v>530</v>
+      </c>
+      <c r="C26" s="6" t="str">
+        <f aca="false">TEXT(C15+2*'1 ข้อมูล'!$C$44,"0.00")&amp;" / "&amp;TEXT('3 ขนาดบ่อ'!$E$13+2*'1 ข้อมูล'!$C$44,"0.00")</f>
+        <v>2.90 / 1.90</v>
+      </c>
+      <c r="D26" s="6" t="str">
+        <f aca="false">TEXT(D15+2*'1 ข้อมูล'!$C$44,"0.00")&amp;" / "&amp;TEXT('3 ขนาดบ่อ'!$E$13+2*'1 ข้อมูล'!$C$44,"0.00")</f>
+        <v>1.90 / 1.90</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F26" s="6"/>
+      <c r="G26" s="6"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="4" t="s">
+        <v>531</v>
+      </c>
+      <c r="C28" s="5"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="5"/>
+      <c r="G28" s="5"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="3" t="s">
+        <v>532</v>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F29" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G29" s="3" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="12" t="n">
+        <f aca="false">$C$9/(C$29*($C$8-$B30))</f>
+        <v>11.0406585607889</v>
+      </c>
+      <c r="D30" s="12" t="n">
+        <f aca="false">$C$9/(D$29*($C$8-$B30))</f>
+        <v>8.28049392059167</v>
+      </c>
+      <c r="E30" s="12" t="n">
+        <f aca="false">$C$9/(E$29*($C$8-$B30))</f>
+        <v>6.62439513647334</v>
+      </c>
+      <c r="F30" s="12" t="n">
+        <f aca="false">$C$9/(F$29*($C$8-$B30))</f>
+        <v>5.52032928039445</v>
+      </c>
+      <c r="G30" s="12" t="n">
+        <f aca="false">$C$8-B30</f>
+        <v>0.953319742642753</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="36" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="C31" s="12" t="n">
+        <f aca="false">$C$9/(C$29*($C$8-$B31))</f>
+        <v>7.2422313335112</v>
+      </c>
+      <c r="D31" s="12" t="n">
+        <f aca="false">$C$9/(D$29*($C$8-$B31))</f>
+        <v>5.4316735001334</v>
+      </c>
+      <c r="E31" s="12" t="n">
+        <f aca="false">$C$9/(E$29*($C$8-$B31))</f>
+        <v>4.34533880010672</v>
+      </c>
+      <c r="F31" s="12" t="n">
+        <f aca="false">$C$9/(F$29*($C$8-$B31))</f>
+        <v>3.6211156667556</v>
+      </c>
+      <c r="G31" s="12" t="n">
+        <f aca="false">$C$8-B31</f>
+        <v>1.45331974264275</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="36" t="n">
+        <v>-1</v>
+      </c>
+      <c r="C32" s="12" t="n">
+        <f aca="false">$C$9/(C$29*($C$8-$B32))</f>
+        <v>5.3884049538851</v>
+      </c>
+      <c r="D32" s="12" t="n">
+        <f aca="false">$C$9/(D$29*($C$8-$B32))</f>
+        <v>4.04130371541382</v>
+      </c>
+      <c r="E32" s="12" t="n">
+        <f aca="false">$C$9/(E$29*($C$8-$B32))</f>
+        <v>3.23304297233106</v>
+      </c>
+      <c r="F32" s="12" t="n">
+        <f aca="false">$C$9/(F$29*($C$8-$B32))</f>
+        <v>2.69420247694255</v>
+      </c>
+      <c r="G32" s="12" t="n">
+        <f aca="false">$C$8-B32</f>
+        <v>1.95331974264275</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="36" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="C33" s="12" t="n">
+        <f aca="false">$C$9/(C$29*($C$8-$B33))</f>
+        <v>4.29021851283021</v>
+      </c>
+      <c r="D33" s="12" t="n">
+        <f aca="false">$C$9/(D$29*($C$8-$B33))</f>
+        <v>3.21766388462266</v>
+      </c>
+      <c r="E33" s="12" t="n">
+        <f aca="false">$C$9/(E$29*($C$8-$B33))</f>
+        <v>2.57413110769812</v>
+      </c>
+      <c r="F33" s="12" t="n">
+        <f aca="false">$C$9/(F$29*($C$8-$B33))</f>
+        <v>2.1451092564151</v>
+      </c>
+      <c r="G33" s="12" t="n">
+        <f aca="false">$C$8-B33</f>
+        <v>2.45331974264275</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="36" t="n">
+        <v>-2</v>
+      </c>
+      <c r="C34" s="12" t="n">
+        <f aca="false">$C$9/(C$29*($C$8-$B34))</f>
+        <v>3.56388020768768</v>
+      </c>
+      <c r="D34" s="12" t="n">
+        <f aca="false">$C$9/(D$29*($C$8-$B34))</f>
+        <v>2.67291015576576</v>
+      </c>
+      <c r="E34" s="12" t="n">
+        <f aca="false">$C$9/(E$29*($C$8-$B34))</f>
+        <v>2.13832812461261</v>
+      </c>
+      <c r="F34" s="12" t="n">
+        <f aca="false">$C$9/(F$29*($C$8-$B34))</f>
+        <v>1.78194010384384</v>
+      </c>
+      <c r="G34" s="12" t="n">
+        <f aca="false">$C$8-B34</f>
+        <v>2.95331974264275</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B36" s="22" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B37" s="22" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B38" s="22" t="s">
+        <v>536</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Make compartment 3 baffle and sill RC 0.10 m as specified
Tank external length 8.60 m. Workbook, drawings and animation updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXLmoKkgGBxM2QbbegGKn7
</commit_message>
<xml_diff>
--- a/weir_design.xlsx
+++ b/weir_design.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="773" uniqueCount="579">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="776" uniqueCount="582">
   <si>
     <t xml:space="preserve">1) ข้อมูลออกแบบ — บ่อ 3 ช่อง: ปั๊มจุ่ม | โชว์น้ำใส | V-notch 90°</t>
   </si>
@@ -208,6 +208,12 @@
   </si>
   <si>
     <t xml:space="preserve">ปั๊ม 0.40 × 0.40 × 0.55</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ผนังลอดใต้ / สันล้น ช่อง 3 หนา (คสล.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">หล่อพร้อมบ่อ</t>
   </si>
   <si>
     <t xml:space="preserve">ความเร็วลอยตัวฟองอากาศ</t>
@@ -672,7 +678,7 @@
     <t xml:space="preserve">ม่านน้ำพุ่งไกล + เผื่อ 0.20</t>
   </si>
   <si>
-    <t xml:space="preserve">ค. โซนรับน้ำตก + ผนังลอดใต้ + สันล้น ช่อง 3 (แผ่น SS 6 mm อยู่ในโซนรับน้ำตก ไม่ยืดบ่อ)</t>
+    <t xml:space="preserve">ค. โซนรับน้ำตก + ผนังลอดใต้ + สันล้น ช่อง 3 (คสล. หนา 0.10)</t>
   </si>
   <si>
     <t xml:space="preserve">ความลึกน้ำช่อง 3 สูงสุด</t>
@@ -1134,7 +1140,7 @@
     <t xml:space="preserve">ความยาวช่อง 3</t>
   </si>
   <si>
-    <t xml:space="preserve">รับน้ำตก + ช่วงตรง + กำแพงเวียร์ + ท้ายเวียร์</t>
+    <t xml:space="preserve">รับน้ำตก 0.30 + ① 0.10 + ห่าง 0.20 + ② 0.10 + ช่วงตรง + กำแพงเวียร์ + ท้ายเวียร์</t>
   </si>
   <si>
     <t xml:space="preserve">ความยาวภายใน</t>
@@ -1381,6 +1387,9 @@
   </si>
   <si>
     <t xml:space="preserve">แถว 2: รวม</t>
+  </si>
+  <si>
+    <t xml:space="preserve">รับน้ำตก + ช่วงตรง + กำแพงเวียร์ + ท้ายเวียร์</t>
   </si>
   <si>
     <t xml:space="preserve">ความยาวภายในบ่อ</t>
@@ -2402,7 +2411,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:E67"/>
+  <dimension ref="B1:E68"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -2797,7 +2806,7 @@
         <v>0.1</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>61</v>
@@ -2808,10 +2817,10 @@
         <v>62</v>
       </c>
       <c r="C33" s="10" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="E33" s="6" t="s">
         <v>63</v>
@@ -2822,7 +2831,7 @@
         <v>64</v>
       </c>
       <c r="C34" s="10" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="D34" s="6" t="s">
         <v>19</v>
@@ -2841,21 +2850,21 @@
       <c r="D35" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E35" s="6"/>
+      <c r="E35" s="6" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C36" s="10" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E36" s="6" t="s">
-        <v>68</v>
-      </c>
+      <c r="E36" s="6"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="6" t="s">
@@ -2867,11 +2876,13 @@
       <c r="D37" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E37" s="6"/>
+      <c r="E37" s="6" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C38" s="10" t="n">
         <v>0.1</v>
@@ -2879,9 +2890,7 @@
       <c r="D38" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E38" s="6" t="s">
-        <v>71</v>
-      </c>
+      <c r="E38" s="6"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="6" t="s">
@@ -2901,34 +2910,34 @@
       <c r="B40" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="C40" s="11" t="n">
-        <v>0.006</v>
+      <c r="C40" s="10" t="n">
+        <v>0.1</v>
       </c>
       <c r="D40" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E40" s="6"/>
+      <c r="E40" s="6" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="C41" s="10" t="n">
-        <v>0.3</v>
+        <v>76</v>
+      </c>
+      <c r="C41" s="11" t="n">
+        <v>0.006</v>
       </c>
       <c r="D41" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E41" s="6" t="s">
-        <v>76</v>
-      </c>
+      <c r="E41" s="6"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="6" t="s">
         <v>77</v>
       </c>
       <c r="C42" s="10" t="n">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="D42" s="6" t="s">
         <v>19</v>
@@ -2942,7 +2951,7 @@
         <v>79</v>
       </c>
       <c r="C43" s="10" t="n">
-        <v>0.25</v>
+        <v>0.15</v>
       </c>
       <c r="D43" s="6" t="s">
         <v>19</v>
@@ -2956,7 +2965,7 @@
         <v>81</v>
       </c>
       <c r="C44" s="10" t="n">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="D44" s="6" t="s">
         <v>19</v>
@@ -2970,7 +2979,7 @@
         <v>83</v>
       </c>
       <c r="C45" s="10" t="n">
-        <v>1.1</v>
+        <v>0.2</v>
       </c>
       <c r="D45" s="6" t="s">
         <v>19</v>
@@ -2984,7 +2993,7 @@
         <v>85</v>
       </c>
       <c r="C46" s="10" t="n">
-        <v>0.05</v>
+        <v>1.1</v>
       </c>
       <c r="D46" s="6" t="s">
         <v>19</v>
@@ -2998,26 +3007,26 @@
         <v>87</v>
       </c>
       <c r="C47" s="10" t="n">
-        <v>1.25</v>
+        <v>0.05</v>
       </c>
       <c r="D47" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E47" s="6"/>
+      <c r="E47" s="6" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C48" s="10" t="n">
-        <v>0.2</v>
+        <v>1.25</v>
       </c>
       <c r="D48" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E48" s="6" t="s">
-        <v>89</v>
-      </c>
+      <c r="E48" s="6"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="6" t="s">
@@ -3029,41 +3038,43 @@
       <c r="D49" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E49" s="6"/>
+      <c r="E49" s="6" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C50" s="10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D50" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E50" s="6"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B51" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C51" s="10" t="n">
         <v>0.05</v>
       </c>
-      <c r="D50" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E50" s="6" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B52" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="C52" s="5"/>
-      <c r="D52" s="5"/>
-      <c r="E52" s="5"/>
+      <c r="D51" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E51" s="6" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="C53" s="13" t="n">
-        <v>9.81</v>
-      </c>
-      <c r="D53" s="6" t="s">
+      <c r="B53" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="E53" s="6"/>
+      <c r="C53" s="5"/>
+      <c r="D53" s="5"/>
+      <c r="E53" s="5"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="6" t="s">
@@ -3081,25 +3092,23 @@
       <c r="B55" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="C55" s="14" t="n">
-        <v>1.38</v>
+      <c r="C55" s="13" t="n">
+        <v>9.81</v>
       </c>
       <c r="D55" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="E55" s="6" t="s">
-        <v>100</v>
-      </c>
+      <c r="E55" s="6"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C56" s="14" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="D56" s="6" t="s">
         <v>101</v>
-      </c>
-      <c r="C56" s="14" t="n">
-        <v>0.578</v>
-      </c>
-      <c r="D56" s="6" t="s">
-        <v>99</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>102</v>
@@ -3109,28 +3118,28 @@
       <c r="B57" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="C57" s="15" t="n">
-        <v>0.00085</v>
+      <c r="C57" s="14" t="n">
+        <v>0.578</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>19</v>
+        <v>101</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="C58" s="15" t="n">
+        <v>0.00085</v>
+      </c>
+      <c r="D58" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E58" s="6" t="s">
         <v>104</v>
-      </c>
-      <c r="C58" s="13" t="n">
-        <v>1.84</v>
-      </c>
-      <c r="D58" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="E58" s="6" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3138,10 +3147,10 @@
         <v>106</v>
       </c>
       <c r="C59" s="13" t="n">
-        <v>0.6</v>
+        <v>1.84</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E59" s="6" t="s">
         <v>107</v>
@@ -3151,80 +3160,94 @@
       <c r="B60" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="C60" s="16" t="n">
-        <v>205</v>
+      <c r="C60" s="13" t="n">
+        <v>0.6</v>
       </c>
       <c r="D60" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="E60" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="E60" s="6"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="6" t="s">
         <v>110</v>
       </c>
       <c r="C61" s="16" t="n">
-        <v>400</v>
+        <v>205</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E61" s="6"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="C62" s="16" t="n">
+        <v>400</v>
+      </c>
+      <c r="D62" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="C62" s="9" t="n">
+      <c r="E62" s="6"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B63" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="C63" s="9" t="n">
         <v>1.7</v>
       </c>
-      <c r="D62" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="E62" s="6"/>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B64" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="C64" s="5"/>
-      <c r="D64" s="5"/>
-      <c r="E64" s="5"/>
+      <c r="D63" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="E63" s="6"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B65" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="C65" s="17" t="s">
+      <c r="B65" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="D65" s="6"/>
-      <c r="E65" s="6" t="s">
-        <v>115</v>
-      </c>
+      <c r="C65" s="5"/>
+      <c r="D65" s="5"/>
+      <c r="E65" s="5"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="C66" s="17" t="s">
         <v>116</v>
-      </c>
-      <c r="C66" s="18" t="s">
-        <v>117</v>
       </c>
       <c r="D66" s="6"/>
       <c r="E66" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C67" s="18" t="s">
         <v>119</v>
-      </c>
-      <c r="C67" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="D67" s="6"/>
       <c r="E67" s="6" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B68" s="6" t="s">
         <v>121</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="D68" s="6"/>
+      <c r="E68" s="6" t="s">
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -3258,17 +3281,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="4" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="5"/>
@@ -3279,17 +3302,17 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C5" s="14" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$55</f>
+        <f aca="false">'1 ข้อมูล'!$C$56</f>
         <v>1.38</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
@@ -3297,17 +3320,17 @@
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C6" s="19" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$56*(8/15)*SQRT(2*'1 ข้อมูล'!$C$53)</f>
+        <f aca="false">'1 ข้อมูล'!$C$57*(8/15)*SQRT(2*'1 ข้อมูล'!$C$54)</f>
         <v>1.36545083661038</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
@@ -3315,7 +3338,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="4" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
@@ -3326,30 +3349,30 @@
     </row>
     <row r="9" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C10" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$7-'1 ข้อมูล'!$C$9</f>
@@ -3364,7 +3387,7 @@
         <v>14.532869095236</v>
       </c>
       <c r="F10" s="9" t="n">
-        <f aca="false">((D10/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$57)*100</f>
+        <f aca="false">((D10/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$58)*100</f>
         <v>14.5096125168743</v>
       </c>
       <c r="G10" s="21" t="n">
@@ -3375,7 +3398,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C11" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$10-'1 ข้อมูล'!$C$9</f>
@@ -3390,7 +3413,7 @@
         <v>16.2387843483091</v>
       </c>
       <c r="F11" s="9" t="n">
-        <f aca="false">((D11/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$57)*100</f>
+        <f aca="false">((D11/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$58)*100</f>
         <v>16.2227754127948</v>
       </c>
       <c r="G11" s="21" t="n">
@@ -3398,12 +3421,12 @@
         <v>0.0160089355143072</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C12" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8-'1 ข้อมูล'!$C$9</f>
@@ -3418,7 +3441,7 @@
         <v>20.1013103538681</v>
       </c>
       <c r="F12" s="9" t="n">
-        <f aca="false">((D12/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$57)*100</f>
+        <f aca="false">((D12/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$58)*100</f>
         <v>20.1017115002301</v>
       </c>
       <c r="G12" s="21" t="n">
@@ -3429,7 +3452,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="22" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C13" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8</f>
@@ -3444,7 +3467,7 @@
         <v>20.9665688762588</v>
       </c>
       <c r="F13" s="9" t="n">
-        <f aca="false">((D13/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$57)*100</f>
+        <f aca="false">((D13/'2 เวียร์'!$C$6)^0.4-'1 ข้อมูล'!$C$58)*100</f>
         <v>20.9706461048468</v>
       </c>
       <c r="G13" s="21" t="n">
@@ -3452,22 +3475,22 @@
         <v>-0.00407722858800952</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="23" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="23" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="23" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>
@@ -3499,12 +3522,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3512,24 +3535,24 @@
         <v>2</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>4</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="4" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -3539,10 +3562,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D7" s="14"/>
       <c r="E7" s="24" t="n">
@@ -3553,15 +3576,15 @@
         <v>19</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D8" s="14" t="n">
         <f aca="false">MAX(0.45,'3 ขนาดบ่อ'!$E$7/0.4)+'1 ข้อมูล'!$C$14</f>
@@ -3575,15 +3598,15 @@
         <v>19</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="6" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D9" s="14" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$7+'1 ข้อมูล'!$C$15</f>
@@ -3597,15 +3620,15 @@
         <v>19</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D10" s="14"/>
       <c r="E10" s="24" t="n">
@@ -3616,15 +3639,15 @@
         <v>19</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D11" s="14"/>
       <c r="E11" s="24" t="n">
@@ -3635,15 +3658,15 @@
         <v>19</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D12" s="14"/>
       <c r="E12" s="24" t="n">
@@ -3654,15 +3677,15 @@
         <v>19</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="6" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D13" s="14" t="n">
         <f aca="false">MAX('3 ขนาดบ่อ'!$E$12,'1 ข้อมูล'!$C$19)</f>
@@ -3676,15 +3699,15 @@
         <v>19</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="6" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D14" s="14" t="n">
         <f aca="false">10*'3 ขนาดบ่อ'!$E$7</f>
@@ -3698,15 +3721,15 @@
         <v>19</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="6" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D15" s="14" t="n">
         <f aca="false">4.5*'3 ขนาดบ่อ'!$E$7</f>
@@ -3720,15 +3743,15 @@
         <v>19</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="D16" s="14" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$7/'3 ขนาดบ่อ'!$E$8</f>
@@ -3743,10 +3766,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D17" s="14" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$7/'3 ขนาดบ่อ'!$E$13</f>
@@ -3761,10 +3784,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="6" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="D18" s="14" t="n">
         <f aca="false">('3 ขนาดบ่อ'!$E$13-'3 ขนาดบ่อ'!$E$10)/2</f>
@@ -3776,34 +3799,34 @@
       </c>
       <c r="F18" s="6"/>
       <c r="G18" s="6" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D19" s="9"/>
       <c r="E19" s="20" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$55*(('3 ขนาดบ่อ'!$E$13-'3 ขนาดบ่อ'!$E$10)/4)^2.5*3600</f>
+        <f aca="false">'1 ข้อมูล'!$C$56*(('3 ขนาดบ่อ'!$E$13-'3 ขนาดบ่อ'!$E$10)/4)^2.5*3600</f>
         <v>119.299296438097</v>
       </c>
       <c r="F19" s="6" t="s">
         <v>11</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="6" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="D20" s="14" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$15/'3 ขนาดบ่อ'!$E$7</f>
@@ -3818,10 +3841,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="6" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D21" s="14" t="n">
         <f aca="false">'2 เวียร์'!$E$10/100</f>
@@ -3833,12 +3856,12 @@
       </c>
       <c r="F21" s="6"/>
       <c r="G21" s="6" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="4" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="5"/>
@@ -3848,14 +3871,14 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="6" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="D24" s="14"/>
       <c r="E24" s="24" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$35/2+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$59*PI()*'1 ข้อมูล'!$C$35^2/4))^2/(2*'1 ข้อมูล'!$C$53)</f>
+        <f aca="false">'1 ข้อมูล'!$C$36/2+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$60*PI()*'1 ข้อมูล'!$C$36^2/4))^2/(2*'1 ข้อมูล'!$C$54)</f>
         <v>0.210686269183871</v>
       </c>
       <c r="F24" s="6" t="s">
@@ -3865,10 +3888,10 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D25" s="14" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8-'3 ขนาดบ่อ'!$E$24</f>
@@ -3880,34 +3903,34 @@
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="6" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="6" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="D26" s="14"/>
       <c r="E26" s="24" t="n">
-        <f aca="false">SQRT(2*'1 ข้อมูล'!$C$53*'3 ขนาดบ่อ'!$E$7)</f>
+        <f aca="false">SQRT(2*'1 ข้อมูล'!$C$54*'3 ขนาดบ่อ'!$E$7)</f>
         <v>2.02821123493634</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>36</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="6" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D27" s="14"/>
       <c r="E27" s="24" t="n">
@@ -3921,32 +3944,32 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="6" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D28" s="14"/>
       <c r="E28" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$26*SQRT(2*'3 ขนาดบ่อ'!$E$27/'1 ข้อมูล'!$C$53)</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$26*SQRT(2*'3 ขนาดบ่อ'!$E$27/'1 ข้อมูล'!$C$54)</f>
         <v>0.708760700266562</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="6" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D29" s="14" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$28+'1 ข้อมูล'!$C$34</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$28+'1 ข้อมูล'!$C$35</f>
         <v>0.908760700266562</v>
       </c>
       <c r="E29" s="24" t="n">
@@ -3960,7 +3983,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="4" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C31" s="5"/>
       <c r="D31" s="5"/>
@@ -3970,10 +3993,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="6" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D32" s="14"/>
       <c r="E32" s="24" t="n">
@@ -3987,10 +4010,10 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="6" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D33" s="14"/>
       <c r="E33" s="24" t="n">
@@ -4004,14 +4027,14 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="6" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D34" s="14"/>
       <c r="E34" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$32/'1 ข้อมูล'!$C$32*'3 ขนาดบ่อ'!$E$33</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$32/'1 ข้อมูล'!$C$33*'3 ขนาดบ่อ'!$E$33</f>
         <v>0.185185185185185</v>
       </c>
       <c r="F34" s="6" t="s">
@@ -4021,13 +4044,13 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="6" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D35" s="14" t="n">
-        <f aca="false">MAX('1 ข้อมูล'!$C$33,'3 ขนาดบ่อ'!$E$34)</f>
+        <f aca="false">MAX('1 ข้อมูล'!$C$34,'3 ขนาดบ่อ'!$E$34)</f>
         <v>0.5</v>
       </c>
       <c r="E35" s="24" t="n">
@@ -4038,15 +4061,15 @@
         <v>19</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="6" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D36" s="14" t="n">
         <f aca="false">'2 เวียร์'!$D$13/('3 ขนาดบ่อ'!$E$13*'1 ข้อมูล'!$C$21)</f>
@@ -4060,15 +4083,15 @@
         <v>19</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="6" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="D37" s="14"/>
       <c r="E37" s="24" t="n">
@@ -4082,10 +4105,10 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="6" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="D38" s="14" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$36+'1 ข้อมูล'!$C$27</f>
@@ -4099,15 +4122,15 @@
         <v>19</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="6" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D39" s="14"/>
       <c r="E39" s="24" t="n">
@@ -4118,12 +4141,12 @@
         <v>19</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="6" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C40" s="6"/>
       <c r="D40" s="14" t="n">
@@ -4136,15 +4159,15 @@
       </c>
       <c r="F40" s="6"/>
       <c r="G40" s="6" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="6" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="D41" s="14"/>
       <c r="E41" s="24" t="n">
@@ -4158,7 +4181,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="6" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C42" s="6"/>
       <c r="D42" s="14" t="n">
@@ -4174,10 +4197,10 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="6" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="D43" s="14" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8+'2 เวียร์'!$E$10/100-'3 ขนาดบ่อ'!$E$38</f>
@@ -4192,7 +4215,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="4" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C45" s="5"/>
       <c r="D45" s="5"/>
@@ -4202,29 +4225,29 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="6" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D46" s="14"/>
       <c r="E46" s="24" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$17+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$58*'3 ขนาดบ่อ'!$E$13))^(2/3)</f>
+        <f aca="false">'1 ข้อมูล'!$C$17+('2 เวียร์'!$D$13/('1 ข้อมูล'!$C$59*'3 ขนาดบ่อ'!$E$13))^(2/3)</f>
         <v>0.0666149917231983</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G46" s="6" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="6" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="D47" s="14" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$32+'1 ข้อมูล'!$C$16-'1 ข้อมูล'!$C$17</f>
@@ -4243,10 +4266,10 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="6" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="D48" s="14" t="n">
         <f aca="false">10*'3 ขนาดบ่อ'!$E$46</f>
@@ -4260,15 +4283,15 @@
         <v>19</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="6" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D49" s="14"/>
       <c r="E49" s="24" t="n">
@@ -4282,7 +4305,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="6" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C50" s="6"/>
       <c r="D50" s="14" t="n">
@@ -4298,7 +4321,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="4" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C52" s="5"/>
       <c r="D52" s="5"/>
@@ -4308,10 +4331,10 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="6" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="D53" s="14" t="n">
         <f aca="false">MAX(0.3,'2 เวียร์'!$D$13/('1 ข้อมูล'!$C$30*'1 ข้อมูล'!$C$21))</f>
@@ -4325,15 +4348,15 @@
         <v>19</v>
       </c>
       <c r="G53" s="6" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="6" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="D54" s="14" t="n">
         <f aca="false">'1 ข้อมูล'!$C$22+2*'1 ข้อมูล'!$C$23</f>
@@ -4350,10 +4373,10 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="6" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="D55" s="14"/>
       <c r="E55" s="24" t="n">
@@ -4367,10 +4390,10 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="6" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D56" s="14" t="n">
         <f aca="false">'1 ข้อมูล'!$C$25+2*'1 ข้อมูล'!$C$26</f>
@@ -4387,10 +4410,10 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="6" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="D57" s="14"/>
       <c r="E57" s="24" t="n">
@@ -4404,33 +4427,33 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="6" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="D58" s="14"/>
       <c r="E58" s="24" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$17+(('1 ข้อมูล'!$C$10-'1 ข้อมูล'!$C$9)/3600/('1 ข้อมูล'!$C$58*'3 ขนาดบ่อ'!$E$13))^(2/3)</f>
+        <f aca="false">'1 ข้อมูล'!$C$17+(('1 ข้อมูล'!$C$10-'1 ข้อมูล'!$C$9)/3600/('1 ข้อมูล'!$C$59*'3 ขนาดบ่อ'!$E$13))^(2/3)</f>
         <v>0.0504487307291521</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="6" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="D59" s="14"/>
       <c r="E59" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$47+'3 ขนาดบ่อ'!$E$58+1.5*(('1 ข้อมูล'!$C$10-'1 ข้อมูล'!$C$9)/3600/('3 ขนาดบ่อ'!$E$13*'3 ขนาดบ่อ'!$E$58))^2/(2*'1 ข้อมูล'!$C$53)</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$47+'3 ขนาดบ่อ'!$E$58+1.5*(('1 ข้อมูล'!$C$10-'1 ข้อมูล'!$C$9)/3600/('3 ขนาดบ่อ'!$E$13*'3 ขนาดบ่อ'!$E$58))^2/(2*'1 ข้อมูล'!$C$54)</f>
         <v>0.953319742642753</v>
       </c>
       <c r="F59" s="6" t="s">
@@ -4440,10 +4463,10 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="6" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="D60" s="14"/>
       <c r="E60" s="24" t="n">
@@ -4457,10 +4480,10 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="6" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="D61" s="14" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$60/('1 ข้อมูล'!$C$30*('3 ขนาดบ่อ'!$E$59-'1 ข้อมูล'!$C$29))</f>
@@ -4477,10 +4500,10 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="6" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D62" s="14"/>
       <c r="E62" s="24" t="n">
@@ -4491,15 +4514,15 @@
         <v>19</v>
       </c>
       <c r="G62" s="6" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="6" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="D63" s="9"/>
       <c r="E63" s="20" t="n">
@@ -4513,7 +4536,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B64" s="6" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C64" s="6"/>
       <c r="D64" s="14" t="n">
@@ -4529,7 +4552,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="6" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C65" s="6"/>
       <c r="D65" s="9"/>
@@ -4541,15 +4564,15 @@
         <v>51</v>
       </c>
       <c r="G65" s="6" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="6" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="D66" s="14"/>
       <c r="E66" s="24" t="n">
@@ -4563,26 +4586,26 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="6" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="D67" s="14"/>
       <c r="E67" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$47+'3 ขนาดบ่อ'!$E$46+1.5*'3 ขนาดบ่อ'!$E$66^2/(2*'1 ข้อมูล'!$C$53)</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$47+'3 ขนาดบ่อ'!$E$46+1.5*'3 ขนาดบ่อ'!$E$66^2/(2*'1 ข้อมูล'!$C$54)</f>
         <v>0.972523267791535</v>
       </c>
       <c r="F67" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G67" s="6" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B69" s="4" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C69" s="5"/>
       <c r="D69" s="5"/>
@@ -4592,10 +4615,10 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B70" s="6" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="D70" s="14" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$67+'1 ข้อมูล'!$C$20</f>
@@ -4609,12 +4632,12 @@
         <v>19</v>
       </c>
       <c r="G70" s="6" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B72" s="4" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C72" s="5"/>
       <c r="D72" s="5"/>
@@ -4624,33 +4647,33 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B73" s="6" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D73" s="14"/>
       <c r="E73" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$8-'1 ข้อมูล'!$C$36</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$8-'1 ข้อมูล'!$C$37</f>
         <v>0.5</v>
       </c>
       <c r="F73" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G73" s="6" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B74" s="6" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D74" s="14"/>
       <c r="E74" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$13+2*'1 ข้อมูล'!$C$39</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$13+2*'1 ข้อมูล'!$C$40</f>
         <v>1.7</v>
       </c>
       <c r="F74" s="6" t="s">
@@ -4660,33 +4683,33 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B75" s="6" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D75" s="14"/>
       <c r="E75" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$73-'1 ข้อมูล'!$C$37</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$73-'1 ข้อมูล'!$C$38</f>
         <v>0.4</v>
       </c>
       <c r="F75" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G75" s="6" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B76" s="6" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D76" s="14"/>
       <c r="E76" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$9+'1 ข้อมูล'!$C$38</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$9+'1 ข้อมูล'!$C$39</f>
         <v>1</v>
       </c>
       <c r="F76" s="6" t="s">
@@ -4696,10 +4719,10 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B77" s="6" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D77" s="14"/>
       <c r="E77" s="24" t="n">
@@ -4713,10 +4736,10 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B78" s="6" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="C78" s="6" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="D78" s="14"/>
       <c r="E78" s="24" t="n">
@@ -4730,63 +4753,63 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B79" s="6" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="D79" s="14"/>
       <c r="E79" s="24" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$54*'3 ขนาดบ่อ'!$E$78^3/6</f>
+        <f aca="false">'1 ข้อมูล'!$C$55*'3 ขนาดบ่อ'!$E$78^3/6</f>
         <v>0.0485508704265308</v>
       </c>
       <c r="F79" s="6" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="G79" s="6" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B80" s="6" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="D80" s="14"/>
       <c r="E80" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$79/('1 ข้อมูล'!$C$40^2/6)/1000</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$79/('1 ข้อมูล'!$C$41^2/6)/1000</f>
         <v>8.09181173775513</v>
       </c>
       <c r="F80" s="6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="G80" s="6"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B81" s="6" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C81" s="6" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="D81" s="14" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$80</f>
         <v>8.09181173775513</v>
       </c>
       <c r="E81" s="18" t="str">
-        <f aca="false">IF(D81&lt;=0.6*'1 ข้อมูล'!$C$60,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <f aca="false">IF(D81&lt;=0.6*'1 ข้อมูล'!$C$61,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
       <c r="F81" s="6"/>
       <c r="G81" s="6" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B83" s="4" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="C83" s="5"/>
       <c r="D83" s="5"/>
@@ -4796,101 +4819,101 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B84" s="6" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="C84" s="6" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="D84" s="14"/>
       <c r="E84" s="24" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$54*'3 ขนาดบ่อ'!$E$70^3/6</f>
+        <f aca="false">'1 ข้อมูล'!$C$55*'3 ขนาดบ่อ'!$E$70^3/6</f>
         <v>2.82528</v>
       </c>
       <c r="F84" s="6" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="G84" s="6" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B85" s="6" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="C85" s="6" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="D85" s="14"/>
       <c r="E85" s="24" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$62*'3 ขนาดบ่อ'!$E$84</f>
+        <f aca="false">'1 ข้อมูล'!$C$63*'3 ขนาดบ่อ'!$E$84</f>
         <v>4.802976</v>
       </c>
       <c r="F85" s="6" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="G85" s="6"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B86" s="6" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="C86" s="6" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="D86" s="14"/>
       <c r="E86" s="24" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$48-'1 ข้อมูล'!$C$50-0.006</f>
+        <f aca="false">'1 ข้อมูล'!$C$49-'1 ข้อมูล'!$C$51-0.006</f>
         <v>0.144</v>
       </c>
       <c r="F86" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G86" s="6" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B87" s="6" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="C87" s="6" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="D87" s="14"/>
       <c r="E87" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$85/(0.9*'1 ข้อมูล'!$C$61*1000*0.9*'3 ขนาดบ่อ'!$E$86)*1000000</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$85/(0.9*'1 ข้อมูล'!$C$62*1000*0.9*'3 ขนาดบ่อ'!$E$86)*1000000</f>
         <v>102.944444444444</v>
       </c>
       <c r="F87" s="6" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="G87" s="6"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B88" s="6" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="C88" s="6" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="D88" s="14"/>
       <c r="E88" s="24" t="n">
-        <f aca="false">0.003*1000*'1 ข้อมูล'!$C$48*1000</f>
+        <f aca="false">0.003*1000*'1 ข้อมูล'!$C$49*1000</f>
         <v>600</v>
       </c>
       <c r="F88" s="6" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="G88" s="6" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B89" s="6" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="C89" s="6" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="D89" s="14"/>
       <c r="E89" s="24" t="n">
@@ -4898,13 +4921,13 @@
         <v>175</v>
       </c>
       <c r="F89" s="6" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="G89" s="6"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B90" s="6" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="C90" s="6"/>
       <c r="D90" s="14" t="n">
@@ -4917,15 +4940,15 @@
       </c>
       <c r="F90" s="6"/>
       <c r="G90" s="6" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B91" s="6" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="C91" s="6" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="D91" s="14"/>
       <c r="E91" s="24" t="n">
@@ -4939,41 +4962,41 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B92" s="6" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="C92" s="6" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="D92" s="14"/>
       <c r="E92" s="24" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$62*'1 ข้อมูล'!$C$54*'3 ขนาดบ่อ'!$E$91^3/6</f>
+        <f aca="false">'1 ข้อมูล'!$C$63*'1 ข้อมูล'!$C$55*'3 ขนาดบ่อ'!$E$91^3/6</f>
         <v>29.596116</v>
       </c>
       <c r="F92" s="6" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="G92" s="6"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B93" s="6" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="C93" s="6" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="D93" s="14"/>
       <c r="E93" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$92/(0.9*'1 ข้อมูล'!$C$61*1000*0.9*'3 ขนาดบ่อ'!$E$86)*1000000</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$92/(0.9*'1 ข้อมูล'!$C$62*1000*0.9*'3 ขนาดบ่อ'!$E$86)*1000000</f>
         <v>634.347479423868</v>
       </c>
       <c r="F93" s="6" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="G93" s="6"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B94" s="6" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C94" s="6"/>
       <c r="D94" s="14"/>
@@ -4982,15 +5005,15 @@
         <v>175</v>
       </c>
       <c r="F94" s="6" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="G94" s="6" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B95" s="6" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="C95" s="6"/>
       <c r="D95" s="14" t="n">
@@ -5003,12 +5026,12 @@
       </c>
       <c r="F95" s="6"/>
       <c r="G95" s="6" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B97" s="4" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="C97" s="5"/>
       <c r="D97" s="5"/>
@@ -5018,56 +5041,56 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B98" s="6" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="C98" s="6" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="D98" s="14"/>
       <c r="E98" s="24" t="n">
-        <f aca="false">ROUND(('1 ข้อมูล'!$C$44+'3 ขนาดบ่อ'!$E$8-'1 ข้อมูล'!$C$43)/2/0.05,0)*0.05</f>
+        <f aca="false">ROUND(('1 ข้อมูล'!$C$45+'3 ขนาดบ่อ'!$E$8-'1 ข้อมูล'!$C$44)/2/0.05,0)*0.05</f>
         <v>0.3</v>
       </c>
       <c r="F98" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G98" s="6" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B99" s="6" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="C99" s="6" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="D99" s="14" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8-'3 ขนาดบ่อ'!$E$98</f>
         <v>0.3</v>
       </c>
       <c r="E99" s="18" t="str">
-        <f aca="false">IF(D99&gt;='1 ข้อมูล'!$C$43-0.0001,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <f aca="false">IF(D99&gt;='1 ข้อมูล'!$C$44-0.0001,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
       <c r="F99" s="6"/>
       <c r="G99" s="6" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B100" s="6" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="C100" s="6" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="D100" s="14" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$98</f>
         <v>0.3</v>
       </c>
       <c r="E100" s="18" t="str">
-        <f aca="false">IF(D100&gt;='1 ข้อมูล'!$C$44-0.0001,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <f aca="false">IF(D100&gt;='1 ข้อมูล'!$C$45-0.0001,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
       <c r="F100" s="6"/>
@@ -5075,14 +5098,14 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B101" s="6" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="C101" s="6" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D101" s="14"/>
       <c r="E101" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$14-'1 ข้อมูล'!$C$41</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$14-'1 ข้อมูล'!$C$42</f>
         <v>1.8</v>
       </c>
       <c r="F101" s="6" t="s">
@@ -5092,10 +5115,10 @@
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B102" s="6" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="C102" s="6" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="D102" s="14" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$101-'3 ขนาดบ่อ'!$E$15</f>
@@ -5107,19 +5130,19 @@
       </c>
       <c r="F102" s="6"/>
       <c r="G102" s="6" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B103" s="6" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="C103" s="6" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="D103" s="14"/>
       <c r="E103" s="24" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$45-'3 ขนาดบ่อ'!$E$32</f>
+        <f aca="false">'1 ข้อมูล'!$C$46-'3 ขนาดบ่อ'!$E$32</f>
         <v>0.290334311237412</v>
       </c>
       <c r="F103" s="6" t="s">
@@ -5129,14 +5152,14 @@
     </row>
     <row r="104" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B104" s="6" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="C104" s="6" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="D104" s="14"/>
       <c r="E104" s="24" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$45-'3 ขนาดบ่อ'!$E$8</f>
+        <f aca="false">'1 ข้อมูล'!$C$46-'3 ขนาดบ่อ'!$E$8</f>
         <v>0.5</v>
       </c>
       <c r="F104" s="6" t="s">
@@ -5146,17 +5169,17 @@
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B105" s="6" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="C105" s="6" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="D105" s="14" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$103</f>
         <v>0.290334311237412</v>
       </c>
       <c r="E105" s="18" t="str">
-        <f aca="false">IF(AND(D105&gt;='1 ข้อมูล'!$C$46,'3 ขนาดบ่อ'!$E$104&lt;='1 ข้อมูล'!$C$47),"ผ่าน ✔","ไม่ผ่าน ✘")</f>
+        <f aca="false">IF(AND(D105&gt;='1 ข้อมูล'!$C$47,'3 ขนาดบ่อ'!$E$104&lt;='1 ข้อมูล'!$C$48),"ผ่าน ✔","ไม่ผ่าน ✘")</f>
         <v>ผ่าน ✔</v>
       </c>
       <c r="F105" s="6"/>
@@ -5164,11 +5187,11 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B106" s="6" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="C106" s="6"/>
       <c r="D106" s="14" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$70-'1 ข้อมูล'!$C$45</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$70-'1 ข้อมูล'!$C$46</f>
         <v>0.1</v>
       </c>
       <c r="E106" s="18" t="str">
@@ -5177,12 +5200,12 @@
       </c>
       <c r="F106" s="6"/>
       <c r="G106" s="6" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B108" s="4" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C108" s="5"/>
       <c r="D108" s="5"/>
@@ -5190,17 +5213,17 @@
       <c r="F108" s="5"/>
       <c r="G108" s="5"/>
     </row>
-    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B109" s="6" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="C109" s="6" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="D109" s="14"/>
       <c r="E109" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$35+'3 ขนาดบ่อ'!$E$14+'1 ข้อมูล'!$C$48+'3 ขนาดบ่อ'!$E$29</f>
-        <v>3.75</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$39+'3 ขนาดบ่อ'!$E$37+2*'1 ข้อมูล'!$C$32+'3 ขนาดบ่อ'!$E$14+'1 ข้อมูล'!$C$49+'3 ขนาดบ่อ'!$E$29</f>
+        <v>3.95</v>
       </c>
       <c r="F109" s="6" t="s">
         <v>19</v>
@@ -5209,15 +5232,15 @@
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B110" s="6" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="C110" s="6" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="D110" s="14"/>
       <c r="E110" s="24" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$62+'3 ขนาดบ่อ'!$E$49+'3 ขนาดบ่อ'!$E$109</f>
-        <v>8</v>
+        <v>8.2</v>
       </c>
       <c r="F110" s="6" t="s">
         <v>19</v>
@@ -5226,10 +5249,10 @@
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B111" s="6" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C111" s="6" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="D111" s="14"/>
       <c r="E111" s="24" t="n">
@@ -5243,7 +5266,7 @@
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B112" s="6" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="C112" s="6"/>
       <c r="D112" s="14"/>
@@ -5258,10 +5281,10 @@
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B113" s="6" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C113" s="6" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="D113" s="14"/>
       <c r="E113" s="24" t="n">
@@ -5275,15 +5298,15 @@
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B114" s="6" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="C114" s="6" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="D114" s="14"/>
       <c r="E114" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$110+2*'1 ข้อมูล'!$C$48</f>
-        <v>8.4</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$110+2*'1 ข้อมูล'!$C$49</f>
+        <v>8.6</v>
       </c>
       <c r="F114" s="6" t="s">
         <v>19</v>
@@ -5292,14 +5315,14 @@
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B115" s="6" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="C115" s="6" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="D115" s="14"/>
       <c r="E115" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$111+2*'1 ข้อมูล'!$C$48</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$111+2*'1 ข้อมูล'!$C$49</f>
         <v>1.9</v>
       </c>
       <c r="F115" s="6" t="s">
@@ -5309,14 +5332,14 @@
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B116" s="6" t="s">
+        <v>378</v>
+      </c>
+      <c r="C116" s="6" t="s">
         <v>376</v>
-      </c>
-      <c r="C116" s="6" t="s">
-        <v>374</v>
       </c>
       <c r="D116" s="14"/>
       <c r="E116" s="24" t="n">
-        <f aca="false">'1 ข้อมูล'!$C$30+2*'1 ข้อมูล'!$C$48</f>
+        <f aca="false">'1 ข้อมูล'!$C$30+2*'1 ข้อมูล'!$C$49</f>
         <v>2.9</v>
       </c>
       <c r="F116" s="6" t="s">
@@ -5326,14 +5349,14 @@
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B117" s="6" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="C117" s="6" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="D117" s="14"/>
       <c r="E117" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$70-'1 ข้อมูล'!$C$29+'1 ข้อมูล'!$C$49</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$70-'1 ข้อมูล'!$C$29+'1 ข้อมูล'!$C$50</f>
         <v>2.4</v>
       </c>
       <c r="F117" s="6" t="s">
@@ -5343,14 +5366,14 @@
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B118" s="6" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="C118" s="6" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="D118" s="14"/>
       <c r="E118" s="24" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$113+'1 ข้อมูล'!$C$49</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$113+'1 ข้อมูล'!$C$50</f>
         <v>1.4</v>
       </c>
       <c r="F118" s="6" t="s">
@@ -5390,43 +5413,43 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="6" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C5" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$7-'1 ข้อมูล'!$C$9</f>
@@ -5437,7 +5460,7 @@
         <v>0.0111111111111111</v>
       </c>
       <c r="E5" s="9" t="n">
-        <f aca="false">(D5/('1 ข้อมูล'!$C$58*'3 ขนาดบ่อ'!$E$13))^(2/3)*100</f>
+        <f aca="false">(D5/('1 ข้อมูล'!$C$59*'3 ขนาดบ่อ'!$E$13))^(2/3)*100</f>
         <v>2.53065109461751</v>
       </c>
       <c r="F5" s="20" t="n">
@@ -5449,7 +5472,7 @@
         <v>0.163495428200321</v>
       </c>
       <c r="H5" s="13" t="n">
-        <f aca="false">G5/SQRT('1 ข้อมูล'!$C$53*F5/100)</f>
+        <f aca="false">G5/SQRT('1 ข้อมูล'!$C$54*F5/100)</f>
         <v>0.24523971352263</v>
       </c>
       <c r="I5" s="18" t="str">
@@ -5459,7 +5482,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C6" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$10-'1 ข้อมูล'!$C$9</f>
@@ -5470,7 +5493,7 @@
         <v>0.0146643518518519</v>
       </c>
       <c r="E6" s="9" t="n">
-        <f aca="false">(D6/('1 ข้อมูล'!$C$58*'3 ขนาดบ่อ'!$E$13))^(2/3)*100</f>
+        <f aca="false">(D6/('1 ข้อมูล'!$C$59*'3 ขนาดบ่อ'!$E$13))^(2/3)*100</f>
         <v>3.04487307291521</v>
       </c>
       <c r="F6" s="20" t="n">
@@ -5482,7 +5505,7 @@
         <v>0.193785540817422</v>
       </c>
       <c r="H6" s="13" t="n">
-        <f aca="false">G6/SQRT('1 ข้อมูล'!$C$53*F6/100)</f>
+        <f aca="false">G6/SQRT('1 ข้อมูล'!$C$54*F6/100)</f>
         <v>0.275462029969398</v>
       </c>
       <c r="I6" s="18" t="str">
@@ -5492,7 +5515,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C7" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8-'1 ข้อมูล'!$C$9</f>
@@ -5503,7 +5526,7 @@
         <v>0.025</v>
       </c>
       <c r="E7" s="9" t="n">
-        <f aca="false">(D7/('1 ข้อมูล'!$C$58*'3 ขนาดบ่อ'!$E$13))^(2/3)*100</f>
+        <f aca="false">(D7/('1 ข้อมูล'!$C$59*'3 ขนาดบ่อ'!$E$13))^(2/3)*100</f>
         <v>4.34530852641276</v>
       </c>
       <c r="F7" s="20" t="n">
@@ -5515,7 +5538,7 @@
         <v>0.262661249603397</v>
       </c>
       <c r="H7" s="13" t="n">
-        <f aca="false">G7/SQRT('1 ข้อมูล'!$C$53*F7/100)</f>
+        <f aca="false">G7/SQRT('1 ข้อมูล'!$C$54*F7/100)</f>
         <v>0.332916354683497</v>
       </c>
       <c r="I7" s="18" t="str">
@@ -5525,7 +5548,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C8" s="9" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8</f>
@@ -5536,7 +5559,7 @@
         <v>0.0277777777777778</v>
       </c>
       <c r="E8" s="9" t="n">
-        <f aca="false">(D8/('1 ข้อมูล'!$C$58*'3 ขนาดบ่อ'!$E$13))^(2/3)*100</f>
+        <f aca="false">(D8/('1 ข้อมูล'!$C$59*'3 ขนาดบ่อ'!$E$13))^(2/3)*100</f>
         <v>4.66149917231983</v>
       </c>
       <c r="F8" s="20" t="n">
@@ -5548,7 +5571,7 @@
         <v>0.277993257065429</v>
       </c>
       <c r="H8" s="13" t="n">
-        <f aca="false">G8/SQRT('1 ข้อมูล'!$C$53*F8/100)</f>
+        <f aca="false">G8/SQRT('1 ข้อมูล'!$C$54*F8/100)</f>
         <v>0.343885424767124</v>
       </c>
       <c r="I8" s="18" t="str">
@@ -5558,17 +5581,17 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="23" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="23" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="23" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
     </row>
   </sheetData>
@@ -5598,196 +5621,196 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>19</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="6" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="C5" s="25" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$70</f>
         <v>1.2</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="C6" s="25" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$67</f>
         <v>0.972523267791535</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="C7" s="25" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$47+'1 ข้อมูล'!$C$17</f>
         <v>0.92</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="C8" s="25" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$47</f>
         <v>0.9</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="6" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="C9" s="25" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$76</f>
         <v>1</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C10" s="25" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8+'3 ขนาดบ่อ'!$E$9</f>
         <v>0.9</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="C11" s="25" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$32</f>
         <v>0.809665688762588</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="C12" s="25" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8</f>
         <v>0.6</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="6" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="C13" s="25" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$73</f>
         <v>0.5</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="6" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="C14" s="25" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$75</f>
         <v>0.4</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="6" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="C15" s="25" t="n">
         <f aca="false">'1 ข้อมูล'!$C$29+'3 ขนาดบ่อ'!$E$53</f>
         <v>-0.7</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="C16" s="25" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$24</f>
         <v>0.210686269183871</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="C17" s="25" t="n">
         <f aca="false">'1 ข้อมูล'!$C$29+0.6</f>
         <v>-0.4</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="6" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="C18" s="25" t="n">
         <f aca="false">'1 ข้อมูล'!$C$29+0.5</f>
         <v>-0.5</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="6" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="C19" s="25" t="n">
         <f aca="false">0</f>
@@ -5797,14 +5820,14 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="6" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="C20" s="25" t="n">
         <f aca="false">'1 ข้อมูล'!$C$29</f>
         <v>-1</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
     </row>
   </sheetData>
@@ -5835,32 +5858,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5872,7 +5895,7 @@
         <v>2.77719642805474</v>
       </c>
       <c r="D5" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B5/100+'1 ข้อมูล'!$C$57)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B5/100+'1 ข้อมูล'!$C$58)^2.5*3600</f>
         <v>2.86619650300861</v>
       </c>
       <c r="E5" s="26" t="n">
@@ -5897,7 +5920,7 @@
         <v>4.38086341517286</v>
       </c>
       <c r="D6" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B6/100+'1 ข้อมูล'!$C$57)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B6/100+'1 ข้อมูล'!$C$58)^2.5*3600</f>
         <v>4.48983131905459</v>
       </c>
       <c r="E6" s="26" t="n">
@@ -5922,7 +5945,7 @@
         <v>6.44060533155076</v>
       </c>
       <c r="D7" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B7/100+'1 ข้อมูล'!$C$57)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B7/100+'1 ข้อมูล'!$C$58)^2.5*3600</f>
         <v>6.56792530595593</v>
       </c>
       <c r="E7" s="26" t="n">
@@ -5947,7 +5970,7 @@
         <v>8.99304061167301</v>
       </c>
       <c r="D8" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B8/100+'1 ข้อมูล'!$C$57)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B8/100+'1 ข้อมูล'!$C$58)^2.5*3600</f>
         <v>9.13647413844802</v>
       </c>
       <c r="E8" s="26" t="n">
@@ -5972,7 +5995,7 @@
         <v>12.07224</v>
       </c>
       <c r="D9" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B9/100+'1 ข้อมูล'!$C$57)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B9/100+'1 ข้อมูล'!$C$58)^2.5*3600</f>
         <v>12.2289986697729</v>
       </c>
       <c r="E9" s="26" t="n">
@@ -5997,7 +6020,7 @@
         <v>15.7101954157165</v>
       </c>
       <c r="D10" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B10/100+'1 ข้อมูล'!$C$57)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B10/100+'1 ข้อมูล'!$C$58)^2.5*3600</f>
         <v>15.8769956216084</v>
       </c>
       <c r="E10" s="26" t="n">
@@ -6022,7 +6045,7 @@
         <v>19.9371602697676</v>
       </c>
       <c r="D11" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B11/100+'1 ข้อมูล'!$C$57)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B11/100+'1 ข้อมูล'!$C$58)^2.5*3600</f>
         <v>20.1102658699656</v>
       </c>
       <c r="E11" s="26" t="n">
@@ -6047,7 +6070,7 @@
         <v>24.7819058265663</v>
       </c>
       <c r="D12" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B12/100+'1 ข้อมูล'!$C$57)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B12/100+'1 ข้อมูล'!$C$58)^2.5*3600</f>
         <v>24.9571624264048</v>
       </c>
       <c r="E12" s="26" t="n">
@@ -6072,7 +6095,7 @@
         <v>30.2719200646936</v>
       </c>
       <c r="D13" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B13/100+'1 ข้อมูล'!$C$57)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B13/100+'1 ข้อมูล'!$C$58)^2.5*3600</f>
         <v>30.4447832233961</v>
       </c>
       <c r="E13" s="26" t="n">
@@ -6097,7 +6120,7 @@
         <v>36.4335656390862</v>
       </c>
       <c r="D14" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B14/100+'1 ข้อมูล'!$C$57)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B14/100+'1 ข้อมูล'!$C$58)^2.5*3600</f>
         <v>36.599124528368</v>
       </c>
       <c r="E14" s="26" t="n">
@@ -6122,7 +6145,7 @@
         <v>43.2922078439065</v>
       </c>
       <c r="D15" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B15/100+'1 ข้อมูล'!$C$57)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B15/100+'1 ข้อมูล'!$C$58)^2.5*3600</f>
         <v>43.4452054104805</v>
       </c>
       <c r="E15" s="26" t="n">
@@ -6147,7 +6170,7 @@
         <v>50.87232</v>
       </c>
       <c r="D16" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B16/100+'1 ข้อมูล'!$C$57)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B16/100+'1 ข้อมูล'!$C$58)^2.5*3600</f>
         <v>51.0071703805085</v>
       </c>
       <c r="E16" s="26" t="n">
@@ -6172,7 +6195,7 @@
         <v>59.1975714819181</v>
       </c>
       <c r="D17" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B17/100+'1 ข้อมูล'!$C$57)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B17/100+'1 ข้อมูล'!$C$58)^2.5*3600</f>
         <v>59.3083752175669</v>
       </c>
       <c r="E17" s="26" t="n">
@@ -6197,7 +6220,7 @@
         <v>68.2909021448919</v>
       </c>
       <c r="D18" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B18/100+'1 ข้อมูล'!$C$57)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B18/100+'1 ข้อมูล'!$C$58)^2.5*3600</f>
         <v>68.3714596053392</v>
       </c>
       <c r="E18" s="26" t="n">
@@ -6222,7 +6245,7 @@
         <v>78.1745859249513</v>
       </c>
       <c r="D19" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B19/100+'1 ข้อมูล'!$C$57)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B19/100+'1 ข้อมูล'!$C$58)^2.5*3600</f>
         <v>78.2184092541632</v>
       </c>
       <c r="E19" s="26" t="n">
@@ -6247,7 +6270,7 @@
         <v>88.8702856977516</v>
       </c>
       <c r="D20" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B20/100+'1 ข้อมูล'!$C$57)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B20/100+'1 ข้อมูล'!$C$58)^2.5*3600</f>
         <v>88.8706095248216</v>
       </c>
       <c r="E20" s="26" t="n">
@@ -6272,7 +6295,7 @@
         <v>100.399100991704</v>
       </c>
       <c r="D21" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B21/100+'1 ข้อมูล'!$C$57)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B21/100+'1 ข้อมูล'!$C$58)^2.5*3600</f>
         <v>100.348892098404</v>
       </c>
       <c r="E21" s="26" t="n">
@@ -6297,7 +6320,7 @@
         <v>112.781609794846</v>
       </c>
       <c r="D22" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B22/100+'1 ข้อมูล'!$C$57)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B22/100+'1 ข้อมูล'!$C$58)^2.5*3600</f>
         <v>112.673575893332</v>
       </c>
       <c r="E22" s="26" t="n">
@@ -6322,7 +6345,7 @@
         <v>126.037905431355</v>
       </c>
       <c r="D23" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B23/100+'1 ข้อมูล'!$C$57)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B23/100+'1 ข้อมูล'!$C$58)^2.5*3600</f>
         <v>125.864503176292</v>
       </c>
       <c r="E23" s="26" t="n">
@@ -6347,7 +6370,7 @@
         <v>140.187629285531</v>
       </c>
       <c r="D24" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B24/100+'1 ข้อมูล'!$C$57)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B24/100+'1 ข้อมูล'!$C$58)^2.5*3600</f>
         <v>139.941071622383</v>
       </c>
       <c r="E24" s="26" t="n">
@@ -6372,7 +6395,7 @@
         <v>155.25</v>
       </c>
       <c r="D25" s="9" t="n">
-        <f aca="false">'2 เวียร์'!$C$6*(B25/100+'1 ข้อมูล'!$C$57)^2.5*3600</f>
+        <f aca="false">'2 เวียร์'!$C$6*(B25/100+'1 ข้อมูล'!$C$58)^2.5*3600</f>
         <v>154.922262933655</v>
       </c>
       <c r="E25" s="26" t="n">
@@ -6416,12 +6439,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6429,7 +6452,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>3</v>
@@ -6438,12 +6461,12 @@
         <v>4</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="4" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -6452,10 +6475,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="D7" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$62</f>
@@ -6468,10 +6491,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="D8" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$49</f>
@@ -6481,15 +6504,15 @@
         <v>19</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="6" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="D9" s="28" t="n">
         <f aca="false">'7 แบบพับ'!$D$7+'7 แบบพับ'!$D$8</f>
@@ -6502,10 +6525,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="D10" s="13" t="n">
         <f aca="false">MAX('7 แบบพับ'!$D$8,'3 ขนาดบ่อ'!$E$35)</f>
@@ -6515,18 +6538,18 @@
         <v>19</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>365</v>
+        <v>446</v>
       </c>
       <c r="D11" s="28" t="n">
-        <f aca="false">'7 แบบพับ'!$D$10+'3 ขนาดบ่อ'!$E$14+'1 ข้อมูล'!$C$48+'3 ขนาดบ่อ'!$E$29</f>
+        <f aca="false">'7 แบบพับ'!$D$10+'3 ขนาดบ่อ'!$E$14+'1 ข้อมูล'!$C$49+'3 ขนาดบ่อ'!$E$29</f>
         <v>4.25</v>
       </c>
       <c r="E11" s="6" t="s">
@@ -6536,10 +6559,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="D12" s="28" t="n">
         <f aca="false">MAX('7 แบบพับ'!$D$9,'7 แบบพับ'!$D$11)</f>
@@ -6552,10 +6575,10 @@
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="6" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="D13" s="13" t="n">
         <f aca="false">'7 แบบพับ'!$D$12-'7 แบบพับ'!$D$9</f>
@@ -6565,18 +6588,18 @@
         <v>19</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="6" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="D14" s="13" t="n">
-        <f aca="false">2*'3 ขนาดบ่อ'!$E$13+'1 ข้อมูล'!$C$48</f>
+        <f aca="false">2*'3 ขนาดบ่อ'!$E$13+'1 ข้อมูล'!$C$49</f>
         <v>3.2</v>
       </c>
       <c r="E14" s="6" t="s">
@@ -6586,7 +6609,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="4" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
@@ -6596,131 +6619,131 @@
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="29"/>
       <c r="C17" s="29" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="D17" s="29" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="E17" s="29" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="F17" s="29"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="6" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="C18" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$114</f>
-        <v>8.4</v>
+        <v>8.6</v>
       </c>
       <c r="D18" s="13" t="n">
-        <f aca="false">'7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$48</f>
+        <f aca="false">'7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$49</f>
         <v>4.65</v>
       </c>
       <c r="E18" s="13" t="n">
-        <f aca="false">'7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$48</f>
+        <f aca="false">'7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$49</f>
         <v>4.65</v>
       </c>
       <c r="F18" s="6"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="6" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="C19" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$115</f>
         <v>1.9</v>
       </c>
       <c r="D19" s="13" t="n">
-        <f aca="false">'7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$48</f>
+        <f aca="false">'7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$49</f>
         <v>3.6</v>
       </c>
       <c r="E19" s="13" t="n">
-        <f aca="false">'7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$48</f>
+        <f aca="false">'7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$49</f>
         <v>3.6</v>
       </c>
       <c r="F19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="6" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="C20" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$114*'3 ขนาดบ่อ'!$E$115</f>
-        <v>15.96</v>
+        <v>16.34</v>
       </c>
       <c r="D20" s="13" t="n">
-        <f aca="false">('7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$48)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$48)</f>
+        <f aca="false">('7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$49)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$49)</f>
         <v>16.74</v>
       </c>
       <c r="E20" s="13" t="n">
-        <f aca="false">('7 แบบพับ'!$D$9+2*'1 ข้อมูล'!$C$48)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$48)+('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$9)*('3 ขนาดบ่อ'!$E$13+2*'1 ข้อมูล'!$C$48)</f>
+        <f aca="false">('7 แบบพับ'!$D$9+2*'1 ข้อมูล'!$C$49)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$49)+('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$9)*('3 ขนาดบ่อ'!$E$13+2*'1 ข้อมูล'!$C$49)</f>
         <v>16.74</v>
       </c>
       <c r="F20" s="6"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="6" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="C21" s="13" t="n">
-        <f aca="false">2*('3 ขนาดบ่อ'!$E$110+'1 ข้อมูล'!$C$48+'3 ขนาดบ่อ'!$E$111+'1 ข้อมูล'!$C$48)*'1 ข้อมูล'!$C$48*'3 ขนาดบ่อ'!$E$70</f>
-        <v>4.752</v>
+        <f aca="false">2*('3 ขนาดบ่อ'!$E$110+'1 ข้อมูล'!$C$49+'3 ขนาดบ่อ'!$E$111+'1 ข้อมูล'!$C$49)*'1 ข้อมูล'!$C$49*'3 ขนาดบ่อ'!$E$70</f>
+        <v>4.848</v>
       </c>
       <c r="D21" s="13" t="n">
-        <f aca="false">2*('7 แบบพับ'!$D$12+'1 ข้อมูล'!$C$48+'7 แบบพับ'!$D$14+'1 ข้อมูล'!$C$48)*'1 ข้อมูล'!$C$48*'3 ขนาดบ่อ'!$E$70</f>
+        <f aca="false">2*('7 แบบพับ'!$D$12+'1 ข้อมูล'!$C$49+'7 แบบพับ'!$D$14+'1 ข้อมูล'!$C$49)*'1 ข้อมูล'!$C$49*'3 ขนาดบ่อ'!$E$70</f>
         <v>3.768</v>
       </c>
       <c r="E21" s="13" t="n">
-        <f aca="false">2*('7 แบบพับ'!$D$12+'1 ข้อมูล'!$C$48+'7 แบบพับ'!$D$14+'1 ข้อมูล'!$C$48)*'1 ข้อมูล'!$C$48*'3 ขนาดบ่อ'!$E$70</f>
+        <f aca="false">2*('7 แบบพับ'!$D$12+'1 ข้อมูล'!$C$49+'7 แบบพับ'!$D$14+'1 ข้อมูล'!$C$49)*'1 ข้อมูล'!$C$49*'3 ขนาดบ่อ'!$E$70</f>
         <v>3.768</v>
       </c>
       <c r="F21" s="6"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="6" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="C22" s="13" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
       <c r="D22" s="13" t="n">
-        <f aca="false">('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$8)*'1 ข้อมูล'!$C$48*'3 ขนาดบ่อ'!$E$70</f>
+        <f aca="false">('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$8)*'1 ข้อมูล'!$C$49*'3 ขนาดบ่อ'!$E$70</f>
         <v>0.78</v>
       </c>
       <c r="E22" s="13" t="n">
-        <f aca="false">'7 แบบพับ'!$D$7*'1 ข้อมูล'!$C$48*'3 ขนาดบ่อ'!$E$70</f>
+        <f aca="false">'7 แบบพับ'!$D$7*'1 ข้อมูล'!$C$49*'3 ขนาดบ่อ'!$E$70</f>
         <v>0.78</v>
       </c>
       <c r="F22" s="6"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="6" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="C23" s="13" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$114*'3 ขนาดบ่อ'!$E$115*'1 ข้อมูล'!$C$49</f>
-        <v>3.192</v>
+        <f aca="false">'3 ขนาดบ่อ'!$E$114*'3 ขนาดบ่อ'!$E$115*'1 ข้อมูล'!$C$50</f>
+        <v>3.268</v>
       </c>
       <c r="D23" s="13" t="n">
-        <f aca="false">('7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$48)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$48)*'1 ข้อมูล'!$C$49</f>
+        <f aca="false">('7 แบบพับ'!$D$12+2*'1 ข้อมูล'!$C$49)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$49)*'1 ข้อมูล'!$C$50</f>
         <v>3.348</v>
       </c>
       <c r="E23" s="13" t="n">
-        <f aca="false">(('7 แบบพับ'!$D$9+2*'1 ข้อมูล'!$C$48)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$48)+('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$9)*('3 ขนาดบ่อ'!$E$13+2*'1 ข้อมูล'!$C$48))*'1 ข้อมูล'!$C$49</f>
+        <f aca="false">(('7 แบบพับ'!$D$9+2*'1 ข้อมูล'!$C$49)*('7 แบบพับ'!$D$14+2*'1 ข้อมูล'!$C$49)+('7 แบบพับ'!$D$12-'7 แบบพับ'!$D$9)*('3 ขนาดบ่อ'!$E$13+2*'1 ข้อมูล'!$C$49))*'1 ข้อมูล'!$C$50</f>
         <v>3.348</v>
       </c>
       <c r="F23" s="6"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="6" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="C24" s="28" t="n">
         <f aca="false">SUM(C21:C23)</f>
-        <v>7.944</v>
+        <v>8.116</v>
       </c>
       <c r="D24" s="28" t="n">
         <f aca="false">SUM(D21:D23)</f>
@@ -6731,29 +6754,29 @@
         <v>7.896</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="6" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D25" s="30" t="n">
         <f aca="false">1-D18/C18</f>
-        <v>0.446428571428571</v>
+        <v>0.459302325581395</v>
       </c>
       <c r="E25" s="30" t="n">
         <f aca="false">1-E18/C18</f>
-        <v>0.446428571428571</v>
+        <v>0.459302325581395</v>
       </c>
       <c r="F25" s="6"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="4" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="C28" s="5"/>
       <c r="D28" s="5"/>
@@ -6762,10 +6785,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="31" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="D29" s="6"/>
       <c r="E29" s="6"/>
@@ -6773,10 +6796,10 @@
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="31" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="D30" s="6"/>
       <c r="E30" s="6"/>
@@ -6784,10 +6807,10 @@
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="31" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="D31" s="6"/>
       <c r="E31" s="6"/>
@@ -6795,10 +6818,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="31" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="D32" s="6"/>
       <c r="E32" s="6"/>
@@ -6806,10 +6829,10 @@
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="32" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="D33" s="6"/>
       <c r="E33" s="6"/>
@@ -6817,10 +6840,10 @@
     </row>
     <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="32" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="D34" s="6"/>
       <c r="E34" s="6"/>
@@ -6828,10 +6851,10 @@
     </row>
     <row r="35" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="32" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
       <c r="D35" s="6"/>
       <c r="E35" s="6"/>
@@ -6839,10 +6862,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="32" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="D36" s="6"/>
       <c r="E36" s="6"/>
@@ -6880,150 +6903,150 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="33" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="F5" s="24" t="n">
         <f aca="false">'1 ข้อมูล'!$C$10/3600</f>
         <v>0.0174421296296296</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="H5" s="13"/>
       <c r="I5" s="18"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="33" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="C6" s="6" t="s">
+        <v>500</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>501</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>497</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>498</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>494</v>
       </c>
       <c r="F6" s="24" t="n">
         <f aca="false">1.5*F5</f>
         <v>0.0261631944444444</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="H6" s="13"/>
       <c r="I6" s="18"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="33" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="F7" s="24" t="n">
         <f aca="false">'1 ข้อมูล'!$C$8/3600</f>
         <v>0.0277777777777778</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="H7" s="13"/>
       <c r="I7" s="18"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="33" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="E8" s="6"/>
       <c r="F8" s="24" t="n">
         <v>1</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="H8" s="13" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="I8" s="18"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="33" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="F9" s="24" t="n">
         <f aca="false">MAX(F6,F7)/F8</f>
         <v>0.0277777777777778</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
       <c r="H9" s="13" t="n">
         <f aca="false">'2 เวียร์'!$D$13</f>
@@ -7033,10 +7056,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="33" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="6" t="s">
@@ -7047,7 +7070,7 @@
         <v>0.458178826795053</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="H10" s="13" t="n">
         <f aca="false">('3 ขนาดบ่อ'!$E$13-'3 ขนาดบ่อ'!$E$10)/2</f>
@@ -7060,10 +7083,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="33" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="D11" s="6"/>
       <c r="E11" s="6" t="s">
@@ -7074,7 +7097,7 @@
         <v>0.416526206177321</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="H11" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$8</f>
@@ -7087,10 +7110,10 @@
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="33" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6" t="s">
@@ -7101,22 +7124,22 @@
         <v>0.208263103088661</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="H12" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$7</f>
         <v>0.209665688762588</v>
       </c>
       <c r="I12" s="18" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="33" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="6"/>
@@ -7133,10 +7156,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="33" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
@@ -7153,10 +7176,10 @@
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="33" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="6" t="s">
@@ -7167,7 +7190,7 @@
         <v>0.624789309265982</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="H15" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$15</f>
@@ -7180,10 +7203,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="33" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="D16" s="6"/>
       <c r="E16" s="6" t="s">
@@ -7194,7 +7217,7 @@
         <v>0.249915723706393</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="H16" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$9</f>
@@ -7207,10 +7230,10 @@
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="33" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="D17" s="6"/>
       <c r="E17" s="6" t="s">
@@ -7221,7 +7244,7 @@
         <v>1.41618910100289</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="H17" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$13</f>
@@ -7234,7 +7257,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="4" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5"/>
@@ -7246,17 +7269,17 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="23" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="23" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="23" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
     </row>
   </sheetData>
@@ -7286,17 +7309,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>3</v>
@@ -7307,12 +7330,12 @@
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
       <c r="G4" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="6" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="C5" s="16" t="n">
         <f aca="false">'1 ข้อมูล'!$C$28</f>
@@ -7324,12 +7347,12 @@
       <c r="E5" s="6"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="C6" s="34" t="n">
         <f aca="false">'1 ข้อมูล'!$C$10</f>
@@ -7341,12 +7364,12 @@
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="C7" s="10" t="n">
         <v>0.09</v>
@@ -7362,10 +7385,10 @@
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="C8" s="35" t="n">
-        <f aca="false">'3 ขนาดบ่อ'!$E$47+'4 ช่องโชว์น้ำ'!$F$6/100+1.5*'4 ช่องโชว์น้ำ'!$G$6^2/(2*'1 ข้อมูล'!$C$53)</f>
+        <f aca="false">'3 ขนาดบ่อ'!$E$47+'4 ช่องโชว์น้ำ'!$F$6/100+1.5*'4 ช่องโชว์น้ำ'!$G$6^2/(2*'1 ข้อมูล'!$C$54)</f>
         <v>0.953319742642753</v>
       </c>
       <c r="D8" s="6" t="s">
@@ -7374,12 +7397,12 @@
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
       <c r="G8" s="6" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="6" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">C6*C5/60+C7</f>
@@ -7391,12 +7414,12 @@
       <c r="E9" s="6"/>
       <c r="F9" s="6"/>
       <c r="G9" s="6" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
       <c r="C10" s="9" t="n">
         <f aca="false">('3 ขนาดบ่อ'!$E$62*'3 ขนาดบ่อ'!$E$13*C8-C7)/C6*60</f>
@@ -7408,12 +7431,12 @@
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>
       <c r="G10" s="6" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="4" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
@@ -7426,17 +7449,17 @@
         <v>2</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>4</v>
       </c>
       <c r="F13" s="3"/>
       <c r="G13" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7455,12 +7478,12 @@
       </c>
       <c r="F14" s="6"/>
       <c r="G14" s="6" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="6" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="C15" s="13" t="n">
         <f aca="false">'1 ข้อมูล'!$C$30</f>
@@ -7475,12 +7498,12 @@
       </c>
       <c r="F15" s="6"/>
       <c r="G15" s="6" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="C16" s="13" t="n">
         <f aca="false">$C$8-C14</f>
@@ -7495,12 +7518,12 @@
       </c>
       <c r="F16" s="6"/>
       <c r="G16" s="6" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="C17" s="13" t="n">
         <f aca="false">$C$9/(C15*C16)</f>
@@ -7515,12 +7538,12 @@
       </c>
       <c r="F17" s="6"/>
       <c r="G17" s="6" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="6" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="C18" s="28" t="n">
         <f aca="false">CEILING(ROUND(C17,4),'1 ข้อมูล'!$C$13)</f>
@@ -7535,12 +7558,12 @@
       </c>
       <c r="F18" s="6"/>
       <c r="G18" s="6" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="6" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="C19" s="9" t="n">
         <f aca="false">C18*C15*C16-$C$7</f>
@@ -7558,7 +7581,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="6" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="C20" s="20" t="n">
         <f aca="false">C19/$C$6*60</f>
@@ -7576,7 +7599,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="6" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="C21" s="18" t="str">
         <f aca="false">IF(C20&gt;=$C$5,"ผ่าน ✔","ไม่ผ่าน ✘")</f>
@@ -7592,7 +7615,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="6" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="C22" s="9" t="n">
         <f aca="false">C19/'1 ข้อมูล'!$C$8*60</f>
@@ -7607,12 +7630,12 @@
       </c>
       <c r="F22" s="6"/>
       <c r="G22" s="6" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="6" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="C23" s="16" t="n">
         <f aca="false">C18*C15*($C$8-(C14+0.6))/'1 ข้อมูล'!$C$9*60</f>
@@ -7627,12 +7650,12 @@
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="6" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="6" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="C24" s="13" t="n">
         <f aca="false">'3 ขนาดบ่อ'!$E$70-C14</f>
@@ -7647,39 +7670,39 @@
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="6" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="6" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
       <c r="C25" s="28" t="n">
-        <f aca="false">C18+'3 ขนาดบ่อ'!$E$49+'3 ขนาดบ่อ'!$E$109+2*'1 ข้อมูล'!$C$48</f>
-        <v>8.4</v>
+        <f aca="false">C18+'3 ขนาดบ่อ'!$E$49+'3 ขนาดบ่อ'!$E$109+2*'1 ข้อมูล'!$C$49</f>
+        <v>8.6</v>
       </c>
       <c r="D25" s="28" t="n">
-        <f aca="false">D18+'3 ขนาดบ่อ'!$E$49+'3 ขนาดบ่อ'!$E$109+2*'1 ข้อมูล'!$C$48</f>
-        <v>9.45</v>
+        <f aca="false">D18+'3 ขนาดบ่อ'!$E$49+'3 ขนาดบ่อ'!$E$109+2*'1 ข้อมูล'!$C$49</f>
+        <v>9.65</v>
       </c>
       <c r="E25" s="6" t="s">
         <v>19</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="6" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="6" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="C26" s="6" t="str">
-        <f aca="false">TEXT(C15+2*'1 ข้อมูล'!$C$48,"0.00")&amp;" / "&amp;TEXT('3 ขนาดบ่อ'!$E$13+2*'1 ข้อมูล'!$C$48,"0.00")</f>
+        <f aca="false">TEXT(C15+2*'1 ข้อมูล'!$C$49,"0.00")&amp;" / "&amp;TEXT('3 ขนาดบ่อ'!$E$13+2*'1 ข้อมูล'!$C$49,"0.00")</f>
         <v>2.90 / 1.90</v>
       </c>
       <c r="D26" s="6" t="str">
-        <f aca="false">TEXT(D15+2*'1 ข้อมูล'!$C$48,"0.00")&amp;" / "&amp;TEXT('3 ขนาดบ่อ'!$E$13+2*'1 ข้อมูล'!$C$48,"0.00")</f>
+        <f aca="false">TEXT(D15+2*'1 ข้อมูล'!$C$49,"0.00")&amp;" / "&amp;TEXT('3 ขนาดบ่อ'!$E$13+2*'1 ข้อมูล'!$C$49,"0.00")</f>
         <v>1.90 / 1.90</v>
       </c>
       <c r="E26" s="6" t="s">
@@ -7690,7 +7713,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="4" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="C28" s="5"/>
       <c r="D28" s="5"/>
@@ -7700,7 +7723,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="3" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="C29" s="3" t="n">
         <v>1.5</v>
@@ -7715,7 +7738,7 @@
         <v>3</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7845,17 +7868,17 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="23" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="23" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="23" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
     </row>
   </sheetData>

</xml_diff>